<commit_message>
test(tenancy): TSC-9 mark RED describe blocks as todo for CI non-blocking execution
</commit_message>
<xml_diff>
--- a/.agents/coral-roadmap.xlsx
+++ b/.agents/coral-roadmap.xlsx
@@ -594,7 +594,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I492"/>
+  <dimension ref="A1:I500"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -22266,6 +22266,382 @@
       <c r="I492" t="inlineStr">
         <is>
           <t>Identity</t>
+        </is>
+      </c>
+    </row>
+    <row r="493">
+      <c r="A493" t="inlineStr">
+        <is>
+          <t>KERN-6</t>
+        </is>
+      </c>
+      <c r="B493" t="inlineStr">
+        <is>
+          <t>PASS 3a: one SYSTEM_DATABASES table; the other four lists become derived</t>
+        </is>
+      </c>
+      <c r="C493" t="inlineStr">
+        <is>
+          <t>Kernel</t>
+        </is>
+      </c>
+      <c r="D493" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E493" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F493" t="inlineStr">
+        <is>
+          <t>coral-id-parsing-decomposition.md</t>
+        </is>
+      </c>
+      <c r="G493" t="inlineStr">
+        <is>
+          <t>Five lists, five lengths: 16/16/14/8/6. Not five bugs — one missing table with columns (role, legacyBase, displayName, module).</t>
+        </is>
+      </c>
+      <c r="H493" t="inlineStr">
+        <is>
+          <t>L0 Kernel</t>
+        </is>
+      </c>
+      <c r="I493" t="inlineStr">
+        <is>
+          <t>Identity</t>
+        </is>
+      </c>
+    </row>
+    <row r="494">
+      <c r="A494" t="inlineStr">
+        <is>
+          <t>KERN-6a</t>
+        </is>
+      </c>
+      <c r="B494" t="inlineStr">
+        <is>
+          <t>LIVE: SYSTEM_DB_PREFIXES omits journal-general and hr (14 of 16)</t>
+        </is>
+      </c>
+      <c r="C494" t="inlineStr">
+        <is>
+          <t>Kernel</t>
+        </is>
+      </c>
+      <c r="D494" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E494" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F494" t="inlineStr">
+        <is>
+          <t>coral-id-parsing-decomposition.md</t>
+        </is>
+      </c>
+      <c r="G494" t="inlineStr">
+        <is>
+          <t>isSystemDatabase('db-hr') === false -&gt; createPageServerFirst does not resolve them through the book; requiredModuleForDb does not gate them.</t>
+        </is>
+      </c>
+      <c r="H494" t="inlineStr">
+        <is>
+          <t>L0 Kernel</t>
+        </is>
+      </c>
+      <c r="I494" t="inlineStr">
+        <is>
+          <t>Identity</t>
+        </is>
+      </c>
+    </row>
+    <row r="495">
+      <c r="A495" t="inlineStr">
+        <is>
+          <t>KERN-6b</t>
+        </is>
+      </c>
+      <c r="B495" t="inlineStr">
+        <is>
+          <t>SERVER_PROVISIONED_BASES (8) now disagrees with reality — pass 1 provisions 16</t>
+        </is>
+      </c>
+      <c r="C495" t="inlineStr">
+        <is>
+          <t>Kernel</t>
+        </is>
+      </c>
+      <c r="D495" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E495" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F495" t="inlineStr">
+        <is>
+          <t>coral-id-parsing-decomposition.md</t>
+        </is>
+      </c>
+      <c r="G495" t="inlineStr">
+        <is>
+          <t>Stale Set left behind by pass 1.</t>
+        </is>
+      </c>
+      <c r="H495" t="inlineStr">
+        <is>
+          <t>L0 Kernel</t>
+        </is>
+      </c>
+      <c r="I495" t="inlineStr">
+        <is>
+          <t>Identity</t>
+        </is>
+      </c>
+    </row>
+    <row r="496">
+      <c r="A496" t="inlineStr">
+        <is>
+          <t>KERN-6c</t>
+        </is>
+      </c>
+      <c r="B496" t="inlineStr">
+        <is>
+          <t>ENTITLEMENT decided by prefix-match: requiredModuleForDb (pages.ts:26)</t>
+        </is>
+      </c>
+      <c r="C496" t="inlineStr">
+        <is>
+          <t>Kernel</t>
+        </is>
+      </c>
+      <c r="D496" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E496" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F496" t="inlineStr">
+        <is>
+          <t>coral-id-parsing-decomposition.md</t>
+        </is>
+      </c>
+      <c r="G496" t="inlineStr">
+        <is>
+          <t>A permission decision made by string comparison. AUTHORITY DIRECTIVE — authority is never inferred from a substring. The careful batch (3b-2).</t>
+        </is>
+      </c>
+      <c r="H496" t="inlineStr">
+        <is>
+          <t>L1 Core</t>
+        </is>
+      </c>
+      <c r="I496" t="inlineStr">
+        <is>
+          <t>Entitlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="497">
+      <c r="A497" t="inlineStr">
+        <is>
+          <t>KERN-7</t>
+        </is>
+      </c>
+      <c r="B497" t="inlineStr">
+        <is>
+          <t>PASS 3b: ESLint parse ratchet — 28 files grandfathered, length is the metric</t>
+        </is>
+      </c>
+      <c r="C497" t="inlineStr">
+        <is>
+          <t>Kernel</t>
+        </is>
+      </c>
+      <c r="D497" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E497" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F497" t="inlineStr">
+        <is>
+          <t>coral-id-parsing-decomposition.md</t>
+        </is>
+      </c>
+      <c r="G497" t="inlineStr">
+        <is>
+          <t>74 parse sites across 28 files. Same mechanism as PRE-1d's prisma allowlist (121).</t>
+        </is>
+      </c>
+      <c r="H497" t="inlineStr">
+        <is>
+          <t>L0 Kernel</t>
+        </is>
+      </c>
+      <c r="I497" t="inlineStr">
+        <is>
+          <t>Identity</t>
+        </is>
+      </c>
+    </row>
+    <row r="498">
+      <c r="A498" t="inlineStr">
+        <is>
+          <t>KERN-8</t>
+        </is>
+      </c>
+      <c r="B498" t="inlineStr">
+        <is>
+          <t>PASS 3c: delete getLockedDbId + lockedDbUtils + resolve.ts prefix searches</t>
+        </is>
+      </c>
+      <c r="C498" t="inlineStr">
+        <is>
+          <t>Kernel</t>
+        </is>
+      </c>
+      <c r="D498" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E498" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F498" t="inlineStr">
+        <is>
+          <t>coral-id-parsing-decomposition.md</t>
+        </is>
+      </c>
+      <c r="G498" t="inlineStr">
+        <is>
+          <t>Only when 3b's allowlist reaches zero. Gated on the R1-1b relation-target measurement.</t>
+        </is>
+      </c>
+      <c r="H498" t="inlineStr">
+        <is>
+          <t>L0 Kernel</t>
+        </is>
+      </c>
+      <c r="I498" t="inlineStr">
+        <is>
+          <t>Identity</t>
+        </is>
+      </c>
+    </row>
+    <row r="499">
+      <c r="A499" t="inlineStr">
+        <is>
+          <t>R1-1b-M</t>
+        </is>
+      </c>
+      <c r="B499" t="inlineStr">
+        <is>
+          <t>MEASURE: relation properties whose targetDatabaseId is a legacy base id</t>
+        </is>
+      </c>
+      <c r="C499" t="inlineStr">
+        <is>
+          <t>Tenancy (R1)</t>
+        </is>
+      </c>
+      <c r="D499" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E499" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F499" t="inlineStr">
+        <is>
+          <t>coral-id-parsing-decomposition.md</t>
+        </is>
+      </c>
+      <c r="G499" t="inlineStr">
+        <is>
+          <t>Florin, production, read-only. resolve.ts:94 proves stored relation targets may hold base ids. Decides whether logicalKey is a backfill or a no-op. Gates pass 3c.</t>
+        </is>
+      </c>
+      <c r="H499" t="inlineStr">
+        <is>
+          <t>L1 Core</t>
+        </is>
+      </c>
+      <c r="I499" t="inlineStr">
+        <is>
+          <t>Relations</t>
+        </is>
+      </c>
+    </row>
+    <row r="500">
+      <c r="A500" t="inlineStr">
+        <is>
+          <t>PLAN-2</t>
+        </is>
+      </c>
+      <c r="B500" t="inlineStr">
+        <is>
+          <t>Planner verified 'one array' by grepping its own three names, not the concept</t>
+        </is>
+      </c>
+      <c r="C500" t="inlineStr">
+        <is>
+          <t>Process</t>
+        </is>
+      </c>
+      <c r="D500" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E500" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F500" t="inlineStr">
+        <is>
+          <t>coral-id-parsing-decomposition.md</t>
+        </is>
+      </c>
+      <c r="G500" t="inlineStr">
+        <is>
+          <t>Missed SYSTEM_DB_PREFIXES, SERVER_PROVISIONED_BASES and DB_ID_MODULE_MAP in the pass-1 check. Verify the claim, not the wording of the claim.</t>
+        </is>
+      </c>
+      <c r="H500" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I500" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(kernel): KERN-6 pass 3a - SYSTEM_DATABASES canonical spec table with four derived lists
</commit_message>
<xml_diff>
--- a/.agents/coral-roadmap.xlsx
+++ b/.agents/coral-roadmap.xlsx
@@ -594,7 +594,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I500"/>
+  <dimension ref="A1:I504"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -10345,7 +10345,7 @@
       </c>
       <c r="G225" s="11" t="inlineStr">
         <is>
-          <t>[P3.2] Backfill source: getBaseDbId(id) — exact, already exists</t>
+          <t>CLARIFIED 2026-09-26: logicalKey is the REVERSE binding. Tenant.lockedDbIds answers role-&gt;id; NOTHING answers id-&gt;role, so every reverse-lookup site parses the id. That is the root of all 74 parse sites. Backfill from lockedDbIds (authoritative) — NEVER by parsing ids. @@unique([tenantId, logicalKey]). Moves EARLIER: it is the storage pass 3b spends.</t>
         </is>
       </c>
       <c r="H225" s="28" t="inlineStr">
@@ -12158,7 +12158,7 @@
       </c>
       <c r="G264" s="11" t="inlineStr">
         <is>
-          <t>[P3.1] NEW FINDING 2026-09-12</t>
+          <t>SAME TASK AS KERN-6 / pass 3a. Planner rediscovered this independently on 2026-09-25 and wrote it up as new (KERN-6a). Tonight's version is wider: five lists, 74 parse sites.</t>
         </is>
       </c>
       <c r="H264" s="28" t="inlineStr">
@@ -22574,7 +22574,7 @@
       </c>
       <c r="E499" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F499" t="inlineStr">
@@ -22584,7 +22584,7 @@
       </c>
       <c r="G499" t="inlineStr">
         <is>
-          <t>Florin, production, read-only. resolve.ts:94 proves stored relation targets may hold base ids. Decides whether logicalKey is a backfill or a no-op. Gates pass 3c.</t>
+          <t>MEASURED 2026-09-26 prod: 36 resolve, 3 LEGACY ALIAS, 0 CROSS-TENANT. R1-1b is 3 JSON edits, not 9,226 pages. Planner's spec had the wrong JSON key (targetDatabaseId); real key is config.relationDatabaseId — the wrong query would have returned 0 rows as a false all-clear.</t>
         </is>
       </c>
       <c r="H499" t="inlineStr">
@@ -22640,6 +22640,194 @@
         </is>
       </c>
       <c r="I500" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="501">
+      <c r="A501" t="inlineStr">
+        <is>
+          <t>R1-1b-R1</t>
+        </is>
+      </c>
+      <c r="B501" t="inlineStr">
+        <is>
+          <t>REPAIR (Florin, UI): BV CORAL Projects -&gt; 'Klant' points at bare db-clients</t>
+        </is>
+      </c>
+      <c r="C501" t="inlineStr">
+        <is>
+          <t>Tenancy (R1)</t>
+        </is>
+      </c>
+      <c r="D501" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="E501" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F501" t="inlineStr">
+        <is>
+          <t>coral-id-parsing-decomposition.md</t>
+        </is>
+      </c>
+      <c r="G501" t="inlineStr">
+        <is>
+          <t>Fix via Settings &gt; Databases &gt; Projects &gt; Klant &gt; re-pick Contacts. No SQL, no snapshot — the normal path writes the bound id.</t>
+        </is>
+      </c>
+      <c r="H501" t="inlineStr">
+        <is>
+          <t>L1 Core</t>
+        </is>
+      </c>
+      <c r="I501" t="inlineStr">
+        <is>
+          <t>Relations</t>
+        </is>
+      </c>
+    </row>
+    <row r="502">
+      <c r="A502" t="inlineStr">
+        <is>
+          <t>R1-1b-R2</t>
+        </is>
+      </c>
+      <c r="B502" t="inlineStr">
+        <is>
+          <t>REPAIR (code, R1-1b): Murgu's 2 invoice dbs -&gt; 'Project' points at fabricated db-1-cmoa44mj</t>
+        </is>
+      </c>
+      <c r="C502" t="inlineStr">
+        <is>
+          <t>Tenancy (R1)</t>
+        </is>
+      </c>
+      <c r="D502" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E502" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F502" t="inlineStr">
+        <is>
+          <t>coral-id-parsing-decomposition.md</t>
+        </is>
+      </c>
+      <c r="G502" t="inlineStr">
+        <is>
+          <t>Proof the getLockedDbId suffix-synthesis branch fired in production AND persisted. Repoint to the tenant's real projects binding via reviewed code, not hand-edited JSON.</t>
+        </is>
+      </c>
+      <c r="H502" t="inlineStr">
+        <is>
+          <t>L1 Core</t>
+        </is>
+      </c>
+      <c r="I502" t="inlineStr">
+        <is>
+          <t>Relations</t>
+        </is>
+      </c>
+    </row>
+    <row r="503">
+      <c r="A503" t="inlineStr">
+        <is>
+          <t>KERN-9</t>
+        </is>
+      </c>
+      <c r="B503" t="inlineStr">
+        <is>
+          <t>'db-' is NOT a reliable database-id marker — it occurs inside random UUIDs</t>
+        </is>
+      </c>
+      <c r="C503" t="inlineStr">
+        <is>
+          <t>Kernel</t>
+        </is>
+      </c>
+      <c r="D503" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E503" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F503" t="inlineStr">
+        <is>
+          <t>coral-id-parsing-decomposition.md</t>
+        </is>
+      </c>
+      <c r="G503" t="inlineStr">
+        <is>
+          <t>Property/view UUIDs like 1b1dd3d1-94ee-4cdb-a8b9-... contain 'db-'. No lint rule, helper or migration in pass 3b may detect a database id by pattern. The binding is the only answer.</t>
+        </is>
+      </c>
+      <c r="H503" t="inlineStr">
+        <is>
+          <t>L0 Kernel</t>
+        </is>
+      </c>
+      <c r="I503" t="inlineStr">
+        <is>
+          <t>Identity</t>
+        </is>
+      </c>
+    </row>
+    <row r="504">
+      <c r="A504" t="inlineStr">
+        <is>
+          <t>PLAN-3</t>
+        </is>
+      </c>
+      <c r="B504" t="inlineStr">
+        <is>
+          <t>Planner produced 4 false findings from a regex matching 'db-' inside UUIDs</t>
+        </is>
+      </c>
+      <c r="C504" t="inlineStr">
+        <is>
+          <t>Process</t>
+        </is>
+      </c>
+      <c r="D504" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E504" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F504" t="inlineStr">
+        <is>
+          <t>coral-id-parsing-decomposition.md</t>
+        </is>
+      </c>
+      <c r="G504" t="inlineStr">
+        <is>
+          <t>Third measurement error on one question: wrong JSON key (targetDatabaseId), then properties-only scope, then a regex manufacturing matches. Real damage was 3 rows, not 7.</t>
+        </is>
+      </c>
+      <c r="H504" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I504" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
fix(workhub): bridge time-tracker AuthContext signOut to next-auth with local cache wipe
</commit_message>
<xml_diff>
--- a/.agents/coral-roadmap.xlsx
+++ b/.agents/coral-roadmap.xlsx
@@ -594,7 +594,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I504"/>
+  <dimension ref="A1:I534"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -22443,7 +22443,7 @@
       </c>
       <c r="G496" t="inlineStr">
         <is>
-          <t>A permission decision made by string comparison. AUTHORITY DIRECTIVE — authority is never inferred from a substring. The careful batch (3b-2).</t>
+          <t>A permission decision made by string comparison. AUTHORITY DIRECTIVE — authority is never inferred from a substring. The careful batch (3b-2). | WIDER THAN LABELLED: not just how the gate reads an id — there are FOUR gates and no module vocabulary. Superseded by ENT-1..5.</t>
         </is>
       </c>
       <c r="H496" t="inlineStr">
@@ -22830,6 +22830,1416 @@
       <c r="I504" t="inlineStr">
         <is>
           <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="505">
+      <c r="A505" t="inlineStr">
+        <is>
+          <t>ENT-3</t>
+        </is>
+      </c>
+      <c r="B505" t="inlineStr">
+        <is>
+          <t>SERAPH: scope.may(module) — one reader, reads the DB, JWT is a hint not a gate</t>
+        </is>
+      </c>
+      <c r="C505" t="inlineStr">
+        <is>
+          <t>Entitlement</t>
+        </is>
+      </c>
+      <c r="D505" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E505" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F505" t="inlineStr">
+        <is>
+          <t>coral-walkdown-entitlement.md</t>
+        </is>
+      </c>
+      <c r="G505" t="inlineStr">
+        <is>
+          <t>LEAK: middleware gates on the JWT, moduleGuard reads the DB to avoid the stale-token window. Revoking a module leaves route access open until token expiry. Revenue leak on free-tier-per-prospect.</t>
+        </is>
+      </c>
+      <c r="H505" t="inlineStr">
+        <is>
+          <t>L1 Core</t>
+        </is>
+      </c>
+      <c r="I505" t="inlineStr">
+        <is>
+          <t>Tenant gate</t>
+        </is>
+      </c>
+    </row>
+    <row r="506">
+      <c r="A506" t="inlineStr">
+        <is>
+          <t>ENT-4</t>
+        </is>
+      </c>
+      <c r="B506" t="inlineStr">
+        <is>
+          <t>CORE: requireModule() — one primitive; superadmin bypass lives here ONCE</t>
+        </is>
+      </c>
+      <c r="C506" t="inlineStr">
+        <is>
+          <t>Entitlement</t>
+        </is>
+      </c>
+      <c r="D506" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E506" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F506" t="inlineStr">
+        <is>
+          <t>coral-walkdown-entitlement.md</t>
+        </is>
+      </c>
+      <c r="G506" t="inlineStr">
+        <is>
+          <t>Bypass is currently re-implemented in middleware, moduleGuard and pages.ts — three copies of a privilege escalation.</t>
+        </is>
+      </c>
+      <c r="H506" t="inlineStr">
+        <is>
+          <t>L1 Core</t>
+        </is>
+      </c>
+      <c r="I506" t="inlineStr">
+        <is>
+          <t>Entitlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="507">
+      <c r="A507" t="inlineStr">
+        <is>
+          <t>ENT-5</t>
+        </is>
+      </c>
+      <c r="B507" t="inlineStr">
+        <is>
+          <t>Gate the CRM pipeline (Florin 2026-09-26: 'there's business logic behind this')</t>
+        </is>
+      </c>
+      <c r="C507" t="inlineStr">
+        <is>
+          <t>Entitlement</t>
+        </is>
+      </c>
+      <c r="D507" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E507" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F507" t="inlineStr">
+        <is>
+          <t>coral-walkdown-entitlement.md</t>
+        </is>
+      </c>
+      <c r="G507" t="inlineStr">
+        <is>
+          <t>UNBLOCKED: BV CORAL holds CRM, so gating the pipeline does not lock Florin out.</t>
+        </is>
+      </c>
+      <c r="H507" t="inlineStr">
+        <is>
+          <t>L2 Module</t>
+        </is>
+      </c>
+      <c r="I507" t="inlineStr">
+        <is>
+          <t>CRM</t>
+        </is>
+      </c>
+    </row>
+    <row r="508">
+      <c r="A508" t="inlineStr">
+        <is>
+          <t>ENT-0</t>
+        </is>
+      </c>
+      <c r="B508" t="inlineStr">
+        <is>
+          <t>CENSUS: activeModules + planType per tenant (Florin, read-only)</t>
+        </is>
+      </c>
+      <c r="C508" t="inlineStr">
+        <is>
+          <t>Entitlement</t>
+        </is>
+      </c>
+      <c r="D508" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E508" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F508" t="inlineStr">
+        <is>
+          <t>coral-walkdown-entitlement.md</t>
+        </is>
+      </c>
+      <c r="G508" t="inlineStr">
+        <is>
+          <t>MEASURED 2026-09-26: BV CORAL = ENTERPRISE, 9 modules incl CRM (gating the pipeline is SAFE). Murgu = FREE, INVOICING only.</t>
+        </is>
+      </c>
+      <c r="H508" t="inlineStr">
+        <is>
+          <t>L1 Core</t>
+        </is>
+      </c>
+      <c r="I508" t="inlineStr">
+        <is>
+          <t>Entitlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="509">
+      <c r="A509" t="inlineStr">
+        <is>
+          <t>ENT-6</t>
+        </is>
+      </c>
+      <c r="B509" t="inlineStr">
+        <is>
+          <t>🔴 FREE tenant can CREATE in 14 of 16 system databases — 8 roles have no gate</t>
+        </is>
+      </c>
+      <c r="C509" t="inlineStr">
+        <is>
+          <t>Entitlement</t>
+        </is>
+      </c>
+      <c r="D509" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E509" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F509" t="inlineStr">
+        <is>
+          <t>coral-walkdown-entitlement.md</t>
+        </is>
+      </c>
+      <c r="G509" t="inlineStr">
+        <is>
+          <t>Murgu (FREE, INVOICING only) has write access to projects, tasks, articles, crm, bobex, bestek, journal-general, hr. Not a decision anyone made — absence of a gate read as permission.</t>
+        </is>
+      </c>
+      <c r="H509" t="inlineStr">
+        <is>
+          <t>L1 Core</t>
+        </is>
+      </c>
+      <c r="I509" t="inlineStr">
+        <is>
+          <t>Entitlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="510">
+      <c r="A510" t="inlineStr">
+        <is>
+          <t>ENT-7</t>
+        </is>
+      </c>
+      <c r="B510" t="inlineStr">
+        <is>
+          <t>🔴 FREE tenant CANNOT create a client — 'clients' is gated on CRM, FREE grants only INVOICING</t>
+        </is>
+      </c>
+      <c r="C510" t="inlineStr">
+        <is>
+          <t>Entitlement</t>
+        </is>
+      </c>
+      <c r="D510" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E510" t="inlineStr">
+        <is>
+          <t>Resolved by design</t>
+        </is>
+      </c>
+      <c r="F510" t="inlineStr">
+        <is>
+          <t>coral-walkdown-entitlement.md</t>
+        </is>
+      </c>
+      <c r="G510" t="inlineStr">
+        <is>
+          <t>An invoice needs a customer. A free-tier prospect can invoice but cannot create the client to invoice. Breaks the free-tier-per-prospect acquisition model at the first step. FLORIN: is clients an INVOICING database or a CRM one? | RESOLVED by ENT-10/11: clients need not move to INVOICING, and CRM need not be granted whole. FREE gets CRM:['clients']. Exactly what the submodule level is for.</t>
+        </is>
+      </c>
+      <c r="H510" t="inlineStr">
+        <is>
+          <t>L2 Module</t>
+        </is>
+      </c>
+      <c r="I510" t="inlineStr">
+        <is>
+          <t>Invoicing</t>
+        </is>
+      </c>
+    </row>
+    <row r="511">
+      <c r="A511" t="inlineStr">
+        <is>
+          <t>ENT-8</t>
+        </is>
+      </c>
+      <c r="B511" t="inlineStr">
+        <is>
+          <t>WEBSITES and EMAIL are granted to BV CORAL but ungrantable via the settings UI</t>
+        </is>
+      </c>
+      <c r="C511" t="inlineStr">
+        <is>
+          <t>Entitlement</t>
+        </is>
+      </c>
+      <c r="D511" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E511" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F511" t="inlineStr">
+        <is>
+          <t>coral-walkdown-entitlement.md</t>
+        </is>
+      </c>
+      <c r="G511" t="inlineStr">
+        <is>
+          <t>A one-way door: present in data, cannot be re-granted if ever removed. MODULES (7) omits both.</t>
+        </is>
+      </c>
+      <c r="H511" t="inlineStr">
+        <is>
+          <t>L1 Core</t>
+        </is>
+      </c>
+      <c r="I511" t="inlineStr">
+        <is>
+          <t>Entitlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="512">
+      <c r="A512" t="inlineStr">
+        <is>
+          <t>ENT-9</t>
+        </is>
+      </c>
+      <c r="B512" t="inlineStr">
+        <is>
+          <t>Superadmin bypass re-implemented in middleware.ts, moduleGuard.ts, pages.ts</t>
+        </is>
+      </c>
+      <c r="C512" t="inlineStr">
+        <is>
+          <t>Entitlement</t>
+        </is>
+      </c>
+      <c r="D512" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E512" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F512" t="inlineStr">
+        <is>
+          <t>coral-walkdown-entitlement.md</t>
+        </is>
+      </c>
+      <c r="G512" t="inlineStr">
+        <is>
+          <t>pd.md directive 5a (Florin 2026-09-26): a component must not decide its own privilege. Three copies of a privilege escalation. Collapses into requireModule().</t>
+        </is>
+      </c>
+      <c r="H512" t="inlineStr">
+        <is>
+          <t>L1 Core</t>
+        </is>
+      </c>
+      <c r="I512" t="inlineStr">
+        <is>
+          <t>Entitlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="513">
+      <c r="A513" t="inlineStr">
+        <is>
+          <t>ENT-10</t>
+        </is>
+      </c>
+      <c r="B513" t="inlineStr">
+        <is>
+          <t>SUBMODULE level: Tenant.entitlements Json replaces flat activeModules</t>
+        </is>
+      </c>
+      <c r="C513" t="inlineStr">
+        <is>
+          <t>Entitlement</t>
+        </is>
+      </c>
+      <c r="D513" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E513" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F513" t="inlineStr">
+        <is>
+          <t>coral-submodule-entitlement.md</t>
+        </is>
+      </c>
+      <c r="G513" t="inlineStr">
+        <is>
+          <t>Florin 2026-09-26. One field, not two: a module granted with zero submodules becomes UNREPRESENTABLE rather than merely invalid. activeModules survives as derived, then drops.</t>
+        </is>
+      </c>
+      <c r="H513" t="inlineStr">
+        <is>
+          <t>L0 Kernel</t>
+        </is>
+      </c>
+      <c r="I513" t="inlineStr">
+        <is>
+          <t>Entitlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="514">
+      <c r="A514" t="inlineStr">
+        <is>
+          <t>ENT-11</t>
+        </is>
+      </c>
+      <c r="B514" t="inlineStr">
+        <is>
+          <t>Routes and dbRoles attach to SUBMODULES, not modules</t>
+        </is>
+      </c>
+      <c r="C514" t="inlineStr">
+        <is>
+          <t>Entitlement</t>
+        </is>
+      </c>
+      <c r="D514" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E514" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F514" t="inlineStr">
+        <is>
+          <t>coral-submodule-entitlement.md</t>
+        </is>
+      </c>
+      <c r="G514" t="inlineStr">
+        <is>
+          <t>The gate gets finer because the map does. A submodule IS a sidebar entry — if it is not in the nav it is not a submodule. That bound stops this becoming a permission system.</t>
+        </is>
+      </c>
+      <c r="H514" t="inlineStr">
+        <is>
+          <t>L0 Kernel</t>
+        </is>
+      </c>
+      <c r="I514" t="inlineStr">
+        <is>
+          <t>Entitlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="515">
+      <c r="A515" t="inlineStr">
+        <is>
+          <t>ENT-12</t>
+        </is>
+      </c>
+      <c r="B515" t="inlineStr">
+        <is>
+          <t>TIER_DEFAULTS: planType is a TEMPLATE, never a gate</t>
+        </is>
+      </c>
+      <c r="C515" t="inlineStr">
+        <is>
+          <t>Entitlement</t>
+        </is>
+      </c>
+      <c r="D515" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E515" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F515" t="inlineStr">
+        <is>
+          <t>coral-submodule-entitlement.md</t>
+        </is>
+      </c>
+      <c r="G515" t="inlineStr">
+        <is>
+          <t>planType decides what a tenant is GIVEN; entitlements decide what it MAY USE. No gate reads planType (pd.md 5a). Entitlements may exceed the tier default — Florin grants, nothing recomputes behind him.</t>
+        </is>
+      </c>
+      <c r="H515" t="inlineStr">
+        <is>
+          <t>L0 Kernel</t>
+        </is>
+      </c>
+      <c r="I515" t="inlineStr">
+        <is>
+          <t>Entitlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="516">
+      <c r="A516" t="inlineStr">
+        <is>
+          <t>ENT-13</t>
+        </is>
+      </c>
+      <c r="B516" t="inlineStr">
+        <is>
+          <t>Sidebar renders from the grant — empty links impossible by construction</t>
+        </is>
+      </c>
+      <c r="C516" t="inlineStr">
+        <is>
+          <t>Entitlement</t>
+        </is>
+      </c>
+      <c r="D516" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E516" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F516" t="inlineStr">
+        <is>
+          <t>coral-submodule-entitlement.md</t>
+        </is>
+      </c>
+      <c r="G516" t="inlineStr">
+        <is>
+          <t>Module link iff &gt;=1 granted submodule. Florin's stated reason for the minimum-one invariant.</t>
+        </is>
+      </c>
+      <c r="H516" t="inlineStr">
+        <is>
+          <t>L2 Module</t>
+        </is>
+      </c>
+      <c r="I516" t="inlineStr">
+        <is>
+          <t>Navigation</t>
+        </is>
+      </c>
+    </row>
+    <row r="517">
+      <c r="A517" t="inlineStr">
+        <is>
+          <t>ENT-14</t>
+        </is>
+      </c>
+      <c r="B517" t="inlineStr">
+        <is>
+          <t>MIGRATION: backfill entitlements from activeModules x TIER_DEFAULTS, nobody loses access</t>
+        </is>
+      </c>
+      <c r="C517" t="inlineStr">
+        <is>
+          <t>Entitlement</t>
+        </is>
+      </c>
+      <c r="D517" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E517" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F517" t="inlineStr">
+        <is>
+          <t>coral-submodule-entitlement.md</t>
+        </is>
+      </c>
+      <c r="G517" t="inlineStr">
+        <is>
+          <t>Existing tenants default to ALL submodules of each granted module. BV CORAL's reachable surface must be byte-identical after backfill. Additive nullable column first.</t>
+        </is>
+      </c>
+      <c r="H517" t="inlineStr">
+        <is>
+          <t>L0 Kernel</t>
+        </is>
+      </c>
+      <c r="I517" t="inlineStr">
+        <is>
+          <t>Entitlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="518">
+      <c r="A518" t="inlineStr">
+        <is>
+          <t>ENT-15</t>
+        </is>
+      </c>
+      <c r="B518" t="inlineStr">
+        <is>
+          <t>QUOTA is the second axis of entitlement — KEEP AND IMPLEMENT (Florin 2026-09-26)</t>
+        </is>
+      </c>
+      <c r="C518" t="inlineStr">
+        <is>
+          <t>Entitlement</t>
+        </is>
+      </c>
+      <c r="D518" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E518" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F518" t="inlineStr">
+        <is>
+          <t>coral-submodule-entitlement.md</t>
+        </is>
+      </c>
+      <c r="G518" t="inlineStr">
+        <is>
+          <t>Reach (submodule grant, yes/no) and Quota (a number, checked at the action) fail differently: no reach = the door is not there; over quota = the door says not this month. Matrix has 5/mo invoices, 20 projects, 2 employees, 5GB, 1 pipeline.</t>
+        </is>
+      </c>
+      <c r="H518" t="inlineStr">
+        <is>
+          <t>L0 Kernel</t>
+        </is>
+      </c>
+      <c r="I518" t="inlineStr">
+        <is>
+          <t>Entitlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="519">
+      <c r="A519" t="inlineStr">
+        <is>
+          <t>ENT-16</t>
+        </is>
+      </c>
+      <c r="B519" t="inlineStr">
+        <is>
+          <t>FOUR tiers after FOUNDER removal: FREE / PRO / ENTERPRISE / CUSTOM</t>
+        </is>
+      </c>
+      <c r="C519" t="inlineStr">
+        <is>
+          <t>Entitlement</t>
+        </is>
+      </c>
+      <c r="D519" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E519" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F519" t="inlineStr">
+        <is>
+          <t>coral-submodule-entitlement.md</t>
+        </is>
+      </c>
+      <c r="G519" t="inlineStr">
+        <is>
+          <t>Plan vocabularies disagree FOUR ways: PLAN_LIMITS (4), PLAN_PRICING (3, no FREE), PLAN_SCAN_QUOTAS (5), Tenant.planType default FREE.</t>
+        </is>
+      </c>
+      <c r="H519" t="inlineStr">
+        <is>
+          <t>L0 Kernel</t>
+        </is>
+      </c>
+      <c r="I519" t="inlineStr">
+        <is>
+          <t>Entitlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="520">
+      <c r="A520" t="inlineStr">
+        <is>
+          <t>ENT-17</t>
+        </is>
+      </c>
+      <c r="B520" t="inlineStr">
+        <is>
+          <t>Roles encode the tier: TENANT_FREE / TENANT_PRO_OWNER / TENANT_ENTERPRISE_*</t>
+        </is>
+      </c>
+      <c r="C520" t="inlineStr">
+        <is>
+          <t>Entitlement</t>
+        </is>
+      </c>
+      <c r="D520" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E520" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F520" t="inlineStr">
+        <is>
+          <t>coral-submodule-entitlement.md</t>
+        </is>
+      </c>
+      <c r="G520" t="inlineStr">
+        <is>
+          <t>Plan baked into identity — authority asserted rather than asked (pd.md AUTHORITY + 5a). A role should say what someone does, not what plan they are on. User-count limits currently ride on the role name.</t>
+        </is>
+      </c>
+      <c r="H520" t="inlineStr">
+        <is>
+          <t>L1 Core</t>
+        </is>
+      </c>
+      <c r="I520" t="inlineStr">
+        <is>
+          <t>Entitlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="521">
+      <c r="A521" t="inlineStr">
+        <is>
+          <t>ENT-18</t>
+        </is>
+      </c>
+      <c r="B521" t="inlineStr">
+        <is>
+          <t>7 of 10 April implementation gaps still open — every one is a feature reaching a tier that should not have it</t>
+        </is>
+      </c>
+      <c r="C521" t="inlineStr">
+        <is>
+          <t>Entitlement</t>
+        </is>
+      </c>
+      <c r="D521" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E521" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F521" t="inlineStr">
+        <is>
+          <t>coral-submodule-entitlement.md</t>
+        </is>
+      </c>
+      <c r="G521" t="inlineStr">
+        <is>
+          <t>Bestek+Library on FREE, Sales on FREE, Email on PRO, File manager on PRO, TASKS module key missing, 1-pipeline cap unenforced. Same defect as ENT-6 measured independently in Sept.</t>
+        </is>
+      </c>
+      <c r="H521" t="inlineStr">
+        <is>
+          <t>L2 Module</t>
+        </is>
+      </c>
+      <c r="I521" t="inlineStr">
+        <is>
+          <t>Entitlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="522">
+      <c r="A522" t="inlineStr">
+        <is>
+          <t>ENT-19</t>
+        </is>
+      </c>
+      <c r="B522" t="inlineStr">
+        <is>
+          <t>Free-tier pricing consequence: unlimited invoicing removes volume upgrade pressure</t>
+        </is>
+      </c>
+      <c r="C522" t="inlineStr">
+        <is>
+          <t>Entitlement</t>
+        </is>
+      </c>
+      <c r="D522" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E522" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F522" t="inlineStr">
+        <is>
+          <t>coral-submodule-entitlement.md</t>
+        </is>
+      </c>
+      <c r="G522" t="inlineStr">
+        <is>
+          <t>Matrix sold FREE as 5 invoices/mo. 'Full financial module' makes it unlimited. Upgrade pressure must then come from projects, team size and library instead. Florin's call, flagged not challenged.</t>
+        </is>
+      </c>
+      <c r="H522" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I522" t="inlineStr">
+        <is>
+          <t>Pricing</t>
+        </is>
+      </c>
+    </row>
+    <row r="523">
+      <c r="A523" t="inlineStr">
+        <is>
+          <t>ENT-20</t>
+        </is>
+      </c>
+      <c r="B523" t="inlineStr">
+        <is>
+          <t>REMOVE FOUNDER tier — 56 references across 15 files incl. terms/page.tsx (legal copy)</t>
+        </is>
+      </c>
+      <c r="C523" t="inlineStr">
+        <is>
+          <t>Entitlement</t>
+        </is>
+      </c>
+      <c r="D523" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E523" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F523" t="inlineStr">
+        <is>
+          <t>coralos-feature-matrix artifact</t>
+        </is>
+      </c>
+      <c r="G523" t="inlineStr">
+        <is>
+          <t>Florin 2026-09-26: 'remove founder, it is useless'. store/page.tsx (12), feature-flags.ts, TenantContext, plan-limits, stripe, tabs.ts, superadmin. Legal copy means this is a real pass.</t>
+        </is>
+      </c>
+      <c r="H523" t="inlineStr">
+        <is>
+          <t>L0 Kernel</t>
+        </is>
+      </c>
+      <c r="I523" t="inlineStr">
+        <is>
+          <t>Entitlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="524">
+      <c r="A524" t="inlineStr">
+        <is>
+          <t>ENT-21</t>
+        </is>
+      </c>
+      <c r="B524" t="inlineStr">
+        <is>
+          <t>🔴 DEAD QUOTA TABLE: PLAN_PEPPOL_LIMITS (stripe.ts) has ZERO readers, 10x the live numbers</t>
+        </is>
+      </c>
+      <c r="C524" t="inlineStr">
+        <is>
+          <t>Entitlement</t>
+        </is>
+      </c>
+      <c r="D524" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E524" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F524" t="inlineStr">
+        <is>
+          <t>coralos-feature-matrix artifact</t>
+        </is>
+      </c>
+      <c r="G524" t="inlineStr">
+        <is>
+          <t>Says FREE 50/mo, PRO 250, ENTERPRISE 1000. Live table PLAN_LIMITS says FREE 5 sent/10 recv, ENTERPRISE unlimited. Danger is plausibility: someone finds it first and 'fixes' the enforcing table. Delete one.</t>
+        </is>
+      </c>
+      <c r="H524" t="inlineStr">
+        <is>
+          <t>L1 Core</t>
+        </is>
+      </c>
+      <c r="I524" t="inlineStr">
+        <is>
+          <t>Entitlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="525">
+      <c r="A525" t="inlineStr">
+        <is>
+          <t>ENT-22</t>
+        </is>
+      </c>
+      <c r="B525" t="inlineStr">
+        <is>
+          <t>G2: invoice + quotation monthly caps unenforced — the meter that is not running</t>
+        </is>
+      </c>
+      <c r="C525" t="inlineStr">
+        <is>
+          <t>Entitlement</t>
+        </is>
+      </c>
+      <c r="D525" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E525" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F525" t="inlineStr">
+        <is>
+          <t>coral-free-tier-readiness.md</t>
+        </is>
+      </c>
+      <c r="G525" t="inlineStr">
+        <is>
+          <t>PLAN_LIMITS holds Peppol counters only. Reuse the SAME shape (counter, 1st-of-month UTC reset, named refusal). Do not invent a second mechanism. Collides with 'free gets full financials'.</t>
+        </is>
+      </c>
+      <c r="H525" t="inlineStr">
+        <is>
+          <t>L1 Core</t>
+        </is>
+      </c>
+      <c r="I525" t="inlineStr">
+        <is>
+          <t>Entitlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="526">
+      <c r="A526" t="inlineStr">
+        <is>
+          <t>ENT-23</t>
+        </is>
+      </c>
+      <c r="B526" t="inlineStr">
+        <is>
+          <t>Batiprix: priced as a TIER (ENTERPRISE_BATIPRIX €199) but described as an opt-in add-on</t>
+        </is>
+      </c>
+      <c r="C526" t="inlineStr">
+        <is>
+          <t>Entitlement</t>
+        </is>
+      </c>
+      <c r="D526" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E526" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F526" t="inlineStr">
+        <is>
+          <t>coralos-feature-matrix artifact</t>
+        </is>
+      </c>
+      <c r="G526" t="inlineStr">
+        <is>
+          <t>Florin 2026-09-26: 'optionally, against an opt-in, a connection to batiprix'. Add-on vs tier changes the billing model and the entitlement shape.</t>
+        </is>
+      </c>
+      <c r="H526" t="inlineStr">
+        <is>
+          <t>L1 Core</t>
+        </is>
+      </c>
+      <c r="I526" t="inlineStr">
+        <is>
+          <t>Entitlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="527">
+      <c r="A527" t="inlineStr">
+        <is>
+          <t>ENT-24</t>
+        </is>
+      </c>
+      <c r="B527" t="inlineStr">
+        <is>
+          <t>FREE is not a trial outcome — the two concepts are separate (Florin 2026-09-26)</t>
+        </is>
+      </c>
+      <c r="C527" t="inlineStr">
+        <is>
+          <t>Entitlement</t>
+        </is>
+      </c>
+      <c r="D527" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E527" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F527" t="inlineStr">
+        <is>
+          <t>coral-free-tier-readiness.md</t>
+        </is>
+      </c>
+      <c r="G527" t="inlineStr">
+        <is>
+          <t>Planner had described FREE as 'only reachable by a lapse' — that described the CODE's confusion (trial -&gt; PAST_DUE -&gt; INACTIVE), not the business logic. FREE is a product; the trial is a temporary grant of a higher tier. See coral-trial-vs-free.md.</t>
+        </is>
+      </c>
+      <c r="H527" t="inlineStr">
+        <is>
+          <t>L1 Core</t>
+        </is>
+      </c>
+      <c r="I527" t="inlineStr">
+        <is>
+          <t>Entitlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="528">
+      <c r="A528" t="inlineStr">
+        <is>
+          <t>LIB-1</t>
+        </is>
+      </c>
+      <c r="B528" t="inlineStr">
+        <is>
+          <t>Library tiering: FREE none · PRO empty (self-filled) · ENTERPRISE populated + Batiprix opt-in</t>
+        </is>
+      </c>
+      <c r="C528" t="inlineStr">
+        <is>
+          <t>Library</t>
+        </is>
+      </c>
+      <c r="D528" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E528" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F528" t="inlineStr">
+        <is>
+          <t>coralos-feature-matrix artifact</t>
+        </is>
+      </c>
+      <c r="G528" t="inlineStr">
+        <is>
+          <t>Florin 2026-09-26. Free gets the quote ENGINE with no catalogue — nothing persists to articles/bestek. That is the upgrade pressure replacing the April volume cap.</t>
+        </is>
+      </c>
+      <c r="H528" t="inlineStr">
+        <is>
+          <t>L2 Module</t>
+        </is>
+      </c>
+      <c r="I528" t="inlineStr">
+        <is>
+          <t>Library</t>
+        </is>
+      </c>
+    </row>
+    <row r="529">
+      <c r="A529" t="inlineStr">
+        <is>
+          <t>TRIAL-1</t>
+        </is>
+      </c>
+      <c r="B529" t="inlineStr">
+        <is>
+          <t>Trial is an ENTITLEMENT OVERLAY — it must never write planType</t>
+        </is>
+      </c>
+      <c r="C529" t="inlineStr">
+        <is>
+          <t>Billing</t>
+        </is>
+      </c>
+      <c r="D529" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E529" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F529" t="inlineStr">
+        <is>
+          <t>coral-trial-vs-free.md</t>
+        </is>
+      </c>
+      <c r="G529" t="inlineStr">
+        <is>
+          <t>trial.ts:40 startTrial calls syncPlanToTenant: a tenant trialling PRO BECOMES PRO, destroying their real tier. Replace with Tenant.trialGrant {tier, entitlements, expiresAt}. Expiry = overlay lapses, nothing downgraded.</t>
+        </is>
+      </c>
+      <c r="H529" t="inlineStr">
+        <is>
+          <t>L1 Core</t>
+        </is>
+      </c>
+      <c r="I529" t="inlineStr">
+        <is>
+          <t>Entitlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="530">
+      <c r="A530" t="inlineStr">
+        <is>
+          <t>TRIAL-2</t>
+        </is>
+      </c>
+      <c r="B530" t="inlineStr">
+        <is>
+          <t>🔴 Trial expiry currently sets PAST_DUE then INACTIVE — a payment failure, then a block</t>
+        </is>
+      </c>
+      <c r="C530" t="inlineStr">
+        <is>
+          <t>Billing</t>
+        </is>
+      </c>
+      <c r="D530" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E530" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F530" t="inlineStr">
+        <is>
+          <t>coral-trial-vs-free.md</t>
+        </is>
+      </c>
+      <c r="G530" t="inlineStr">
+        <is>
+          <t>trial.ts:121-160. Nothing was owed and no payment failed. A lapsed trial must leave a working tenant on their own tier. Blocking a FREE tenant because they tried PRO is the bug this design prevents.</t>
+        </is>
+      </c>
+      <c r="H530" t="inlineStr">
+        <is>
+          <t>L1 Core</t>
+        </is>
+      </c>
+      <c r="I530" t="inlineStr">
+        <is>
+          <t>Entitlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="531">
+      <c r="A531" t="inlineStr">
+        <is>
+          <t>TRIAL-3</t>
+        </is>
+      </c>
+      <c r="B531" t="inlineStr">
+        <is>
+          <t>subscriptionStatus must mean PAYMENT only — it currently also encodes TRIAL</t>
+        </is>
+      </c>
+      <c r="C531" t="inlineStr">
+        <is>
+          <t>Billing</t>
+        </is>
+      </c>
+      <c r="D531" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E531" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F531" t="inlineStr">
+        <is>
+          <t>coral-trial-vs-free.md</t>
+        </is>
+      </c>
+      <c r="G531" t="inlineStr">
+        <is>
+          <t>planType says PRO, subscriptionStatus says TRIAL: two fields carrying one fact, agreeing by convention.</t>
+        </is>
+      </c>
+      <c r="H531" t="inlineStr">
+        <is>
+          <t>L1 Core</t>
+        </is>
+      </c>
+      <c r="I531" t="inlineStr">
+        <is>
+          <t>Entitlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="532">
+      <c r="A532" t="inlineStr">
+        <is>
+          <t>TRIAL-4</t>
+        </is>
+      </c>
+      <c r="B532" t="inlineStr">
+        <is>
+          <t>PRO tenant trialling ENTERPRISE is INEXPRESSIBLE in the current model</t>
+        </is>
+      </c>
+      <c r="C532" t="inlineStr">
+        <is>
+          <t>Billing</t>
+        </is>
+      </c>
+      <c r="D532" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E532" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F532" t="inlineStr">
+        <is>
+          <t>coral-trial-vs-free.md</t>
+        </is>
+      </c>
+      <c r="G532" t="inlineStr">
+        <is>
+          <t>Because planType is overwritten there is nothing to revert to. This case is the proof the overlay works. Florin 2026-09-26: a client may want to try the higher tier directly.</t>
+        </is>
+      </c>
+      <c r="H532" t="inlineStr">
+        <is>
+          <t>L1 Core</t>
+        </is>
+      </c>
+      <c r="I532" t="inlineStr">
+        <is>
+          <t>Entitlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="533">
+      <c r="A533" t="inlineStr">
+        <is>
+          <t>TRIAL-5</t>
+        </is>
+      </c>
+      <c r="B533" t="inlineStr">
+        <is>
+          <t>TWO different things are called 'trial': entitlement trial vs Stripe payment trial</t>
+        </is>
+      </c>
+      <c r="C533" t="inlineStr">
+        <is>
+          <t>Billing</t>
+        </is>
+      </c>
+      <c r="D533" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E533" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F533" t="inlineStr">
+        <is>
+          <t>coral-trial-vs-free.md</t>
+        </is>
+      </c>
+      <c r="G533" t="inlineStr">
+        <is>
+          <t>P10 retired the Stripe payment trial (trial_period_days) and should never have touched the entitlement trial. Keep checkout/route.ts parked; un-park only the entitlement side.</t>
+        </is>
+      </c>
+      <c r="H533" t="inlineStr">
+        <is>
+          <t>L1 Core</t>
+        </is>
+      </c>
+      <c r="I533" t="inlineStr">
+        <is>
+          <t>Entitlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="534">
+      <c r="A534" t="inlineStr">
+        <is>
+          <t>TRIAL-6</t>
+        </is>
+      </c>
+      <c r="B534" t="inlineStr">
+        <is>
+          <t>trialHistory: one trial per tenant per tier, remembered after the grant is cleared</t>
+        </is>
+      </c>
+      <c r="C534" t="inlineStr">
+        <is>
+          <t>Billing</t>
+        </is>
+      </c>
+      <c r="D534" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="E534" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F534" t="inlineStr">
+        <is>
+          <t>coral-trial-vs-free.md</t>
+        </is>
+      </c>
+      <c r="G534" t="inlineStr">
+        <is>
+          <t>Checking whether trialGrant is null forgets. Durations already derive correctly from PLAN_PRICING.trialMonths (PRO 3 / ENTERPRISE 2).</t>
+        </is>
+      </c>
+      <c r="H534" t="inlineStr">
+        <is>
+          <t>L1 Core</t>
+        </is>
+      </c>
+      <c r="I534" t="inlineStr">
+        <is>
+          <t>Entitlement</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(deps): SUPA-1 remove @supabase/supabase-js and clean stale comments
</commit_message>
<xml_diff>
--- a/.agents/coral-roadmap.xlsx
+++ b/.agents/coral-roadmap.xlsx
@@ -594,7 +594,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I534"/>
+  <dimension ref="A1:I540"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -24240,6 +24240,288 @@
       <c r="I534" t="inlineStr">
         <is>
           <t>Entitlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="535">
+      <c r="A535" t="inlineStr">
+        <is>
+          <t>WORKHUB-LOGOUT</t>
+        </is>
+      </c>
+      <c r="B535" t="inlineStr">
+        <is>
+          <t>Time-tracker logout did nothing — AuthContext signOut was an empty stub</t>
+        </is>
+      </c>
+      <c r="C535" t="inlineStr">
+        <is>
+          <t>WorkHub</t>
+        </is>
+      </c>
+      <c r="D535" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E535" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F535" t="inlineStr">
+        <is>
+          <t>coral-supa-2-shape.md</t>
+        </is>
+      </c>
+      <c r="G535" t="inlineStr">
+        <is>
+          <t>Live defect 2026-09-26. Bridge to next-auth + cache wipe landed 696d5c7. Also left the cached tenant DB on the device — a shared-site-device data-hygiene issue, not just UX.</t>
+        </is>
+      </c>
+      <c r="H535" t="inlineStr">
+        <is>
+          <t>L2 Module</t>
+        </is>
+      </c>
+      <c r="I535" t="inlineStr">
+        <is>
+          <t>WorkHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="536">
+      <c r="A536" t="inlineStr">
+        <is>
+          <t>SUPA-1</t>
+        </is>
+      </c>
+      <c r="B536" t="inlineStr">
+        <is>
+          <t>Remove the dead @supabase/supabase-js dependency + 2 stale comments</t>
+        </is>
+      </c>
+      <c r="C536" t="inlineStr">
+        <is>
+          <t>Housekeeping</t>
+        </is>
+      </c>
+      <c r="D536" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="E536" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F536" t="inlineStr">
+        <is>
+          <t>coral-supa-2-shape.md</t>
+        </is>
+      </c>
+      <c r="G536" t="inlineStr">
+        <is>
+          <t>Imported nowhere, src/integrations gone, no SUPABASE_* env read. One line + lockfile. Do NOT touch the snake_case shape.</t>
+        </is>
+      </c>
+      <c r="H536" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I536" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="537">
+      <c r="A537" t="inlineStr">
+        <is>
+          <t>SUPA-2</t>
+        </is>
+      </c>
+      <c r="B537" t="inlineStr">
+        <is>
+          <t>The Supabase SHAPE: ~250 snake_case field accesses across 28 files</t>
+        </is>
+      </c>
+      <c r="C537" t="inlineStr">
+        <is>
+          <t>Housekeeping</t>
+        </is>
+      </c>
+      <c r="D537" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E537" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F537" t="inlineStr">
+        <is>
+          <t>coral-supa-2-shape.md</t>
+        </is>
+      </c>
+      <c r="G537" t="inlineStr">
+        <is>
+          <t>Not a deletion, a rename — and full_name is SEMANTIC (maps to User.name; Employee splits it in two). Find-and-replace compiles and renders blank.</t>
+        </is>
+      </c>
+      <c r="H537" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I537" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="538">
+      <c r="A538" t="inlineStr">
+        <is>
+          <t>SUPA-2.0</t>
+        </is>
+      </c>
+      <c r="B538" t="inlineStr">
+        <is>
+          <t>INVENTORY THE MANUFACTURERS: where snake_case is WRITTEN, not read</t>
+        </is>
+      </c>
+      <c r="C538" t="inlineStr">
+        <is>
+          <t>Housekeeping</t>
+        </is>
+      </c>
+      <c r="D538" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E538" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F538" t="inlineStr">
+        <is>
+          <t>coral-supa-2-shape.md</t>
+        </is>
+      </c>
+      <c r="G538" t="inlineStr">
+        <is>
+          <t>Two confirmed: AuthContext bridgedProfile:95, actions/timesheets.ts:97. useScheduledShifts.ts (17 sites) is the prime suspect. Kill the manufacturer and consumers break VISIBLY; convert consumers first and the old shape keeps feeding them silently.</t>
+        </is>
+      </c>
+      <c r="H538" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I538" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="539">
+      <c r="A539" t="inlineStr">
+        <is>
+          <t>SUPA-2.6</t>
+        </is>
+      </c>
+      <c r="B539" t="inlineStr">
+        <is>
+          <t>🔴 TimesheetView + ClockButton convert LAST — payable hours</t>
+        </is>
+      </c>
+      <c r="C539" t="inlineStr">
+        <is>
+          <t>Housekeeping</t>
+        </is>
+      </c>
+      <c r="D539" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E539" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F539" t="inlineStr">
+        <is>
+          <t>coral-supa-2-shape.md</t>
+        </is>
+      </c>
+      <c r="G539" t="inlineStr">
+        <is>
+          <t>17 of 250 sites in TimesheetView alone. A wrong mapping renders a blank or a wrong duration, and a wrong duration is a wrong wage. Verification is a FIGURE: total hours for a named worker over a named week, before and after.</t>
+        </is>
+      </c>
+      <c r="H539" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I539" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="540">
+      <c r="A540" t="inlineStr">
+        <is>
+          <t>DOC-1</t>
+        </is>
+      </c>
+      <c r="B540" t="inlineStr">
+        <is>
+          <t>board-v2:748 describes a live Supabase split-brain — five months out of date</t>
+        </is>
+      </c>
+      <c r="C540" t="inlineStr">
+        <is>
+          <t>Housekeeping</t>
+        </is>
+      </c>
+      <c r="D540" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="E540" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F540" t="inlineStr">
+        <is>
+          <t>coral-supa-2-shape.md</t>
+        </is>
+      </c>
+      <c r="G540" t="inlineStr">
+        <is>
+          <t>The migration happened and nobody recorded it. The stale description is what made a cold corpse look like a live system.</t>
+        </is>
+      </c>
+      <c r="H540" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I540" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(workhub): WH-5a server-side project labour aggregate and decouple ProjectDetailView
</commit_message>
<xml_diff>
--- a/.agents/coral-roadmap.xlsx
+++ b/.agents/coral-roadmap.xlsx
@@ -594,7 +594,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I540"/>
+  <dimension ref="A1:I579"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -10340,7 +10340,7 @@
       </c>
       <c r="F225" s="11" t="inlineStr">
         <is>
-          <t>coral-r1-tenancy.md</t>
+          <t>coder-directive-r1-1b-logicalkey.md</t>
         </is>
       </c>
       <c r="G225" s="11" t="inlineStr">
@@ -20679,7 +20679,7 @@
       </c>
       <c r="B459" t="inlineStr">
         <is>
-          <t>DECIDED (Florin 2026-09-24): ONE projects database. All workforce-side links point at the project page.</t>
+          <t>DECIDED 2026-09-27: the PAGE is the project. InternalProject and HrProject are deleted.</t>
         </is>
       </c>
       <c r="C459" t="inlineStr">
@@ -20694,7 +20694,7 @@
       </c>
       <c r="E459" t="inlineStr">
         <is>
-          <t>Decided — execution open</t>
+          <t>Decided</t>
         </is>
       </c>
       <c r="F459" t="inlineStr">
@@ -20704,7 +20704,7 @@
       </c>
       <c r="G459" t="inlineStr">
         <is>
-          <t>Florin's decision, not the coder's. Blocks PROJ-1..7: every cockpit aggregate joins on an undeclared projectId. Options A/B/C in the spec.</t>
+          <t>Census: 0 pages have an InternalProject twin; exactly 1 InternalProject exists (no page); 73 project pages. The quote-service id pun essentially never executed. Option B' is dead — a 1-row model cannot be canonical for 73 pages. Florin: 'quote acceptance must simply add a row in a db and prefill the needed data.' CMS_Project is a separate entity living in the CMS only.</t>
         </is>
       </c>
       <c r="H459" t="inlineStr">
@@ -24522,6 +24522,1839 @@
       <c r="I540" t="inlineStr">
         <is>
           <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="541">
+      <c r="A541" t="inlineStr">
+        <is>
+          <t>WH-0</t>
+        </is>
+      </c>
+      <c r="B541" t="inlineStr">
+        <is>
+          <t>🔴 KEYSTONE: the app's shadcn kit (52 files) imports cn() from INSIDE the time-tracker</t>
+        </is>
+      </c>
+      <c r="C541" t="inlineStr">
+        <is>
+          <t>WorkHub</t>
+        </is>
+      </c>
+      <c r="D541" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E541" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F541" t="inlineStr">
+        <is>
+          <t>coral-workhub-scope.md</t>
+        </is>
+      </c>
+      <c r="G541" t="inlineStr">
+        <is>
+          <t>src/lib/utils.ts does not exist. time-tracker/lib/utils.ts is 7 lines of cn(). The design system depends on the module we are deciding whether to delete. Fixing this removes 73% of the apparent coupling.</t>
+        </is>
+      </c>
+      <c r="H541" t="inlineStr">
+        <is>
+          <t>L0 Kernel</t>
+        </is>
+      </c>
+      <c r="I541" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+    </row>
+    <row r="542">
+      <c r="A542" t="inlineStr">
+        <is>
+          <t>WH-1</t>
+        </is>
+      </c>
+      <c r="B542" t="inlineStr">
+        <is>
+          <t>STEP 1: extract the plumbing — cn, use-toast, use-mobile, ThemeContext, hr-api</t>
+        </is>
+      </c>
+      <c r="C542" t="inlineStr">
+        <is>
+          <t>WorkHub</t>
+        </is>
+      </c>
+      <c r="D542" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E542" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F542" t="inlineStr">
+        <is>
+          <t>coral-workhub-scope.md</t>
+        </is>
+      </c>
+      <c r="G542" t="inlineStr">
+        <is>
+          <t>Do this whatever is decided. Moves and repoints, no logic. Afterwards the module has 8 inbound imports and repair-vs-rebuild becomes reversible.</t>
+        </is>
+      </c>
+      <c r="H542" t="inlineStr">
+        <is>
+          <t>L0 Kernel</t>
+        </is>
+      </c>
+      <c r="I542" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+    </row>
+    <row r="543">
+      <c r="A543" t="inlineStr">
+        <is>
+          <t>WH-2</t>
+        </is>
+      </c>
+      <c r="B543" t="inlineStr">
+        <is>
+          <t>DECISION: repair / rebuild-the-editor / rebuild-the-module</t>
+        </is>
+      </c>
+      <c r="C543" t="inlineStr">
+        <is>
+          <t>WorkHub</t>
+        </is>
+      </c>
+      <c r="D543" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E543" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F543" t="inlineStr">
+        <is>
+          <t>coral-workhub-scope.md</t>
+        </is>
+      </c>
+      <c r="G543" t="inlineStr">
+        <is>
+          <t>Planner recommends Step 1 then B: rewrite the 3 shift-editor files (3,508 lines, 22%) against the corrected kernel; repair the display layer in place. A = tail-chasing, C = premature (kernel mid-repair, PROJ-0 undecided, R1-4 four gates out).</t>
+        </is>
+      </c>
+      <c r="H543" t="inlineStr">
+        <is>
+          <t>L2 Module</t>
+        </is>
+      </c>
+      <c r="I543" t="inlineStr">
+        <is>
+          <t>WorkHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="544">
+      <c r="A544" t="inlineStr">
+        <is>
+          <t>WH-3</t>
+        </is>
+      </c>
+      <c r="B544" t="inlineStr">
+        <is>
+          <t>PARK SUPA-2 batches 2.2-2.6 pending WH-2</t>
+        </is>
+      </c>
+      <c r="C544" t="inlineStr">
+        <is>
+          <t>WorkHub</t>
+        </is>
+      </c>
+      <c r="D544" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E544" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F544" t="inlineStr">
+        <is>
+          <t>coral-workhub-scope.md</t>
+        </is>
+      </c>
+      <c r="G544" t="inlineStr">
+        <is>
+          <t>Converting 40 files' field names is throwaway if those files are rewritten — the same 'fix it twice' argument made for GRID-REPLACE. Ratchet + WORKHUB-CLOCKLINK are kept; the batch march is parked.</t>
+        </is>
+      </c>
+      <c r="H544" t="inlineStr">
+        <is>
+          <t>L2 Module</t>
+        </is>
+      </c>
+      <c r="I544" t="inlineStr">
+        <is>
+          <t>WorkHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="545">
+      <c r="A545" t="inlineStr">
+        <is>
+          <t>WH-4</t>
+        </is>
+      </c>
+      <c r="B545" t="inlineStr">
+        <is>
+          <t>METRIC: @ts-nocheck 21 of 68 files (31% of the module never compiled)</t>
+        </is>
+      </c>
+      <c r="C545" t="inlineStr">
+        <is>
+          <t>WorkHub</t>
+        </is>
+      </c>
+      <c r="D545" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E545" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F545" t="inlineStr">
+        <is>
+          <t>coral-workhub-scope.md</t>
+        </is>
+      </c>
+      <c r="G545" t="inlineStr">
+        <is>
+          <t>The honest health number. Should only fall. Overlaps almost entirely with the 38 files carrying the Supabase shape.</t>
+        </is>
+      </c>
+      <c r="H545" t="inlineStr">
+        <is>
+          <t>L2 Module</t>
+        </is>
+      </c>
+      <c r="I545" t="inlineStr">
+        <is>
+          <t>WorkHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="546">
+      <c r="A546" t="inlineStr">
+        <is>
+          <t>DOC-2</t>
+        </is>
+      </c>
+      <c r="B546" t="inlineStr">
+        <is>
+          <t>🔴 board-v2:748 describes a system that no longer exists — correct or delete it</t>
+        </is>
+      </c>
+      <c r="C546" t="inlineStr">
+        <is>
+          <t>Housekeeping</t>
+        </is>
+      </c>
+      <c r="D546" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E546" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F546" t="inlineStr">
+        <is>
+          <t>coral-workhub-scope.md</t>
+        </is>
+      </c>
+      <c r="G546" t="inlineStr">
+        <is>
+          <t>Claims duplicate shadcn set (0 files), integrations/supabase (gone), split-brain data (gone). Still true: own i18n (5 locales incl ro/ru for the crews), own pages/contexts. A stale map costs more than no map.</t>
+        </is>
+      </c>
+      <c r="H546" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I546" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="547">
+      <c r="A547" t="inlineStr">
+        <is>
+          <t>CLEAN-11</t>
+        </is>
+      </c>
+      <c r="B547" t="inlineStr">
+        <is>
+          <t>Clock entry cmrm3n2rd has -2.00 hours and is APPROVED</t>
+        </is>
+      </c>
+      <c r="C547" t="inlineStr">
+        <is>
+          <t>HR · Timesheets</t>
+        </is>
+      </c>
+      <c r="D547" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E547" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F547" t="inlineStr">
+        <is>
+          <t>coral-workhub-scope.md</t>
+        </is>
+      </c>
+      <c r="G547" t="inlineStr">
+        <is>
+          <t>Vasile Ucraina, 2026-07-10, clockOutTime before clockInTime. Two hours subtracted from a paid week. Florin's data repair.</t>
+        </is>
+      </c>
+      <c r="H547" t="inlineStr">
+        <is>
+          <t>L2 Module</t>
+        </is>
+      </c>
+      <c r="I547" t="inlineStr">
+        <is>
+          <t>Timesheets</t>
+        </is>
+      </c>
+    </row>
+    <row r="548">
+      <c r="A548" t="inlineStr">
+        <is>
+          <t>WH-5</t>
+        </is>
+      </c>
+      <c r="B548" t="inlineStr">
+        <is>
+          <t>BOUNDARY AUDIT: files imported by BOTH /workhub and /admin; payload + reachability leaks</t>
+        </is>
+      </c>
+      <c r="C548" t="inlineStr">
+        <is>
+          <t>WorkHub</t>
+        </is>
+      </c>
+      <c r="D548" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E548" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F548" t="inlineStr">
+        <is>
+          <t>coral-workhub-structure.md</t>
+        </is>
+      </c>
+      <c r="G548" t="inlineStr">
+        <is>
+          <t>A measurement, not a refactor. Sizes WH-6/7/8 and makes 'zero visible connection with the ERP' checkable. The two modules may share the CORE, never COMPONENTS.</t>
+        </is>
+      </c>
+      <c r="H548" t="inlineStr">
+        <is>
+          <t>L2 Module</t>
+        </is>
+      </c>
+      <c r="I548" t="inlineStr">
+        <is>
+          <t>WorkHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="549">
+      <c r="A549" t="inlineStr">
+        <is>
+          <t>WH-6</t>
+        </is>
+      </c>
+      <c r="B549" t="inlineStr">
+        <is>
+          <t>🔴 ACTOR REACH is the second gate below the seraph — and it does not exist structurally</t>
+        </is>
+      </c>
+      <c r="C549" t="inlineStr">
+        <is>
+          <t>WorkHub</t>
+        </is>
+      </c>
+      <c r="D549" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E549" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F549" t="inlineStr">
+        <is>
+          <t>coral-workhub-structure.md</t>
+        </is>
+      </c>
+      <c r="G549" t="inlineStr">
+        <is>
+          <t>getAccessibleUserIds(tenantId, userId) NEVER USES tenantId. HrTeamMember has no tenantId (Class B via team), so neither query is tenant-constrained. Decorative tenancy in the function deciding who sees whose hours. Becomes scope.reach()/scope.reachableUserIds(), rides with R1-4.</t>
+        </is>
+      </c>
+      <c r="H549" t="inlineStr">
+        <is>
+          <t>L1 Core</t>
+        </is>
+      </c>
+      <c r="I549" t="inlineStr">
+        <is>
+          <t>Tenant gate</t>
+        </is>
+      </c>
+    </row>
+    <row r="550">
+      <c r="A550" t="inlineStr">
+        <is>
+          <t>WH-7</t>
+        </is>
+      </c>
+      <c r="B550" t="inlineStr">
+        <is>
+          <t>REBUILD the shift editor — 3,508 lines, 22% of the module, where the defects cluster</t>
+        </is>
+      </c>
+      <c r="C550" t="inlineStr">
+        <is>
+          <t>WorkHub</t>
+        </is>
+      </c>
+      <c r="D550" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E550" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F550" t="inlineStr">
+        <is>
+          <t>coral-workhub-structure.md</t>
+        </is>
+      </c>
+      <c r="G550" t="inlineStr">
+        <is>
+          <t>CreateShiftForm 1967 + EditShiftDialog 915 + ShiftViewDialog 626. BLOCKED on PROJ-0 and R1-4 — starting earlier rebuilds the [ERP] prefix and the 74 parse sites into new code.</t>
+        </is>
+      </c>
+      <c r="H550" t="inlineStr">
+        <is>
+          <t>L2 Module</t>
+        </is>
+      </c>
+      <c r="I550" t="inlineStr">
+        <is>
+          <t>WorkHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="551">
+      <c r="A551" t="inlineStr">
+        <is>
+          <t>WH-8</t>
+        </is>
+      </c>
+      <c r="B551" t="inlineStr">
+        <is>
+          <t>Display layer repaired in place, opportunistically, ratchet holding the line</t>
+        </is>
+      </c>
+      <c r="C551" t="inlineStr">
+        <is>
+          <t>WorkHub</t>
+        </is>
+      </c>
+      <c r="D551" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="E551" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F551" t="inlineStr">
+        <is>
+          <t>coral-workhub-structure.md</t>
+        </is>
+      </c>
+      <c r="G551" t="inlineStr">
+        <is>
+          <t>The other 78% is presentation. @ts-nocheck (21) only falls.</t>
+        </is>
+      </c>
+      <c r="H551" t="inlineStr">
+        <is>
+          <t>L2 Module</t>
+        </is>
+      </c>
+      <c r="I551" t="inlineStr">
+        <is>
+          <t>WorkHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="552">
+      <c r="A552" t="inlineStr">
+        <is>
+          <t>WH-9</t>
+        </is>
+      </c>
+      <c r="B552" t="inlineStr">
+        <is>
+          <t>KERNEL: the offline intent queue is a WRITE PRIMITIVE, not an HR feature</t>
+        </is>
+      </c>
+      <c r="C552" t="inlineStr">
+        <is>
+          <t>WorkHub</t>
+        </is>
+      </c>
+      <c r="D552" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E552" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F552" t="inlineStr">
+        <is>
+          <t>coral-workhub-structure.md</t>
+        </is>
+      </c>
+      <c r="G552" t="inlineStr">
+        <is>
+          <t>The ERP store needs the same thing (R2-4). One queue, or the phone and the desk will disagree about what happened. Clock-in must succeed on a dead network.</t>
+        </is>
+      </c>
+      <c r="H552" t="inlineStr">
+        <is>
+          <t>L0 Kernel</t>
+        </is>
+      </c>
+      <c r="I552" t="inlineStr">
+        <is>
+          <t>Write path</t>
+        </is>
+      </c>
+    </row>
+    <row r="553">
+      <c r="A553" t="inlineStr">
+        <is>
+          <t>WH-10</t>
+        </is>
+      </c>
+      <c r="B553" t="inlineStr">
+        <is>
+          <t>KERNEL: a negative duration must be a kernel REFUSAL, not a UI check</t>
+        </is>
+      </c>
+      <c r="C553" t="inlineStr">
+        <is>
+          <t>WorkHub</t>
+        </is>
+      </c>
+      <c r="D553" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E553" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F553" t="inlineStr">
+        <is>
+          <t>coral-workhub-structure.md</t>
+        </is>
+      </c>
+      <c r="G553" t="inlineStr">
+        <is>
+          <t>CLEAN-11 proves nothing refuses it: entry cmrm3n2rd holds -2.00 hours and is APPROVED. duration.test.ts is already pure and tested — the model for the rest.</t>
+        </is>
+      </c>
+      <c r="H553" t="inlineStr">
+        <is>
+          <t>L0 Kernel</t>
+        </is>
+      </c>
+      <c r="I553" t="inlineStr">
+        <is>
+          <t>Time</t>
+        </is>
+      </c>
+    </row>
+    <row r="554">
+      <c r="A554" t="inlineStr">
+        <is>
+          <t>WH-11</t>
+        </is>
+      </c>
+      <c r="B554" t="inlineStr">
+        <is>
+          <t>ONE WRITE PATH: phone clock-in and back-office manual entry are the SAME intent</t>
+        </is>
+      </c>
+      <c r="C554" t="inlineStr">
+        <is>
+          <t>WorkHub</t>
+        </is>
+      </c>
+      <c r="D554" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E554" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F554" t="inlineStr">
+        <is>
+          <t>coral-workhub-structure.md</t>
+        </is>
+      </c>
+      <c r="G554" t="inlineStr">
+        <is>
+          <t>Differ only in actor and reason. Two doors is how the phone and the desk start disagreeing. Rides with R2-1.</t>
+        </is>
+      </c>
+      <c r="H554" t="inlineStr">
+        <is>
+          <t>L1 Core</t>
+        </is>
+      </c>
+      <c r="I554" t="inlineStr">
+        <is>
+          <t>Write path</t>
+        </is>
+      </c>
+    </row>
+    <row r="555">
+      <c r="A555" t="inlineStr">
+        <is>
+          <t>WH-12</t>
+        </is>
+      </c>
+      <c r="B555" t="inlineStr">
+        <is>
+          <t>DECIDE which 'employee' is canonical: User, Employee model, or the db-hr projection</t>
+        </is>
+      </c>
+      <c r="C555" t="inlineStr">
+        <is>
+          <t>WorkHub</t>
+        </is>
+      </c>
+      <c r="D555" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E555" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F555" t="inlineStr">
+        <is>
+          <t>coral-workhub-structure.md</t>
+        </is>
+      </c>
+      <c r="G555" t="inlineStr">
+        <is>
+          <t>Three representations of one concept. db-hr holds no data — it synthesises rows from User at read time behind a 14-role allowlist.</t>
+        </is>
+      </c>
+      <c r="H555" t="inlineStr">
+        <is>
+          <t>L1 Core</t>
+        </is>
+      </c>
+      <c r="I555" t="inlineStr">
+        <is>
+          <t>Identity</t>
+        </is>
+      </c>
+    </row>
+    <row r="556">
+      <c r="A556" t="inlineStr">
+        <is>
+          <t>WH-13</t>
+        </is>
+      </c>
+      <c r="B556" t="inlineStr">
+        <is>
+          <t>REQUIREMENT: clock WITHOUT a shift must remain — Florin: 'very important'</t>
+        </is>
+      </c>
+      <c r="C556" t="inlineStr">
+        <is>
+          <t>WorkHub</t>
+        </is>
+      </c>
+      <c r="D556" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E556" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F556" t="inlineStr">
+        <is>
+          <t>coral-workhub-structure.md</t>
+        </is>
+      </c>
+      <c r="G556" t="inlineStr">
+        <is>
+          <t>Reachable today only from ClockButton on the workhub home; NOT from a shift card. Any rebuild must preserve it as a first-class path.</t>
+        </is>
+      </c>
+      <c r="H556" t="inlineStr">
+        <is>
+          <t>L2 Module</t>
+        </is>
+      </c>
+      <c r="I556" t="inlineStr">
+        <is>
+          <t>WorkHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="557">
+      <c r="A557" t="inlineStr">
+        <is>
+          <t>WH-13a</t>
+        </is>
+      </c>
+      <c r="B557" t="inlineStr">
+        <is>
+          <t>🔴 ad-hoc shift fabricates shiftEnd '17:00' and carries NO projectId</t>
+        </is>
+      </c>
+      <c r="C557" t="inlineStr">
+        <is>
+          <t>WorkHub</t>
+        </is>
+      </c>
+      <c r="D557" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E557" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F557" t="inlineStr">
+        <is>
+          <t>coral-workhub-structure.md</t>
+        </is>
+      </c>
+      <c r="G557" t="inlineStr">
+        <is>
+          <t>useScheduledShifts.ts:214. Hours attach to a shift attached to no job — 'mid air' by construction. The end time is invented regardless of reality.</t>
+        </is>
+      </c>
+      <c r="H557" t="inlineStr">
+        <is>
+          <t>L2 Module</t>
+        </is>
+      </c>
+      <c r="I557" t="inlineStr">
+        <is>
+          <t>WorkHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="558">
+      <c r="A558" t="inlineStr">
+        <is>
+          <t>WH-13b</t>
+        </is>
+      </c>
+      <c r="B558" t="inlineStr">
+        <is>
+          <t>🔴 ORPHAN GENERATOR: entry created first, linked by a separate PATCH afterwards</t>
+        </is>
+      </c>
+      <c r="C558" t="inlineStr">
+        <is>
+          <t>WorkHub</t>
+        </is>
+      </c>
+      <c r="D558" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E558" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F558" t="inlineStr">
+        <is>
+          <t>coral-workhub-structure.md</t>
+        </is>
+      </c>
+      <c r="G558" t="inlineStr">
+        <is>
+          <t>ClockButton:117-122. If the PATCH fails (dead network — the exact condition) the entry is saved unlinked. Likely source of some of the 11 orphans alongside late entry. Must be ONE atomic intent (WH-11).</t>
+        </is>
+      </c>
+      <c r="H558" t="inlineStr">
+        <is>
+          <t>L1 Core</t>
+        </is>
+      </c>
+      <c r="I558" t="inlineStr">
+        <is>
+          <t>Write path</t>
+        </is>
+      </c>
+    </row>
+    <row r="559">
+      <c r="A559" t="inlineStr">
+        <is>
+          <t>WH-14</t>
+        </is>
+      </c>
+      <c r="B559" t="inlineStr">
+        <is>
+          <t>REQUIREMENT: no way to create a shift in the PAST — late entries orphan as a result</t>
+        </is>
+      </c>
+      <c r="C559" t="inlineStr">
+        <is>
+          <t>WorkHub</t>
+        </is>
+      </c>
+      <c r="D559" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E559" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F559" t="inlineStr">
+        <is>
+          <t>coral-workhub-structure.md</t>
+        </is>
+      </c>
+      <c r="G559" t="inlineStr">
+        <is>
+          <t>Florin created some of the 11 orphans this way: late entry accepted, no retrospective shift to attach it to. Either allow a past shift, or let late entry create one.</t>
+        </is>
+      </c>
+      <c r="H559" t="inlineStr">
+        <is>
+          <t>L2 Module</t>
+        </is>
+      </c>
+      <c r="I559" t="inlineStr">
+        <is>
+          <t>WorkHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="560">
+      <c r="A560" t="inlineStr">
+        <is>
+          <t>WH-15</t>
+        </is>
+      </c>
+      <c r="B560" t="inlineStr">
+        <is>
+          <t>REQUIREMENT: the shift brief — opening a shift shows everything needed to work it</t>
+        </is>
+      </c>
+      <c r="C560" t="inlineStr">
+        <is>
+          <t>WorkHub</t>
+        </is>
+      </c>
+      <c r="D560" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E560" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F560" t="inlineStr">
+        <is>
+          <t>coral-workhub-structure.md</t>
+        </is>
+      </c>
+      <c r="G560" t="inlineStr">
+        <is>
+          <t>Florin 2026-09-27: address as a clickable navigation link, phone of the client or other relevant contact, photos, files. This is ShiftViewDialog's purpose and it is one of the 3 files WH-7 rebuilds.</t>
+        </is>
+      </c>
+      <c r="H560" t="inlineStr">
+        <is>
+          <t>L2 Module</t>
+        </is>
+      </c>
+      <c r="I560" t="inlineStr">
+        <is>
+          <t>WorkHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="561">
+      <c r="A561" t="inlineStr">
+        <is>
+          <t>WH-16</t>
+        </is>
+      </c>
+      <c r="B561" t="inlineStr">
+        <is>
+          <t>REQUIREMENT: GPS stays, and becomes a NOT-OVERCOMPLICATED geofence</t>
+        </is>
+      </c>
+      <c r="C561" t="inlineStr">
+        <is>
+          <t>WorkHub</t>
+        </is>
+      </c>
+      <c r="D561" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="E561" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F561" t="inlineStr">
+        <is>
+          <t>coral-workhub-structure.md</t>
+        </is>
+      </c>
+      <c r="G561" t="inlineStr">
+        <is>
+          <t>Already partially built: validateGeofence at ClockButton with a 200m radius against the shift's project lat/lng, warning + override rather than a hard block. Keep that shape — warn and record, do not refuse.</t>
+        </is>
+      </c>
+      <c r="H561" t="inlineStr">
+        <is>
+          <t>L2 Module</t>
+        </is>
+      </c>
+      <c r="I561" t="inlineStr">
+        <is>
+          <t>WorkHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="562">
+      <c r="A562" t="inlineStr">
+        <is>
+          <t>WH-17</t>
+        </is>
+      </c>
+      <c r="B562" t="inlineStr">
+        <is>
+          <t>Offline clocking — LAST in sequence, NOT dropped (Florin 2026-09-27)</t>
+        </is>
+      </c>
+      <c r="C562" t="inlineStr">
+        <is>
+          <t>WorkHub</t>
+        </is>
+      </c>
+      <c r="D562" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E562" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F562" t="inlineStr">
+        <is>
+          <t>coral-workhub-structure.md</t>
+        </is>
+      </c>
+      <c r="G562" t="inlineStr">
+        <is>
+          <t>Florin: 'rare, but still very much counts in EUR... me, client or crew member... so even if at the end, we do not leave it behind.' A lost hour is always PAID BY SOMEONE. sw-workhub.js:58 handles GET only; /api/* always network; the shell caches so the app LOOKS alive offline and a clock-in dies with a toast. Sequenced last, never dropped.</t>
+        </is>
+      </c>
+      <c r="H562" t="inlineStr">
+        <is>
+          <t>L0 Kernel</t>
+        </is>
+      </c>
+      <c r="I562" t="inlineStr">
+        <is>
+          <t>Write path</t>
+        </is>
+      </c>
+    </row>
+    <row r="563">
+      <c r="A563" t="inlineStr">
+        <is>
+          <t>WH-17a</t>
+        </is>
+      </c>
+      <c r="B563" t="inlineStr">
+        <is>
+          <t>Offline queue must be VISIBLE, not silent — rare failures are never noticed</t>
+        </is>
+      </c>
+      <c r="C563" t="inlineStr">
+        <is>
+          <t>WorkHub</t>
+        </is>
+      </c>
+      <c r="D563" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E563" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F563" t="inlineStr">
+        <is>
+          <t>coral-workhub-structure.md</t>
+        </is>
+      </c>
+      <c r="G563" t="inlineStr">
+        <is>
+          <t>Because it is rare, nobody develops a habit of checking. The worker must be told 'stored, not sent' at the moment it happens, and told again when it lands. A pending count on the surface so a stuck item surfaces itself.</t>
+        </is>
+      </c>
+      <c r="H563" t="inlineStr">
+        <is>
+          <t>L2 Module</t>
+        </is>
+      </c>
+      <c r="I563" t="inlineStr">
+        <is>
+          <t>WorkHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="564">
+      <c r="A564" t="inlineStr">
+        <is>
+          <t>WH-17b</t>
+        </is>
+      </c>
+      <c r="B564" t="inlineStr">
+        <is>
+          <t>Offline queue must be DELIBERATELY TESTABLE — rare paths are rarely exercised</t>
+        </is>
+      </c>
+      <c r="C564" t="inlineStr">
+        <is>
+          <t>WorkHub</t>
+        </is>
+      </c>
+      <c r="D564" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E564" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F564" t="inlineStr">
+        <is>
+          <t>coral-workhub-structure.md</t>
+        </is>
+      </c>
+      <c r="G564" t="inlineStr">
+        <is>
+          <t>A queue nobody exercises is a queue that breaks silently. Needs an explicit offline-mode test in the verify steps (airplane mode / SW offline), not just 'it worked once'. Same class as PRE-1c: an untested gate is not a gate.</t>
+        </is>
+      </c>
+      <c r="H564" t="inlineStr">
+        <is>
+          <t>L2 Module</t>
+        </is>
+      </c>
+      <c r="I564" t="inlineStr">
+        <is>
+          <t>WorkHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="565">
+      <c r="A565" t="inlineStr">
+        <is>
+          <t>PROJ-1a</t>
+        </is>
+      </c>
+      <c r="B565" t="inlineStr">
+        <is>
+          <t>DELETE InternalProject — 1 row, 19 touch points across 8 files</t>
+        </is>
+      </c>
+      <c r="C565" t="inlineStr">
+        <is>
+          <t>Projects</t>
+        </is>
+      </c>
+      <c r="D565" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E565" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F565" t="inlineStr">
+        <is>
+          <t>coral-project-module.md</t>
+        </is>
+      </c>
+      <c r="G565" t="inlineStr">
+        <is>
+          <t>superadmin (4), timesheets.ts:67, internal-projects.ts (3), crm.ts (2), hr/[entity] erp-projects merge (6), quote-service (3). Quote acceptance writes a row in the projects DATABASE instead.</t>
+        </is>
+      </c>
+      <c r="H565" t="inlineStr">
+        <is>
+          <t>L2 Module</t>
+        </is>
+      </c>
+      <c r="I565" t="inlineStr">
+        <is>
+          <t>Projects</t>
+        </is>
+      </c>
+    </row>
+    <row r="566">
+      <c r="A566" t="inlineStr">
+        <is>
+          <t>PROJ-1b</t>
+        </is>
+      </c>
+      <c r="B566" t="inlineStr">
+        <is>
+          <t>D-A stands and must be enforced at write: GlobalPage is polymorphic</t>
+        </is>
+      </c>
+      <c r="C566" t="inlineStr">
+        <is>
+          <t>Projects</t>
+        </is>
+      </c>
+      <c r="D566" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E566" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F566" t="inlineStr">
+        <is>
+          <t>coral-decision-one-project.md</t>
+        </is>
+      </c>
+      <c r="G566" t="inlineStr">
+        <is>
+          <t>With the page as the project, no FK can enforce 'is a project page' — the type lives in databaseId, which is user data. Verify databaseId === scope.systemDatabase('projects') on every write that sets a project reference. Written once, in R1-4.</t>
+        </is>
+      </c>
+      <c r="H566" t="inlineStr">
+        <is>
+          <t>L1 Core</t>
+        </is>
+      </c>
+      <c r="I566" t="inlineStr">
+        <is>
+          <t>Projects</t>
+        </is>
+      </c>
+    </row>
+    <row r="567">
+      <c r="A567" t="inlineStr">
+        <is>
+          <t>PORTAL-1</t>
+        </is>
+      </c>
+      <c r="B567" t="inlineStr">
+        <is>
+          <t>🔴 ClientPortal password is enforced CLIENT-SIDE ONLY — the payload is returned unauthenticated</t>
+        </is>
+      </c>
+      <c r="C567" t="inlineStr">
+        <is>
+          <t>Portals</t>
+        </is>
+      </c>
+      <c r="D567" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E567" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F567" t="inlineStr">
+        <is>
+          <t>coder-directive-portal-1-server-auth.md</t>
+        </is>
+      </c>
+      <c r="G567" t="inlineStr">
+        <is>
+          <t>api/portals/slug/[slug]/route.ts:129-136 returns tasks, linkedProjectData, QUOTES, INVOICES, budget and paidAmount, with hasPassword as a mere flag. The password is never verified in that route; portal/[slug]/page.tsx:30 does the gating. Anyone holding the link sees everything regardless of the password.</t>
+        </is>
+      </c>
+      <c r="H567" t="inlineStr">
+        <is>
+          <t>L2 Module</t>
+        </is>
+      </c>
+      <c r="I567" t="inlineStr">
+        <is>
+          <t>Portals</t>
+        </is>
+      </c>
+    </row>
+    <row r="568">
+      <c r="A568" t="inlineStr">
+        <is>
+          <t>PORTAL-2</t>
+        </is>
+      </c>
+      <c r="B568" t="inlineStr">
+        <is>
+          <t>The slug IS the credential — nanoid(10), ~60 bits, not brute-forceable</t>
+        </is>
+      </c>
+      <c r="C568" t="inlineStr">
+        <is>
+          <t>Portals</t>
+        </is>
+      </c>
+      <c r="D568" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E568" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F568" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G568" t="inlineStr">
+        <is>
+          <t>Materially limits severity: not enumerable. But a forwarded email, screenshot, chat link or shared browser history grants full access, and the password adds nothing against any of them.</t>
+        </is>
+      </c>
+      <c r="H568" t="inlineStr">
+        <is>
+          <t>L2 Module</t>
+        </is>
+      </c>
+      <c r="I568" t="inlineStr">
+        <is>
+          <t>Portals</t>
+        </is>
+      </c>
+    </row>
+    <row r="569">
+      <c r="A569" t="inlineStr">
+        <is>
+          <t>PORTAL-3</t>
+        </is>
+      </c>
+      <c r="B569" t="inlineStr">
+        <is>
+          <t>2FA on ClientPortal (Florin 2026-09-27) — AFTER server-side verification</t>
+        </is>
+      </c>
+      <c r="C569" t="inlineStr">
+        <is>
+          <t>Portals</t>
+        </is>
+      </c>
+      <c r="D569" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E569" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F569" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G569" t="inlineStr">
+        <is>
+          <t>A second factor on top of a client-side gate is decoration on decoration. Order: verify password server-side and issue a scoped session, THEN add the second factor.</t>
+        </is>
+      </c>
+      <c r="H569" t="inlineStr">
+        <is>
+          <t>L2 Module</t>
+        </is>
+      </c>
+      <c r="I569" t="inlineStr">
+        <is>
+          <t>Portals</t>
+        </is>
+      </c>
+    </row>
+    <row r="570">
+      <c r="A570" t="inlineStr">
+        <is>
+          <t>PORTAL-4</t>
+        </is>
+      </c>
+      <c r="B570" t="inlineStr">
+        <is>
+          <t>ClientPortal.password is nullable — a portal may exist with no credential at all</t>
+        </is>
+      </c>
+      <c r="C570" t="inlineStr">
+        <is>
+          <t>Portals</t>
+        </is>
+      </c>
+      <c r="D570" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E570" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F570" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G570" t="inlineStr">
+        <is>
+          <t>Combined with PORTAL-1 this means link-only access by design for some portals. Decide whether that is intended (a public progress page) or an oversight.</t>
+        </is>
+      </c>
+      <c r="H570" t="inlineStr">
+        <is>
+          <t>L2 Module</t>
+        </is>
+      </c>
+      <c r="I570" t="inlineStr">
+        <is>
+          <t>Portals</t>
+        </is>
+      </c>
+    </row>
+    <row r="571">
+      <c r="A571" t="inlineStr">
+        <is>
+          <t>PT-0</t>
+        </is>
+      </c>
+      <c r="B571" t="inlineStr">
+        <is>
+          <t>🔴 AUTHORSHIP DOES NOT EXIST: Message.sender is free text from the body; the other 4 records have no author at all</t>
+        </is>
+      </c>
+      <c r="C571" t="inlineStr">
+        <is>
+          <t>Portals</t>
+        </is>
+      </c>
+      <c r="D571" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E571" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F571" t="inlineStr">
+        <is>
+          <t>coral-portal-two-party-record.md</t>
+        </is>
+      </c>
+      <c r="G571" t="inlineStr">
+        <is>
+          <t>ProjectUpdate, Document, ProjectMedia, Task have NO author field. The two-party rule cannot be enforced until the data records which side wrote each row. Schema first, then the gate, then the UI.</t>
+        </is>
+      </c>
+      <c r="H571" t="inlineStr">
+        <is>
+          <t>L1 Core</t>
+        </is>
+      </c>
+      <c r="I571" t="inlineStr">
+        <is>
+          <t>Portals</t>
+        </is>
+      </c>
+    </row>
+    <row r="572">
+      <c r="A572" t="inlineStr">
+        <is>
+          <t>PT-1</t>
+        </is>
+      </c>
+      <c r="B572" t="inlineStr">
+        <is>
+          <t>authorSide (NOT NULL) + authorId + frozen authorLabel on all five portal records</t>
+        </is>
+      </c>
+      <c r="C572" t="inlineStr">
+        <is>
+          <t>Portals</t>
+        </is>
+      </c>
+      <c r="D572" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E572" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F572" t="inlineStr">
+        <is>
+          <t>coral-portal-two-party-record.md</t>
+        </is>
+      </c>
+      <c r="G572" t="inlineStr">
+        <is>
+          <t>Set by the SCOPE, never the payload (R1-3). authorLabel frozen at write time. NO BACKFILL NEEDED — Florin 2026-09-27: portals are not yet properly in use, one or two created, UI still clumsy. So authorSide goes in NOT NULL from the start; no nullable-then-tighten dance, no inferred-author flag.</t>
+        </is>
+      </c>
+      <c r="H572" t="inlineStr">
+        <is>
+          <t>L1 Core</t>
+        </is>
+      </c>
+      <c r="I572" t="inlineStr">
+        <is>
+          <t>Portals</t>
+        </is>
+      </c>
+    </row>
+    <row r="573">
+      <c r="A573" t="inlineStr">
+        <is>
+          <t>PT-2</t>
+        </is>
+      </c>
+      <c r="B573" t="inlineStr">
+        <is>
+          <t>Cross-side mutation refused in the scoped client — append-only for the other side</t>
+        </is>
+      </c>
+      <c r="C573" t="inlineStr">
+        <is>
+          <t>Portals</t>
+        </is>
+      </c>
+      <c r="D573" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E573" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F573" t="inlineStr">
+        <is>
+          <t>coral-portal-two-party-record.md</t>
+        </is>
+      </c>
+      <c r="G573" t="inlineStr">
+        <is>
+          <t>The tenant cannot edit or delete a client message. Not soft-delete, not hide. If it can vanish it was never evidence. A correction is a new entry. Not conditional on plan or role.</t>
+        </is>
+      </c>
+      <c r="H573" t="inlineStr">
+        <is>
+          <t>L1 Core</t>
+        </is>
+      </c>
+      <c r="I573" t="inlineStr">
+        <is>
+          <t>Portals</t>
+        </is>
+      </c>
+    </row>
+    <row r="574">
+      <c r="A574" t="inlineStr">
+        <is>
+          <t>PT-3</t>
+        </is>
+      </c>
+      <c r="B574" t="inlineStr">
+        <is>
+          <t>Task.status is CHANGEABLE, with every change logged (Florin 2026-09-27)</t>
+        </is>
+      </c>
+      <c r="C574" t="inlineStr">
+        <is>
+          <t>Portals</t>
+        </is>
+      </c>
+      <c r="D574" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E574" t="inlineStr">
+        <is>
+          <t>Decided</t>
+        </is>
+      </c>
+      <c r="F574" t="inlineStr">
+        <is>
+          <t>coral-portal-two-party-record.md</t>
+        </is>
+      </c>
+      <c r="G574" t="inlineStr">
+        <is>
+          <t>Not prohibited — logged. Use the EXISTING AuditLog (entityType 'portalTask', field 'status', before/after). Do NOT create a fourth audit model: AuditLog and RateChangeAudit already exist.</t>
+        </is>
+      </c>
+      <c r="H574" t="inlineStr">
+        <is>
+          <t>L1 Core</t>
+        </is>
+      </c>
+      <c r="I574" t="inlineStr">
+        <is>
+          <t>Portals</t>
+        </is>
+      </c>
+    </row>
+    <row r="575">
+      <c r="A575" t="inlineStr">
+        <is>
+          <t>PT-4</t>
+        </is>
+      </c>
+      <c r="B575" t="inlineStr">
+        <is>
+          <t>Loud UI both ways — no edit affordance on the other side's entries</t>
+        </is>
+      </c>
+      <c r="C575" t="inlineStr">
+        <is>
+          <t>Portals</t>
+        </is>
+      </c>
+      <c r="D575" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E575" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F575" t="inlineStr">
+        <is>
+          <t>coral-portal-two-party-record.md</t>
+        </is>
+      </c>
+      <c r="G575" t="inlineStr">
+        <is>
+          <t>Florin: 'it has to be loud, obvious in the ui'. Absent, not greyed out — a disabled edit button invites a support request. Inferred authorship marked until confirmed.</t>
+        </is>
+      </c>
+      <c r="H575" t="inlineStr">
+        <is>
+          <t>L2 Module</t>
+        </is>
+      </c>
+      <c r="I575" t="inlineStr">
+        <is>
+          <t>Portals</t>
+        </is>
+      </c>
+    </row>
+    <row r="576">
+      <c r="A576" t="inlineStr">
+        <is>
+          <t>PT-5</t>
+        </is>
+      </c>
+      <c r="B576" t="inlineStr">
+        <is>
+          <t>portalScope(portalId, secret) — a THIRD constructor of the same scope</t>
+        </is>
+      </c>
+      <c r="C576" t="inlineStr">
+        <is>
+          <t>Portals</t>
+        </is>
+      </c>
+      <c r="D576" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E576" t="inlineStr">
+        <is>
+          <t>Decided</t>
+        </is>
+      </c>
+      <c r="F576" t="inlineStr">
+        <is>
+          <t>coral-portal-two-party-record.md</t>
+        </is>
+      </c>
+      <c r="G576" t="inlineStr">
+        <is>
+          <t>Beside scopeFromSession and systemScope (TSC-0 D3/D5). Carries tenant AND side. No new principal type — what flows downstream is the identical TenantScopedClient. Rejected: a restricted User row (seats, db-hr projection, team pickers, 'a user who is not a user'). | CONFIRMED by Florin 2026-09-27: 'no new user then.'</t>
+        </is>
+      </c>
+      <c r="H576" t="inlineStr">
+        <is>
+          <t>L1 Core</t>
+        </is>
+      </c>
+      <c r="I576" t="inlineStr">
+        <is>
+          <t>Tenant gate</t>
+        </is>
+      </c>
+    </row>
+    <row r="577">
+      <c r="A577" t="inlineStr">
+        <is>
+          <t>PORTAL-5</t>
+        </is>
+      </c>
+      <c r="B577" t="inlineStr">
+        <is>
+          <t>🔴 THREE auth models in one feature: password server-side / ERP session / nothing</t>
+        </is>
+      </c>
+      <c r="C577" t="inlineStr">
+        <is>
+          <t>Portals</t>
+        </is>
+      </c>
+      <c r="D577" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E577" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F577" t="inlineStr">
+        <is>
+          <t>coral-portal-two-party-record.md</t>
+        </is>
+      </c>
+      <c r="G577" t="inlineStr">
+        <is>
+          <t>documents+media verify the portal password server-side; messages+tasks+updates demand auth() an ERP session the client lacks; slug read checks nothing. So a client CAN upload a document and CANNOT post a message. portalScope collapses all three.</t>
+        </is>
+      </c>
+      <c r="H577" t="inlineStr">
+        <is>
+          <t>L1 Core</t>
+        </is>
+      </c>
+      <c r="I577" t="inlineStr">
+        <is>
+          <t>Portals</t>
+        </is>
+      </c>
+    </row>
+    <row r="578">
+      <c r="A578" t="inlineStr">
+        <is>
+          <t>CORE-2</t>
+        </is>
+      </c>
+      <c r="B578" t="inlineStr">
+        <is>
+          <t>🔴 AuditLog.actorUserId is NOT NULL — cannot record a system, portal or operator actor</t>
+        </is>
+      </c>
+      <c r="C578" t="inlineStr">
+        <is>
+          <t>Audit</t>
+        </is>
+      </c>
+      <c r="D578" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E578" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F578" t="inlineStr">
+        <is>
+          <t>coder-directive-core-2-audit-actor.md</t>
+        </is>
+      </c>
+      <c r="G578" t="inlineStr">
+        <is>
+          <t>Blocks portal writes (no user by design), cron/webhook writes (TSC-3 systemScope), and impersonation tracking. The 'reason' column already anticipates system writes but there is nowhere to put the actor. Needs actorUserId String? + an actor KIND: user | system | portal | operator-impersonating. Serves portals, scheduled work and impersonation at once.</t>
+        </is>
+      </c>
+      <c r="H578" t="inlineStr">
+        <is>
+          <t>L1 Core</t>
+        </is>
+      </c>
+      <c r="I578" t="inlineStr">
+        <is>
+          <t>Audit</t>
+        </is>
+      </c>
+    </row>
+    <row r="579">
+      <c r="A579" t="inlineStr">
+        <is>
+          <t>WH-5a</t>
+        </is>
+      </c>
+      <c r="B579" t="inlineStr">
+        <is>
+          <t>Core accessor labourForProject — the last ERP-&gt;workhub wire</t>
+        </is>
+      </c>
+      <c r="C579" t="inlineStr">
+        <is>
+          <t>WorkHub</t>
+        </is>
+      </c>
+      <c r="D579" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E579" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F579" t="inlineStr">
+        <is>
+          <t>coder-directive-wh-5a-project-hours.md</t>
+        </is>
+      </c>
+      <c r="G579" t="inlineStr">
+        <is>
+          <t>ProjectDetailView loads the tenant's ENTIRE clock-entry and shift history into the browser to compute one project's labour, and carries the last project_id fallback outside the time-tracker. Replaced by a server-side aggregate. Closes WH-5 and answers PROJ-6 from the core.</t>
+        </is>
+      </c>
+      <c r="H579" t="inlineStr">
+        <is>
+          <t>L1 Core</t>
+        </is>
+      </c>
+      <c r="I579" t="inlineStr">
+        <is>
+          <t>Projects</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(kernel): R1-1c provisionLockedDatabases ongoing logicalKey write, binding verification, and self-heal
</commit_message>
<xml_diff>
--- a/.agents/coral-roadmap.xlsx
+++ b/.agents/coral-roadmap.xlsx
@@ -594,7 +594,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I579"/>
+  <dimension ref="A1:I582"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -21822,7 +21822,7 @@
       </c>
       <c r="E483" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Confirmed live</t>
         </is>
       </c>
       <c r="F483" t="inlineStr">
@@ -21832,7 +21832,7 @@
       </c>
       <c r="G483" t="inlineStr">
         <is>
-          <t>A bound role pointing at a non-existent database. scope.systemDatabase('hr') must throw; today code queries a ghost id and gets silence.</t>
+          <t>A bound role pointing at a non-existent database. scope.systemDatabase('hr') must throw; today code queries a ghost id and gets silence. | CONFIRMED 2026-09-27: it is the single missing logicalKey (31 of 32). Pass 2 could not repair it — idempotency by binding skips a bound-but-dangling role. Fixed by R1-1c.2.</t>
         </is>
       </c>
       <c r="H483" t="inlineStr">
@@ -22465,7 +22465,7 @@
       </c>
       <c r="B497" t="inlineStr">
         <is>
-          <t>PASS 3b: ESLint parse ratchet — 28 files grandfathered, length is the metric</t>
+          <t>PASS 3b SPLIT: 7a ratchet (ready now) · 7b conversions (blocked on the R1-1b migration)</t>
         </is>
       </c>
       <c r="C497" t="inlineStr">
@@ -22485,12 +22485,12 @@
       </c>
       <c r="F497" t="inlineStr">
         <is>
-          <t>coral-id-parsing-decomposition.md</t>
+          <t>coder-directive-kern-7a-parse-ratchet.md</t>
         </is>
       </c>
       <c r="G497" t="inlineStr">
         <is>
-          <t>74 parse sites across 28 files. Same mechanism as PRE-1d's prisma allowlist (121).</t>
+          <t>74 sites / 28 files. split('-') deliberately EXCLUDED from the rule: only 2 of its 9 sites parse a database id (both in lockedDbUtils.ts, deleted in 3c); the other 7 parse dates, projectCode and payment terms. A blanket ban would be 7 false positives — a rule that over-reaches gets disabled.</t>
         </is>
       </c>
       <c r="H497" t="inlineStr">
@@ -26355,6 +26355,147 @@
       <c r="I579" t="inlineStr">
         <is>
           <t>Projects</t>
+        </is>
+      </c>
+    </row>
+    <row r="580">
+      <c r="A580" t="inlineStr">
+        <is>
+          <t>KERN-7b</t>
+        </is>
+      </c>
+      <c r="B580" t="inlineStr">
+        <is>
+          <t>Convert the 74 parse sites to roleOfDatabase — batch by batch, allowlist falling</t>
+        </is>
+      </c>
+      <c r="C580" t="inlineStr">
+        <is>
+          <t>Kernel</t>
+        </is>
+      </c>
+      <c r="D580" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E580" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="F580" t="inlineStr">
+        <is>
+          <t>coder-directive-kern-7a-parse-ratchet.md</t>
+        </is>
+      </c>
+      <c r="G580" t="inlineStr">
+        <is>
+          <t>BLOCKED on Florin applying the R1-1b migration. roleOfDatabase reads logicalKey; until backfilled it returns null for every database and any conversion built on it is silently wrong. Confirm with: SELECT COUNT(*) FROM GlobalDatabase WHERE logicalKey IS NOT NULL -&gt; expect 32. | ALSO blocked on R1-1c: without the ongoing write, conversions break for every tenant provisioned after today.</t>
+        </is>
+      </c>
+      <c r="H580" t="inlineStr">
+        <is>
+          <t>L0 Kernel</t>
+        </is>
+      </c>
+      <c r="I580" t="inlineStr">
+        <is>
+          <t>Identity</t>
+        </is>
+      </c>
+    </row>
+    <row r="581">
+      <c r="A581" t="inlineStr">
+        <is>
+          <t>R1-1c</t>
+        </is>
+      </c>
+      <c r="B581" t="inlineStr">
+        <is>
+          <t>🔴 Provisioning does not write logicalKey — new tenants get the forward binding only</t>
+        </is>
+      </c>
+      <c r="C581" t="inlineStr">
+        <is>
+          <t>Kernel</t>
+        </is>
+      </c>
+      <c r="D581" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E581" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F581" t="inlineStr">
+        <is>
+          <t>coder-directive-r1-1c-provision-logicalkey.md</t>
+        </is>
+      </c>
+      <c r="G581" t="inlineStr">
+        <is>
+          <t>R1-1b landed the column and a one-time backfill, not the ongoing write. roleOfDatabase returns null for anything provisioned after today, so KERN-7b's conversions would be silently wrong for every new tenant. Two lines, atomic with the create.</t>
+        </is>
+      </c>
+      <c r="H581" t="inlineStr">
+        <is>
+          <t>L0 Kernel</t>
+        </is>
+      </c>
+      <c r="I581" t="inlineStr">
+        <is>
+          <t>Identity</t>
+        </is>
+      </c>
+    </row>
+    <row r="582">
+      <c r="A582" t="inlineStr">
+        <is>
+          <t>R1-1c.2</t>
+        </is>
+      </c>
+      <c r="B582" t="inlineStr">
+        <is>
+          <t>🔴 Idempotency-by-binding skips a BROKEN binding forever</t>
+        </is>
+      </c>
+      <c r="C582" t="inlineStr">
+        <is>
+          <t>Kernel</t>
+        </is>
+      </c>
+      <c r="D582" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E582" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F582" t="inlineStr">
+        <is>
+          <t>coder-directive-r1-1c-provision-logicalkey.md</t>
+        </is>
+      </c>
+      <c r="G582" t="inlineStr">
+        <is>
+          <t>This is how hr -&gt; db-hr survived KERN-5 pass 2: the binding existed so provisioning skipped it, and the id had no row. Measured: 31 keyed where 32 expected. Skip only if the bound id RESOLVES; otherwise provision a replacement and REPORT the repair.</t>
+        </is>
+      </c>
+      <c r="H582" t="inlineStr">
+        <is>
+          <t>L0 Kernel</t>
+        </is>
+      </c>
+      <c r="I582" t="inlineStr">
+        <is>
+          <t>Identity</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(kernel): KERN-7a parse ratchet ESLint rule and grandfathered allowlist
</commit_message>
<xml_diff>
--- a/.agents/coral-roadmap.xlsx
+++ b/.agents/coral-roadmap.xlsx
@@ -594,7 +594,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I582"/>
+  <dimension ref="A1:I583"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -10335,7 +10335,7 @@
       </c>
       <c r="E225" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F225" s="11" t="inlineStr">
@@ -10345,7 +10345,7 @@
       </c>
       <c r="G225" s="11" t="inlineStr">
         <is>
-          <t>CLARIFIED 2026-09-26: logicalKey is the REVERSE binding. Tenant.lockedDbIds answers role-&gt;id; NOTHING answers id-&gt;role, so every reverse-lookup site parses the id. That is the root of all 74 parse sites. Backfill from lockedDbIds (authoritative) — NEVER by parsing ids. @@unique([tenantId, logicalKey]). Moves EARLIER: it is the storage pass 3b spends.</t>
+          <t>CLARIFIED 2026-09-26: logicalKey is the REVERSE binding. Tenant.lockedDbIds answers role-&gt;id; NOTHING answers id-&gt;role, so every reverse-lookup site parses the id. That is the root of all 74 parse sites. Backfill from lockedDbIds (authoritative) — NEVER by parsing ids. @@unique([tenantId, logicalKey]). Moves EARLIER: it is the storage pass 3b spends. | logicalKey column + accessor landed 9ca8bb1; migration applied; 32 keyed.</t>
         </is>
       </c>
       <c r="H225" s="28" t="inlineStr">
@@ -21822,7 +21822,7 @@
       </c>
       <c r="E483" t="inlineStr">
         <is>
-          <t>Confirmed live</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F483" t="inlineStr">
@@ -21832,7 +21832,7 @@
       </c>
       <c r="G483" t="inlineStr">
         <is>
-          <t>A bound role pointing at a non-existent database. scope.systemDatabase('hr') must throw; today code queries a ghost id and gets silence. | CONFIRMED 2026-09-27: it is the single missing logicalKey (31 of 32). Pass 2 could not repair it — idempotency by binding skips a bound-but-dangling role. Fixed by R1-1c.2.</t>
+          <t>A bound role pointing at a non-existent database. scope.systemDatabase('hr') must throw; today code queries a ghost id and gets silence. | CONFIRMED 2026-09-27: it is the single missing logicalKey (31 of 32). Pass 2 could not repair it — idempotency by binding skips a bound-but-dangling role. Fixed by R1-1c.2. | CLOSED by R1-1c: hr repointed to an opaque cuid with logicalKey set.</t>
         </is>
       </c>
       <c r="H483" t="inlineStr">
@@ -24595,7 +24595,7 @@
       </c>
       <c r="E542" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F542" t="inlineStr">
@@ -24605,7 +24605,7 @@
       </c>
       <c r="G542" t="inlineStr">
         <is>
-          <t>Do this whatever is decided. Moves and repoints, no logic. Afterwards the module has 8 inbound imports and repair-vs-rebuild becomes reversible.</t>
+          <t>Do this whatever is decided. Moves and repoints, no logic. Afterwards the module has 8 inbound imports and repair-vs-rebuild becomes reversible. | Landed 1ea37cf — inbound imports 71 -&gt; 12.</t>
         </is>
       </c>
       <c r="H542" t="inlineStr">
@@ -25770,7 +25770,7 @@
       </c>
       <c r="E567" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F567" t="inlineStr">
@@ -25780,7 +25780,7 @@
       </c>
       <c r="G567" t="inlineStr">
         <is>
-          <t>api/portals/slug/[slug]/route.ts:129-136 returns tasks, linkedProjectData, QUOTES, INVOICES, budget and paidAmount, with hasPassword as a mere flag. The password is never verified in that route; portal/[slug]/page.tsx:30 does the gating. Anyone holding the link sees everything regardless of the password.</t>
+          <t>api/portals/slug/[slug]/route.ts:129-136 returns tasks, linkedProjectData, QUOTES, INVOICES, budget and paidAmount, with hasPassword as a mere flag. The password is never verified in that route; portal/[slug]/page.tsx:30 does the gating. Anyone holding the link sees everything regardless of the password. | Landed 7b79e36.</t>
         </is>
       </c>
       <c r="H567" t="inlineStr">
@@ -26287,7 +26287,7 @@
       </c>
       <c r="E578" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F578" t="inlineStr">
@@ -26297,7 +26297,7 @@
       </c>
       <c r="G578" t="inlineStr">
         <is>
-          <t>Blocks portal writes (no user by design), cron/webhook writes (TSC-3 systemScope), and impersonation tracking. The 'reason' column already anticipates system writes but there is nowhere to put the actor. Needs actorUserId String? + an actor KIND: user | system | portal | operator-impersonating. Serves portals, scheduled work and impersonation at once.</t>
+          <t>Blocks portal writes (no user by design), cron/webhook writes (TSC-3 systemScope), and impersonation tracking. The 'reason' column already anticipates system writes but there is nowhere to put the actor. Needs actorUserId String? + an actor KIND: user | system | portal | operator-impersonating. Serves portals, scheduled work and impersonation at once. | Landed f1ad3a9.</t>
         </is>
       </c>
       <c r="H578" t="inlineStr">
@@ -26334,7 +26334,7 @@
       </c>
       <c r="E579" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F579" t="inlineStr">
@@ -26344,7 +26344,7 @@
       </c>
       <c r="G579" t="inlineStr">
         <is>
-          <t>ProjectDetailView loads the tenant's ENTIRE clock-entry and shift history into the browser to compute one project's labour, and carries the last project_id fallback outside the time-tracker. Replaced by a server-side aggregate. Closes WH-5 and answers PROJ-6 from the core.</t>
+          <t>ProjectDetailView loads the tenant's ENTIRE clock-entry and shift history into the browser to compute one project's labour, and carries the last project_id fallback outside the time-tracker. Replaced by a server-side aggregate. Closes WH-5 and answers PROJ-6 from the core. | Landed ed7572d.</t>
         </is>
       </c>
       <c r="H579" t="inlineStr">
@@ -26381,17 +26381,17 @@
       </c>
       <c r="E580" t="inlineStr">
         <is>
-          <t>Blocked</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="F580" t="inlineStr">
         <is>
-          <t>coder-directive-kern-7a-parse-ratchet.md</t>
+          <t>coder-directive-kern-7b-conversions.md</t>
         </is>
       </c>
       <c r="G580" t="inlineStr">
         <is>
-          <t>BLOCKED on Florin applying the R1-1b migration. roleOfDatabase reads logicalKey; until backfilled it returns null for every database and any conversion built on it is silently wrong. Confirm with: SELECT COUNT(*) FROM GlobalDatabase WHERE logicalKey IS NOT NULL -&gt; expect 32. | ALSO blocked on R1-1c: without the ongoing write, conversions break for every tenant provisioned after today.</t>
+          <t>UNBLOCKED: logicalKey populated (32). Batch 0 = carry logicalKey to the client Database interface + every mapper (the query already returns it; a field-by-field mapper drops it). TRAP: getBaseDbId returns a BASE ID, logicalKey returns a ROLE — a swap that keeps the comparison string compiles and is always false. 7b.2 (pages.ts) is entitlement + the write path; 7b.5 (schema-cleanup) is destructive.</t>
         </is>
       </c>
       <c r="H580" t="inlineStr">
@@ -26428,7 +26428,7 @@
       </c>
       <c r="E581" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F581" t="inlineStr">
@@ -26438,7 +26438,7 @@
       </c>
       <c r="G581" t="inlineStr">
         <is>
-          <t>R1-1b landed the column and a one-time backfill, not the ongoing write. roleOfDatabase returns null for anything provisioned after today, so KERN-7b's conversions would be silently wrong for every new tenant. Two lines, atomic with the create.</t>
+          <t>R1-1b landed the column and a one-time backfill, not the ongoing write. roleOfDatabase returns null for anything provisioned after today, so KERN-7b's conversions would be silently wrong for every new tenant. Two lines, atomic with the create. | Landed 5ba9630. Repaired the dangling hr-&gt;db-hr binding on first page load; keyed count 31 -&gt; 32.</t>
         </is>
       </c>
       <c r="H581" t="inlineStr">
@@ -26475,7 +26475,7 @@
       </c>
       <c r="E582" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F582" t="inlineStr">
@@ -26485,7 +26485,7 @@
       </c>
       <c r="G582" t="inlineStr">
         <is>
-          <t>This is how hr -&gt; db-hr survived KERN-5 pass 2: the binding existed so provisioning skipped it, and the id had no row. Measured: 31 keyed where 32 expected. Skip only if the bound id RESOLVES; otherwise provision a replacement and REPORT the repair.</t>
+          <t>This is how hr -&gt; db-hr survived KERN-5 pass 2: the binding existed so provisioning skipped it, and the id had no row. Measured: 31 keyed where 32 expected. Skip only if the bound id RESOLVES; otherwise provision a replacement and REPORT the repair. | Landed — idempotency now verifies the bound id resolves.</t>
         </is>
       </c>
       <c r="H582" t="inlineStr">
@@ -26494,6 +26494,53 @@
         </is>
       </c>
       <c r="I582" t="inlineStr">
+        <is>
+          <t>Identity</t>
+        </is>
+      </c>
+    </row>
+    <row r="583">
+      <c r="A583" t="inlineStr">
+        <is>
+          <t>KERN-7b.0</t>
+        </is>
+      </c>
+      <c r="B583" t="inlineStr">
+        <is>
+          <t>Carry logicalKey across the server/client boundary — gates every conversion</t>
+        </is>
+      </c>
+      <c r="C583" t="inlineStr">
+        <is>
+          <t>Kernel</t>
+        </is>
+      </c>
+      <c r="D583" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E583" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F583" t="inlineStr">
+        <is>
+          <t>coder-directive-kern-7b-conversions.md</t>
+        </is>
+      </c>
+      <c r="G583" t="inlineStr">
+        <is>
+          <t>global-databases.ts findMany returns logicalKey (no select) and the field-by-field mapper drops it. Add it to the client Database interface and EVERY mapper (at least 2 findMany sites). A missed mapper yields undefined, which reads as 'custom database' and is silently wrong. Verify all 16 roles present, none undefined, BEFORE converting anything.</t>
+        </is>
+      </c>
+      <c r="H583" t="inlineStr">
+        <is>
+          <t>L1 Core</t>
+        </is>
+      </c>
+      <c r="I583" t="inlineStr">
         <is>
           <t>Identity</t>
         </is>

</xml_diff>

<commit_message>
fix(workhub): INC-1 restore shift snake_case bridge to unbreak production
</commit_message>
<xml_diff>
--- a/.agents/coral-roadmap.xlsx
+++ b/.agents/coral-roadmap.xlsx
@@ -594,7 +594,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I583"/>
+  <dimension ref="A1:I595"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -24652,7 +24652,7 @@
       </c>
       <c r="G543" t="inlineStr">
         <is>
-          <t>Planner recommends Step 1 then B: rewrite the 3 shift-editor files (3,508 lines, 22%) against the corrected kernel; repair the display layer in place. A = tail-chasing, C = premature (kernel mid-repair, PROJ-0 undecided, R1-4 four gates out).</t>
+          <t>Planner recommends Step 1 then B: rewrite the 3 shift-editor files (3,508 lines, 22%) against the corrected kernel; repair the display layer in place. A = tail-chasing, C = premature (kernel mid-repair, PROJ-0 undecided, R1-4 four gates out). | BETTER DECIDED AFTER TD-0: the real error count across 21 files is the missing input. A file needing 40 exceptions argues rebuild; one needing 3 argues repair.</t>
         </is>
       </c>
       <c r="H543" t="inlineStr">
@@ -24699,7 +24699,7 @@
       </c>
       <c r="G544" t="inlineStr">
         <is>
-          <t>Converting 40 files' field names is throwaway if those files are rewritten — the same 'fix it twice' argument made for GRID-REPLACE. Ratchet + WORKHUB-CLOCKLINK are kept; the batch march is parked.</t>
+          <t>Converting 40 files' field names is throwaway if those files are rewritten — the same 'fix it twice' argument made for GRID-REPLACE. Ratchet + WORKHUB-CLOCKLINK are kept; the batch march is parked. | OVERTAKEN 2026-09-28 by INC-1: the shift-consuming files are correctness work now, not tidying.</t>
         </is>
       </c>
       <c r="H544" t="inlineStr">
@@ -26381,7 +26381,7 @@
       </c>
       <c r="E580" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Paused</t>
         </is>
       </c>
       <c r="F580" t="inlineStr">
@@ -26391,7 +26391,7 @@
       </c>
       <c r="G580" t="inlineStr">
         <is>
-          <t>UNBLOCKED: logicalKey populated (32). Batch 0 = carry logicalKey to the client Database interface + every mapper (the query already returns it; a field-by-field mapper drops it). TRAP: getBaseDbId returns a BASE ID, logicalKey returns a ROLE — a swap that keeps the comparison string compiles and is always false. 7b.2 (pages.ts) is entitlement + the write path; 7b.5 (schema-cleanup) is destructive.</t>
+          <t>UNBLOCKED: logicalKey populated (32). Batch 0 = carry logicalKey to the client Database interface + every mapper (the query already returns it; a field-by-field mapper drops it). TRAP: getBaseDbId returns a BASE ID, logicalKey returns a ROLE — a swap that keeps the comparison string compiles and is always false. 7b.2 (pages.ts) is entitlement + the write path; 7b.5 (schema-cleanup) is destructive. | PAUSED until INC-1 closes — same tree, and two conversions in flight over one surface makes a revert impossible.</t>
         </is>
       </c>
       <c r="H580" t="inlineStr">
@@ -26543,6 +26543,570 @@
       <c r="I583" t="inlineStr">
         <is>
           <t>Identity</t>
+        </is>
+      </c>
+    </row>
+    <row r="584">
+      <c r="A584" t="inlineStr">
+        <is>
+          <t>INC-1</t>
+        </is>
+      </c>
+      <c r="B584" t="inlineStr">
+        <is>
+          <t>🔴 PRODUCTION BROKEN: shift_date write removed, 12 blind readers remain</t>
+        </is>
+      </c>
+      <c r="C584" t="inlineStr">
+        <is>
+          <t>Incident</t>
+        </is>
+      </c>
+      <c r="D584" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E584" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F584" t="inlineStr">
+        <is>
+          <t>coder-directive-shift-shape-incident.md</t>
+        </is>
+      </c>
+      <c r="G584" t="inlineStr">
+        <is>
+          <t>TypeError 'e.split' on the workhub for every tenant. addSnakeCase stopped writing shift_date/start/end; 12 @ts-nocheck files still read them. The one file tsc could see is the one that did not break.</t>
+        </is>
+      </c>
+      <c r="H584" t="inlineStr">
+        <is>
+          <t>L2 Module</t>
+        </is>
+      </c>
+      <c r="I584" t="inlineStr">
+        <is>
+          <t>WorkHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="585">
+      <c r="A585" t="inlineStr">
+        <is>
+          <t>PROC-1</t>
+        </is>
+      </c>
+      <c r="B585" t="inlineStr">
+        <is>
+          <t>🔴 ROOT: no gate between landed and live — main == develop, 0 commits apart</t>
+        </is>
+      </c>
+      <c r="C585" t="inlineStr">
+        <is>
+          <t>Process</t>
+        </is>
+      </c>
+      <c r="D585" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E585" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F585" t="inlineStr">
+        <is>
+          <t>coder-directive-shift-shape-incident.md</t>
+        </is>
+      </c>
+      <c r="G585" t="inlineStr">
+        <is>
+          <t>Every pass this week went straight to production. coral-promotion-plan.md describes a release branch, staging pass and 48h watch — none happened and nobody noticed it stopped. This is the only defect that made the others reach a user.</t>
+        </is>
+      </c>
+      <c r="H585" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I585" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="586">
+      <c r="A586" t="inlineStr">
+        <is>
+          <t>KERN-TIME</t>
+        </is>
+      </c>
+      <c r="B586" t="inlineStr">
+        <is>
+          <t>L0: shift time is TEXT, and stored two ways in one module</t>
+        </is>
+      </c>
+      <c r="C586" t="inlineStr">
+        <is>
+          <t>Kernel</t>
+        </is>
+      </c>
+      <c r="D586" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E586" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F586" t="inlineStr">
+        <is>
+          <t>coder-directive-shift-shape-incident.md</t>
+        </is>
+      </c>
+      <c r="G586" t="inlineStr">
+        <is>
+          <t>ScheduledShift.shiftDate/Start/End are String; ClockEntry.clockInTime is DateTime. 25 hand-parse sites (split('-')/split(':')) exist because the text form forces every consumer to parse. The kernel owns the arithmetic (computeWorkedDuration) but no TYPE. A kernel time type makes this crash class unrepresentable.</t>
+        </is>
+      </c>
+      <c r="H586" t="inlineStr">
+        <is>
+          <t>L0 Kernel</t>
+        </is>
+      </c>
+      <c r="I586" t="inlineStr">
+        <is>
+          <t>Time</t>
+        </is>
+      </c>
+    </row>
+    <row r="587">
+      <c r="A587" t="inlineStr">
+        <is>
+          <t>CORE-DTO</t>
+        </is>
+      </c>
+      <c r="B587" t="inlineStr">
+        <is>
+          <t>L1: nothing owns the record shape that crosses to a module</t>
+        </is>
+      </c>
+      <c r="C587" t="inlineStr">
+        <is>
+          <t>Kernel</t>
+        </is>
+      </c>
+      <c r="D587" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E587" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F587" t="inlineStr">
+        <is>
+          <t>coder-directive-shift-shape-incident.md</t>
+        </is>
+      </c>
+      <c r="G587" t="inlineStr">
+        <is>
+          <t>API returns Prisma camelCase; a CLIENT hook invents a second snake_case shape. A client file unilaterally defines the contract, so editing it changes production.</t>
+        </is>
+      </c>
+      <c r="H587" t="inlineStr">
+        <is>
+          <t>L1 Core</t>
+        </is>
+      </c>
+      <c r="I587" t="inlineStr">
+        <is>
+          <t>Write path</t>
+        </is>
+      </c>
+    </row>
+    <row r="588">
+      <c r="A588" t="inlineStr">
+        <is>
+          <t>PLAN-4</t>
+        </is>
+      </c>
+      <c r="B588" t="inlineStr">
+        <is>
+          <t>Planner treated @ts-nocheck as debt, not as an INTERLOCK</t>
+        </is>
+      </c>
+      <c r="C588" t="inlineStr">
+        <is>
+          <t>Process</t>
+        </is>
+      </c>
+      <c r="D588" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E588" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F588" t="inlineStr">
+        <is>
+          <t>coder-directive-shift-shape-incident.md</t>
+        </is>
+      </c>
+      <c r="G588" t="inlineStr">
+        <is>
+          <t>While a file carries @ts-nocheck its reads are unverifiable, so the data it consumes must not change. Refused the coder's proposal to restore the aliases on type-purity grounds — the type declarations were safe to remove, the writes were not. New rule: a write may be removed only in the commit that converts its readers.</t>
+        </is>
+      </c>
+      <c r="H588" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I588" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="589">
+      <c r="A589" t="inlineStr">
+        <is>
+          <t>TD-0</t>
+        </is>
+      </c>
+      <c r="B589" t="inlineStr">
+        <is>
+          <t>MEASURE: lift all 37 directives on a scratch branch, count, categorise, revert</t>
+        </is>
+      </c>
+      <c r="C589" t="inlineStr">
+        <is>
+          <t>Type debt</t>
+        </is>
+      </c>
+      <c r="D589" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E589" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F589" t="inlineStr">
+        <is>
+          <t>coral-typecheck-debt-plan.md</t>
+        </is>
+      </c>
+      <c r="G589" t="inlineStr">
+        <is>
+          <t>The only honest input to sequencing. Per file, by category: casing rename / semantic mapping / phantom field / real bug / type debt. Fix nothing. One file gave 24 errors — do not extrapolate.</t>
+        </is>
+      </c>
+      <c r="H589" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I589" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="590">
+      <c r="A590" t="inlineStr">
+        <is>
+          <t>TD-1</t>
+        </is>
+      </c>
+      <c r="B590" t="inlineStr">
+        <is>
+          <t>🔴 REAL BUGS found under @ts-nocheck — fix immediately, each its own commit</t>
+        </is>
+      </c>
+      <c r="C590" t="inlineStr">
+        <is>
+          <t>Type debt</t>
+        </is>
+      </c>
+      <c r="D590" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E590" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F590" t="inlineStr">
+        <is>
+          <t>coral-typecheck-debt-plan.md</t>
+        </is>
+      </c>
+      <c r="G590" t="inlineStr">
+        <is>
+          <t>EditShiftDialog:785 'Cannot find name fileInputRef' — an undefined variable in shipping code, a crash if that path runs. Plus a missing ProjectAttachment export. These are why the plan is urgent rather than tidy.</t>
+        </is>
+      </c>
+      <c r="H590" t="inlineStr">
+        <is>
+          <t>L2 Module</t>
+        </is>
+      </c>
+      <c r="I590" t="inlineStr">
+        <is>
+          <t>WorkHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="591">
+      <c r="A591" t="inlineStr">
+        <is>
+          <t>TD-2</t>
+        </is>
+      </c>
+      <c r="B591" t="inlineStr">
+        <is>
+          <t>PHANTOM FIELDS: reads of fields that exist in no model</t>
+        </is>
+      </c>
+      <c r="C591" t="inlineStr">
+        <is>
+          <t>Type debt</t>
+        </is>
+      </c>
+      <c r="D591" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E591" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F591" t="inlineStr">
+        <is>
+          <t>coral-typecheck-debt-plan.md</t>
+        </is>
+      </c>
+      <c r="G591" t="inlineStr">
+        <is>
+          <t>source_project_id is read on ScheduleAttachment and exists in neither Prisma nor the client type — the feature it drives is already dead. Implement or delete. NEVER rename a phantom.</t>
+        </is>
+      </c>
+      <c r="H591" t="inlineStr">
+        <is>
+          <t>L2 Module</t>
+        </is>
+      </c>
+      <c r="I591" t="inlineStr">
+        <is>
+          <t>WorkHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="592">
+      <c r="A592" t="inlineStr">
+        <is>
+          <t>TD-3</t>
+        </is>
+      </c>
+      <c r="B592" t="inlineStr">
+        <is>
+          <t>@ts-nocheck → line-level @ts-expect-error, one file per commit</t>
+        </is>
+      </c>
+      <c r="C592" t="inlineStr">
+        <is>
+          <t>Type debt</t>
+        </is>
+      </c>
+      <c r="D592" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E592" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F592" t="inlineStr">
+        <is>
+          <t>coral-typecheck-debt-plan.md</t>
+        </is>
+      </c>
+      <c r="G592" t="inlineStr">
+        <is>
+          <t>THE CORE MOVE. Blanket silence makes readers unenumerable — that is INC-1. Line-level makes them greppable and countable WITHOUT converting one. The file becomes type-checked immediately; a new error fails the build. Order: fewest errors first.</t>
+        </is>
+      </c>
+      <c r="H592" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I592" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="593">
+      <c r="A593" t="inlineStr">
+        <is>
+          <t>TD-4</t>
+        </is>
+      </c>
+      <c r="B593" t="inlineStr">
+        <is>
+          <t>Convert by CATEGORY, not by file — casing in bulk, semantic one at a time</t>
+        </is>
+      </c>
+      <c r="C593" t="inlineStr">
+        <is>
+          <t>Type debt</t>
+        </is>
+      </c>
+      <c r="D593" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E593" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F593" t="inlineStr">
+        <is>
+          <t>coral-typecheck-debt-plan.md</t>
+        </is>
+      </c>
+      <c r="G593" t="inlineStr">
+        <is>
+          <t>file_path → ShiftAttachment.url is a semantic mapping, not a rename. No find-and-replace ever (the full_name lesson). Each converted read deletes its @ts-expect-error — and a stale expect-error FAILS the build, so the ratchet maintains itself.</t>
+        </is>
+      </c>
+      <c r="H593" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I593" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="594">
+      <c r="A594" t="inlineStr">
+        <is>
+          <t>TD-5</t>
+        </is>
+      </c>
+      <c r="B594" t="inlineStr">
+        <is>
+          <t>RULE: a write is removed only in the commit that converts its LAST reader</t>
+        </is>
+      </c>
+      <c r="C594" t="inlineStr">
+        <is>
+          <t>Type debt</t>
+        </is>
+      </c>
+      <c r="D594" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E594" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F594" t="inlineStr">
+        <is>
+          <t>coral-typecheck-debt-plan.md</t>
+        </is>
+      </c>
+      <c r="G594" t="inlineStr">
+        <is>
+          <t>Readers become countable via grep on the @ts-expect-error comments. Zero readers, then the write goes. 'Strip the type, remove the write, convert later' is INC-1 stated as a sentence.</t>
+        </is>
+      </c>
+      <c r="H594" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I594" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="595">
+      <c r="A595" t="inlineStr">
+        <is>
+          <t>TD-6</t>
+        </is>
+      </c>
+      <c r="B595" t="inlineStr">
+        <is>
+          <t>RATCHET: @ts-nocheck forbidden by ESLint, 21 files grandfathered, allowlist only falls</t>
+        </is>
+      </c>
+      <c r="C595" t="inlineStr">
+        <is>
+          <t>Type debt</t>
+        </is>
+      </c>
+      <c r="D595" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E595" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F595" t="inlineStr">
+        <is>
+          <t>coral-typecheck-debt-plan.md</t>
+        </is>
+      </c>
+      <c r="G595" t="inlineStr">
+        <is>
+          <t>ban-ts-comment already warns; make nocheck an error. Two monotonic numbers: files unchecked -&gt; 0, expected errors -&gt; 0.</t>
+        </is>
+      </c>
+      <c r="H595" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I595" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(time-tracker): TD-1 resolve latent bugs uncovered by typecheck surface measurement
- EditShiftDialog: declare fileInputRef and attach to file input element
- AllSchedulesView: fix undefined employeeMap to use worker.full_name
- useApprovalRequests: support parameters in createRequest signature
- useScheduleAttachments: export ProjectAttachment interface
- useWorkerSchedules: implement upsertSchedule, toggleScheduleActive, and profile aliases
- useTimeOffRequests: implement fetchRequests, refetch, and deleteRequest
- usePushNotifications: provide permission and error properties
- CreateShiftForm: safe cast on onCreateShift result data access
</commit_message>
<xml_diff>
--- a/.agents/coral-roadmap.xlsx
+++ b/.agents/coral-roadmap.xlsx
@@ -20521,12 +20521,12 @@
       </c>
       <c r="H455" t="inlineStr">
         <is>
-          <t>L1 Core</t>
+          <t>GATE</t>
         </is>
       </c>
       <c r="I455" t="inlineStr">
         <is>
-          <t>Tenant gate</t>
+          <t>the seraph — resolver, logicalKey, scoped accessor</t>
         </is>
       </c>
     </row>
@@ -20568,12 +20568,12 @@
       </c>
       <c r="H456" t="inlineStr">
         <is>
-          <t>L1 Core</t>
+          <t>GATE</t>
         </is>
       </c>
       <c r="I456" t="inlineStr">
         <is>
-          <t>Tenant gate</t>
+          <t>the seraph — resolver, logicalKey, scoped accessor</t>
         </is>
       </c>
     </row>
@@ -20615,12 +20615,12 @@
       </c>
       <c r="H457" t="inlineStr">
         <is>
-          <t>L1 Core</t>
+          <t>GATE</t>
         </is>
       </c>
       <c r="I457" t="inlineStr">
         <is>
-          <t>Tenant gate</t>
+          <t>the seraph — resolver, logicalKey, scoped accessor</t>
         </is>
       </c>
     </row>
@@ -20662,12 +20662,12 @@
       </c>
       <c r="H458" t="inlineStr">
         <is>
-          <t>L0 Kernel</t>
+          <t>L0</t>
         </is>
       </c>
       <c r="I458" t="inlineStr">
         <is>
-          <t>Storage</t>
+          <t>storage — the one blob door</t>
         </is>
       </c>
     </row>
@@ -20709,7 +20709,7 @@
       </c>
       <c r="H459" t="inlineStr">
         <is>
-          <t>L2 Module</t>
+          <t>L2</t>
         </is>
       </c>
       <c r="I459" t="inlineStr">
@@ -20756,12 +20756,12 @@
       </c>
       <c r="H460" t="inlineStr">
         <is>
-          <t>L1 Core</t>
+          <t>GATE</t>
         </is>
       </c>
       <c r="I460" t="inlineStr">
         <is>
-          <t>Tenant gate</t>
+          <t>the seraph — resolver, logicalKey, scoped accessor</t>
         </is>
       </c>
     </row>
@@ -20803,7 +20803,7 @@
       </c>
       <c r="H461" t="inlineStr">
         <is>
-          <t>L2 Module</t>
+          <t>L2</t>
         </is>
       </c>
       <c r="I461" t="inlineStr">
@@ -20850,12 +20850,12 @@
       </c>
       <c r="H462" t="inlineStr">
         <is>
-          <t>L1 Core</t>
+          <t>L1</t>
         </is>
       </c>
       <c r="I462" t="inlineStr">
         <is>
-          <t>Resolution</t>
+          <t>identity — ids, roles, bindings</t>
         </is>
       </c>
     </row>
@@ -20897,7 +20897,7 @@
       </c>
       <c r="H463" t="inlineStr">
         <is>
-          <t>L2 Module</t>
+          <t>L2</t>
         </is>
       </c>
       <c r="I463" t="inlineStr">
@@ -20944,7 +20944,7 @@
       </c>
       <c r="H464" t="inlineStr">
         <is>
-          <t>L2 Module</t>
+          <t>L2</t>
         </is>
       </c>
       <c r="I464" t="inlineStr">
@@ -20991,7 +20991,7 @@
       </c>
       <c r="H465" t="inlineStr">
         <is>
-          <t>L2 Module</t>
+          <t>L2</t>
         </is>
       </c>
       <c r="I465" t="inlineStr">
@@ -21038,7 +21038,7 @@
       </c>
       <c r="H466" t="inlineStr">
         <is>
-          <t>L2 Module</t>
+          <t>L2</t>
         </is>
       </c>
       <c r="I466" t="inlineStr">
@@ -21085,12 +21085,12 @@
       </c>
       <c r="H467" t="inlineStr">
         <is>
-          <t>L1 Core</t>
+          <t>GATE</t>
         </is>
       </c>
       <c r="I467" t="inlineStr">
         <is>
-          <t>Tenant gate</t>
+          <t>the seraph — resolver, logicalKey, scoped accessor</t>
         </is>
       </c>
     </row>
@@ -21132,12 +21132,12 @@
       </c>
       <c r="H468" t="inlineStr">
         <is>
-          <t>L1 Core</t>
+          <t>GATE</t>
         </is>
       </c>
       <c r="I468" t="inlineStr">
         <is>
-          <t>Tenant gate</t>
+          <t>the seraph — resolver, logicalKey, scoped accessor</t>
         </is>
       </c>
     </row>
@@ -21179,12 +21179,12 @@
       </c>
       <c r="H469" t="inlineStr">
         <is>
-          <t>L1 Core</t>
+          <t>GATE</t>
         </is>
       </c>
       <c r="I469" t="inlineStr">
         <is>
-          <t>Tenant gate</t>
+          <t>the seraph — resolver, logicalKey, scoped accessor</t>
         </is>
       </c>
     </row>
@@ -21226,12 +21226,12 @@
       </c>
       <c r="H470" t="inlineStr">
         <is>
-          <t>L1 Core</t>
+          <t>L1</t>
         </is>
       </c>
       <c r="I470" t="inlineStr">
         <is>
-          <t>Refusals</t>
+          <t>refusals — visible, never swallowed</t>
         </is>
       </c>
     </row>
@@ -21273,12 +21273,12 @@
       </c>
       <c r="H471" t="inlineStr">
         <is>
-          <t>L1 Core</t>
+          <t>GATE</t>
         </is>
       </c>
       <c r="I471" t="inlineStr">
         <is>
-          <t>Tenant gate</t>
+          <t>the seraph — resolver, logicalKey, scoped accessor</t>
         </is>
       </c>
     </row>
@@ -21320,12 +21320,12 @@
       </c>
       <c r="H472" t="inlineStr">
         <is>
-          <t>L1 Core</t>
+          <t>GATE</t>
         </is>
       </c>
       <c r="I472" t="inlineStr">
         <is>
-          <t>Tenant gate</t>
+          <t>the seraph — resolver, logicalKey, scoped accessor</t>
         </is>
       </c>
     </row>
@@ -21367,7 +21367,7 @@
       </c>
       <c r="H473" t="inlineStr">
         <is>
-          <t>L2 Module</t>
+          <t>L2</t>
         </is>
       </c>
       <c r="I473" t="inlineStr">
@@ -21414,12 +21414,12 @@
       </c>
       <c r="H474" t="inlineStr">
         <is>
-          <t>L1 Core</t>
+          <t>GATE</t>
         </is>
       </c>
       <c r="I474" t="inlineStr">
         <is>
-          <t>Tenant gate</t>
+          <t>the seraph — resolver, logicalKey, scoped accessor</t>
         </is>
       </c>
     </row>
@@ -21461,7 +21461,7 @@
       </c>
       <c r="H475" t="inlineStr">
         <is>
-          <t>L2 Module</t>
+          <t>L2</t>
         </is>
       </c>
       <c r="I475" t="inlineStr">
@@ -21508,7 +21508,7 @@
       </c>
       <c r="H476" t="inlineStr">
         <is>
-          <t>L2 Module</t>
+          <t>L2</t>
         </is>
       </c>
       <c r="I476" t="inlineStr">
@@ -21555,12 +21555,12 @@
       </c>
       <c r="H477" t="inlineStr">
         <is>
-          <t>L0 Kernel</t>
+          <t>L0</t>
         </is>
       </c>
       <c r="I477" t="inlineStr">
         <is>
-          <t>Identity</t>
+          <t>identity — ids, roles, bindings</t>
         </is>
       </c>
     </row>
@@ -21602,12 +21602,12 @@
       </c>
       <c r="H478" t="inlineStr">
         <is>
-          <t>L0 Kernel</t>
+          <t>L0</t>
         </is>
       </c>
       <c r="I478" t="inlineStr">
         <is>
-          <t>Identity</t>
+          <t>identity — ids, roles, bindings</t>
         </is>
       </c>
     </row>
@@ -21649,12 +21649,12 @@
       </c>
       <c r="H479" t="inlineStr">
         <is>
-          <t>L0 Kernel</t>
+          <t>L0</t>
         </is>
       </c>
       <c r="I479" t="inlineStr">
         <is>
-          <t>Identity</t>
+          <t>identity — ids, roles, bindings</t>
         </is>
       </c>
     </row>
@@ -21696,12 +21696,12 @@
       </c>
       <c r="H480" t="inlineStr">
         <is>
-          <t>L0 Kernel</t>
+          <t>L0</t>
         </is>
       </c>
       <c r="I480" t="inlineStr">
         <is>
-          <t>Identity</t>
+          <t>identity — ids, roles, bindings</t>
         </is>
       </c>
     </row>
@@ -21743,12 +21743,12 @@
       </c>
       <c r="H481" t="inlineStr">
         <is>
-          <t>L1 Core</t>
+          <t>GATE</t>
         </is>
       </c>
       <c r="I481" t="inlineStr">
         <is>
-          <t>Tenant gate</t>
+          <t>the seraph — resolver, logicalKey, scoped accessor</t>
         </is>
       </c>
     </row>
@@ -21790,12 +21790,12 @@
       </c>
       <c r="H482" t="inlineStr">
         <is>
-          <t>L0 Kernel</t>
+          <t>L0</t>
         </is>
       </c>
       <c r="I482" t="inlineStr">
         <is>
-          <t>Identity</t>
+          <t>identity — ids, roles, bindings</t>
         </is>
       </c>
     </row>
@@ -21837,12 +21837,12 @@
       </c>
       <c r="H483" t="inlineStr">
         <is>
-          <t>L0 Kernel</t>
+          <t>L0</t>
         </is>
       </c>
       <c r="I483" t="inlineStr">
         <is>
-          <t>Identity</t>
+          <t>identity — ids, roles, bindings</t>
         </is>
       </c>
     </row>
@@ -21884,12 +21884,12 @@
       </c>
       <c r="H484" t="inlineStr">
         <is>
-          <t>L0 Kernel</t>
+          <t>L0</t>
         </is>
       </c>
       <c r="I484" t="inlineStr">
         <is>
-          <t>Identity</t>
+          <t>identity — ids, roles, bindings</t>
         </is>
       </c>
     </row>
@@ -21931,12 +21931,12 @@
       </c>
       <c r="H485" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>⟂</t>
         </is>
       </c>
       <c r="I485" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>process &amp; housekeeping</t>
         </is>
       </c>
     </row>
@@ -21978,12 +21978,12 @@
       </c>
       <c r="H486" t="inlineStr">
         <is>
-          <t>L0 Kernel</t>
+          <t>L0</t>
         </is>
       </c>
       <c r="I486" t="inlineStr">
         <is>
-          <t>Identity</t>
+          <t>identity — ids, roles, bindings</t>
         </is>
       </c>
     </row>
@@ -22025,12 +22025,12 @@
       </c>
       <c r="H487" t="inlineStr">
         <is>
-          <t>L0 Kernel</t>
+          <t>L0</t>
         </is>
       </c>
       <c r="I487" t="inlineStr">
         <is>
-          <t>Identity</t>
+          <t>identity — ids, roles, bindings</t>
         </is>
       </c>
     </row>
@@ -22072,12 +22072,12 @@
       </c>
       <c r="H488" t="inlineStr">
         <is>
-          <t>L0 Kernel</t>
+          <t>L0</t>
         </is>
       </c>
       <c r="I488" t="inlineStr">
         <is>
-          <t>Identity</t>
+          <t>identity — ids, roles, bindings</t>
         </is>
       </c>
     </row>
@@ -22119,12 +22119,12 @@
       </c>
       <c r="H489" t="inlineStr">
         <is>
-          <t>L0 Kernel</t>
+          <t>L0</t>
         </is>
       </c>
       <c r="I489" t="inlineStr">
         <is>
-          <t>Identity</t>
+          <t>identity — ids, roles, bindings</t>
         </is>
       </c>
     </row>
@@ -22166,7 +22166,7 @@
       </c>
       <c r="H490" t="inlineStr">
         <is>
-          <t>L1 Core</t>
+          <t>L1</t>
         </is>
       </c>
       <c r="I490" t="inlineStr">
@@ -22213,12 +22213,12 @@
       </c>
       <c r="H491" t="inlineStr">
         <is>
-          <t>L0 Kernel</t>
+          <t>L0</t>
         </is>
       </c>
       <c r="I491" t="inlineStr">
         <is>
-          <t>Identity</t>
+          <t>identity — ids, roles, bindings</t>
         </is>
       </c>
     </row>
@@ -22260,12 +22260,12 @@
       </c>
       <c r="H492" t="inlineStr">
         <is>
-          <t>L0 Kernel</t>
+          <t>L0</t>
         </is>
       </c>
       <c r="I492" t="inlineStr">
         <is>
-          <t>Identity</t>
+          <t>identity — ids, roles, bindings</t>
         </is>
       </c>
     </row>
@@ -22307,12 +22307,12 @@
       </c>
       <c r="H493" t="inlineStr">
         <is>
-          <t>L0 Kernel</t>
+          <t>L0</t>
         </is>
       </c>
       <c r="I493" t="inlineStr">
         <is>
-          <t>Identity</t>
+          <t>identity — ids, roles, bindings</t>
         </is>
       </c>
     </row>
@@ -22354,12 +22354,12 @@
       </c>
       <c r="H494" t="inlineStr">
         <is>
-          <t>L0 Kernel</t>
+          <t>L0</t>
         </is>
       </c>
       <c r="I494" t="inlineStr">
         <is>
-          <t>Identity</t>
+          <t>identity — ids, roles, bindings</t>
         </is>
       </c>
     </row>
@@ -22401,12 +22401,12 @@
       </c>
       <c r="H495" t="inlineStr">
         <is>
-          <t>L0 Kernel</t>
+          <t>L0</t>
         </is>
       </c>
       <c r="I495" t="inlineStr">
         <is>
-          <t>Identity</t>
+          <t>identity — ids, roles, bindings</t>
         </is>
       </c>
     </row>
@@ -22448,12 +22448,12 @@
       </c>
       <c r="H496" t="inlineStr">
         <is>
-          <t>L1 Core</t>
+          <t>MODULE GATE</t>
         </is>
       </c>
       <c r="I496" t="inlineStr">
         <is>
-          <t>Entitlement</t>
+          <t>entitlement — vocabulary &amp; grants</t>
         </is>
       </c>
     </row>
@@ -22495,12 +22495,12 @@
       </c>
       <c r="H497" t="inlineStr">
         <is>
-          <t>L0 Kernel</t>
+          <t>L0</t>
         </is>
       </c>
       <c r="I497" t="inlineStr">
         <is>
-          <t>Identity</t>
+          <t>identity — ids, roles, bindings</t>
         </is>
       </c>
     </row>
@@ -22542,12 +22542,12 @@
       </c>
       <c r="H498" t="inlineStr">
         <is>
-          <t>L0 Kernel</t>
+          <t>L0</t>
         </is>
       </c>
       <c r="I498" t="inlineStr">
         <is>
-          <t>Identity</t>
+          <t>identity — ids, roles, bindings</t>
         </is>
       </c>
     </row>
@@ -22589,12 +22589,12 @@
       </c>
       <c r="H499" t="inlineStr">
         <is>
-          <t>L1 Core</t>
+          <t>L1</t>
         </is>
       </c>
       <c r="I499" t="inlineStr">
         <is>
-          <t>Relations</t>
+          <t>relations — targets &amp; resolution</t>
         </is>
       </c>
     </row>
@@ -22636,12 +22636,12 @@
       </c>
       <c r="H500" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>⟂</t>
         </is>
       </c>
       <c r="I500" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>process &amp; housekeeping</t>
         </is>
       </c>
     </row>
@@ -22683,12 +22683,12 @@
       </c>
       <c r="H501" t="inlineStr">
         <is>
-          <t>L1 Core</t>
+          <t>L1</t>
         </is>
       </c>
       <c r="I501" t="inlineStr">
         <is>
-          <t>Relations</t>
+          <t>relations — targets &amp; resolution</t>
         </is>
       </c>
     </row>
@@ -22730,12 +22730,12 @@
       </c>
       <c r="H502" t="inlineStr">
         <is>
-          <t>L1 Core</t>
+          <t>L1</t>
         </is>
       </c>
       <c r="I502" t="inlineStr">
         <is>
-          <t>Relations</t>
+          <t>relations — targets &amp; resolution</t>
         </is>
       </c>
     </row>
@@ -22777,12 +22777,12 @@
       </c>
       <c r="H503" t="inlineStr">
         <is>
-          <t>L0 Kernel</t>
+          <t>L0</t>
         </is>
       </c>
       <c r="I503" t="inlineStr">
         <is>
-          <t>Identity</t>
+          <t>identity — ids, roles, bindings</t>
         </is>
       </c>
     </row>
@@ -22824,12 +22824,12 @@
       </c>
       <c r="H504" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>⟂</t>
         </is>
       </c>
       <c r="I504" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>process &amp; housekeeping</t>
         </is>
       </c>
     </row>
@@ -22871,12 +22871,12 @@
       </c>
       <c r="H505" t="inlineStr">
         <is>
-          <t>L1 Core</t>
+          <t>GATE</t>
         </is>
       </c>
       <c r="I505" t="inlineStr">
         <is>
-          <t>Tenant gate</t>
+          <t>the seraph — resolver, logicalKey, scoped accessor</t>
         </is>
       </c>
     </row>
@@ -22918,12 +22918,12 @@
       </c>
       <c r="H506" t="inlineStr">
         <is>
-          <t>L1 Core</t>
+          <t>MODULE GATE</t>
         </is>
       </c>
       <c r="I506" t="inlineStr">
         <is>
-          <t>Entitlement</t>
+          <t>entitlement — vocabulary &amp; grants</t>
         </is>
       </c>
     </row>
@@ -22965,12 +22965,12 @@
       </c>
       <c r="H507" t="inlineStr">
         <is>
-          <t>L2 Module</t>
+          <t>L2</t>
         </is>
       </c>
       <c r="I507" t="inlineStr">
         <is>
-          <t>CRM</t>
+          <t>CRM / pipeline</t>
         </is>
       </c>
     </row>
@@ -23012,12 +23012,12 @@
       </c>
       <c r="H508" t="inlineStr">
         <is>
-          <t>L1 Core</t>
+          <t>MODULE GATE</t>
         </is>
       </c>
       <c r="I508" t="inlineStr">
         <is>
-          <t>Entitlement</t>
+          <t>entitlement — vocabulary &amp; grants</t>
         </is>
       </c>
     </row>
@@ -23059,12 +23059,12 @@
       </c>
       <c r="H509" t="inlineStr">
         <is>
-          <t>L1 Core</t>
+          <t>MODULE GATE</t>
         </is>
       </c>
       <c r="I509" t="inlineStr">
         <is>
-          <t>Entitlement</t>
+          <t>entitlement — vocabulary &amp; grants</t>
         </is>
       </c>
     </row>
@@ -23106,12 +23106,12 @@
       </c>
       <c r="H510" t="inlineStr">
         <is>
-          <t>L2 Module</t>
+          <t>L2</t>
         </is>
       </c>
       <c r="I510" t="inlineStr">
         <is>
-          <t>Invoicing</t>
+          <t>Finance — invoicing</t>
         </is>
       </c>
     </row>
@@ -23153,12 +23153,12 @@
       </c>
       <c r="H511" t="inlineStr">
         <is>
-          <t>L1 Core</t>
+          <t>MODULE GATE</t>
         </is>
       </c>
       <c r="I511" t="inlineStr">
         <is>
-          <t>Entitlement</t>
+          <t>entitlement — vocabulary &amp; grants</t>
         </is>
       </c>
     </row>
@@ -23200,12 +23200,12 @@
       </c>
       <c r="H512" t="inlineStr">
         <is>
-          <t>L1 Core</t>
+          <t>MODULE GATE</t>
         </is>
       </c>
       <c r="I512" t="inlineStr">
         <is>
-          <t>Entitlement</t>
+          <t>entitlement — vocabulary &amp; grants</t>
         </is>
       </c>
     </row>
@@ -23247,12 +23247,12 @@
       </c>
       <c r="H513" t="inlineStr">
         <is>
-          <t>L0 Kernel</t>
+          <t>L0</t>
         </is>
       </c>
       <c r="I513" t="inlineStr">
         <is>
-          <t>Entitlement</t>
+          <t>entitlement — vocabulary &amp; grants</t>
         </is>
       </c>
     </row>
@@ -23294,12 +23294,12 @@
       </c>
       <c r="H514" t="inlineStr">
         <is>
-          <t>L0 Kernel</t>
+          <t>L0</t>
         </is>
       </c>
       <c r="I514" t="inlineStr">
         <is>
-          <t>Entitlement</t>
+          <t>entitlement — vocabulary &amp; grants</t>
         </is>
       </c>
     </row>
@@ -23341,12 +23341,12 @@
       </c>
       <c r="H515" t="inlineStr">
         <is>
-          <t>L0 Kernel</t>
+          <t>L0</t>
         </is>
       </c>
       <c r="I515" t="inlineStr">
         <is>
-          <t>Entitlement</t>
+          <t>entitlement — vocabulary &amp; grants</t>
         </is>
       </c>
     </row>
@@ -23388,12 +23388,12 @@
       </c>
       <c r="H516" t="inlineStr">
         <is>
-          <t>L2 Module</t>
+          <t>L2</t>
         </is>
       </c>
       <c r="I516" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>shells &amp; navigation — WorkHubShell</t>
         </is>
       </c>
     </row>
@@ -23435,12 +23435,12 @@
       </c>
       <c r="H517" t="inlineStr">
         <is>
-          <t>L0 Kernel</t>
+          <t>L0</t>
         </is>
       </c>
       <c r="I517" t="inlineStr">
         <is>
-          <t>Entitlement</t>
+          <t>entitlement — vocabulary &amp; grants</t>
         </is>
       </c>
     </row>
@@ -23482,12 +23482,12 @@
       </c>
       <c r="H518" t="inlineStr">
         <is>
-          <t>L0 Kernel</t>
+          <t>L0</t>
         </is>
       </c>
       <c r="I518" t="inlineStr">
         <is>
-          <t>Entitlement</t>
+          <t>entitlement — vocabulary &amp; grants</t>
         </is>
       </c>
     </row>
@@ -23529,12 +23529,12 @@
       </c>
       <c r="H519" t="inlineStr">
         <is>
-          <t>L0 Kernel</t>
+          <t>L0</t>
         </is>
       </c>
       <c r="I519" t="inlineStr">
         <is>
-          <t>Entitlement</t>
+          <t>entitlement — vocabulary &amp; grants</t>
         </is>
       </c>
     </row>
@@ -23576,12 +23576,12 @@
       </c>
       <c r="H520" t="inlineStr">
         <is>
-          <t>L1 Core</t>
+          <t>MODULE GATE</t>
         </is>
       </c>
       <c r="I520" t="inlineStr">
         <is>
-          <t>Entitlement</t>
+          <t>entitlement — vocabulary &amp; grants</t>
         </is>
       </c>
     </row>
@@ -23623,12 +23623,12 @@
       </c>
       <c r="H521" t="inlineStr">
         <is>
-          <t>L2 Module</t>
+          <t>L2</t>
         </is>
       </c>
       <c r="I521" t="inlineStr">
         <is>
-          <t>Entitlement</t>
+          <t>entitlement — vocabulary &amp; grants</t>
         </is>
       </c>
     </row>
@@ -23670,12 +23670,12 @@
       </c>
       <c r="H522" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>⟂</t>
         </is>
       </c>
       <c r="I522" t="inlineStr">
         <is>
-          <t>Pricing</t>
+          <t>pricing &amp; tiers</t>
         </is>
       </c>
     </row>
@@ -23717,12 +23717,12 @@
       </c>
       <c r="H523" t="inlineStr">
         <is>
-          <t>L0 Kernel</t>
+          <t>L0</t>
         </is>
       </c>
       <c r="I523" t="inlineStr">
         <is>
-          <t>Entitlement</t>
+          <t>entitlement — vocabulary &amp; grants</t>
         </is>
       </c>
     </row>
@@ -23764,12 +23764,12 @@
       </c>
       <c r="H524" t="inlineStr">
         <is>
-          <t>L1 Core</t>
+          <t>MODULE GATE</t>
         </is>
       </c>
       <c r="I524" t="inlineStr">
         <is>
-          <t>Entitlement</t>
+          <t>entitlement — vocabulary &amp; grants</t>
         </is>
       </c>
     </row>
@@ -23811,12 +23811,12 @@
       </c>
       <c r="H525" t="inlineStr">
         <is>
-          <t>L1 Core</t>
+          <t>MODULE GATE</t>
         </is>
       </c>
       <c r="I525" t="inlineStr">
         <is>
-          <t>Entitlement</t>
+          <t>entitlement — vocabulary &amp; grants</t>
         </is>
       </c>
     </row>
@@ -23858,12 +23858,12 @@
       </c>
       <c r="H526" t="inlineStr">
         <is>
-          <t>L1 Core</t>
+          <t>MODULE GATE</t>
         </is>
       </c>
       <c r="I526" t="inlineStr">
         <is>
-          <t>Entitlement</t>
+          <t>entitlement — vocabulary &amp; grants</t>
         </is>
       </c>
     </row>
@@ -23905,12 +23905,12 @@
       </c>
       <c r="H527" t="inlineStr">
         <is>
-          <t>L1 Core</t>
+          <t>MODULE GATE</t>
         </is>
       </c>
       <c r="I527" t="inlineStr">
         <is>
-          <t>Entitlement</t>
+          <t>entitlement — vocabulary &amp; grants</t>
         </is>
       </c>
     </row>
@@ -23952,12 +23952,12 @@
       </c>
       <c r="H528" t="inlineStr">
         <is>
-          <t>L2 Module</t>
+          <t>L2</t>
         </is>
       </c>
       <c r="I528" t="inlineStr">
         <is>
-          <t>Library</t>
+          <t>Library module</t>
         </is>
       </c>
     </row>
@@ -23999,12 +23999,12 @@
       </c>
       <c r="H529" t="inlineStr">
         <is>
-          <t>L1 Core</t>
+          <t>MODULE GATE</t>
         </is>
       </c>
       <c r="I529" t="inlineStr">
         <is>
-          <t>Entitlement</t>
+          <t>entitlement — vocabulary &amp; grants</t>
         </is>
       </c>
     </row>
@@ -24046,12 +24046,12 @@
       </c>
       <c r="H530" t="inlineStr">
         <is>
-          <t>L1 Core</t>
+          <t>MODULE GATE</t>
         </is>
       </c>
       <c r="I530" t="inlineStr">
         <is>
-          <t>Entitlement</t>
+          <t>entitlement — vocabulary &amp; grants</t>
         </is>
       </c>
     </row>
@@ -24093,12 +24093,12 @@
       </c>
       <c r="H531" t="inlineStr">
         <is>
-          <t>L1 Core</t>
+          <t>MODULE GATE</t>
         </is>
       </c>
       <c r="I531" t="inlineStr">
         <is>
-          <t>Entitlement</t>
+          <t>entitlement — vocabulary &amp; grants</t>
         </is>
       </c>
     </row>
@@ -24140,12 +24140,12 @@
       </c>
       <c r="H532" t="inlineStr">
         <is>
-          <t>L1 Core</t>
+          <t>MODULE GATE</t>
         </is>
       </c>
       <c r="I532" t="inlineStr">
         <is>
-          <t>Entitlement</t>
+          <t>entitlement — vocabulary &amp; grants</t>
         </is>
       </c>
     </row>
@@ -24187,12 +24187,12 @@
       </c>
       <c r="H533" t="inlineStr">
         <is>
-          <t>L1 Core</t>
+          <t>MODULE GATE</t>
         </is>
       </c>
       <c r="I533" t="inlineStr">
         <is>
-          <t>Entitlement</t>
+          <t>entitlement — vocabulary &amp; grants</t>
         </is>
       </c>
     </row>
@@ -24234,12 +24234,12 @@
       </c>
       <c r="H534" t="inlineStr">
         <is>
-          <t>L1 Core</t>
+          <t>MODULE GATE</t>
         </is>
       </c>
       <c r="I534" t="inlineStr">
         <is>
-          <t>Entitlement</t>
+          <t>entitlement — vocabulary &amp; grants</t>
         </is>
       </c>
     </row>
@@ -24281,12 +24281,12 @@
       </c>
       <c r="H535" t="inlineStr">
         <is>
-          <t>L2 Module</t>
+          <t>L2</t>
         </is>
       </c>
       <c r="I535" t="inlineStr">
         <is>
-          <t>WorkHub</t>
+          <t>WorkHub / time-tracker</t>
         </is>
       </c>
     </row>
@@ -24328,12 +24328,12 @@
       </c>
       <c r="H536" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>⟂</t>
         </is>
       </c>
       <c r="I536" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>process &amp; housekeeping</t>
         </is>
       </c>
     </row>
@@ -24375,12 +24375,12 @@
       </c>
       <c r="H537" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>⟂</t>
         </is>
       </c>
       <c r="I537" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>process &amp; housekeeping</t>
         </is>
       </c>
     </row>
@@ -24422,12 +24422,12 @@
       </c>
       <c r="H538" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>⟂</t>
         </is>
       </c>
       <c r="I538" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>process &amp; housekeeping</t>
         </is>
       </c>
     </row>
@@ -24469,12 +24469,12 @@
       </c>
       <c r="H539" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>⟂</t>
         </is>
       </c>
       <c r="I539" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>process &amp; housekeeping</t>
         </is>
       </c>
     </row>
@@ -24516,12 +24516,12 @@
       </c>
       <c r="H540" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>⟂</t>
         </is>
       </c>
       <c r="I540" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>process &amp; housekeeping</t>
         </is>
       </c>
     </row>
@@ -24563,12 +24563,12 @@
       </c>
       <c r="H541" t="inlineStr">
         <is>
-          <t>L0 Kernel</t>
+          <t>L0</t>
         </is>
       </c>
       <c r="I541" t="inlineStr">
         <is>
-          <t>Plumbing</t>
+          <t>shared plumbing — cn, theme, hr-api</t>
         </is>
       </c>
     </row>
@@ -24610,12 +24610,12 @@
       </c>
       <c r="H542" t="inlineStr">
         <is>
-          <t>L0 Kernel</t>
+          <t>L0</t>
         </is>
       </c>
       <c r="I542" t="inlineStr">
         <is>
-          <t>Plumbing</t>
+          <t>shared plumbing — cn, theme, hr-api</t>
         </is>
       </c>
     </row>
@@ -24657,12 +24657,12 @@
       </c>
       <c r="H543" t="inlineStr">
         <is>
-          <t>L2 Module</t>
+          <t>L2</t>
         </is>
       </c>
       <c r="I543" t="inlineStr">
         <is>
-          <t>WorkHub</t>
+          <t>WorkHub / time-tracker</t>
         </is>
       </c>
     </row>
@@ -24704,12 +24704,12 @@
       </c>
       <c r="H544" t="inlineStr">
         <is>
-          <t>L2 Module</t>
+          <t>L2</t>
         </is>
       </c>
       <c r="I544" t="inlineStr">
         <is>
-          <t>WorkHub</t>
+          <t>WorkHub / time-tracker</t>
         </is>
       </c>
     </row>
@@ -24751,12 +24751,12 @@
       </c>
       <c r="H545" t="inlineStr">
         <is>
-          <t>L2 Module</t>
+          <t>L2</t>
         </is>
       </c>
       <c r="I545" t="inlineStr">
         <is>
-          <t>WorkHub</t>
+          <t>WorkHub / time-tracker</t>
         </is>
       </c>
     </row>
@@ -24798,12 +24798,12 @@
       </c>
       <c r="H546" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>⟂</t>
         </is>
       </c>
       <c r="I546" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>process &amp; housekeeping</t>
         </is>
       </c>
     </row>
@@ -24845,12 +24845,12 @@
       </c>
       <c r="H547" t="inlineStr">
         <is>
-          <t>L2 Module</t>
+          <t>L2</t>
         </is>
       </c>
       <c r="I547" t="inlineStr">
         <is>
-          <t>Timesheets</t>
+          <t>HR — timesheets</t>
         </is>
       </c>
     </row>
@@ -24892,12 +24892,12 @@
       </c>
       <c r="H548" t="inlineStr">
         <is>
-          <t>L2 Module</t>
+          <t>L2</t>
         </is>
       </c>
       <c r="I548" t="inlineStr">
         <is>
-          <t>WorkHub</t>
+          <t>WorkHub / time-tracker</t>
         </is>
       </c>
     </row>
@@ -24939,12 +24939,12 @@
       </c>
       <c r="H549" t="inlineStr">
         <is>
-          <t>L1 Core</t>
+          <t>GATE</t>
         </is>
       </c>
       <c r="I549" t="inlineStr">
         <is>
-          <t>Tenant gate</t>
+          <t>the seraph — resolver, logicalKey, scoped accessor</t>
         </is>
       </c>
     </row>
@@ -24986,12 +24986,12 @@
       </c>
       <c r="H550" t="inlineStr">
         <is>
-          <t>L2 Module</t>
+          <t>L2</t>
         </is>
       </c>
       <c r="I550" t="inlineStr">
         <is>
-          <t>WorkHub</t>
+          <t>WorkHub / time-tracker</t>
         </is>
       </c>
     </row>
@@ -25033,12 +25033,12 @@
       </c>
       <c r="H551" t="inlineStr">
         <is>
-          <t>L2 Module</t>
+          <t>L2</t>
         </is>
       </c>
       <c r="I551" t="inlineStr">
         <is>
-          <t>WorkHub</t>
+          <t>WorkHub / time-tracker</t>
         </is>
       </c>
     </row>
@@ -25080,12 +25080,12 @@
       </c>
       <c r="H552" t="inlineStr">
         <is>
-          <t>L0 Kernel</t>
+          <t>L0</t>
         </is>
       </c>
       <c r="I552" t="inlineStr">
         <is>
-          <t>Write path</t>
+          <t>write path — one door</t>
         </is>
       </c>
     </row>
@@ -25127,12 +25127,12 @@
       </c>
       <c r="H553" t="inlineStr">
         <is>
-          <t>L0 Kernel</t>
+          <t>L0</t>
         </is>
       </c>
       <c r="I553" t="inlineStr">
         <is>
-          <t>Time</t>
+          <t>time — duration, the break rule</t>
         </is>
       </c>
     </row>
@@ -25174,12 +25174,12 @@
       </c>
       <c r="H554" t="inlineStr">
         <is>
-          <t>L1 Core</t>
+          <t>L1</t>
         </is>
       </c>
       <c r="I554" t="inlineStr">
         <is>
-          <t>Write path</t>
+          <t>write path — one door</t>
         </is>
       </c>
     </row>
@@ -25221,12 +25221,12 @@
       </c>
       <c r="H555" t="inlineStr">
         <is>
-          <t>L1 Core</t>
+          <t>L1</t>
         </is>
       </c>
       <c r="I555" t="inlineStr">
         <is>
-          <t>Identity</t>
+          <t>identity — ids, roles, bindings</t>
         </is>
       </c>
     </row>
@@ -25268,12 +25268,12 @@
       </c>
       <c r="H556" t="inlineStr">
         <is>
-          <t>L2 Module</t>
+          <t>L2</t>
         </is>
       </c>
       <c r="I556" t="inlineStr">
         <is>
-          <t>WorkHub</t>
+          <t>WorkHub / time-tracker</t>
         </is>
       </c>
     </row>
@@ -25315,12 +25315,12 @@
       </c>
       <c r="H557" t="inlineStr">
         <is>
-          <t>L2 Module</t>
+          <t>L2</t>
         </is>
       </c>
       <c r="I557" t="inlineStr">
         <is>
-          <t>WorkHub</t>
+          <t>WorkHub / time-tracker</t>
         </is>
       </c>
     </row>
@@ -25362,12 +25362,12 @@
       </c>
       <c r="H558" t="inlineStr">
         <is>
-          <t>L1 Core</t>
+          <t>L1</t>
         </is>
       </c>
       <c r="I558" t="inlineStr">
         <is>
-          <t>Write path</t>
+          <t>write path — one door</t>
         </is>
       </c>
     </row>
@@ -25409,12 +25409,12 @@
       </c>
       <c r="H559" t="inlineStr">
         <is>
-          <t>L2 Module</t>
+          <t>L2</t>
         </is>
       </c>
       <c r="I559" t="inlineStr">
         <is>
-          <t>WorkHub</t>
+          <t>WorkHub / time-tracker</t>
         </is>
       </c>
     </row>
@@ -25456,12 +25456,12 @@
       </c>
       <c r="H560" t="inlineStr">
         <is>
-          <t>L2 Module</t>
+          <t>L2</t>
         </is>
       </c>
       <c r="I560" t="inlineStr">
         <is>
-          <t>WorkHub</t>
+          <t>WorkHub / time-tracker</t>
         </is>
       </c>
     </row>
@@ -25503,12 +25503,12 @@
       </c>
       <c r="H561" t="inlineStr">
         <is>
-          <t>L2 Module</t>
+          <t>L2</t>
         </is>
       </c>
       <c r="I561" t="inlineStr">
         <is>
-          <t>WorkHub</t>
+          <t>WorkHub / time-tracker</t>
         </is>
       </c>
     </row>
@@ -25550,12 +25550,12 @@
       </c>
       <c r="H562" t="inlineStr">
         <is>
-          <t>L0 Kernel</t>
+          <t>L0</t>
         </is>
       </c>
       <c r="I562" t="inlineStr">
         <is>
-          <t>Write path</t>
+          <t>write path — one door</t>
         </is>
       </c>
     </row>
@@ -25597,12 +25597,12 @@
       </c>
       <c r="H563" t="inlineStr">
         <is>
-          <t>L2 Module</t>
+          <t>L2</t>
         </is>
       </c>
       <c r="I563" t="inlineStr">
         <is>
-          <t>WorkHub</t>
+          <t>WorkHub / time-tracker</t>
         </is>
       </c>
     </row>
@@ -25644,12 +25644,12 @@
       </c>
       <c r="H564" t="inlineStr">
         <is>
-          <t>L2 Module</t>
+          <t>L2</t>
         </is>
       </c>
       <c r="I564" t="inlineStr">
         <is>
-          <t>WorkHub</t>
+          <t>WorkHub / time-tracker</t>
         </is>
       </c>
     </row>
@@ -25691,7 +25691,7 @@
       </c>
       <c r="H565" t="inlineStr">
         <is>
-          <t>L2 Module</t>
+          <t>L2</t>
         </is>
       </c>
       <c r="I565" t="inlineStr">
@@ -25738,7 +25738,7 @@
       </c>
       <c r="H566" t="inlineStr">
         <is>
-          <t>L1 Core</t>
+          <t>L1</t>
         </is>
       </c>
       <c r="I566" t="inlineStr">
@@ -25785,12 +25785,12 @@
       </c>
       <c r="H567" t="inlineStr">
         <is>
-          <t>L2 Module</t>
+          <t>L2</t>
         </is>
       </c>
       <c r="I567" t="inlineStr">
         <is>
-          <t>Portals</t>
+          <t>Client Portal</t>
         </is>
       </c>
     </row>
@@ -25832,12 +25832,12 @@
       </c>
       <c r="H568" t="inlineStr">
         <is>
-          <t>L2 Module</t>
+          <t>L2</t>
         </is>
       </c>
       <c r="I568" t="inlineStr">
         <is>
-          <t>Portals</t>
+          <t>Client Portal</t>
         </is>
       </c>
     </row>
@@ -25879,12 +25879,12 @@
       </c>
       <c r="H569" t="inlineStr">
         <is>
-          <t>L2 Module</t>
+          <t>L2</t>
         </is>
       </c>
       <c r="I569" t="inlineStr">
         <is>
-          <t>Portals</t>
+          <t>Client Portal</t>
         </is>
       </c>
     </row>
@@ -25926,12 +25926,12 @@
       </c>
       <c r="H570" t="inlineStr">
         <is>
-          <t>L2 Module</t>
+          <t>L2</t>
         </is>
       </c>
       <c r="I570" t="inlineStr">
         <is>
-          <t>Portals</t>
+          <t>Client Portal</t>
         </is>
       </c>
     </row>
@@ -25973,12 +25973,12 @@
       </c>
       <c r="H571" t="inlineStr">
         <is>
-          <t>L1 Core</t>
+          <t>L1</t>
         </is>
       </c>
       <c r="I571" t="inlineStr">
         <is>
-          <t>Portals</t>
+          <t>Client Portal</t>
         </is>
       </c>
     </row>
@@ -26020,12 +26020,12 @@
       </c>
       <c r="H572" t="inlineStr">
         <is>
-          <t>L1 Core</t>
+          <t>L1</t>
         </is>
       </c>
       <c r="I572" t="inlineStr">
         <is>
-          <t>Portals</t>
+          <t>Client Portal</t>
         </is>
       </c>
     </row>
@@ -26067,12 +26067,12 @@
       </c>
       <c r="H573" t="inlineStr">
         <is>
-          <t>L1 Core</t>
+          <t>L1</t>
         </is>
       </c>
       <c r="I573" t="inlineStr">
         <is>
-          <t>Portals</t>
+          <t>Client Portal</t>
         </is>
       </c>
     </row>
@@ -26114,12 +26114,12 @@
       </c>
       <c r="H574" t="inlineStr">
         <is>
-          <t>L1 Core</t>
+          <t>L1</t>
         </is>
       </c>
       <c r="I574" t="inlineStr">
         <is>
-          <t>Portals</t>
+          <t>Client Portal</t>
         </is>
       </c>
     </row>
@@ -26161,12 +26161,12 @@
       </c>
       <c r="H575" t="inlineStr">
         <is>
-          <t>L2 Module</t>
+          <t>L2</t>
         </is>
       </c>
       <c r="I575" t="inlineStr">
         <is>
-          <t>Portals</t>
+          <t>Client Portal</t>
         </is>
       </c>
     </row>
@@ -26208,12 +26208,12 @@
       </c>
       <c r="H576" t="inlineStr">
         <is>
-          <t>L1 Core</t>
+          <t>GATE</t>
         </is>
       </c>
       <c r="I576" t="inlineStr">
         <is>
-          <t>Tenant gate</t>
+          <t>the seraph — resolver, logicalKey, scoped accessor</t>
         </is>
       </c>
     </row>
@@ -26255,12 +26255,12 @@
       </c>
       <c r="H577" t="inlineStr">
         <is>
-          <t>L1 Core</t>
+          <t>L1</t>
         </is>
       </c>
       <c r="I577" t="inlineStr">
         <is>
-          <t>Portals</t>
+          <t>Client Portal</t>
         </is>
       </c>
     </row>
@@ -26302,12 +26302,12 @@
       </c>
       <c r="H578" t="inlineStr">
         <is>
-          <t>L1 Core</t>
+          <t>L1</t>
         </is>
       </c>
       <c r="I578" t="inlineStr">
         <is>
-          <t>Audit</t>
+          <t>audit — the actor</t>
         </is>
       </c>
     </row>
@@ -26349,7 +26349,7 @@
       </c>
       <c r="H579" t="inlineStr">
         <is>
-          <t>L1 Core</t>
+          <t>L1</t>
         </is>
       </c>
       <c r="I579" t="inlineStr">
@@ -26396,12 +26396,12 @@
       </c>
       <c r="H580" t="inlineStr">
         <is>
-          <t>L0 Kernel</t>
+          <t>L0</t>
         </is>
       </c>
       <c r="I580" t="inlineStr">
         <is>
-          <t>Identity</t>
+          <t>identity — ids, roles, bindings</t>
         </is>
       </c>
     </row>
@@ -26443,12 +26443,12 @@
       </c>
       <c r="H581" t="inlineStr">
         <is>
-          <t>L0 Kernel</t>
+          <t>L0</t>
         </is>
       </c>
       <c r="I581" t="inlineStr">
         <is>
-          <t>Identity</t>
+          <t>identity — ids, roles, bindings</t>
         </is>
       </c>
     </row>
@@ -26490,12 +26490,12 @@
       </c>
       <c r="H582" t="inlineStr">
         <is>
-          <t>L0 Kernel</t>
+          <t>L0</t>
         </is>
       </c>
       <c r="I582" t="inlineStr">
         <is>
-          <t>Identity</t>
+          <t>identity — ids, roles, bindings</t>
         </is>
       </c>
     </row>
@@ -26537,12 +26537,12 @@
       </c>
       <c r="H583" t="inlineStr">
         <is>
-          <t>L1 Core</t>
+          <t>L1</t>
         </is>
       </c>
       <c r="I583" t="inlineStr">
         <is>
-          <t>Identity</t>
+          <t>identity — ids, roles, bindings</t>
         </is>
       </c>
     </row>
@@ -26584,12 +26584,12 @@
       </c>
       <c r="H584" t="inlineStr">
         <is>
-          <t>L2 Module</t>
+          <t>L2</t>
         </is>
       </c>
       <c r="I584" t="inlineStr">
         <is>
-          <t>WorkHub</t>
+          <t>WorkHub / time-tracker</t>
         </is>
       </c>
     </row>
@@ -26631,12 +26631,12 @@
       </c>
       <c r="H585" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>⟂</t>
         </is>
       </c>
       <c r="I585" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>process &amp; housekeeping</t>
         </is>
       </c>
     </row>
@@ -26678,12 +26678,12 @@
       </c>
       <c r="H586" t="inlineStr">
         <is>
-          <t>L0 Kernel</t>
+          <t>L0</t>
         </is>
       </c>
       <c r="I586" t="inlineStr">
         <is>
-          <t>Time</t>
+          <t>time — duration, the break rule</t>
         </is>
       </c>
     </row>
@@ -26725,12 +26725,12 @@
       </c>
       <c r="H587" t="inlineStr">
         <is>
-          <t>L1 Core</t>
+          <t>L1</t>
         </is>
       </c>
       <c r="I587" t="inlineStr">
         <is>
-          <t>Write path</t>
+          <t>write path — one door</t>
         </is>
       </c>
     </row>
@@ -26772,12 +26772,12 @@
       </c>
       <c r="H588" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>⟂</t>
         </is>
       </c>
       <c r="I588" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>process &amp; housekeeping</t>
         </is>
       </c>
     </row>
@@ -26819,12 +26819,12 @@
       </c>
       <c r="H589" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>⟂</t>
         </is>
       </c>
       <c r="I589" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>process &amp; housekeeping</t>
         </is>
       </c>
     </row>
@@ -26866,12 +26866,12 @@
       </c>
       <c r="H590" t="inlineStr">
         <is>
-          <t>L2 Module</t>
+          <t>L2</t>
         </is>
       </c>
       <c r="I590" t="inlineStr">
         <is>
-          <t>WorkHub</t>
+          <t>WorkHub / time-tracker</t>
         </is>
       </c>
     </row>
@@ -26913,12 +26913,12 @@
       </c>
       <c r="H591" t="inlineStr">
         <is>
-          <t>L2 Module</t>
+          <t>L2</t>
         </is>
       </c>
       <c r="I591" t="inlineStr">
         <is>
-          <t>WorkHub</t>
+          <t>WorkHub / time-tracker</t>
         </is>
       </c>
     </row>
@@ -26960,12 +26960,12 @@
       </c>
       <c r="H592" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>⟂</t>
         </is>
       </c>
       <c r="I592" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>process &amp; housekeeping</t>
         </is>
       </c>
     </row>
@@ -27007,12 +27007,12 @@
       </c>
       <c r="H593" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>⟂</t>
         </is>
       </c>
       <c r="I593" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>process &amp; housekeeping</t>
         </is>
       </c>
     </row>
@@ -27054,12 +27054,12 @@
       </c>
       <c r="H594" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>⟂</t>
         </is>
       </c>
       <c r="I594" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>process &amp; housekeeping</t>
         </is>
       </c>
     </row>
@@ -27101,12 +27101,12 @@
       </c>
       <c r="H595" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>⟂</t>
         </is>
       </c>
       <c r="I595" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>process &amp; housekeeping</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(workflows): update roadmap, pd.md pre-handover guidelines, and CSF-1 directive
</commit_message>
<xml_diff>
--- a/.agents/coral-roadmap.xlsx
+++ b/.agents/coral-roadmap.xlsx
@@ -594,7 +594,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I595"/>
+  <dimension ref="A1:I603"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -24981,7 +24981,7 @@
       </c>
       <c r="G550" t="inlineStr">
         <is>
-          <t>CreateShiftForm 1967 + EditShiftDialog 915 + ShiftViewDialog 626. BLOCKED on PROJ-0 and R1-4 — starting earlier rebuilds the [ERP] prefix and the 74 parse sites into new code.</t>
+          <t>CreateShiftForm 1967 + EditShiftDialog 915 + ShiftViewDialog 626. BLOCKED on PROJ-0 and R1-4 — starting earlier rebuilds the [ERP] prefix and the 74 parse sites into new code. | STRONGER JUSTIFICATION (CSF-1, 2026-09-28): the ~900-line form exists TWICE in one file. Both CSF-1 defects are a fix that landed on one copy and not the other — and the copy that missed both is the matrix-+ path, which is the one actually used.</t>
         </is>
       </c>
       <c r="H550" t="inlineStr">
@@ -25191,7 +25191,7 @@
       </c>
       <c r="B555" t="inlineStr">
         <is>
-          <t>DECIDE which 'employee' is canonical: User, Employee model, or the db-hr projection</t>
+          <t>IDENTITY MODEL DEFINED (Florin 2026-09-28) — not a collapse</t>
         </is>
       </c>
       <c r="C555" t="inlineStr">
@@ -25206,7 +25206,7 @@
       </c>
       <c r="E555" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Decided</t>
         </is>
       </c>
       <c r="F555" t="inlineStr">
@@ -25216,7 +25216,7 @@
       </c>
       <c r="G555" t="inlineStr">
         <is>
-          <t>Three representations of one concept. db-hr holds no data — it synthesises rows from User at read time behind a 14-role allowlist.</t>
+          <t>User = anyone who logs into the ERP. Two role axes: FUNCTIONAL (superadmin, tenant admin, ERP operator, tenant employee) and OPERATIONAL/HIERARCHICAL (director, HR, team leader, workforce — tenant-specific), the latter governing module access. Employee = a person in the company structure; db-hr = a projection joining them. THREE CONCEPTS, ALL LEGITIMATE. Planner had wrongly proposed collapsing to one — see pd.md 4z.</t>
         </is>
       </c>
       <c r="H555" t="inlineStr">
@@ -26084,7 +26084,7 @@
       </c>
       <c r="B574" t="inlineStr">
         <is>
-          <t>Task.status is CHANGEABLE, with every change logged (Florin 2026-09-27)</t>
+          <t>Task status is OPEN AT BOTH ENDS, with an exact log behind it (Florin 2026-09-28)</t>
         </is>
       </c>
       <c r="C574" t="inlineStr">
@@ -26109,7 +26109,7 @@
       </c>
       <c r="G574" t="inlineStr">
         <is>
-          <t>Not prohibited — logged. Use the EXISTING AuditLog (entityType 'portalTask', field 'status', before/after). Do NOT create a fourth audit model: AuditLog and RateChangeAudit already exist.</t>
+          <t>Not a response-vs-edit distinction: either side may change status, every change logged in AuditLog (entityType portalTask, field status, before/after, actor).</t>
         </is>
       </c>
       <c r="H574" t="inlineStr">
@@ -26616,7 +26616,7 @@
       </c>
       <c r="E585" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F585" t="inlineStr">
@@ -26626,7 +26626,7 @@
       </c>
       <c r="G585" t="inlineStr">
         <is>
-          <t>Every pass this week went straight to production. coral-promotion-plan.md describes a release branch, staging pass and 48h watch — none happened and nobody noticed it stopped. This is the only defect that made the others reach a user.</t>
+          <t>Every pass this week went straight to production. coral-promotion-plan.md describes a release branch, staging pass and 48h watch — none happened and nobody noticed it stopped. This is the only defect that made the others reach a user. | develop -&gt; main separation restored by Florin 2026-09-28.</t>
         </is>
       </c>
       <c r="H585" t="inlineStr">
@@ -27105,6 +27105,382 @@
         </is>
       </c>
       <c r="I595" t="inlineStr">
+        <is>
+          <t>process &amp; housekeeping</t>
+        </is>
+      </c>
+    </row>
+    <row r="596">
+      <c r="A596" t="inlineStr">
+        <is>
+          <t>HRS-1</t>
+        </is>
+      </c>
+      <c r="B596" t="inlineStr">
+        <is>
+          <t>Hours must be assignable to a project AT ANY MOMENT — never fixed at creation</t>
+        </is>
+      </c>
+      <c r="C596" t="inlineStr">
+        <is>
+          <t>WorkHub</t>
+        </is>
+      </c>
+      <c r="D596" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E596" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F596" t="inlineStr">
+        <is>
+          <t>pd.md 4x</t>
+        </is>
+      </c>
+      <c r="G596" t="inlineStr">
+        <is>
+          <t>Florin 2026-09-28: 'do not make assumptions, leave it open with the possibility to set at any moment.' Recorded hours exist independently; attribution is a later, repeatable act. Unattributed hours are a NORMAL TRANSIENT STATE, not an error and not an orphan.</t>
+        </is>
+      </c>
+      <c r="H596" t="inlineStr">
+        <is>
+          <t>L0 Kernel</t>
+        </is>
+      </c>
+      <c r="I596" t="inlineStr">
+        <is>
+          <t>time — duration, the break rule</t>
+        </is>
+      </c>
+    </row>
+    <row r="597">
+      <c r="A597" t="inlineStr">
+        <is>
+          <t>HRS-2</t>
+        </is>
+      </c>
+      <c r="B597" t="inlineStr">
+        <is>
+          <t>A surface to assign / re-assign hours to a project, including retrospectively</t>
+        </is>
+      </c>
+      <c r="C597" t="inlineStr">
+        <is>
+          <t>WorkHub</t>
+        </is>
+      </c>
+      <c r="D597" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E597" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F597" t="inlineStr">
+        <is>
+          <t>pd.md 4x</t>
+        </is>
+      </c>
+      <c r="G597" t="inlineStr">
+        <is>
+          <t>Follows from HRS-1. Applies to late entries AND live clock-ins. Covers the 11 orphaned entries without needing invented shifts.</t>
+        </is>
+      </c>
+      <c r="H597" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="I597" t="inlineStr">
+        <is>
+          <t>WorkHub / time-tracker</t>
+        </is>
+      </c>
+    </row>
+    <row r="598">
+      <c r="A598" t="inlineStr">
+        <is>
+          <t>HRS-3</t>
+        </is>
+      </c>
+      <c r="B598" t="inlineStr">
+        <is>
+          <t>Every project re-assignment of hours is logged</t>
+        </is>
+      </c>
+      <c r="C598" t="inlineStr">
+        <is>
+          <t>WorkHub</t>
+        </is>
+      </c>
+      <c r="D598" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E598" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F598" t="inlineStr">
+        <is>
+          <t>pd.md 4x</t>
+        </is>
+      </c>
+      <c r="G598" t="inlineStr">
+        <is>
+          <t>Hours moving between projects moves money between jobs. AuditLog, one authority (pd.md 5a).</t>
+        </is>
+      </c>
+      <c r="H598" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="I598" t="inlineStr">
+        <is>
+          <t>audit — the actor</t>
+        </is>
+      </c>
+    </row>
+    <row r="599">
+      <c r="A599" t="inlineStr">
+        <is>
+          <t>PLAN-5</t>
+        </is>
+      </c>
+      <c r="B599" t="inlineStr">
+        <is>
+          <t>Planner misused 'canonical' as a collapse rule</t>
+        </is>
+      </c>
+      <c r="C599" t="inlineStr">
+        <is>
+          <t>Process</t>
+        </is>
+      </c>
+      <c r="D599" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E599" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F599" t="inlineStr">
+        <is>
+          <t>pd.md 4z</t>
+        </is>
+      </c>
+      <c r="G599" t="inlineStr">
+        <is>
+          <t>Proposed deleting one of User / Employee / db-hr projection as duplicates. Florin: canonical means each concept DEFINED then FROZEN, not reduced to one. The defect-shape-#1 test is 'one concept, two representations' — not 'two things that sound alike'. Some earlier shape-#1 calls this month deserve re-checking under the correct test.</t>
+        </is>
+      </c>
+      <c r="H599" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I599" t="inlineStr">
+        <is>
+          <t>process &amp; housekeeping</t>
+        </is>
+      </c>
+    </row>
+    <row r="600">
+      <c r="A600" t="inlineStr">
+        <is>
+          <t>CSF-1</t>
+        </is>
+      </c>
+      <c r="B600" t="inlineStr">
+        <is>
+          <t>Shift modal: worker names blank + project unselectable from the matrix +</t>
+        </is>
+      </c>
+      <c r="C600" t="inlineStr">
+        <is>
+          <t>WorkHub</t>
+        </is>
+      </c>
+      <c r="D600" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E600" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F600" t="inlineStr">
+        <is>
+          <t>coder-directive-csf-1-shift-modal.md</t>
+        </is>
+      </c>
+      <c r="G600" t="inlineStr">
+        <is>
+          <t>REV 2 (canonical): both fixes moved to the DEFINITION. (A) WorkerOption is declared THREE times (CreateShiftForm:45, EditShiftDialog:53, ScheduleManagement:19) plus WorkerWithProfile as a fourth shape — one definition in time-tracker/types, name REQUIRED, full_name deleted. (B) 56 SearchableSelect callers, ONE passes portalContainer — the component must self-determine its target (closest('[role=dialog]') ?? body) so all 56 are correct by construction. Rev 1 would have made it 2 of 56.</t>
+        </is>
+      </c>
+      <c r="H600" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="I600" t="inlineStr">
+        <is>
+          <t>WorkHub / time-tracker</t>
+        </is>
+      </c>
+    </row>
+    <row r="601">
+      <c r="A601" t="inlineStr">
+        <is>
+          <t>PLAN-6</t>
+        </is>
+      </c>
+      <c r="B601" t="inlineStr">
+        <is>
+          <t>Planner mistook Employee.schedule for a broken User↔Employee link</t>
+        </is>
+      </c>
+      <c r="C601" t="inlineStr">
+        <is>
+          <t>Process</t>
+        </is>
+      </c>
+      <c r="D601" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E601" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F601" t="inlineStr">
+        <is>
+          <t>coder-directive-csf-1-shift-modal.md</t>
+        </is>
+      </c>
+      <c r="G601" t="inlineStr">
+        <is>
+          <t>Employee.schedule is a deliberate per-employee checkbox in the profile deciding scheduler visibility. Florin manages it. The short employee list was the feature working. Second false alarm today (the other: grepping the WORD @ts-nocheck rather than the directive).</t>
+        </is>
+      </c>
+      <c r="H601" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I601" t="inlineStr">
+        <is>
+          <t>process &amp; housekeeping</t>
+        </is>
+      </c>
+    </row>
+    <row r="602">
+      <c r="A602" t="inlineStr">
+        <is>
+          <t>SS-1</t>
+        </is>
+      </c>
+      <c r="B602" t="inlineStr">
+        <is>
+          <t>🔴 SearchableSelect: 56 callers, 1 passes portalContainer — the component must decide</t>
+        </is>
+      </c>
+      <c r="C602" t="inlineStr">
+        <is>
+          <t>Type debt</t>
+        </is>
+      </c>
+      <c r="D602" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E602" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F602" t="inlineStr">
+        <is>
+          <t>coder-directive-csf-1-shift-modal.md</t>
+        </is>
+      </c>
+      <c r="G602" t="inlineStr">
+        <is>
+          <t>Defaults usePortal=true and falls back to document.body, so ANY SearchableSelect inside ANY Radix dialog is unclickable — the focus trap eats the clicks. Fix at the component: closest('[role=dialog]') ?? body. All 56 callers correct by construction. RISK: position:fixed inside a transformed ancestor — verify placement, not just that it opens.</t>
+        </is>
+      </c>
+      <c r="H602" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="I602" t="inlineStr">
+        <is>
+          <t>shared plumbing — cn, theme, hr-api</t>
+        </is>
+      </c>
+    </row>
+    <row r="603">
+      <c r="A603" t="inlineStr">
+        <is>
+          <t>PLAN-7</t>
+        </is>
+      </c>
+      <c r="B603" t="inlineStr">
+        <is>
+          <t>Planner fixed the instance, not the shape — one message after criticising exactly that</t>
+        </is>
+      </c>
+      <c r="C603" t="inlineStr">
+        <is>
+          <t>Process</t>
+        </is>
+      </c>
+      <c r="D603" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E603" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F603" t="inlineStr">
+        <is>
+          <t>coder-directive-csf-1-shift-modal.md</t>
+        </is>
+      </c>
+      <c r="G603" t="inlineStr">
+        <is>
+          <t>CSF-1 rev 1 patched caller #2 of 56 and froze WorkerOption in a leaf where it is declared three times. Rev 2 moves both to the definition. The canonical check must run BEFORE a directive is handed over, not after Florin asks for it.</t>
+        </is>
+      </c>
+      <c r="H603" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I603" t="inlineStr">
         <is>
           <t>process &amp; housekeeping</t>
         </is>

</xml_diff>

<commit_message>
feat(WH-UI-1): WorkHub Home screen overhaul, brand palette, and formatTime kernel addition
</commit_message>
<xml_diff>
--- a/.agents/coral-roadmap.xlsx
+++ b/.agents/coral-roadmap.xlsx
@@ -594,7 +594,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I603"/>
+  <dimension ref="A1:I606"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -27483,6 +27483,147 @@
       <c r="I603" t="inlineStr">
         <is>
           <t>process &amp; housekeeping</t>
+        </is>
+      </c>
+    </row>
+    <row r="604">
+      <c r="A604" t="inlineStr">
+        <is>
+          <t>WH-UI-1</t>
+        </is>
+      </c>
+      <c r="B604" t="inlineStr">
+        <is>
+          <t>WorkHub home: schedule fills the page, clock button to the bottom as fallback</t>
+        </is>
+      </c>
+      <c r="C604" t="inlineStr">
+        <is>
+          <t>WorkHub</t>
+        </is>
+      </c>
+      <c r="D604" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E604" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F604" t="inlineStr">
+        <is>
+          <t>coder-directive-wh-ui-1-workhub-home.md</t>
+        </is>
+      </c>
+      <c r="G604" t="inlineStr">
+        <is>
+          <t>Florin 2026-09-28. Time Off to nav, QuickLinks deleted, 'Today's Shift' block removed, hero section gone. Shift cards are ALREADY built to bleed (rounded-none border-x-0) and the page px-4 plus an outer Card put them back in a box. | REVISED: Florin decided the shift entry gains project NAME + tappable ADDRESS in this pass; the word 'Shift' is deleted. Clock button FIXED above the nav, green (emerald-600) when a shift is available / brand-orange when not, both labels LOCALIZED in all 5 locales. Text starts at OS default 1rem. Borders between entries kept.</t>
+        </is>
+      </c>
+      <c r="H604" t="inlineStr">
+        <is>
+          <t>L3</t>
+        </is>
+      </c>
+      <c r="I604" t="inlineStr">
+        <is>
+          <t>shells &amp; navigation — WorkHubShell</t>
+        </is>
+      </c>
+    </row>
+    <row r="605">
+      <c r="A605" t="inlineStr">
+        <is>
+          <t>WH-UI-2</t>
+        </is>
+      </c>
+      <c r="B605" t="inlineStr">
+        <is>
+          <t>Files appears in the nav while loading and disappears once loaded</t>
+        </is>
+      </c>
+      <c r="C605" t="inlineStr">
+        <is>
+          <t>WorkHub</t>
+        </is>
+      </c>
+      <c r="D605" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="E605" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F605" t="inlineStr">
+        <is>
+          <t>coder-directive-wh-ui-1-workhub-home.md</t>
+        </is>
+      </c>
+      <c r="G605" t="inlineStr">
+        <is>
+          <t>Unconditional in the WorkHubShell array (line 31) so something filters it after the tenant resolves. This is the 'old screen with five links' Florin saw during the INC-1 crash — not a stale cache. Also: the header shows 'User' as a placeholder before the name loads.</t>
+        </is>
+      </c>
+      <c r="H605" t="inlineStr">
+        <is>
+          <t>L3</t>
+        </is>
+      </c>
+      <c r="I605" t="inlineStr">
+        <is>
+          <t>shells &amp; navigation — WorkHubShell</t>
+        </is>
+      </c>
+    </row>
+    <row r="606">
+      <c r="A606" t="inlineStr">
+        <is>
+          <t>DS-1</t>
+        </is>
+      </c>
+      <c r="B606" t="inlineStr">
+        <is>
+          <t>🔴 The brand palette exists as a decision and NOWHERE as code</t>
+        </is>
+      </c>
+      <c r="C606" t="inlineStr">
+        <is>
+          <t>Design system</t>
+        </is>
+      </c>
+      <c r="D606" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E606" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F606" t="inlineStr">
+        <is>
+          <t>coder-directive-wh-ui-1-workhub-home.md</t>
+        </is>
+      </c>
+      <c r="G606" t="inlineStr">
+        <is>
+          <t>tawny/persian-green/eerie-black/baby-powder/eggshell: 0 occurrences in src. Instead: #d35400 x368 (WRONG orange, ERP surfaces), #d75d00 x158 (tawny, correct, public site), orange-* x522, emerald-* x210. The public site has the brand right; the ERP drifted because no token existed to disagree with. globals.css defines no palette. WH-UI-1 defines the tokens and is the first correct consumer; converting the other ~1,258 sites is this item.</t>
+        </is>
+      </c>
+      <c r="H606" t="inlineStr">
+        <is>
+          <t>L4</t>
+        </is>
+      </c>
+      <c r="I606" t="inlineStr">
+        <is>
+          <t>design system</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(WH-UI-1): delete ShiftViewDialog (§8.0), add shiftBrief server accessor (§8.1), wire Shift Brief modal (§8.2), and apply font-content (§7)
</commit_message>
<xml_diff>
--- a/.agents/coral-roadmap.xlsx
+++ b/.agents/coral-roadmap.xlsx
@@ -594,7 +594,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I606"/>
+  <dimension ref="A1:I608"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -24981,7 +24981,7 @@
       </c>
       <c r="G550" t="inlineStr">
         <is>
-          <t>CreateShiftForm 1967 + EditShiftDialog 915 + ShiftViewDialog 626. BLOCKED on PROJ-0 and R1-4 — starting earlier rebuilds the [ERP] prefix and the 74 parse sites into new code. | STRONGER JUSTIFICATION (CSF-1, 2026-09-28): the ~900-line form exists TWICE in one file. Both CSF-1 defects are a fix that landed on one copy and not the other — and the copy that missed both is the matrix-+ path, which is the one actually used.</t>
+          <t>CreateShiftForm 1967 + EditShiftDialog 915 + ShiftViewDialog 626. BLOCKED on PROJ-0 and R1-4 — starting earlier rebuilds the [ERP] prefix and the 74 parse sites into new code. | STRONGER JUSTIFICATION (CSF-1, 2026-09-28): the ~900-line form exists TWICE in one file. Both CSF-1 defects are a fix that landed on one copy and not the other — and the copy that missed both is the matrix-+ path, which is the one actually used. | SCOPE REDUCED: ShiftViewDialog is deleted by WH-UI-1, so WH-7 is CreateShiftForm + EditShiftDialog — 2,882 lines, not 3,508.</t>
         </is>
       </c>
       <c r="H550" t="inlineStr">
@@ -25426,7 +25426,7 @@
       </c>
       <c r="B560" t="inlineStr">
         <is>
-          <t>REQUIREMENT: the shift brief — opening a shift shows everything needed to work it</t>
+          <t>SPECCED: the shift brief — one server accessor, shiftBrief(scope, shiftId)</t>
         </is>
       </c>
       <c r="C560" t="inlineStr">
@@ -25451,7 +25451,7 @@
       </c>
       <c r="G560" t="inlineStr">
         <is>
-          <t>Florin 2026-09-27: address as a clickable navigation link, phone of the client or other relevant contact, photos, files. This is ShiftViewDialog's purpose and it is one of the 3 files WH-7 rebuilds.</t>
+          <t>Title (3-step fallback), address-&gt;map, contact name+phone-&gt;dial, scheduled, worked (from clockEntries via computeWorkedDuration), photos (clock entry JSON), files (ShiftAttachment). Phone is a TWO-HOP lookup: shift -&gt; project page -&gt; Klant relation -&gt; client page -&gt; Telefoon. Hence ONE server accessor, not 3+ client round trips on a site connection. Follows the WH-5a pattern.</t>
         </is>
       </c>
       <c r="H560" t="inlineStr">
@@ -26955,7 +26955,7 @@
       </c>
       <c r="G592" t="inlineStr">
         <is>
-          <t>THE CORE MOVE. Blanket silence makes readers unenumerable — that is INC-1. Line-level makes them greppable and countable WITHOUT converting one. The file becomes type-checked immediately; a new error fails the build. Order: fewest errors first.</t>
+          <t>THE CORE MOVE. Blanket silence makes readers unenumerable — that is INC-1. Line-level makes them greppable and countable WITHOUT converting one. The file becomes type-checked immediately; a new error fails the build. Order: fewest errors first. | SUPERSEDED AS A METRIC: the markers are gone (TD-4 converted those exact lines) and were never complete — local snake_case interfaces type-check and were never marked.</t>
         </is>
       </c>
       <c r="H592" t="inlineStr">
@@ -26977,7 +26977,7 @@
       </c>
       <c r="B593" t="inlineStr">
         <is>
-          <t>Convert by CATEGORY, not by file — casing in bulk, semantic one at a time</t>
+          <t>Convert the remaining shape — the SUPA-2 allowlist (37) is the metric, not @ts-expect-error</t>
         </is>
       </c>
       <c r="C593" t="inlineStr">
@@ -26997,12 +26997,12 @@
       </c>
       <c r="F593" t="inlineStr">
         <is>
-          <t>coral-typecheck-debt-plan.md</t>
+          <t>coder-directive-td-4-convert.md</t>
         </is>
       </c>
       <c r="G593" t="inlineStr">
         <is>
-          <t>file_path → ShiftAttachment.url is a semantic mapping, not a rename. No find-and-replace ever (the full_name lesson). Each converted read deletes its @ts-expect-error — and a stale expect-error FAILS the build, so the ratchet maintains itself.</t>
+          <t>@ts-expect-error is 0 and CANNOT come back: TimesheetView and Performance declare LOCAL snake_case interfaces, so those reads type-check and tsc never saw them. The ESLint allowlist matches the PATTERN including TSPropertySignature, so a locally-declared wrong shape cannot hide. Surface: 9 files already clean, 17-file tail, 4 local-interface files, 3 SKIPPED (WH-7 rebuilds two, WH-UI-1 deletes one), 3 bridges last.</t>
         </is>
       </c>
       <c r="H593" t="inlineStr">
@@ -27049,7 +27049,7 @@
       </c>
       <c r="G594" t="inlineStr">
         <is>
-          <t>Readers become countable via grep on the @ts-expect-error comments. Zero readers, then the write goes. 'Strip the type, remove the write, convert later' is INC-1 stated as a sentence.</t>
+          <t>Readers become countable via grep on the @ts-expect-error comments. Zero readers, then the write goes. 'Strip the type, remove the write, convert later' is INC-1 stated as a sentence. | Bridges: useScheduledShifts (62) + useScheduleAttachments (30) + actions/timesheets (15). One FIELD at a time, not one file. Zero readers, then the write goes.</t>
         </is>
       </c>
       <c r="H594" t="inlineStr">
@@ -27624,6 +27624,100 @@
       <c r="I606" t="inlineStr">
         <is>
           <t>design system</t>
+        </is>
+      </c>
+    </row>
+    <row r="607">
+      <c r="A607" t="inlineStr">
+        <is>
+          <t>WH-UI-3</t>
+        </is>
+      </c>
+      <c r="B607" t="inlineStr">
+        <is>
+          <t>🔴 Legibility: a DISPLAY font does body work in the workhub</t>
+        </is>
+      </c>
+      <c r="C607" t="inlineStr">
+        <is>
+          <t>WorkHub</t>
+        </is>
+      </c>
+      <c r="D607" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E607" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F607" t="inlineStr">
+        <is>
+          <t>coder-directive-wh-ui-1-workhub-home.md</t>
+        </is>
+      </c>
+      <c r="G607" t="inlineStr">
+        <is>
+          <t>body uses Oxanium (squarish display face, small x-height) while IBM Plex Sans is loaded and assigned to '.font-content — legible for data-heavy areas' and used NOWHERE in the workhub. Plus 119 text-xs + 169 text-sm against 21 at base or above. Apply .font-content to the shell; base 1rem; delete text-xs from crew surfaces.</t>
+        </is>
+      </c>
+      <c r="H607" t="inlineStr">
+        <is>
+          <t>L4</t>
+        </is>
+      </c>
+      <c r="I607" t="inlineStr">
+        <is>
+          <t>design system</t>
+        </is>
+      </c>
+    </row>
+    <row r="608">
+      <c r="A608" t="inlineStr">
+        <is>
+          <t>WH-UI-4</t>
+        </is>
+      </c>
+      <c r="B608" t="inlineStr">
+        <is>
+          <t>DECIDED: delete ShiftViewDialog (626 lines, never rendered, never executed)</t>
+        </is>
+      </c>
+      <c r="C608" t="inlineStr">
+        <is>
+          <t>WorkHub</t>
+        </is>
+      </c>
+      <c r="D608" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E608" t="inlineStr">
+        <is>
+          <t>Decided</t>
+        </is>
+      </c>
+      <c r="F608" t="inlineStr">
+        <is>
+          <t>coder-directive-wh-ui-1-workhub-home.md</t>
+        </is>
+      </c>
+      <c r="G608" t="inlineStr">
+        <is>
+          <t>Its clock-entry rendering was gated behind clock_entry_id, hardcoded null at useScheduledShifts:76 — that code has NEVER run. Not proven work to harvest: unverified code on a removed shape carrying @ts-expect-errors. Delete it.</t>
+        </is>
+      </c>
+      <c r="H608" t="inlineStr">
+        <is>
+          <t>L3</t>
+        </is>
+      </c>
+      <c r="I608" t="inlineStr">
+        <is>
+          <t>shells &amp; navigation — WorkHubShell</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(roadmap): reconcile 29–30 Sep into the record — 38 items added (WHS-1/1b, HR-TS-*, CORE-3, INC-2, ERR-1, RBAC-CE-1, GATE-2, FILES-CREW-1, TASK-CREW-1, SHIFT-SUBMIT, CLOCK-2, KERN-TIME-1, WB-A..E, PEPPOL-1, BRAND-1, …), 5 updated; layer 'L0 Kernel' → 'L0'; Summary formulas counted rows 2–334 of 608 (now to 2000)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/.agents/coral-roadmap.xlsx
+++ b/.agents/coral-roadmap.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roadmap" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Florin - my actions" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Roadmap" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Florin - my actions" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Summary" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Roadmap'!$A$1:$G$334</definedName>
@@ -594,7 +594,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I608"/>
+  <dimension ref="A1:I646"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -24642,7 +24642,7 @@
       </c>
       <c r="E543" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="F543" t="inlineStr">
@@ -24652,7 +24652,7 @@
       </c>
       <c r="G543" t="inlineStr">
         <is>
-          <t>Planner recommends Step 1 then B: rewrite the 3 shift-editor files (3,508 lines, 22%) against the corrected kernel; repair the display layer in place. A = tail-chasing, C = premature (kernel mid-repair, PROJ-0 undecided, R1-4 four gates out). | BETTER DECIDED AFTER TD-0: the real error count across 21 files is the missing input. A file needing 40 exceptions argues rebuild; one needing 3 argues repair.</t>
+          <t>Planner recommends Step 1 then B: rewrite the 3 shift-editor files (3,508 lines, 22%) against the corrected kernel; repair the display layer in place. A = tail-chasing, C = premature (kernel mid-repair, PROJ-0 undecided, R1-4 four gates out). | BETTER DECIDED AFTER TD-0: the real error count across 21 files is the missing input. A file needing 40 exceptions argues rebuild; one needing 3 argues repair. | Planner 2026-09-30: Crew-native screens: Time Off, My hours, My tasks, Documents, Profile, Shift Brief (37e9036…499e165). Home still the admin Index component.</t>
         </is>
       </c>
       <c r="H543" t="inlineStr">
@@ -25253,7 +25253,7 @@
       </c>
       <c r="E556" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F556" t="inlineStr">
@@ -25263,7 +25263,7 @@
       </c>
       <c r="G556" t="inlineStr">
         <is>
-          <t>Reachable today only from ClockButton on the workhub home; NOT from a shift card. Any rebuild must preserve it as a first-class path.</t>
+          <t>Reachable today only from ClockButton on the workhub home; NOT from a shift card. Any rebuild must preserve it as a first-class path. | Planner 2026-09-30: no-shift path kept; clock-in without shift always available (24cec9c)</t>
         </is>
       </c>
       <c r="H556" t="inlineStr">
@@ -26663,7 +26663,7 @@
       </c>
       <c r="E586" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="F586" t="inlineStr">
@@ -26673,7 +26673,7 @@
       </c>
       <c r="G586" t="inlineStr">
         <is>
-          <t>ScheduledShift.shiftDate/Start/End are String; ClockEntry.clockInTime is DateTime. 25 hand-parse sites (split('-')/split(':')) exist because the text form forces every consumer to parse. The kernel owns the arithmetic (computeWorkedDuration) but no TYPE. A kernel time type makes this crash class unrepresentable.</t>
+          <t>ScheduledShift.shiftDate/Start/End are String; ClockEntry.clockInTime is DateTime. 25 hand-parse sites (split('-')/split(':')) exist because the text form forces every consumer to parse. The kernel owns the arithmetic (computeWorkedDuration) but no TYPE. A kernel time type makes this crash class unrepresentable. | Planner 2026-09-30: kernel/shift-time.ts created (KERN-TIME-1)</t>
         </is>
       </c>
       <c r="H586" t="inlineStr">
@@ -26992,7 +26992,7 @@
       </c>
       <c r="E593" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="F593" t="inlineStr">
@@ -27002,7 +27002,7 @@
       </c>
       <c r="G593" t="inlineStr">
         <is>
-          <t>@ts-expect-error is 0 and CANNOT come back: TimesheetView and Performance declare LOCAL snake_case interfaces, so those reads type-check and tsc never saw them. The ESLint allowlist matches the PATTERN including TSPropertySignature, so a locally-declared wrong shape cannot hide. Surface: 9 files already clean, 17-file tail, 4 local-interface files, 3 SKIPPED (WH-7 rebuilds two, WH-UI-1 deletes one), 3 bridges last.</t>
+          <t>@ts-expect-error is 0 and CANNOT come back: TimesheetView and Performance declare LOCAL snake_case interfaces, so those reads type-check and tsc never saw them. The ESLint allowlist matches the PATTERN including TSPropertySignature, so a locally-declared wrong shape cannot hide. Surface: 9 files already clean, 17-file tail, 4 local-interface files, 3 SKIPPED (WH-7 rebuilds two, WH-UI-1 deletes one), 3 bridges last. | Planner 2026-09-30: allowlist 36 → 5</t>
         </is>
       </c>
       <c r="H593" t="inlineStr">
@@ -27148,7 +27148,7 @@
       </c>
       <c r="H596" t="inlineStr">
         <is>
-          <t>L0 Kernel</t>
+          <t>L0</t>
         </is>
       </c>
       <c r="I596" t="inlineStr">
@@ -27509,7 +27509,7 @@
       </c>
       <c r="E604" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F604" t="inlineStr">
@@ -27519,7 +27519,7 @@
       </c>
       <c r="G604" t="inlineStr">
         <is>
-          <t>Florin 2026-09-28. Time Off to nav, QuickLinks deleted, 'Today's Shift' block removed, hero section gone. Shift cards are ALREADY built to bleed (rounded-none border-x-0) and the page px-4 plus an outer Card put them back in a box. | REVISED: Florin decided the shift entry gains project NAME + tappable ADDRESS in this pass; the word 'Shift' is deleted. Clock button FIXED above the nav, green (emerald-600) when a shift is available / brand-orange when not, both labels LOCALIZED in all 5 locales. Text starts at OS default 1rem. Borders between entries kept.</t>
+          <t>Florin 2026-09-28. Time Off to nav, QuickLinks deleted, 'Today's Shift' block removed, hero section gone. Shift cards are ALREADY built to bleed (rounded-none border-x-0) and the page px-4 plus an outer Card put them back in a box. | REVISED: Florin decided the shift entry gains project NAME + tappable ADDRESS in this pass; the word 'Shift' is deleted. Clock button FIXED above the nav, green (emerald-600) when a shift is available / brand-orange when not, both labels LOCALIZED in all 5 locales. Text starts at OS default 1rem. Borders between entries kept. | Planner 2026-09-30: §9 landed; legibility root cause = iOS zoom-out (e16efb7); 1.2rem + cards (285dd63)</t>
         </is>
       </c>
       <c r="H604" t="inlineStr">
@@ -27718,6 +27718,1788 @@
       <c r="I608" t="inlineStr">
         <is>
           <t>shells &amp; navigation — WorkHubShell</t>
+        </is>
+      </c>
+    </row>
+    <row r="609">
+      <c r="A609" t="inlineStr">
+        <is>
+          <t>WHS-1</t>
+        </is>
+      </c>
+      <c r="B609" t="inlineStr">
+        <is>
+          <t>WorkHub stabilisation: allSettled, timeouts, no endless spinner, timer revert, nav</t>
+        </is>
+      </c>
+      <c r="C609" t="inlineStr">
+        <is>
+          <t>WorkHub</t>
+        </is>
+      </c>
+      <c r="D609" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E609" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F609" t="inlineStr">
+        <is>
+          <t>Planner 2026-09-30</t>
+        </is>
+      </c>
+      <c r="G609" t="inlineStr">
+        <is>
+          <t>aff03a0</t>
+        </is>
+      </c>
+      <c r="H609" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="I609" t="inlineStr">
+        <is>
+          <t>WorkHub / time-tracker</t>
+        </is>
+      </c>
+    </row>
+    <row r="610">
+      <c r="A610" t="inlineStr">
+        <is>
+          <t>WHS-1b</t>
+        </is>
+      </c>
+      <c r="B610" t="inlineStr">
+        <is>
+          <t>Clock never acts on unknown state: server refuses a 2nd open entry (409, adopt), no duplicate shift on slow network</t>
+        </is>
+      </c>
+      <c r="C610" t="inlineStr">
+        <is>
+          <t>WorkHub</t>
+        </is>
+      </c>
+      <c r="D610" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E610" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F610" t="inlineStr">
+        <is>
+          <t>Planner 2026-09-30</t>
+        </is>
+      </c>
+      <c r="G610" t="inlineStr">
+        <is>
+          <t>f7659d3</t>
+        </is>
+      </c>
+      <c r="H610" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="I610" t="inlineStr">
+        <is>
+          <t>WorkHub / time-tracker</t>
+        </is>
+      </c>
+    </row>
+    <row r="611">
+      <c r="A611" t="inlineStr">
+        <is>
+          <t>HR-TS-1</t>
+        </is>
+      </c>
+      <c r="B611" t="inlineStr">
+        <is>
+          <t>Timesheet detail: approve/deny visible, approvedBy stamped, werkbon link fixes</t>
+        </is>
+      </c>
+      <c r="C611" t="inlineStr">
+        <is>
+          <t>HR</t>
+        </is>
+      </c>
+      <c r="D611" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E611" t="inlineStr">
+        <is>
+          <t>Done (code)</t>
+        </is>
+      </c>
+      <c r="F611" t="inlineStr">
+        <is>
+          <t>Planner 2026-09-30</t>
+        </is>
+      </c>
+      <c r="G611" t="inlineStr">
+        <is>
+          <t>457f1a1 — not yet Planner-verified</t>
+        </is>
+      </c>
+      <c r="H611" t="inlineStr">
+        <is>
+          <t>L3</t>
+        </is>
+      </c>
+      <c r="I611" t="inlineStr">
+        <is>
+          <t>HR — timesheets, workforce</t>
+        </is>
+      </c>
+    </row>
+    <row r="612">
+      <c r="A612" t="inlineStr">
+        <is>
+          <t>HR-TS-3</t>
+        </is>
+      </c>
+      <c r="B612" t="inlineStr">
+        <is>
+          <t>Thumbnails: one t_ URL resolver for photos + attachments</t>
+        </is>
+      </c>
+      <c r="C612" t="inlineStr">
+        <is>
+          <t>HR</t>
+        </is>
+      </c>
+      <c r="D612" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E612" t="inlineStr">
+        <is>
+          <t>Done (code)</t>
+        </is>
+      </c>
+      <c r="F612" t="inlineStr">
+        <is>
+          <t>Planner 2026-09-30</t>
+        </is>
+      </c>
+      <c r="G612" t="inlineStr">
+        <is>
+          <t>9248788 — not yet Planner-verified</t>
+        </is>
+      </c>
+      <c r="H612" t="inlineStr">
+        <is>
+          <t>L3</t>
+        </is>
+      </c>
+      <c r="I612" t="inlineStr">
+        <is>
+          <t>HR — timesheets, workforce</t>
+        </is>
+      </c>
+    </row>
+    <row r="613">
+      <c r="A613" t="inlineStr">
+        <is>
+          <t>HR-TS-5</t>
+        </is>
+      </c>
+      <c r="B613" t="inlineStr">
+        <is>
+          <t>Timesheet detail edit mode: project picker, billable, audit log shown</t>
+        </is>
+      </c>
+      <c r="C613" t="inlineStr">
+        <is>
+          <t>HR</t>
+        </is>
+      </c>
+      <c r="D613" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E613" t="inlineStr">
+        <is>
+          <t>Done (code)</t>
+        </is>
+      </c>
+      <c r="F613" t="inlineStr">
+        <is>
+          <t>Planner 2026-09-30</t>
+        </is>
+      </c>
+      <c r="G613" t="inlineStr">
+        <is>
+          <t>e87093f — not yet Planner-verified</t>
+        </is>
+      </c>
+      <c r="H613" t="inlineStr">
+        <is>
+          <t>L3</t>
+        </is>
+      </c>
+      <c r="I613" t="inlineStr">
+        <is>
+          <t>HR — timesheets, workforce</t>
+        </is>
+      </c>
+    </row>
+    <row r="614">
+      <c r="A614" t="inlineStr">
+        <is>
+          <t>HR-TS-6</t>
+        </is>
+      </c>
+      <c r="B614" t="inlineStr">
+        <is>
+          <t>Edit pane read in local time (was UTC, 2h early)</t>
+        </is>
+      </c>
+      <c r="C614" t="inlineStr">
+        <is>
+          <t>HR</t>
+        </is>
+      </c>
+      <c r="D614" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E614" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F614" t="inlineStr">
+        <is>
+          <t>Planner 2026-09-30</t>
+        </is>
+      </c>
+      <c r="G614" t="inlineStr">
+        <is>
+          <t>8bed336</t>
+        </is>
+      </c>
+      <c r="H614" t="inlineStr">
+        <is>
+          <t>L3</t>
+        </is>
+      </c>
+      <c r="I614" t="inlineStr">
+        <is>
+          <t>HR — timesheets, workforce</t>
+        </is>
+      </c>
+    </row>
+    <row r="615">
+      <c r="A615" t="inlineStr">
+        <is>
+          <t>HR-TS-7</t>
+        </is>
+      </c>
+      <c r="B615" t="inlineStr">
+        <is>
+          <t>Entry provenance: source, createdBy, derived self-approval, notes (its migration = INC-2)</t>
+        </is>
+      </c>
+      <c r="C615" t="inlineStr">
+        <is>
+          <t>HR</t>
+        </is>
+      </c>
+      <c r="D615" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E615" t="inlineStr">
+        <is>
+          <t>Done (code)</t>
+        </is>
+      </c>
+      <c r="F615" t="inlineStr">
+        <is>
+          <t>Planner 2026-09-30</t>
+        </is>
+      </c>
+      <c r="G615" t="inlineStr">
+        <is>
+          <t>0d56eb9 — not yet Planner-verified</t>
+        </is>
+      </c>
+      <c r="H615" t="inlineStr">
+        <is>
+          <t>L3</t>
+        </is>
+      </c>
+      <c r="I615" t="inlineStr">
+        <is>
+          <t>HR — timesheets, workforce</t>
+        </is>
+      </c>
+    </row>
+    <row r="616">
+      <c r="A616" t="inlineStr">
+        <is>
+          <t>SCH-8</t>
+        </is>
+      </c>
+      <c r="B616" t="inlineStr">
+        <is>
+          <t>Series scope is decorative ("save for all" does nothing) + HR-TS-8 manual-entry project select</t>
+        </is>
+      </c>
+      <c r="C616" t="inlineStr">
+        <is>
+          <t>HR</t>
+        </is>
+      </c>
+      <c r="D616" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E616" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F616" t="inlineStr">
+        <is>
+          <t>Planner 2026-09-30</t>
+        </is>
+      </c>
+      <c r="G616" t="inlineStr">
+        <is>
+          <t>coder-directive-sch-8-series-and-manual-entry.md</t>
+        </is>
+      </c>
+      <c r="H616" t="inlineStr">
+        <is>
+          <t>L3</t>
+        </is>
+      </c>
+      <c r="I616" t="inlineStr">
+        <is>
+          <t>HR — timesheets, workforce</t>
+        </is>
+      </c>
+    </row>
+    <row r="617">
+      <c r="A617" t="inlineStr">
+        <is>
+          <t>PROJ-SSOT-1</t>
+        </is>
+      </c>
+      <c r="B617" t="inlineStr">
+        <is>
+          <t>One project resolver; retire HrProject (export Project column resolves from an empty table). Land before hours are attributed + exported.</t>
+        </is>
+      </c>
+      <c r="C617" t="inlineStr">
+        <is>
+          <t>Projects</t>
+        </is>
+      </c>
+      <c r="D617" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E617" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F617" t="inlineStr">
+        <is>
+          <t>Planner 2026-09-30</t>
+        </is>
+      </c>
+      <c r="G617" t="inlineStr">
+        <is>
+          <t>census 2026-09-30: 26 unattributed by design, 1 dangling cleared</t>
+        </is>
+      </c>
+      <c r="H617" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="I617" t="inlineStr">
+        <is>
+          <t>ERP core — mixed triage</t>
+        </is>
+      </c>
+    </row>
+    <row r="618">
+      <c r="A618" t="inlineStr">
+        <is>
+          <t>CORE-3</t>
+        </is>
+      </c>
+      <c r="B618" t="inlineStr">
+        <is>
+          <t>$transaction received a resolved audit record; every clock-entry PATCH failed; audit rows outside the tx</t>
+        </is>
+      </c>
+      <c r="C618" t="inlineStr">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="D618" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E618" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F618" t="inlineStr">
+        <is>
+          <t>Planner 2026-09-30</t>
+        </is>
+      </c>
+      <c r="G618" t="inlineStr">
+        <is>
+          <t>0e66a1d</t>
+        </is>
+      </c>
+      <c r="H618" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="I618" t="inlineStr">
+        <is>
+          <t>write path — saveRecord, intents, read model</t>
+        </is>
+      </c>
+    </row>
+    <row r="619">
+      <c r="A619" t="inlineStr">
+        <is>
+          <t>INC-2</t>
+        </is>
+      </c>
+      <c r="B619" t="inlineStr">
+        <is>
+          <t>Schema deployed before its migration → P2022 on every clockEntry read; crew could not clock in. Rule pd.md 5e.</t>
+        </is>
+      </c>
+      <c r="C619" t="inlineStr">
+        <is>
+          <t>Process</t>
+        </is>
+      </c>
+      <c r="D619" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E619" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F619" t="inlineStr">
+        <is>
+          <t>Planner 2026-09-30</t>
+        </is>
+      </c>
+      <c r="G619" t="inlineStr">
+        <is>
+          <t>pd.md 5e</t>
+        </is>
+      </c>
+      <c r="H619" t="inlineStr">
+        <is>
+          <t>⟂</t>
+        </is>
+      </c>
+      <c r="I619" t="inlineStr">
+        <is>
+          <t>process &amp; housekeeping</t>
+        </is>
+      </c>
+    </row>
+    <row r="620">
+      <c r="A620" t="inlineStr">
+        <is>
+          <t>ERR-1</t>
+        </is>
+      </c>
+      <c r="B620" t="inlineStr">
+        <is>
+          <t>describeError: one definition of "what went wrong", 49 sites</t>
+        </is>
+      </c>
+      <c r="C620" t="inlineStr">
+        <is>
+          <t>Process</t>
+        </is>
+      </c>
+      <c r="D620" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E620" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F620" t="inlineStr">
+        <is>
+          <t>Planner 2026-09-30</t>
+        </is>
+      </c>
+      <c r="G620" t="inlineStr">
+        <is>
+          <t>ea8cfdb…de6ad3c · report cc20582</t>
+        </is>
+      </c>
+      <c r="H620" t="inlineStr">
+        <is>
+          <t>⟂</t>
+        </is>
+      </c>
+      <c r="I620" t="inlineStr">
+        <is>
+          <t>process &amp; housekeeping</t>
+        </is>
+      </c>
+    </row>
+    <row r="621">
+      <c r="A621" t="inlineStr">
+        <is>
+          <t>RBAC-CE-1</t>
+        </is>
+      </c>
+      <c r="B621" t="inlineStr">
+        <is>
+          <t>Seraph gaps on the hours write path: foreign userId accepted; team-scoping ignored tenantId</t>
+        </is>
+      </c>
+      <c r="C621" t="inlineStr">
+        <is>
+          <t>Seraph</t>
+        </is>
+      </c>
+      <c r="D621" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E621" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F621" t="inlineStr">
+        <is>
+          <t>Planner 2026-09-30</t>
+        </is>
+      </c>
+      <c r="G621" t="inlineStr">
+        <is>
+          <t>b293961</t>
+        </is>
+      </c>
+      <c r="H621" t="inlineStr">
+        <is>
+          <t>GATE</t>
+        </is>
+      </c>
+      <c r="I621" t="inlineStr">
+        <is>
+          <t>the seraph — resolver, logicalKey, scoped accessor</t>
+        </is>
+      </c>
+    </row>
+    <row r="622">
+      <c r="A622" t="inlineStr">
+        <is>
+          <t>GATE-2</t>
+        </is>
+      </c>
+      <c r="B622" t="inlineStr">
+        <is>
+          <t>Actor reach bridge: one authority (actor-reach.ts, isTenantHrRole in lib/roles) + pure write policy (22 tests). Crew could approve own hours/leave. Exit: R1-4 scope.reach().</t>
+        </is>
+      </c>
+      <c r="C622" t="inlineStr">
+        <is>
+          <t>Gates</t>
+        </is>
+      </c>
+      <c r="D622" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E622" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F622" t="inlineStr">
+        <is>
+          <t>Planner 2026-09-30</t>
+        </is>
+      </c>
+      <c r="G622" t="inlineStr">
+        <is>
+          <t>ebb27d6 · f54e0ae · SUPERADMIN everywhere (Florin)</t>
+        </is>
+      </c>
+      <c r="H622" t="inlineStr">
+        <is>
+          <t>GATE</t>
+        </is>
+      </c>
+      <c r="I622" t="inlineStr">
+        <is>
+          <t>actor reach · platform access · operator scopes</t>
+        </is>
+      </c>
+    </row>
+    <row r="623">
+      <c r="A623" t="inlineStr">
+        <is>
+          <t>GATE-2b</t>
+        </is>
+      </c>
+      <c r="B623" t="inlineStr">
+        <is>
+          <t>Crew self-service on shifts / shift-tasks / attachments needs reach-on-parent</t>
+        </is>
+      </c>
+      <c r="C623" t="inlineStr">
+        <is>
+          <t>Gates</t>
+        </is>
+      </c>
+      <c r="D623" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E623" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F623" t="inlineStr">
+        <is>
+          <t>Planner 2026-09-30</t>
+        </is>
+      </c>
+      <c r="G623" t="inlineStr">
+        <is>
+          <t>rides with R1-4</t>
+        </is>
+      </c>
+      <c r="H623" t="inlineStr">
+        <is>
+          <t>GATE</t>
+        </is>
+      </c>
+      <c r="I623" t="inlineStr">
+        <is>
+          <t>actor reach · platform access · operator scopes</t>
+        </is>
+      </c>
+    </row>
+    <row r="624">
+      <c r="A624" t="inlineStr">
+        <is>
+          <t>CE-TIME-1</t>
+        </is>
+      </c>
+      <c r="B624" t="inlineStr">
+        <is>
+          <t>Server stamps live clock-in and crew clock-out (phone could backdate)</t>
+        </is>
+      </c>
+      <c r="C624" t="inlineStr">
+        <is>
+          <t>WorkHub</t>
+        </is>
+      </c>
+      <c r="D624" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E624" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F624" t="inlineStr">
+        <is>
+          <t>Planner 2026-09-30</t>
+        </is>
+      </c>
+      <c r="G624" t="inlineStr">
+        <is>
+          <t>da6977f</t>
+        </is>
+      </c>
+      <c r="H624" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="I624" t="inlineStr">
+        <is>
+          <t>WorkHub / time-tracker</t>
+        </is>
+      </c>
+    </row>
+    <row r="625">
+      <c r="A625" t="inlineStr">
+        <is>
+          <t>FILES-CREW-1</t>
+        </is>
+      </c>
+      <c r="B625" t="inlineStr">
+        <is>
+          <t>Crew could list/delete/overwrite every tenant file; whole ERP dataset shipped to crew phones</t>
+        </is>
+      </c>
+      <c r="C625" t="inlineStr">
+        <is>
+          <t>Storage</t>
+        </is>
+      </c>
+      <c r="D625" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E625" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F625" t="inlineStr">
+        <is>
+          <t>Planner 2026-09-30</t>
+        </is>
+      </c>
+      <c r="G625" t="inlineStr">
+        <is>
+          <t>f8f2aa0 · 3542abb</t>
+        </is>
+      </c>
+      <c r="H625" t="inlineStr">
+        <is>
+          <t>L0</t>
+        </is>
+      </c>
+      <c r="I625" t="inlineStr">
+        <is>
+          <t>storage — the one blob door</t>
+        </is>
+      </c>
+    </row>
+    <row r="626">
+      <c r="A626" t="inlineStr">
+        <is>
+          <t>FILES-GATE-1</t>
+        </is>
+      </c>
+      <c r="B626" t="inlineStr">
+        <is>
+          <t>Office roles still reach every file — folds into ENT (function-confined roles, owner grants per role + person overrides)</t>
+        </is>
+      </c>
+      <c r="C626" t="inlineStr">
+        <is>
+          <t>Entitlement</t>
+        </is>
+      </c>
+      <c r="D626" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E626" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F626" t="inlineStr">
+        <is>
+          <t>Planner 2026-09-30</t>
+        </is>
+      </c>
+      <c r="G626" t="inlineStr">
+        <is>
+          <t>Florin 2026-09-30</t>
+        </is>
+      </c>
+      <c r="H626" t="inlineStr">
+        <is>
+          <t>MODULE GATE</t>
+        </is>
+      </c>
+      <c r="I626" t="inlineStr">
+        <is>
+          <t>entitlement — vocabulary &amp; grants (modules → submodules → quota)</t>
+        </is>
+      </c>
+    </row>
+    <row r="627">
+      <c r="A627" t="inlineStr">
+        <is>
+          <t>TASK-CREW-1</t>
+        </is>
+      </c>
+      <c r="B627" t="inlineStr">
+        <is>
+          <t>Crew task status + notes with photos (draft → submit frozen) + read-only change log in WorkHub and ERP</t>
+        </is>
+      </c>
+      <c r="C627" t="inlineStr">
+        <is>
+          <t>Tasks</t>
+        </is>
+      </c>
+      <c r="D627" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E627" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F627" t="inlineStr">
+        <is>
+          <t>Planner 2026-09-30</t>
+        </is>
+      </c>
+      <c r="G627" t="inlineStr">
+        <is>
+          <t>93bbe1d · TaskNote table migrated by Florin</t>
+        </is>
+      </c>
+      <c r="H627" t="inlineStr">
+        <is>
+          <t>L3</t>
+        </is>
+      </c>
+      <c r="I627" t="inlineStr">
+        <is>
+          <t>Tasks submodule</t>
+        </is>
+      </c>
+    </row>
+    <row r="628">
+      <c r="A628" t="inlineStr">
+        <is>
+          <t>SHIFT-SUBMIT</t>
+        </is>
+      </c>
+      <c r="B628" t="inlineStr">
+        <is>
+          <t>A shift is completed ONLY when its worker submits it (5 automatic completions removed); audited</t>
+        </is>
+      </c>
+      <c r="C628" t="inlineStr">
+        <is>
+          <t>WorkHub</t>
+        </is>
+      </c>
+      <c r="D628" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E628" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F628" t="inlineStr">
+        <is>
+          <t>Planner 2026-09-30</t>
+        </is>
+      </c>
+      <c r="G628" t="inlineStr">
+        <is>
+          <t>bacc329</t>
+        </is>
+      </c>
+      <c r="H628" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="I628" t="inlineStr">
+        <is>
+          <t>WorkHub / time-tracker</t>
+        </is>
+      </c>
+    </row>
+    <row r="629">
+      <c r="A629" t="inlineStr">
+        <is>
+          <t>CLOCK-2</t>
+        </is>
+      </c>
+      <c r="B629" t="inlineStr">
+        <is>
+          <t>Clock into a shift more than once; shifts in time order; "clock in without shift"; clock-out no longer rewrites planned shifts</t>
+        </is>
+      </c>
+      <c r="C629" t="inlineStr">
+        <is>
+          <t>WorkHub</t>
+        </is>
+      </c>
+      <c r="D629" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E629" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F629" t="inlineStr">
+        <is>
+          <t>Planner 2026-09-30</t>
+        </is>
+      </c>
+      <c r="G629" t="inlineStr">
+        <is>
+          <t>24cec9c</t>
+        </is>
+      </c>
+      <c r="H629" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="I629" t="inlineStr">
+        <is>
+          <t>WorkHub / time-tracker</t>
+        </is>
+      </c>
+    </row>
+    <row r="630">
+      <c r="A630" t="inlineStr">
+        <is>
+          <t>KERN-TIME-1</t>
+        </is>
+      </c>
+      <c r="B630" t="inlineStr">
+        <is>
+          <t>Kernel shift-time: moments from parts, local dates, pickShiftNow, zoned server time (Europe/Brussels via Intl)</t>
+        </is>
+      </c>
+      <c r="C630" t="inlineStr">
+        <is>
+          <t>Kernel</t>
+        </is>
+      </c>
+      <c r="D630" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E630" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F630" t="inlineStr">
+        <is>
+          <t>Planner 2026-09-30</t>
+        </is>
+      </c>
+      <c r="G630" t="inlineStr">
+        <is>
+          <t>24cec9c · 8880e5b</t>
+        </is>
+      </c>
+      <c r="H630" t="inlineStr">
+        <is>
+          <t>L0</t>
+        </is>
+      </c>
+      <c r="I630" t="inlineStr">
+        <is>
+          <t>time — duration, the break rule</t>
+        </is>
+      </c>
+    </row>
+    <row r="631">
+      <c r="A631" t="inlineStr">
+        <is>
+          <t>TENANT-TZ</t>
+        </is>
+      </c>
+      <c r="B631" t="inlineStr">
+        <is>
+          <t>Per-tenant timezone setting (kernel assumes Europe/Brussels)</t>
+        </is>
+      </c>
+      <c r="C631" t="inlineStr">
+        <is>
+          <t>Kernel</t>
+        </is>
+      </c>
+      <c r="D631" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="E631" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F631" t="inlineStr">
+        <is>
+          <t>Planner 2026-09-30</t>
+        </is>
+      </c>
+      <c r="G631" t="inlineStr">
+        <is>
+          <t>after KERN-TIME-1</t>
+        </is>
+      </c>
+      <c r="H631" t="inlineStr">
+        <is>
+          <t>L0</t>
+        </is>
+      </c>
+      <c r="I631" t="inlineStr">
+        <is>
+          <t>time — duration, the break rule</t>
+        </is>
+      </c>
+    </row>
+    <row r="632">
+      <c r="A632" t="inlineStr">
+        <is>
+          <t>WH-EXPORT-1</t>
+        </is>
+      </c>
+      <c r="B632" t="inlineStr">
+        <is>
+          <t>Worker-facing timesheet export (My hours: month → Excel/PDF from the official export)</t>
+        </is>
+      </c>
+      <c r="C632" t="inlineStr">
+        <is>
+          <t>WorkHub</t>
+        </is>
+      </c>
+      <c r="D632" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E632" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F632" t="inlineStr">
+        <is>
+          <t>Planner 2026-09-30</t>
+        </is>
+      </c>
+      <c r="G632" t="inlineStr">
+        <is>
+          <t>8880e5b</t>
+        </is>
+      </c>
+      <c r="H632" t="inlineStr">
+        <is>
+          <t>L3</t>
+        </is>
+      </c>
+      <c r="I632" t="inlineStr">
+        <is>
+          <t>HR — timesheets, workforce</t>
+        </is>
+      </c>
+    </row>
+    <row r="633">
+      <c r="A633" t="inlineStr">
+        <is>
+          <t>LATE-1</t>
+        </is>
+      </c>
+      <c r="B633" t="inlineStr">
+        <is>
+          <t>Two late-entry paths (LateEntryCard → server action, LateEntryForm → HR API) — merge into one</t>
+        </is>
+      </c>
+      <c r="C633" t="inlineStr">
+        <is>
+          <t>HR</t>
+        </is>
+      </c>
+      <c r="D633" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="E633" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F633" t="inlineStr">
+        <is>
+          <t>Planner 2026-09-30</t>
+        </is>
+      </c>
+      <c r="G633" t="inlineStr">
+        <is>
+          <t>found 2026-09-30</t>
+        </is>
+      </c>
+      <c r="H633" t="inlineStr">
+        <is>
+          <t>L3</t>
+        </is>
+      </c>
+      <c r="I633" t="inlineStr">
+        <is>
+          <t>HR — timesheets, workforce</t>
+        </is>
+      </c>
+    </row>
+    <row r="634">
+      <c r="A634" t="inlineStr">
+        <is>
+          <t>I18N-TT-1</t>
+        </is>
+      </c>
+      <c r="B634" t="inlineStr">
+        <is>
+          <t>Test guard for the crew i18n instance; Russian completed</t>
+        </is>
+      </c>
+      <c r="C634" t="inlineStr">
+        <is>
+          <t>Process</t>
+        </is>
+      </c>
+      <c r="D634" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E634" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F634" t="inlineStr">
+        <is>
+          <t>Planner 2026-09-30</t>
+        </is>
+      </c>
+      <c r="G634" t="inlineStr">
+        <is>
+          <t>7ed7735</t>
+        </is>
+      </c>
+      <c r="H634" t="inlineStr">
+        <is>
+          <t>⟂</t>
+        </is>
+      </c>
+      <c r="I634" t="inlineStr">
+        <is>
+          <t>CI gates</t>
+        </is>
+      </c>
+    </row>
+    <row r="635">
+      <c r="A635" t="inlineStr">
+        <is>
+          <t>WB-A</t>
+        </is>
+      </c>
+      <c r="B635" t="inlineStr">
+        <is>
+          <t>Werkbon: order giver on the shift (client page, not the empty Contact table)</t>
+        </is>
+      </c>
+      <c r="C635" t="inlineStr">
+        <is>
+          <t>Werkbon</t>
+        </is>
+      </c>
+      <c r="D635" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E635" t="inlineStr">
+        <is>
+          <t>Done (code)</t>
+        </is>
+      </c>
+      <c r="F635" t="inlineStr">
+        <is>
+          <t>Planner 2026-09-30</t>
+        </is>
+      </c>
+      <c r="G635" t="inlineStr">
+        <is>
+          <t>4735871 · column migrated by Florin</t>
+        </is>
+      </c>
+      <c r="H635" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="I635" t="inlineStr">
+        <is>
+          <t>document engine (+ archive, attachments)</t>
+        </is>
+      </c>
+    </row>
+    <row r="636">
+      <c r="A636" t="inlineStr">
+        <is>
+          <t>WB-B</t>
+        </is>
+      </c>
+      <c r="B636" t="inlineStr">
+        <is>
+          <t>Werkbon record + recorded membership + crew picker (no signing)</t>
+        </is>
+      </c>
+      <c r="C636" t="inlineStr">
+        <is>
+          <t>Werkbon</t>
+        </is>
+      </c>
+      <c r="D636" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E636" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F636" t="inlineStr">
+        <is>
+          <t>Planner 2026-09-30</t>
+        </is>
+      </c>
+      <c r="G636" t="inlineStr">
+        <is>
+          <t>phasing A → B → C+D → E (Florin)</t>
+        </is>
+      </c>
+      <c r="H636" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="I636" t="inlineStr">
+        <is>
+          <t>document engine (+ archive, attachments)</t>
+        </is>
+      </c>
+    </row>
+    <row r="637">
+      <c r="A637" t="inlineStr">
+        <is>
+          <t>WB-C</t>
+        </is>
+      </c>
+      <c r="B637" t="inlineStr">
+        <is>
+          <t>Werkbon signing + frozen PDF — ships WITH WB-D</t>
+        </is>
+      </c>
+      <c r="C637" t="inlineStr">
+        <is>
+          <t>Werkbon</t>
+        </is>
+      </c>
+      <c r="D637" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E637" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F637" t="inlineStr">
+        <is>
+          <t>Planner 2026-09-30</t>
+        </is>
+      </c>
+      <c r="G637" t="inlineStr">
+        <is>
+          <t>the lock has the grain of the work order, not the day</t>
+        </is>
+      </c>
+      <c r="H637" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="I637" t="inlineStr">
+        <is>
+          <t>document engine (+ archive, attachments)</t>
+        </is>
+      </c>
+    </row>
+    <row r="638">
+      <c r="A638" t="inlineStr">
+        <is>
+          <t>WB-D</t>
+        </is>
+      </c>
+      <c r="B638" t="inlineStr">
+        <is>
+          <t>Route-level transitive freeze of the work order — ships WITH WB-C</t>
+        </is>
+      </c>
+      <c r="C638" t="inlineStr">
+        <is>
+          <t>Werkbon</t>
+        </is>
+      </c>
+      <c r="D638" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E638" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F638" t="inlineStr">
+        <is>
+          <t>Planner 2026-09-30</t>
+        </is>
+      </c>
+      <c r="G638" t="inlineStr">
+        <is>
+          <t>never freeze by date or worker</t>
+        </is>
+      </c>
+      <c r="H638" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="I638" t="inlineStr">
+        <is>
+          <t>document engine (+ archive, attachments)</t>
+        </is>
+      </c>
+    </row>
+    <row r="639">
+      <c r="A639" t="inlineStr">
+        <is>
+          <t>WB-E</t>
+        </is>
+      </c>
+      <c r="B639" t="inlineStr">
+        <is>
+          <t>Cron send to the order giver + unsent visibility</t>
+        </is>
+      </c>
+      <c r="C639" t="inlineStr">
+        <is>
+          <t>Werkbon</t>
+        </is>
+      </c>
+      <c r="D639" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="E639" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F639" t="inlineStr">
+        <is>
+          <t>Planner 2026-09-30</t>
+        </is>
+      </c>
+      <c r="G639" t="inlineStr"/>
+      <c r="H639" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="I639" t="inlineStr">
+        <is>
+          <t>document engine (+ archive, attachments)</t>
+        </is>
+      </c>
+    </row>
+    <row r="640">
+      <c r="A640" t="inlineStr">
+        <is>
+          <t>PEPPOL-1</t>
+        </is>
+      </c>
+      <c r="B640" t="inlineStr">
+        <is>
+          <t>One Peppol quota table (billing reads enforcement); FREE 5 sent (draft above) / 20 received soft + the payment-method case; PRO/ENT fair use pending the reseller rate</t>
+        </is>
+      </c>
+      <c r="C640" t="inlineStr">
+        <is>
+          <t>Entitlement</t>
+        </is>
+      </c>
+      <c r="D640" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E640" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F640" t="inlineStr">
+        <is>
+          <t>Planner 2026-09-30</t>
+        </is>
+      </c>
+      <c r="G640" t="inlineStr">
+        <is>
+          <t>feature_matrix.md decisions log 2026-09-30</t>
+        </is>
+      </c>
+      <c r="H640" t="inlineStr">
+        <is>
+          <t>MODULE GATE</t>
+        </is>
+      </c>
+      <c r="I640" t="inlineStr">
+        <is>
+          <t>entitlement — vocabulary &amp; grants (modules → submodules → quota)</t>
+        </is>
+      </c>
+    </row>
+    <row r="641">
+      <c r="A641" t="inlineStr">
+        <is>
+          <t>BRAND-1</t>
+        </is>
+      </c>
+      <c r="B641" t="inlineStr">
+        <is>
+          <t>Basic branding (logo, stationery, colour, templates) never gated on any tier</t>
+        </is>
+      </c>
+      <c r="C641" t="inlineStr">
+        <is>
+          <t>Entitlement</t>
+        </is>
+      </c>
+      <c r="D641" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E641" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F641" t="inlineStr">
+        <is>
+          <t>Planner 2026-09-30</t>
+        </is>
+      </c>
+      <c r="G641" t="inlineStr">
+        <is>
+          <t>Florin 2026-09-30</t>
+        </is>
+      </c>
+      <c r="H641" t="inlineStr">
+        <is>
+          <t>MODULE GATE</t>
+        </is>
+      </c>
+      <c r="I641" t="inlineStr">
+        <is>
+          <t>entitlement — vocabulary &amp; grants (modules → submodules → quota)</t>
+        </is>
+      </c>
+    </row>
+    <row r="642">
+      <c r="A642" t="inlineStr">
+        <is>
+          <t>BATIPRIX-1</t>
+        </is>
+      </c>
+      <c r="B642" t="inlineStr">
+        <is>
+          <t>Batiprix = Enterprise-only add-on (retire the ENTERPRISE_BATIPRIX tier)</t>
+        </is>
+      </c>
+      <c r="C642" t="inlineStr">
+        <is>
+          <t>Entitlement</t>
+        </is>
+      </c>
+      <c r="D642" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="E642" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F642" t="inlineStr">
+        <is>
+          <t>Planner 2026-09-30</t>
+        </is>
+      </c>
+      <c r="G642" t="inlineStr">
+        <is>
+          <t>Florin 2026-09-30</t>
+        </is>
+      </c>
+      <c r="H642" t="inlineStr">
+        <is>
+          <t>MODULE GATE</t>
+        </is>
+      </c>
+      <c r="I642" t="inlineStr">
+        <is>
+          <t>entitlement — vocabulary &amp; grants (modules → submodules → quota)</t>
+        </is>
+      </c>
+    </row>
+    <row r="643">
+      <c r="A643" t="inlineStr">
+        <is>
+          <t>PRO-DEF</t>
+        </is>
+      </c>
+      <c r="B643" t="inlineStr">
+        <is>
+          <t>Define PRO — draft with three shapes (the HR/WorkHub contradiction)</t>
+        </is>
+      </c>
+      <c r="C643" t="inlineStr">
+        <is>
+          <t>Entitlement</t>
+        </is>
+      </c>
+      <c r="D643" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E643" t="inlineStr">
+        <is>
+          <t>Decided</t>
+        </is>
+      </c>
+      <c r="F643" t="inlineStr">
+        <is>
+          <t>Planner 2026-09-30</t>
+        </is>
+      </c>
+      <c r="G643" t="inlineStr">
+        <is>
+          <t>coral-draft-pro-tier.md — awaiting Florin</t>
+        </is>
+      </c>
+      <c r="H643" t="inlineStr">
+        <is>
+          <t>MODULE GATE</t>
+        </is>
+      </c>
+      <c r="I643" t="inlineStr">
+        <is>
+          <t>entitlement — vocabulary &amp; grants (modules → submodules → quota)</t>
+        </is>
+      </c>
+    </row>
+    <row r="644">
+      <c r="A644" t="inlineStr">
+        <is>
+          <t>OPEN-ENTRY-IDX</t>
+        </is>
+      </c>
+      <c r="B644" t="inlineStr">
+        <is>
+          <t>Partial unique index: one open clock entry per worker (durable form of WHS-1b)</t>
+        </is>
+      </c>
+      <c r="C644" t="inlineStr">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="D644" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="E644" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F644" t="inlineStr">
+        <is>
+          <t>Planner 2026-09-30</t>
+        </is>
+      </c>
+      <c r="G644" t="inlineStr">
+        <is>
+          <t>Florin's migration, when wanted</t>
+        </is>
+      </c>
+      <c r="H644" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="I644" t="inlineStr">
+        <is>
+          <t>write path — concurrency</t>
+        </is>
+      </c>
+    </row>
+    <row r="645">
+      <c r="A645" t="inlineStr">
+        <is>
+          <t>BRANCH-PROTECT</t>
+        </is>
+      </c>
+      <c r="B645" t="inlineStr">
+        <is>
+          <t>Branch protection on main requiring CI green (red commits reached main 27 + 28 Sep)</t>
+        </is>
+      </c>
+      <c r="C645" t="inlineStr">
+        <is>
+          <t>Process</t>
+        </is>
+      </c>
+      <c r="D645" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E645" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F645" t="inlineStr">
+        <is>
+          <t>Planner 2026-09-30</t>
+        </is>
+      </c>
+      <c r="G645" t="inlineStr">
+        <is>
+          <t>GitHub setting — Florin</t>
+        </is>
+      </c>
+      <c r="H645" t="inlineStr">
+        <is>
+          <t>⟂</t>
+        </is>
+      </c>
+      <c r="I645" t="inlineStr">
+        <is>
+          <t>CI gates</t>
+        </is>
+      </c>
+    </row>
+    <row r="646">
+      <c r="A646" t="inlineStr">
+        <is>
+          <t>ROADMAP-SUM</t>
+        </is>
+      </c>
+      <c r="B646" t="inlineStr">
+        <is>
+          <t>Summary sheet counted rows 2–334 of 608</t>
+        </is>
+      </c>
+      <c r="C646" t="inlineStr">
+        <is>
+          <t>Process</t>
+        </is>
+      </c>
+      <c r="D646" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="E646" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F646" t="inlineStr">
+        <is>
+          <t>Planner 2026-09-30</t>
+        </is>
+      </c>
+      <c r="G646" t="inlineStr">
+        <is>
+          <t>fixed 2026-09-30</t>
+        </is>
+      </c>
+      <c r="H646" t="inlineStr">
+        <is>
+          <t>⟂</t>
+        </is>
+      </c>
+      <c r="I646" t="inlineStr">
+        <is>
+          <t>process &amp; housekeeping</t>
         </is>
       </c>
     </row>
@@ -28318,7 +30100,7 @@
         </is>
       </c>
       <c r="B2" s="3">
-        <f>COUNTA(Roadmap!A2:A334)</f>
+        <f>COUNTA(Roadmap!A2:A2000)</f>
         <v/>
       </c>
     </row>
@@ -28329,7 +30111,7 @@
         </is>
       </c>
       <c r="B3" s="3">
-        <f>COUNTIF(Roadmap!E2:E334,"Open")</f>
+        <f>COUNTIF(Roadmap!E2:E2000,"Open")</f>
         <v/>
       </c>
     </row>
@@ -28340,7 +30122,7 @@
         </is>
       </c>
       <c r="B4" s="3">
-        <f>COUNTIF(Roadmap!E2:E334,"In progress")</f>
+        <f>COUNTIF(Roadmap!E2:E2000,"In progress")</f>
         <v/>
       </c>
     </row>
@@ -28351,7 +30133,7 @@
         </is>
       </c>
       <c r="B5" s="3">
-        <f>COUNTIF(Roadmap!E2:E334,"Done")</f>
+        <f>COUNTIF(Roadmap!E2:E2000,"Done")</f>
         <v/>
       </c>
     </row>
@@ -28366,7 +30148,7 @@
         </is>
       </c>
       <c r="B7" s="3">
-        <f>COUNTIF(Roadmap!D2:D334,"P0")</f>
+        <f>COUNTIF(Roadmap!D2:D2000,"P0")</f>
         <v/>
       </c>
     </row>
@@ -28377,7 +30159,7 @@
         </is>
       </c>
       <c r="B8" s="3">
-        <f>COUNTIFS(Roadmap!D2:D334,"P0",Roadmap!E2:E334,"Open")</f>
+        <f>COUNTIFS(Roadmap!D2:D2000,"P0",Roadmap!E2:E2000,"Open")</f>
         <v/>
       </c>
     </row>
@@ -28388,7 +30170,7 @@
         </is>
       </c>
       <c r="B9" s="3">
-        <f>COUNTIF(Roadmap!D2:D334,"P1")</f>
+        <f>COUNTIF(Roadmap!D2:D2000,"P1")</f>
         <v/>
       </c>
     </row>
@@ -28399,7 +30181,7 @@
         </is>
       </c>
       <c r="B10" s="3">
-        <f>COUNTIFS(Roadmap!D2:D334,"P1",Roadmap!E2:E334,"Open")</f>
+        <f>COUNTIFS(Roadmap!D2:D2000,"P1",Roadmap!E2:E2000,"Open")</f>
         <v/>
       </c>
     </row>
@@ -28410,7 +30192,7 @@
         </is>
       </c>
       <c r="B11" s="3">
-        <f>COUNTIF(Roadmap!D2:D334,"P2")</f>
+        <f>COUNTIF(Roadmap!D2:D2000,"P2")</f>
         <v/>
       </c>
     </row>
@@ -28421,7 +30203,7 @@
         </is>
       </c>
       <c r="B12" s="3">
-        <f>COUNTIFS(Roadmap!D2:D334,"P2",Roadmap!E2:E334,"Open")</f>
+        <f>COUNTIFS(Roadmap!D2:D2000,"P2",Roadmap!E2:E2000,"Open")</f>
         <v/>
       </c>
     </row>
@@ -28432,7 +30214,7 @@
         </is>
       </c>
       <c r="B13" s="3">
-        <f>COUNTIF(Roadmap!D2:D334,"P3")</f>
+        <f>COUNTIF(Roadmap!D2:D2000,"P3")</f>
         <v/>
       </c>
     </row>
@@ -28443,7 +30225,7 @@
         </is>
       </c>
       <c r="B14" s="3">
-        <f>COUNTIFS(Roadmap!D2:D334,"P3",Roadmap!E2:E334,"Open")</f>
+        <f>COUNTIFS(Roadmap!D2:D2000,"P3",Roadmap!E2:E2000,"Open")</f>
         <v/>
       </c>
     </row>
@@ -28454,7 +30236,7 @@
         </is>
       </c>
       <c r="B15" s="3">
-        <f>COUNTIF(Roadmap!D2:D334,"P4")</f>
+        <f>COUNTIF(Roadmap!D2:D2000,"P4")</f>
         <v/>
       </c>
     </row>
@@ -28465,7 +30247,7 @@
         </is>
       </c>
       <c r="B16" s="3">
-        <f>COUNTIFS(Roadmap!D2:D334,"P4",Roadmap!E2:E334,"Open")</f>
+        <f>COUNTIFS(Roadmap!D2:D2000,"P4",Roadmap!E2:E2000,"Open")</f>
         <v/>
       </c>
     </row>
@@ -28488,7 +30270,7 @@
         </is>
       </c>
       <c r="B19" s="3">
-        <f>COUNTIFS(Roadmap!C2:C334,"Automations",Roadmap!E2:E334,"Open")</f>
+        <f>COUNTIFS(Roadmap!C2:C2000,"Automations",Roadmap!E2:E2000,"Open")</f>
         <v/>
       </c>
     </row>
@@ -28499,7 +30281,7 @@
         </is>
       </c>
       <c r="B20" s="3">
-        <f>COUNTIFS(Roadmap!C2:C334,"Calendar",Roadmap!E2:E334,"Open")</f>
+        <f>COUNTIFS(Roadmap!C2:C2000,"Calendar",Roadmap!E2:E2000,"Open")</f>
         <v/>
       </c>
     </row>
@@ -28510,7 +30292,7 @@
         </is>
       </c>
       <c r="B21" s="3">
-        <f>COUNTIFS(Roadmap!C2:C334,"Email attachments",Roadmap!E2:E334,"Open")</f>
+        <f>COUNTIFS(Roadmap!C2:C2000,"Email attachments",Roadmap!E2:E2000,"Open")</f>
         <v/>
       </c>
     </row>
@@ -28521,7 +30303,7 @@
         </is>
       </c>
       <c r="B22" s="3">
-        <f>COUNTIFS(Roadmap!C2:C334,"Engine · Grid",Roadmap!E2:E334,"Open")</f>
+        <f>COUNTIFS(Roadmap!C2:C2000,"Engine · Grid",Roadmap!E2:E2000,"Open")</f>
         <v/>
       </c>
     </row>
@@ -28532,7 +30314,7 @@
         </is>
       </c>
       <c r="B23" s="3">
-        <f>COUNTIFS(Roadmap!C2:C334,"Engine · Relations",Roadmap!E2:E334,"Open")</f>
+        <f>COUNTIFS(Roadmap!C2:C2000,"Engine · Relations",Roadmap!E2:E2000,"Open")</f>
         <v/>
       </c>
     </row>
@@ -28543,7 +30325,7 @@
         </is>
       </c>
       <c r="B24" s="3">
-        <f>COUNTIFS(Roadmap!C2:C334,"Finance · Invoice protest",Roadmap!E2:E334,"Open")</f>
+        <f>COUNTIFS(Roadmap!C2:C2000,"Finance · Invoice protest",Roadmap!E2:E2000,"Open")</f>
         <v/>
       </c>
     </row>
@@ -28554,7 +30336,7 @@
         </is>
       </c>
       <c r="B25" s="3">
-        <f>COUNTIFS(Roadmap!C2:C334,"Finance · Purchase invoices",Roadmap!E2:E334,"Open")</f>
+        <f>COUNTIFS(Roadmap!C2:C2000,"Finance · Purchase invoices",Roadmap!E2:E2000,"Open")</f>
         <v/>
       </c>
     </row>
@@ -28565,7 +30347,7 @@
         </is>
       </c>
       <c r="B26" s="3">
-        <f>COUNTIFS(Roadmap!C2:C334,"Finance · Purchase orders",Roadmap!E2:E334,"Open")</f>
+        <f>COUNTIFS(Roadmap!C2:C2000,"Finance · Purchase orders",Roadmap!E2:E2000,"Open")</f>
         <v/>
       </c>
     </row>
@@ -28576,7 +30358,7 @@
         </is>
       </c>
       <c r="B27" s="3">
-        <f>COUNTIFS(Roadmap!C2:C334,"HR · Timesheet reporting",Roadmap!E2:E334,"Open")</f>
+        <f>COUNTIFS(Roadmap!C2:C2000,"HR · Timesheet reporting",Roadmap!E2:E2000,"Open")</f>
         <v/>
       </c>
     </row>
@@ -28587,7 +30369,7 @@
         </is>
       </c>
       <c r="B28" s="3">
-        <f>COUNTIFS(Roadmap!C2:C334,"HR · Timesheets page",Roadmap!E2:E334,"Open")</f>
+        <f>COUNTIFS(Roadmap!C2:C2000,"HR · Timesheets page",Roadmap!E2:E2000,"Open")</f>
         <v/>
       </c>
     </row>
@@ -28598,7 +30380,7 @@
         </is>
       </c>
       <c r="B29" s="3">
-        <f>COUNTIFS(Roadmap!C2:C334,"Mobile",Roadmap!E2:E334,"Open")</f>
+        <f>COUNTIFS(Roadmap!C2:C2000,"Mobile",Roadmap!E2:E2000,"Open")</f>
         <v/>
       </c>
     </row>
@@ -28609,7 +30391,7 @@
         </is>
       </c>
       <c r="B30" s="3">
-        <f>COUNTIFS(Roadmap!C2:C334,"Mobile / PWA",Roadmap!E2:E334,"Open")</f>
+        <f>COUNTIFS(Roadmap!C2:C2000,"Mobile / PWA",Roadmap!E2:E2000,"Open")</f>
         <v/>
       </c>
     </row>
@@ -28620,7 +30402,7 @@
         </is>
       </c>
       <c r="B31" s="3">
-        <f>COUNTIFS(Roadmap!C2:C334,"Performance · Memory",Roadmap!E2:E334,"Open")</f>
+        <f>COUNTIFS(Roadmap!C2:C2000,"Performance · Memory",Roadmap!E2:E2000,"Open")</f>
         <v/>
       </c>
     </row>
@@ -28631,7 +30413,7 @@
         </is>
       </c>
       <c r="B32" s="3">
-        <f>COUNTIFS(Roadmap!C2:C334,"Pro Hardening",Roadmap!E2:E334,"Open")</f>
+        <f>COUNTIFS(Roadmap!C2:C2000,"Pro Hardening",Roadmap!E2:E2000,"Open")</f>
         <v/>
       </c>
     </row>
@@ -28642,7 +30424,7 @@
         </is>
       </c>
       <c r="B33" s="3">
-        <f>COUNTIFS(Roadmap!C2:C334,"Projects",Roadmap!E2:E334,"Open")</f>
+        <f>COUNTIFS(Roadmap!C2:C2000,"Projects",Roadmap!E2:E2000,"Open")</f>
         <v/>
       </c>
     </row>
@@ -28653,7 +30435,7 @@
         </is>
       </c>
       <c r="B34" s="3">
-        <f>COUNTIFS(Roadmap!C2:C334,"Reliability",Roadmap!E2:E334,"Open")</f>
+        <f>COUNTIFS(Roadmap!C2:C2000,"Reliability",Roadmap!E2:E2000,"Open")</f>
         <v/>
       </c>
     </row>
@@ -28664,7 +30446,7 @@
         </is>
       </c>
       <c r="B35" s="3">
-        <f>COUNTIFS(Roadmap!C2:C334,"Scan · Receipt bulk",Roadmap!E2:E334,"Open")</f>
+        <f>COUNTIFS(Roadmap!C2:C2000,"Scan · Receipt bulk",Roadmap!E2:E2000,"Open")</f>
         <v/>
       </c>
     </row>
@@ -28675,10 +30457,11 @@
         </is>
       </c>
       <c r="B36" s="3">
-        <f>COUNTIFS(Roadmap!C2:C334,"Triage / core",Roadmap!E2:E334,"Open")</f>
+        <f>COUNTIFS(Roadmap!C2:C2000,"Triage / core",Roadmap!E2:E2000,"Open")</f>
         <v/>
       </c>
     </row>
+    <row r="37"/>
     <row r="38">
       <c r="A38" s="29" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
docs(roadmap): night of 30 Sep → 1 Oct — KERN-7b Done, KERN-8/R1-2 on track-b (gated on census), R1-3 measured done, R1-4 scopeWhere + client built (not adopted), PROJ-SSOT-1 phase 1, CREW-ERP-1, SHIFT-DST-1
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/.agents/coral-roadmap.xlsx
+++ b/.agents/coral-roadmap.xlsx
@@ -594,7 +594,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I646"/>
+  <dimension ref="A1:I649"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -10382,7 +10382,7 @@
       </c>
       <c r="E226" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="F226" s="11" t="inlineStr">
@@ -10392,7 +10392,7 @@
       </c>
       <c r="G226" s="11" t="inlineStr">
         <is>
-          <t>[P3.3] Was: denormalise tenantId column — WITHDRAWN</t>
+          <t>[P3.3] Was: denormalise tenantId column — WITHDRAWN | Planner 2026-10-01: resolveDatabaseId fail-closed in the kernel, all 11 callers converted — branch track-b/r1-2-kern-8. GATED on .agents/workflows/r1-2-binding-census.sql (Florin)</t>
         </is>
       </c>
       <c r="H226" s="28" t="inlineStr">
@@ -10429,7 +10429,7 @@
       </c>
       <c r="E227" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F227" s="11" t="inlineStr">
@@ -10439,7 +10439,7 @@
       </c>
       <c r="G227" s="11" t="inlineStr">
         <is>
-          <t>[P3.4] Revised after Florin review 2026-09-12</t>
+          <t>[P3.4] Revised after Florin review 2026-09-12 | Planner 2026-10-01: measured: the per-id ERP doors (pages.ts, global-databases.ts) already verify tenant ownership (TSC-4 era). Actor gap found → CREW-ERP-1</t>
         </is>
       </c>
       <c r="H227" s="28" t="inlineStr">
@@ -10476,7 +10476,7 @@
       </c>
       <c r="E228" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="F228" s="11" t="inlineStr">
@@ -10486,7 +10486,7 @@
       </c>
       <c r="G228" s="11" t="inlineStr">
         <is>
-          <t>[P3.5] Revised after Florin review 2026-09-12</t>
+          <t>[P3.5] Revised after Florin review 2026-09-12 | Planner 2026-10-01: scopeWhere implemented + §2B/§2C contract now a build gate (6b0a37a); TenantScopedClient built + 14 tests (bd56156) — NOT adopted; branch track-b/r1-2-kern-8</t>
         </is>
       </c>
       <c r="H228" s="28" t="inlineStr">
@@ -10533,7 +10533,7 @@
       </c>
       <c r="G229" s="11" t="inlineStr">
         <is>
-          <t>[P3.5] Revised after Florin review 2026-09-12</t>
+          <t>[P3.5] Revised after Florin review 2026-09-12 | Planner 2026-10-01: next: adopt scopeFromSession file by file; direct prisma outside lib/data → CI failure. Florin decides the rollout</t>
         </is>
       </c>
       <c r="H229" s="28" t="inlineStr">
@@ -22527,7 +22527,7 @@
       </c>
       <c r="E498" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="F498" t="inlineStr">
@@ -22537,7 +22537,7 @@
       </c>
       <c r="G498" t="inlineStr">
         <is>
-          <t>Only when 3b's allowlist reaches zero. Gated on the R1-1b relation-target measurement.</t>
+          <t>Only when 3b's allowlist reaches zero. Gated on the R1-1b relation-target measurement. | Planner 2026-10-01: getLockedDbId + lockedDbUtils deleted, resolve.ts prefix searches deleted — on branch track-b/r1-2-kern-8 (b7e5853); ships with R1-2</t>
         </is>
       </c>
       <c r="H498" t="inlineStr">
@@ -26381,7 +26381,7 @@
       </c>
       <c r="E580" t="inlineStr">
         <is>
-          <t>Paused</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F580" t="inlineStr">
@@ -26391,7 +26391,7 @@
       </c>
       <c r="G580" t="inlineStr">
         <is>
-          <t>UNBLOCKED: logicalKey populated (32). Batch 0 = carry logicalKey to the client Database interface + every mapper (the query already returns it; a field-by-field mapper drops it). TRAP: getBaseDbId returns a BASE ID, logicalKey returns a ROLE — a swap that keeps the comparison string compiles and is always false. 7b.2 (pages.ts) is entitlement + the write path; 7b.5 (schema-cleanup) is destructive. | PAUSED until INC-1 closes — same tree, and two conversions in flight over one surface makes a revert impossible.</t>
+          <t>UNBLOCKED: logicalKey populated (32). Batch 0 = carry logicalKey to the client Database interface + every mapper (the query already returns it; a field-by-field mapper drops it). TRAP: getBaseDbId returns a BASE ID, logicalKey returns a ROLE — a swap that keeps the comparison string compiles and is always false. 7b.2 (pages.ts) is entitlement + the write path; 7b.5 (schema-cleanup) is destructive. | PAUSED until INC-1 closes — same tree, and two conversions in flight over one surface makes a revert impossible. | Planner 2026-10-01: allowlist reached 0 on 28 Sep (53023a5) — the roadmap still said Paused</t>
         </is>
       </c>
       <c r="H580" t="inlineStr">
@@ -28120,7 +28120,7 @@
       </c>
       <c r="E617" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="F617" t="inlineStr">
@@ -28130,7 +28130,7 @@
       </c>
       <c r="G617" t="inlineStr">
         <is>
-          <t>census 2026-09-30: 26 unattributed by design, 1 dangling cleared</t>
+          <t>census 2026-09-30: 26 unattributed by design, 1 dangling cleared | Planner 2026-10-01: phase 1 done (9ef6a6d): one resolver lib/data/projects.ts, HrProject read nowhere. Phase 2 (drop) gated: code first, snapshot, Florin's migration</t>
         </is>
       </c>
       <c r="H617" t="inlineStr">
@@ -28966,7 +28966,7 @@
       </c>
       <c r="E635" t="inlineStr">
         <is>
-          <t>Done (code)</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F635" t="inlineStr">
@@ -28976,7 +28976,7 @@
       </c>
       <c r="G635" t="inlineStr">
         <is>
-          <t>4735871 · column migrated by Florin</t>
+          <t>4735871 · column migrated by Florin | Planner 2026-10-01: 4735871 live</t>
         </is>
       </c>
       <c r="H635" t="inlineStr">
@@ -29162,7 +29162,6 @@
           <t>Planner 2026-09-30</t>
         </is>
       </c>
-      <c r="G639" t="inlineStr"/>
       <c r="H639" t="inlineStr">
         <is>
           <t>L1</t>
@@ -29500,6 +29499,143 @@
       <c r="I646" t="inlineStr">
         <is>
           <t>process &amp; housekeeping</t>
+        </is>
+      </c>
+    </row>
+    <row r="647">
+      <c r="A647" t="inlineStr">
+        <is>
+          <t>CREW-ERP-1</t>
+        </is>
+      </c>
+      <c r="B647" t="inlineStr">
+        <is>
+          <t>ERP database doors (12 server actions) had no actor check — a crew phone held the tenant's db ids and could delete a database; crew phones also received IBAN/VAT/Peppol id/invoice numbering</t>
+        </is>
+      </c>
+      <c r="C647" t="inlineStr">
+        <is>
+          <t>Gates</t>
+        </is>
+      </c>
+      <c r="D647" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E647" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F647" t="inlineStr">
+        <is>
+          <t>Planner 2026-10-01</t>
+        </is>
+      </c>
+      <c r="G647" t="inlineStr">
+        <is>
+          <t>51039bc</t>
+        </is>
+      </c>
+      <c r="H647" t="inlineStr">
+        <is>
+          <t>GATE</t>
+        </is>
+      </c>
+      <c r="I647" t="inlineStr">
+        <is>
+          <t>actor reach · platform access · operator scopes</t>
+        </is>
+      </c>
+    </row>
+    <row r="648">
+      <c r="A648" t="inlineStr">
+        <is>
+          <t>SHIFT-DST-1</t>
+        </is>
+      </c>
+      <c r="B648" t="inlineStr">
+        <is>
+          <t>Recurring/multi-day shift creation slipped one day after the spring clock change (UTC midnight + local days + toISOString)</t>
+        </is>
+      </c>
+      <c r="C648" t="inlineStr">
+        <is>
+          <t>HR</t>
+        </is>
+      </c>
+      <c r="D648" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E648" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F648" t="inlineStr">
+        <is>
+          <t>Planner 2026-10-01</t>
+        </is>
+      </c>
+      <c r="G648" t="inlineStr">
+        <is>
+          <t>4735871</t>
+        </is>
+      </c>
+      <c r="H648" t="inlineStr">
+        <is>
+          <t>L3</t>
+        </is>
+      </c>
+      <c r="I648" t="inlineStr">
+        <is>
+          <t>HR — timesheets, workforce</t>
+        </is>
+      </c>
+    </row>
+    <row r="649">
+      <c r="A649" t="inlineStr">
+        <is>
+          <t>SHIFT-FORM-EDIT</t>
+        </is>
+      </c>
+      <c r="B649" t="inlineStr">
+        <is>
+          <t>Order-giver picker on the EDIT shift dialog (WB-A covered creation only)</t>
+        </is>
+      </c>
+      <c r="C649" t="inlineStr">
+        <is>
+          <t>Werkbon</t>
+        </is>
+      </c>
+      <c r="D649" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="E649" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F649" t="inlineStr">
+        <is>
+          <t>Planner 2026-10-01</t>
+        </is>
+      </c>
+      <c r="G649" t="inlineStr"/>
+      <c r="H649" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="I649" t="inlineStr">
+        <is>
+          <t>document engine (+ archive, attachments)</t>
         </is>
       </c>
     </row>
@@ -30461,7 +30597,6 @@
         <v/>
       </c>
     </row>
-    <row r="37"/>
     <row r="38">
       <c r="A38" s="29" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
docs(roadmap): Jibble review — OFFLINE-1, PAYROLL-1, GEO-2 planned; TEAM-1, KIOSK-1, REPORT-1, HR-LIVE-1, AI-1 later; face recognition and live location rejected (Florin 2026-10-02)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/.agents/coral-roadmap.xlsx
+++ b/.agents/coral-roadmap.xlsx
@@ -594,7 +594,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I649"/>
+  <dimension ref="A1:I659"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -29627,7 +29627,6 @@
           <t>Planner 2026-10-01</t>
         </is>
       </c>
-      <c r="G649" t="inlineStr"/>
       <c r="H649" t="inlineStr">
         <is>
           <t>L1</t>
@@ -29636,6 +29635,476 @@
       <c r="I649" t="inlineStr">
         <is>
           <t>document engine (+ archive, attachments)</t>
+        </is>
+      </c>
+    </row>
+    <row r="650">
+      <c r="A650" t="inlineStr">
+        <is>
+          <t>OFFLINE-1</t>
+        </is>
+      </c>
+      <c r="B650" t="inlineStr">
+        <is>
+          <t>Offline clocking: clock in/out without signal, queued on the phone and synced later; every item shows its own sync state, plus a banner while anything is unsynced. Builds on the kernel offline queue (the queued intent carries its own time — CE-TIME-1).</t>
+        </is>
+      </c>
+      <c r="C650" t="inlineStr">
+        <is>
+          <t>HR · WorkHub</t>
+        </is>
+      </c>
+      <c r="D650" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E650" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F650" t="inlineStr">
+        <is>
+          <t>Florin 2026-10-02 · Jibble review (coral-backlog-jibble.md)</t>
+        </is>
+      </c>
+      <c r="G650" t="inlineStr">
+        <is>
+          <t>PLANNED</t>
+        </is>
+      </c>
+      <c r="H650" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="I650" t="inlineStr">
+        <is>
+          <t>HR · WorkHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="651">
+      <c r="A651" t="inlineStr">
+        <is>
+          <t>PAYROLL-1</t>
+        </is>
+      </c>
+      <c r="B651" t="inlineStr">
+        <is>
+          <t>Payroll export to the social secretariat (SD Worx, Acerta, Partena, Securex…) — export only, NO payroll math in-house; a flag for self-employed workers (excluded from the payroll export).</t>
+        </is>
+      </c>
+      <c r="C651" t="inlineStr">
+        <is>
+          <t>HR · Timesheet reporting</t>
+        </is>
+      </c>
+      <c r="D651" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E651" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F651" t="inlineStr">
+        <is>
+          <t>Florin 2026-10-02 · Jibble review (coral-backlog-jibble.md)</t>
+        </is>
+      </c>
+      <c r="G651" t="inlineStr">
+        <is>
+          <t>PLANNED</t>
+        </is>
+      </c>
+      <c r="H651" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="I651" t="inlineStr">
+        <is>
+          <t>HR · Timesheet reporting</t>
+        </is>
+      </c>
+    </row>
+    <row r="652">
+      <c r="A652" t="inlineStr">
+        <is>
+          <t>GEO-2</t>
+        </is>
+      </c>
+      <c r="B652" t="inlineStr">
+        <is>
+          <t>Our own location explanation BEFORE the browser's permission prompt (what is recorded, when, why — clock events only), so the crew understands before the OS asks.</t>
+        </is>
+      </c>
+      <c r="C652" t="inlineStr">
+        <is>
+          <t>HR · WorkHub</t>
+        </is>
+      </c>
+      <c r="D652" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E652" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F652" t="inlineStr">
+        <is>
+          <t>Florin 2026-10-02 · Jibble review (coral-backlog-jibble.md)</t>
+        </is>
+      </c>
+      <c r="G652" t="inlineStr">
+        <is>
+          <t>PLANNED</t>
+        </is>
+      </c>
+      <c r="H652" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="I652" t="inlineStr">
+        <is>
+          <t>HR · WorkHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="653">
+      <c r="A653" t="inlineStr">
+        <is>
+          <t>TEAM-1</t>
+        </is>
+      </c>
+      <c r="B653" t="inlineStr">
+        <is>
+          <t>Teams: foreman role in HrTeamMember; a shift assigned to a team fans out to its members; the foreman enters the crew's hours.</t>
+        </is>
+      </c>
+      <c r="C653" t="inlineStr">
+        <is>
+          <t>HR · Scheduling</t>
+        </is>
+      </c>
+      <c r="D653" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="E653" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F653" t="inlineStr">
+        <is>
+          <t>Florin 2026-10-02 · Jibble review (coral-backlog-jibble.md)</t>
+        </is>
+      </c>
+      <c r="G653" t="inlineStr">
+        <is>
+          <t>LATER</t>
+        </is>
+      </c>
+      <c r="H653" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="I653" t="inlineStr">
+        <is>
+          <t>HR · Scheduling</t>
+        </is>
+      </c>
+    </row>
+    <row r="654">
+      <c r="A654" t="inlineStr">
+        <is>
+          <t>KIOSK-1</t>
+        </is>
+      </c>
+      <c r="B654" t="inlineStr">
+        <is>
+          <t>Kiosk: a shared on-site device where workers clock in (PIN / QR / NFC).</t>
+        </is>
+      </c>
+      <c r="C654" t="inlineStr">
+        <is>
+          <t>HR · WorkHub</t>
+        </is>
+      </c>
+      <c r="D654" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="E654" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F654" t="inlineStr">
+        <is>
+          <t>Florin 2026-10-02 · Jibble review (coral-backlog-jibble.md)</t>
+        </is>
+      </c>
+      <c r="G654" t="inlineStr">
+        <is>
+          <t>LATER</t>
+        </is>
+      </c>
+      <c r="H654" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="I654" t="inlineStr">
+        <is>
+          <t>HR · WorkHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="655">
+      <c r="A655" t="inlineStr">
+        <is>
+          <t>REPORT-1</t>
+        </is>
+      </c>
+      <c r="B655" t="inlineStr">
+        <is>
+          <t>Reports: planned vs actual (shift vs clocked hours) and attendance (late, absent, no-show).</t>
+        </is>
+      </c>
+      <c r="C655" t="inlineStr">
+        <is>
+          <t>HR · Timesheet reporting</t>
+        </is>
+      </c>
+      <c r="D655" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="E655" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F655" t="inlineStr">
+        <is>
+          <t>Florin 2026-10-02 · Jibble review (coral-backlog-jibble.md)</t>
+        </is>
+      </c>
+      <c r="G655" t="inlineStr">
+        <is>
+          <t>LATER</t>
+        </is>
+      </c>
+      <c r="H655" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="I655" t="inlineStr">
+        <is>
+          <t>HR · Timesheet reporting</t>
+        </is>
+      </c>
+    </row>
+    <row r="656">
+      <c r="A656" t="inlineStr">
+        <is>
+          <t>HR-LIVE-1</t>
+        </is>
+      </c>
+      <c r="B656" t="inlineStr">
+        <is>
+          <t>Who is in now — on the HR dashboard (office), NOT in the WorkHub.</t>
+        </is>
+      </c>
+      <c r="C656" t="inlineStr">
+        <is>
+          <t>HR · Dashboard</t>
+        </is>
+      </c>
+      <c r="D656" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="E656" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F656" t="inlineStr">
+        <is>
+          <t>Florin 2026-10-02 · Jibble review (coral-backlog-jibble.md)</t>
+        </is>
+      </c>
+      <c r="G656" t="inlineStr">
+        <is>
+          <t>LATER</t>
+        </is>
+      </c>
+      <c r="H656" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="I656" t="inlineStr">
+        <is>
+          <t>HR · Dashboard</t>
+        </is>
+      </c>
+    </row>
+    <row r="657">
+      <c r="A657" t="inlineStr">
+        <is>
+          <t>AI-1</t>
+        </is>
+      </c>
+      <c r="B657" t="inlineStr">
+        <is>
+          <t>Claude assistant over the tenant's data — only after R1 (tenancy) is closed.</t>
+        </is>
+      </c>
+      <c r="C657" t="inlineStr">
+        <is>
+          <t>Platform</t>
+        </is>
+      </c>
+      <c r="D657" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="E657" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F657" t="inlineStr">
+        <is>
+          <t>Florin 2026-10-02 · Jibble review (coral-backlog-jibble.md)</t>
+        </is>
+      </c>
+      <c r="G657" t="inlineStr">
+        <is>
+          <t>LATER — after R1</t>
+        </is>
+      </c>
+      <c r="H657" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="I657" t="inlineStr">
+        <is>
+          <t>Platform</t>
+        </is>
+      </c>
+    </row>
+    <row r="658">
+      <c r="A658" t="inlineStr">
+        <is>
+          <t>REJ-FACE</t>
+        </is>
+      </c>
+      <c r="B658" t="inlineStr">
+        <is>
+          <t>Face recognition / selfie at clock-in.</t>
+        </is>
+      </c>
+      <c r="C658" t="inlineStr">
+        <is>
+          <t>HR · WorkHub</t>
+        </is>
+      </c>
+      <c r="D658" t="inlineStr">
+        <is>
+          <t>P4</t>
+        </is>
+      </c>
+      <c r="E658" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+      <c r="F658" t="inlineStr">
+        <is>
+          <t>Florin 2026-10-02 · Jibble review (coral-backlog-jibble.md)</t>
+        </is>
+      </c>
+      <c r="G658" t="inlineStr">
+        <is>
+          <t>REJECTED — biometrics (GDPR special category), little value next to signature + location record</t>
+        </is>
+      </c>
+      <c r="H658" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="I658" t="inlineStr">
+        <is>
+          <t>HR · WorkHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="659">
+      <c r="A659" t="inlineStr">
+        <is>
+          <t>REJ-LIVELOC</t>
+        </is>
+      </c>
+      <c r="B659" t="inlineStr">
+        <is>
+          <t>Live location tracking during work.</t>
+        </is>
+      </c>
+      <c r="C659" t="inlineStr">
+        <is>
+          <t>HR · WorkHub</t>
+        </is>
+      </c>
+      <c r="D659" t="inlineStr">
+        <is>
+          <t>P4</t>
+        </is>
+      </c>
+      <c r="E659" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+      <c r="F659" t="inlineStr">
+        <is>
+          <t>Florin 2026-10-02 · Jibble review (coral-backlog-jibble.md)</t>
+        </is>
+      </c>
+      <c r="G659" t="inlineStr">
+        <is>
+          <t>REJECTED — it gets promoted to the single source of truth and conflicts with signed hours</t>
+        </is>
+      </c>
+      <c r="H659" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="I659" t="inlineStr">
+        <is>
+          <t>HR · WorkHub</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(roadmap): 29 rows for the work since 28 Sep; architecture map generator
The map's stack is now computed from the spreadsheet (build.py); the narrative
around it is kept in narrative.html.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/.agents/coral-roadmap.xlsx
+++ b/.agents/coral-roadmap.xlsx
@@ -594,7 +594,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I659"/>
+  <dimension ref="A1:I688"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -10617,7 +10617,7 @@
       </c>
       <c r="E231" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F231" s="11" t="inlineStr">
@@ -10627,7 +10627,7 @@
       </c>
       <c r="G231" s="11" t="inlineStr">
         <is>
-          <t>[P4.1] Written first</t>
+          <t>[P4.1] Written first · Coder c1d4de5 — DONE WITH CORRECTIONS: store tests kept; 11 copy-tests replaced by real occ-merge tests (OCC-MERGE-1).</t>
         </is>
       </c>
       <c r="H231" s="23" t="inlineStr">
@@ -10674,7 +10674,7 @@
       </c>
       <c r="G232" s="11" t="inlineStr">
         <is>
-          <t>[P4.2]</t>
+          <t>[P4.2] · R2-1-CENSUS queued for the coder (33 direct GlobalPage writes, 18 files).</t>
         </is>
       </c>
       <c r="H232" s="23" t="inlineStr">
@@ -25545,7 +25545,7 @@
       </c>
       <c r="G562" t="inlineStr">
         <is>
-          <t>Florin: 'rare, but still very much counts in EUR... me, client or crew member... so even if at the end, we do not leave it behind.' A lost hour is always PAID BY SOMEONE. sw-workhub.js:58 handles GET only; /api/* always network; the shell caches so the app LOOKS alive offline and a clock-in dies with a toast. Sequenced last, never dropped.</t>
+          <t>Florin: 'rare, but still very much counts in EUR... me, client or crew member... so even if at the end, we do not leave it behind.' A lost hour is always PAID BY SOMEONE. sw-workhub.js:58 handles GET only; /api/* always network; the shell caches so the app LOOKS alive offline and a clock-in dies with a toast. Sequenced last, never dropped. · Same as OFFLINE-1 (Planned, Jibble review 2026-10-02).</t>
         </is>
       </c>
       <c r="H562" t="inlineStr">
@@ -26569,7 +26569,7 @@
       </c>
       <c r="E584" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F584" t="inlineStr">
@@ -26579,7 +26579,7 @@
       </c>
       <c r="G584" t="inlineStr">
         <is>
-          <t>TypeError 'e.split' on the workhub for every tenant. addSnakeCase stopped writing shift_date/start/end; 12 @ts-nocheck files still read them. The one file tsc could see is the one that did not break.</t>
+          <t>TypeError 'e.split' on the workhub for every tenant. addSnakeCase stopped writing shift_date/start/end; 12 @ts-nocheck files still read them. The one file tsc could see is the one that did not break. · Fixed 28–29 Sep (shift_date restored, blind reads removed); WorkHub live since. Closed 2026-10-03.</t>
         </is>
       </c>
       <c r="H584" t="inlineStr">
@@ -28073,7 +28073,7 @@
       </c>
       <c r="E616" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F616" t="inlineStr">
@@ -28083,7 +28083,7 @@
       </c>
       <c r="G616" t="inlineStr">
         <is>
-          <t>coder-directive-sch-8-series-and-manual-entry.md</t>
+          <t>coder-directive-sch-8-series-and-manual-entry.md · ff9e5cc + d489204: server-side series scope, one transaction, count shown (2026-10-01/02).</t>
         </is>
       </c>
       <c r="H616" t="inlineStr">
@@ -29013,7 +29013,7 @@
       </c>
       <c r="E636" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Dropped</t>
         </is>
       </c>
       <c r="F636" t="inlineStr">
@@ -29023,7 +29023,7 @@
       </c>
       <c r="G636" t="inlineStr">
         <is>
-          <t>phasing A → B → C+D → E (Florin)</t>
+          <t>phasing A → B → C+D → E (Florin) · Superseded 2026-10-01 (Florin): the work order = shifts created together (seriesId) — no separate Werkbon record.</t>
         </is>
       </c>
       <c r="H636" t="inlineStr">
@@ -29060,7 +29060,7 @@
       </c>
       <c r="E637" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F637" t="inlineStr">
@@ -29070,7 +29070,7 @@
       </c>
       <c r="G637" t="inlineStr">
         <is>
-          <t>the lock has the grain of the work order, not the day</t>
+          <t>the lock has the grain of the work order, not the day · Delivered as WO-3 (d1f24dc): client signs with name, evidence frozen in AuditLog.</t>
         </is>
       </c>
       <c r="H637" t="inlineStr">
@@ -29107,7 +29107,7 @@
       </c>
       <c r="E638" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F638" t="inlineStr">
@@ -29117,7 +29117,7 @@
       </c>
       <c r="G638" t="inlineStr">
         <is>
-          <t>never freeze by date or worker</t>
+          <t>never freeze by date or worker · Delivered as WO-3: the lock by work-order grain, every writer refuses (work-order-lock.ts).</t>
         </is>
       </c>
       <c r="H638" t="inlineStr">
@@ -29162,6 +29162,11 @@
           <t>Planner 2026-09-30</t>
         </is>
       </c>
+      <c r="G639" t="inlineStr">
+        <is>
+          <t>Continues as WO-4b (PDF at signing, stored, cron send, unsent view).</t>
+        </is>
+      </c>
       <c r="H639" t="inlineStr">
         <is>
           <t>L1</t>
@@ -30105,6 +30110,1340 @@
       <c r="I659" t="inlineStr">
         <is>
           <t>HR · WorkHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="660">
+      <c r="A660" t="inlineStr">
+        <is>
+          <t>SHIFT-LINK-1</t>
+        </is>
+      </c>
+      <c r="B660" t="inlineStr">
+        <is>
+          <t>Hours ↔ shifts: auto-link a recorded entry to the one overlapping shift; review card (editable suggestion) in My hours + Timesheets</t>
+        </is>
+      </c>
+      <c r="C660" t="inlineStr">
+        <is>
+          <t>HR · WorkHub</t>
+        </is>
+      </c>
+      <c r="D660" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E660" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F660" t="inlineStr">
+        <is>
+          <t>bf08331</t>
+        </is>
+      </c>
+      <c r="G660" t="inlineStr">
+        <is>
+          <t>Live 2026-10-01</t>
+        </is>
+      </c>
+      <c r="H660" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="I660" t="inlineStr">
+        <is>
+          <t>WorkHub / time-tracker</t>
+        </is>
+      </c>
+    </row>
+    <row r="661">
+      <c r="A661" t="inlineStr">
+        <is>
+          <t>WH-LEAN-1</t>
+        </is>
+      </c>
+      <c r="B661" t="inlineStr">
+        <is>
+          <t>WorkHub stops loading the ERP store at start-up (office roles too); site visit loads on demand</t>
+        </is>
+      </c>
+      <c r="C661" t="inlineStr">
+        <is>
+          <t>HR · WorkHub</t>
+        </is>
+      </c>
+      <c r="D661" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E661" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F661" t="inlineStr">
+        <is>
+          <t>7b77809</t>
+        </is>
+      </c>
+      <c r="G661" t="inlineStr">
+        <is>
+          <t>Live 2026-10-01</t>
+        </is>
+      </c>
+      <c r="H661" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="I661" t="inlineStr">
+        <is>
+          <t>WorkHub / time-tracker</t>
+        </is>
+      </c>
+    </row>
+    <row r="662">
+      <c r="A662" t="inlineStr">
+        <is>
+          <t>LATE-TZ-1</t>
+        </is>
+      </c>
+      <c r="B662" t="inlineStr">
+        <is>
+          <t>Late/manual entries sent without a zone landed 2 h late — the phone sends instants; server refuses zone-less times</t>
+        </is>
+      </c>
+      <c r="C662" t="inlineStr">
+        <is>
+          <t>HR · WorkHub</t>
+        </is>
+      </c>
+      <c r="D662" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E662" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F662" t="inlineStr">
+        <is>
+          <t>32c61f9</t>
+        </is>
+      </c>
+      <c r="G662" t="inlineStr">
+        <is>
+          <t>Live 2026-10-01. Past entries since June: list offered, not fixed</t>
+        </is>
+      </c>
+      <c r="H662" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="I662" t="inlineStr">
+        <is>
+          <t>WorkHub / time-tracker</t>
+        </is>
+      </c>
+    </row>
+    <row r="663">
+      <c r="A663" t="inlineStr">
+        <is>
+          <t>WO-1</t>
+        </is>
+      </c>
+      <c r="B663" t="inlineStr">
+        <is>
+          <t>The shift opens as a work order — tabs Info · Hours · Tasks · Notes · Sign; full-screen on the phone</t>
+        </is>
+      </c>
+      <c r="C663" t="inlineStr">
+        <is>
+          <t>HR · WorkHub</t>
+        </is>
+      </c>
+      <c r="D663" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E663" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F663" t="inlineStr">
+        <is>
+          <t>58f101b, 99bde84</t>
+        </is>
+      </c>
+      <c r="G663" t="inlineStr">
+        <is>
+          <t>Live 2026-10-01</t>
+        </is>
+      </c>
+      <c r="H663" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="I663" t="inlineStr">
+        <is>
+          <t>WorkHub / time-tracker</t>
+        </is>
+      </c>
+    </row>
+    <row r="664">
+      <c r="A664" t="inlineStr">
+        <is>
+          <t>WO-2</t>
+        </is>
+      </c>
+      <c r="B664" t="inlineStr">
+        <is>
+          <t>Scheduler: execution address, materials flag, crew note; shifts created together = one work order (seriesId)</t>
+        </is>
+      </c>
+      <c r="C664" t="inlineStr">
+        <is>
+          <t>HR · Scheduling</t>
+        </is>
+      </c>
+      <c r="D664" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E664" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F664" t="inlineStr">
+        <is>
+          <t>27ceff5</t>
+        </is>
+      </c>
+      <c r="G664" t="inlineStr">
+        <is>
+          <t>Migration 20261001090000 (Florin)</t>
+        </is>
+      </c>
+      <c r="H664" t="inlineStr">
+        <is>
+          <t>L3</t>
+        </is>
+      </c>
+      <c r="I664" t="inlineStr">
+        <is>
+          <t>HR — scheduling</t>
+        </is>
+      </c>
+    </row>
+    <row r="665">
+      <c r="A665" t="inlineStr">
+        <is>
+          <t>WO-3</t>
+        </is>
+      </c>
+      <c r="B665" t="inlineStr">
+        <is>
+          <t>Client signs the work order (name + signature); evidence frozen; the lock by work-order grain, every writer refuses</t>
+        </is>
+      </c>
+      <c r="C665" t="inlineStr">
+        <is>
+          <t>Documents</t>
+        </is>
+      </c>
+      <c r="D665" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E665" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F665" t="inlineStr">
+        <is>
+          <t>d1f24dc, 69f8ddc</t>
+        </is>
+      </c>
+      <c r="G665">
+        <f> WB-C + WB-D; serializable re-check</f>
+        <v/>
+      </c>
+      <c r="H665" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="I665" t="inlineStr">
+        <is>
+          <t>document engine (+ archive, attachments)</t>
+        </is>
+      </c>
+    </row>
+    <row r="666">
+      <c r="A666" t="inlineStr">
+        <is>
+          <t>WO-4a</t>
+        </is>
+      </c>
+      <c r="B666" t="inlineStr">
+        <is>
+          <t>Signed work order PDF renderer (pure: view model → PDF, IBM Plex, Brussels time, page breaks)</t>
+        </is>
+      </c>
+      <c r="C666" t="inlineStr">
+        <is>
+          <t>Documents</t>
+        </is>
+      </c>
+      <c r="D666" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E666" t="inlineStr">
+        <is>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="F666" t="inlineStr">
+        <is>
+          <t>coder plan-first</t>
+        </is>
+      </c>
+      <c r="G666" t="inlineStr">
+        <is>
+          <t>M1 ✅ M2 ✅, M3 next (fr/en, edge cases)</t>
+        </is>
+      </c>
+      <c r="H666" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="I666" t="inlineStr">
+        <is>
+          <t>document engine (+ archive, attachments)</t>
+        </is>
+      </c>
+    </row>
+    <row r="667">
+      <c r="A667" t="inlineStr">
+        <is>
+          <t>WO-4b</t>
+        </is>
+      </c>
+      <c r="B667" t="inlineStr">
+        <is>
+          <t>PDF generated AT signing, stored once; cron send to the order giver; unsent visibility (walkdown §11a)</t>
+        </is>
+      </c>
+      <c r="C667" t="inlineStr">
+        <is>
+          <t>Documents</t>
+        </is>
+      </c>
+      <c r="D667" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E667" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F667" t="inlineStr">
+        <is>
+          <t>coral-work-order-tabs.md</t>
+        </is>
+      </c>
+      <c r="G667" t="inlineStr">
+        <is>
+          <t>Planner. Prints shift description + crew notes (Florin 2026-10-02)</t>
+        </is>
+      </c>
+      <c r="H667" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="I667" t="inlineStr">
+        <is>
+          <t>document engine (+ archive, attachments)</t>
+        </is>
+      </c>
+    </row>
+    <row r="668">
+      <c r="A668" t="inlineStr">
+        <is>
+          <t>GEO-1</t>
+        </is>
+      </c>
+      <c r="B668" t="inlineStr">
+        <is>
+          <t>Clock-in/out address + distance to site (record, never block); Geoapify now, Google later</t>
+        </is>
+      </c>
+      <c r="C668" t="inlineStr">
+        <is>
+          <t>HR · WorkHub</t>
+        </is>
+      </c>
+      <c r="D668" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E668" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F668" t="inlineStr">
+        <is>
+          <t>e125d4a, 70180c2</t>
+        </is>
+      </c>
+      <c r="G668" t="inlineStr">
+        <is>
+          <t>Migration 20261001180000 (Florin)</t>
+        </is>
+      </c>
+      <c r="H668" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="I668" t="inlineStr">
+        <is>
+          <t>WorkHub / time-tracker</t>
+        </is>
+      </c>
+    </row>
+    <row r="669">
+      <c r="A669" t="inlineStr">
+        <is>
+          <t>HR-TS-8</t>
+        </is>
+      </c>
+      <c r="B669" t="inlineStr">
+        <is>
+          <t>Manual entry: searchable project, Belgian date/time pickers; night work = next day</t>
+        </is>
+      </c>
+      <c r="C669" t="inlineStr">
+        <is>
+          <t>HR · Timesheet reporting</t>
+        </is>
+      </c>
+      <c r="D669" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="E669" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F669" t="inlineStr">
+        <is>
+          <t>ff9e5cc, 638bf2c</t>
+        </is>
+      </c>
+      <c r="G669" t="inlineStr"/>
+      <c r="H669" t="inlineStr">
+        <is>
+          <t>L3</t>
+        </is>
+      </c>
+      <c r="I669" t="inlineStr">
+        <is>
+          <t>HR — timesheets</t>
+        </is>
+      </c>
+    </row>
+    <row r="670">
+      <c r="A670" t="inlineStr">
+        <is>
+          <t>TS-INV-1</t>
+        </is>
+      </c>
+      <c r="B670" t="inlineStr">
+        <is>
+          <t>Hour statuses approved · denied · invoiced · non-billable; invoiced locked like approved</t>
+        </is>
+      </c>
+      <c r="C670" t="inlineStr">
+        <is>
+          <t>HR · Timesheet reporting</t>
+        </is>
+      </c>
+      <c r="D670" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E670" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F670" t="inlineStr">
+        <is>
+          <t>48f1d2d</t>
+        </is>
+      </c>
+      <c r="G670" t="inlineStr">
+        <is>
+          <t>Migration 20261002090000</t>
+        </is>
+      </c>
+      <c r="H670" t="inlineStr">
+        <is>
+          <t>L3</t>
+        </is>
+      </c>
+      <c r="I670" t="inlineStr">
+        <is>
+          <t>HR — timesheets</t>
+        </is>
+      </c>
+    </row>
+    <row r="671">
+      <c r="A671" t="inlineStr">
+        <is>
+          <t>TS-INV-2</t>
+        </is>
+      </c>
+      <c r="B671" t="inlineStr">
+        <is>
+          <t>"Factureer selectie": selected hours → draft invoice (one client, rate typed, a line per worker per day)</t>
+        </is>
+      </c>
+      <c r="C671" t="inlineStr">
+        <is>
+          <t>HR · Timesheet reporting</t>
+        </is>
+      </c>
+      <c r="D671" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E671" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F671" t="inlineStr">
+        <is>
+          <t>cd8fba3</t>
+        </is>
+      </c>
+      <c r="G671" t="inlineStr"/>
+      <c r="H671" t="inlineStr">
+        <is>
+          <t>L3</t>
+        </is>
+      </c>
+      <c r="I671" t="inlineStr">
+        <is>
+          <t>HR — timesheets</t>
+        </is>
+      </c>
+    </row>
+    <row r="672">
+      <c r="A672" t="inlineStr">
+        <is>
+          <t>TS-ARCH-1</t>
+        </is>
+      </c>
+      <c r="B672" t="inlineStr">
+        <is>
+          <t>Archive hours (settled only) — out of the view, restorable, still exported</t>
+        </is>
+      </c>
+      <c r="C672" t="inlineStr">
+        <is>
+          <t>HR · Timesheet reporting</t>
+        </is>
+      </c>
+      <c r="D672" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="E672" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F672" t="inlineStr">
+        <is>
+          <t>3131762</t>
+        </is>
+      </c>
+      <c r="G672" t="inlineStr">
+        <is>
+          <t>Migration 20261002120000</t>
+        </is>
+      </c>
+      <c r="H672" t="inlineStr">
+        <is>
+          <t>L3</t>
+        </is>
+      </c>
+      <c r="I672" t="inlineStr">
+        <is>
+          <t>HR — timesheets</t>
+        </is>
+      </c>
+    </row>
+    <row r="673">
+      <c r="A673" t="inlineStr">
+        <is>
+          <t>HOURS-FMT-1</t>
+        </is>
+      </c>
+      <c r="B673" t="inlineStr">
+        <is>
+          <t>Hours as decimals with HH:mm in brackets — screen, export (two columns + TOTAAL from minutes), invoice</t>
+        </is>
+      </c>
+      <c r="C673" t="inlineStr">
+        <is>
+          <t>HR · Timesheet reporting</t>
+        </is>
+      </c>
+      <c r="D673" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E673" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F673" t="inlineStr">
+        <is>
+          <t>18fbec4</t>
+        </is>
+      </c>
+      <c r="G673" t="inlineStr">
+        <is>
+          <t>One conversion (computeWorkedDuration)</t>
+        </is>
+      </c>
+      <c r="H673" t="inlineStr">
+        <is>
+          <t>L3</t>
+        </is>
+      </c>
+      <c r="I673" t="inlineStr">
+        <is>
+          <t>HR — timesheets</t>
+        </is>
+      </c>
+    </row>
+    <row r="674">
+      <c r="A674" t="inlineStr">
+        <is>
+          <t>OWNER-EDIT-1</t>
+        </is>
+      </c>
+      <c r="B674" t="inlineStr">
+        <is>
+          <t>Owner edits approved hours without the unlock; every edit of approved hours needs a written reason</t>
+        </is>
+      </c>
+      <c r="C674" t="inlineStr">
+        <is>
+          <t>HR · Timesheet reporting</t>
+        </is>
+      </c>
+      <c r="D674" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E674" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F674" t="inlineStr">
+        <is>
+          <t>24aa6db</t>
+        </is>
+      </c>
+      <c r="G674" t="inlineStr"/>
+      <c r="H674" t="inlineStr">
+        <is>
+          <t>L3</t>
+        </is>
+      </c>
+      <c r="I674" t="inlineStr">
+        <is>
+          <t>HR — timesheets</t>
+        </is>
+      </c>
+    </row>
+    <row r="675">
+      <c r="A675" t="inlineStr">
+        <is>
+          <t>TS-SHIFT-CTX</t>
+        </is>
+      </c>
+      <c r="B675" t="inlineStr">
+        <is>
+          <t>Timesheet entry shows its shift: planner note, crew note, tasks; "Admin notes"</t>
+        </is>
+      </c>
+      <c r="C675" t="inlineStr">
+        <is>
+          <t>HR · Timesheet reporting</t>
+        </is>
+      </c>
+      <c r="D675" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="E675" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F675" t="inlineStr">
+        <is>
+          <t>aa28cea</t>
+        </is>
+      </c>
+      <c r="G675" t="inlineStr"/>
+      <c r="H675" t="inlineStr">
+        <is>
+          <t>L3</t>
+        </is>
+      </c>
+      <c r="I675" t="inlineStr">
+        <is>
+          <t>HR — timesheets</t>
+        </is>
+      </c>
+    </row>
+    <row r="676">
+      <c r="A676" t="inlineStr">
+        <is>
+          <t>OCC-MERGE-1</t>
+        </is>
+      </c>
+      <c r="B676" t="inlineStr">
+        <is>
+          <t>Stale save no longer overwrites another user's field; no false conflicts after a first save</t>
+        </is>
+      </c>
+      <c r="C676" t="inlineStr">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="D676" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E676" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F676" t="inlineStr">
+        <is>
+          <t>d01dcb5</t>
+        </is>
+      </c>
+      <c r="G676" t="inlineStr">
+        <is>
+          <t>Found via R2-5; one merge rule (lib/records/occ-merge.ts)</t>
+        </is>
+      </c>
+      <c r="H676" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="I676" t="inlineStr">
+        <is>
+          <t>write path — concurrency</t>
+        </is>
+      </c>
+    </row>
+    <row r="677">
+      <c r="A677" t="inlineStr">
+        <is>
+          <t>DOC-LOCK-1</t>
+        </is>
+      </c>
+      <c r="B677" t="inlineStr">
+        <is>
+          <t>Sent / accepted / rejected quote = locked document, enforced in every server write door; "Revise" = -vN draft</t>
+        </is>
+      </c>
+      <c r="C677" t="inlineStr">
+        <is>
+          <t>Documents</t>
+        </is>
+      </c>
+      <c r="D677" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E677" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F677" t="inlineStr">
+        <is>
+          <t>61474cd</t>
+        </is>
+      </c>
+      <c r="G677" t="inlineStr">
+        <is>
+          <t>Florin 2026-10-03; status never back to draft</t>
+        </is>
+      </c>
+      <c r="H677" t="inlineStr">
+        <is>
+          <t>MODULE GATE</t>
+        </is>
+      </c>
+      <c r="I677" t="inlineStr">
+        <is>
+          <t>export lock · accountant export</t>
+        </is>
+      </c>
+    </row>
+    <row r="678">
+      <c r="A678" t="inlineStr">
+        <is>
+          <t>WO-LIB-1</t>
+        </is>
+      </c>
+      <c r="B678" t="inlineStr">
+        <is>
+          <t>Library signal: line remembers its article values; draft = badge + take library values; locked = badge; expired = banner</t>
+        </is>
+      </c>
+      <c r="C678" t="inlineStr">
+        <is>
+          <t>Quotations</t>
+        </is>
+      </c>
+      <c r="D678" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E678" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F678" t="inlineStr">
+        <is>
+          <t>Planner</t>
+        </is>
+      </c>
+      <c r="G678" t="inlineStr">
+        <is>
+          <t>Next (step 3)</t>
+        </is>
+      </c>
+      <c r="H678" t="inlineStr">
+        <is>
+          <t>L3</t>
+        </is>
+      </c>
+      <c r="I678" t="inlineStr">
+        <is>
+          <t>Quotations engine</t>
+        </is>
+      </c>
+    </row>
+    <row r="679">
+      <c r="A679" t="inlineStr">
+        <is>
+          <t>VARIANT-1</t>
+        </is>
+      </c>
+      <c r="B679" t="inlineStr">
+        <is>
+          <t>Variant surcharges: frozen on the line, counted in totals (today 0 in saved totals; db-articles fixed-id lookup)</t>
+        </is>
+      </c>
+      <c r="C679" t="inlineStr">
+        <is>
+          <t>Quotations</t>
+        </is>
+      </c>
+      <c r="D679" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E679" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F679" t="inlineStr">
+        <is>
+          <t>Planner 2026-10-03</t>
+        </is>
+      </c>
+      <c r="G679" t="inlineStr">
+        <is>
+          <t>Found digging the variants logic</t>
+        </is>
+      </c>
+      <c r="H679" t="inlineStr">
+        <is>
+          <t>L3</t>
+        </is>
+      </c>
+      <c r="I679" t="inlineStr">
+        <is>
+          <t>Quotations engine</t>
+        </is>
+      </c>
+    </row>
+    <row r="680">
+      <c r="A680" t="inlineStr">
+        <is>
+          <t>ART-DISC-1</t>
+        </is>
+      </c>
+      <c r="B680" t="inlineStr">
+        <is>
+          <t>One discount meaning (real discount) in articles + quote/invoice lines; article discount reaches the line</t>
+        </is>
+      </c>
+      <c r="C680" t="inlineStr">
+        <is>
+          <t>Library</t>
+        </is>
+      </c>
+      <c r="D680" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E680" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F680" t="inlineStr">
+        <is>
+          <t>7521fb4</t>
+        </is>
+      </c>
+      <c r="G680" t="inlineStr">
+        <is>
+          <t>Data flipped by Florin (SQL, 3 articles)</t>
+        </is>
+      </c>
+      <c r="H680" t="inlineStr">
+        <is>
+          <t>L3</t>
+        </is>
+      </c>
+      <c r="I680" t="inlineStr">
+        <is>
+          <t>Quotations engine</t>
+        </is>
+      </c>
+    </row>
+    <row r="681">
+      <c r="A681" t="inlineStr">
+        <is>
+          <t>GRID-NUM-1</t>
+        </is>
+      </c>
+      <c r="B681" t="inlineStr">
+        <is>
+          <t>Grid number cells stored "[object Object]" — store the number; formulas unwrap legacy; repair SQL run</t>
+        </is>
+      </c>
+      <c r="C681" t="inlineStr">
+        <is>
+          <t>Records</t>
+        </is>
+      </c>
+      <c r="D681" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E681" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F681" t="inlineStr">
+        <is>
+          <t>5a72144</t>
+        </is>
+      </c>
+      <c r="G681" t="inlineStr">
+        <is>
+          <t>12 fields repaired 2026-10-03</t>
+        </is>
+      </c>
+      <c r="H681" t="inlineStr">
+        <is>
+          <t>L3</t>
+        </is>
+      </c>
+      <c r="I681" t="inlineStr">
+        <is>
+          <t>grid / record surface primitives</t>
+        </is>
+      </c>
+    </row>
+    <row r="682">
+      <c r="A682" t="inlineStr">
+        <is>
+          <t>KERN-SCHEMA-1</t>
+        </is>
+      </c>
+      <c r="B682" t="inlineStr">
+        <is>
+          <t>System database columns from the kernel, reconciled server-side per tenant, tier-gated; never rows</t>
+        </is>
+      </c>
+      <c r="C682" t="inlineStr">
+        <is>
+          <t>Kernel</t>
+        </is>
+      </c>
+      <c r="D682" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E682" t="inlineStr">
+        <is>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="F682" t="inlineStr">
+        <is>
+          <t>branch hold/kern-schema-1</t>
+        </is>
+      </c>
+      <c r="G682" t="inlineStr">
+        <is>
+          <t>Waiting Florin; Murgu had 0 fields on 10 DBs</t>
+        </is>
+      </c>
+      <c r="H682" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="I682" t="inlineStr">
+        <is>
+          <t>provisioning capability</t>
+        </is>
+      </c>
+    </row>
+    <row r="683">
+      <c r="A683" t="inlineStr">
+        <is>
+          <t>ENT-FREE-1</t>
+        </is>
+      </c>
+      <c r="B683" t="inlineStr">
+        <is>
+          <t>FREE gets no databases at all; PRO an empty library; ENTERPRISE may get it filled — and close the ungated library</t>
+        </is>
+      </c>
+      <c r="C683" t="inlineStr">
+        <is>
+          <t>Entitlement</t>
+        </is>
+      </c>
+      <c r="D683" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E683" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F683" t="inlineStr">
+        <is>
+          <t>Florin 2026-10-03</t>
+        </is>
+      </c>
+      <c r="G683" t="inlineStr">
+        <is>
+          <t>Provisioning creates 16 for everyone today</t>
+        </is>
+      </c>
+      <c r="H683" t="inlineStr">
+        <is>
+          <t>MODULE GATE</t>
+        </is>
+      </c>
+      <c r="I683" t="inlineStr">
+        <is>
+          <t>entitlement — vocabulary &amp; grants (modules → submodules → quota)</t>
+        </is>
+      </c>
+    </row>
+    <row r="684">
+      <c r="A684" t="inlineStr">
+        <is>
+          <t>DATE-PICKER-1</t>
+        </is>
+      </c>
+      <c r="B684" t="inlineStr">
+        <is>
+          <t>Date picker inside a dialog: calendar now opens in the dialog (days were unclickable)</t>
+        </is>
+      </c>
+      <c r="C684" t="inlineStr">
+        <is>
+          <t>Design system</t>
+        </is>
+      </c>
+      <c r="D684" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E684" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F684" t="inlineStr">
+        <is>
+          <t>b5ec10b</t>
+        </is>
+      </c>
+      <c r="G684" t="inlineStr">
+        <is>
+          <t>Manual hours landed on today</t>
+        </is>
+      </c>
+      <c r="H684" t="inlineStr">
+        <is>
+          <t>L4</t>
+        </is>
+      </c>
+      <c r="I684" t="inlineStr">
+        <is>
+          <t>date display</t>
+        </is>
+      </c>
+    </row>
+    <row r="685">
+      <c r="A685" t="inlineStr">
+        <is>
+          <t>LOC-SWEEP-1</t>
+        </is>
+      </c>
+      <c r="B685" t="inlineStr">
+        <is>
+          <t>Belgian dates/times/numbers in 38 ERP sites</t>
+        </is>
+      </c>
+      <c r="C685" t="inlineStr">
+        <is>
+          <t>Design system</t>
+        </is>
+      </c>
+      <c r="D685" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="E685" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F685" t="inlineStr">
+        <is>
+          <t>03ec24c (coder)</t>
+        </is>
+      </c>
+      <c r="G685" t="inlineStr"/>
+      <c r="H685" t="inlineStr">
+        <is>
+          <t>L4</t>
+        </is>
+      </c>
+      <c r="I685" t="inlineStr">
+        <is>
+          <t>date display</t>
+        </is>
+      </c>
+    </row>
+    <row r="686">
+      <c r="A686" t="inlineStr">
+        <is>
+          <t>FONTS-1</t>
+        </is>
+      </c>
+      <c r="B686" t="inlineStr">
+        <is>
+          <t>Self-hosted fonts — builds no longer fetch Google Fonts (failed twice); Cyrillic for the crew</t>
+        </is>
+      </c>
+      <c r="C686" t="inlineStr">
+        <is>
+          <t>Platform</t>
+        </is>
+      </c>
+      <c r="D686" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E686" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F686" t="inlineStr">
+        <is>
+          <t>5ae807e</t>
+        </is>
+      </c>
+      <c r="G686" t="inlineStr"/>
+      <c r="H686" t="inlineStr">
+        <is>
+          <t>⟂</t>
+        </is>
+      </c>
+      <c r="I686" t="inlineStr">
+        <is>
+          <t>release</t>
+        </is>
+      </c>
+    </row>
+    <row r="687">
+      <c r="A687" t="inlineStr">
+        <is>
+          <t>PLAN-FIRST-1</t>
+        </is>
+      </c>
+      <c r="B687" t="inlineStr">
+        <is>
+          <t>Coder protocol: plan → review → milestones; §3a throw proof; §3b a fence is a wall</t>
+        </is>
+      </c>
+      <c r="C687" t="inlineStr">
+        <is>
+          <t>Process</t>
+        </is>
+      </c>
+      <c r="D687" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E687" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F687" t="inlineStr">
+        <is>
+          <t>77ebd40, 238d618</t>
+        </is>
+      </c>
+      <c r="G687" t="inlineStr"/>
+      <c r="H687" t="inlineStr">
+        <is>
+          <t>⟂</t>
+        </is>
+      </c>
+      <c r="I687" t="inlineStr">
+        <is>
+          <t>process &amp; housekeeping</t>
+        </is>
+      </c>
+    </row>
+    <row r="688">
+      <c r="A688" t="inlineStr">
+        <is>
+          <t>R2-1-CENSUS</t>
+        </is>
+      </c>
+      <c r="B688" t="inlineStr">
+        <is>
+          <t>Coder: census of the 33 direct GlobalPage writes (tenant check, OCC, audit, fate)</t>
+        </is>
+      </c>
+      <c r="C688" t="inlineStr">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="D688" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E688" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F688" t="inlineStr">
+        <is>
+          <t>coder</t>
+        </is>
+      </c>
+      <c r="G688" t="inlineStr">
+        <is>
+          <t>Queued</t>
+        </is>
+      </c>
+      <c r="H688" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="I688" t="inlineStr">
+        <is>
+          <t>write path — saveRecord, intents, read model</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(roadmap): central catalogue (ERP → tenant only), library packs with opt-in nudges, price service, supplier cart import
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/.agents/coral-roadmap.xlsx
+++ b/.agents/coral-roadmap.xlsx
@@ -594,7 +594,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I688"/>
+  <dimension ref="A1:I695"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -30566,7 +30566,6 @@
           <t>ff9e5cc, 638bf2c</t>
         </is>
       </c>
-      <c r="G669" t="inlineStr"/>
       <c r="H669" t="inlineStr">
         <is>
           <t>L3</t>
@@ -30656,7 +30655,6 @@
           <t>cd8fba3</t>
         </is>
       </c>
-      <c r="G671" t="inlineStr"/>
       <c r="H671" t="inlineStr">
         <is>
           <t>L3</t>
@@ -30793,7 +30791,6 @@
           <t>24aa6db</t>
         </is>
       </c>
-      <c r="G674" t="inlineStr"/>
       <c r="H674" t="inlineStr">
         <is>
           <t>L3</t>
@@ -30836,7 +30833,6 @@
           <t>aa28cea</t>
         </is>
       </c>
-      <c r="G675" t="inlineStr"/>
       <c r="H675" t="inlineStr">
         <is>
           <t>L3</t>
@@ -31302,7 +31298,6 @@
           <t>03ec24c (coder)</t>
         </is>
       </c>
-      <c r="G685" t="inlineStr"/>
       <c r="H685" t="inlineStr">
         <is>
           <t>L4</t>
@@ -31345,7 +31340,6 @@
           <t>5ae807e</t>
         </is>
       </c>
-      <c r="G686" t="inlineStr"/>
       <c r="H686" t="inlineStr">
         <is>
           <t>⟂</t>
@@ -31388,7 +31382,6 @@
           <t>77ebd40, 238d618</t>
         </is>
       </c>
-      <c r="G687" t="inlineStr"/>
       <c r="H687" t="inlineStr">
         <is>
           <t>⟂</t>
@@ -31444,6 +31437,335 @@
       <c r="I688" t="inlineStr">
         <is>
           <t>write path — saveRecord, intents, read model</t>
+        </is>
+      </c>
+    </row>
+    <row r="689">
+      <c r="A689" t="inlineStr">
+        <is>
+          <t>CAT-1</t>
+        </is>
+      </c>
+      <c r="B689" t="inlineStr">
+        <is>
+          <t>Central catalogue (articles + bestek), owned and maintained by the platform. Information flows ERP → tenant, NEVER tenant → ERP: no tenant row, price or edit is ever read back into it.</t>
+        </is>
+      </c>
+      <c r="C689" t="inlineStr">
+        <is>
+          <t>Library</t>
+        </is>
+      </c>
+      <c r="D689" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E689" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F689" t="inlineStr">
+        <is>
+          <t>Florin 2026-10-03</t>
+        </is>
+      </c>
+      <c r="G689" t="inlineStr">
+        <is>
+          <t>Indispensable: every new tenant library is hydrated from an up-to-date catalogue, not a stale seed.</t>
+        </is>
+      </c>
+      <c r="H689" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="I689" t="inlineStr">
+        <is>
+          <t>central catalogue — ERP → tenant only</t>
+        </is>
+      </c>
+    </row>
+    <row r="690">
+      <c r="A690" t="inlineStr">
+        <is>
+          <t>CAT-2</t>
+        </is>
+      </c>
+      <c r="B690" t="inlineStr">
+        <is>
+          <t>Hydrate a tenant library from the catalogue: rows are COPIED into the tenant's own articles / bestek; the tenant owns and edits the copy. Each row remembers its catalogue origin (id + version).</t>
+        </is>
+      </c>
+      <c r="C690" t="inlineStr">
+        <is>
+          <t>Library</t>
+        </is>
+      </c>
+      <c r="D690" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E690" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F690" t="inlineStr">
+        <is>
+          <t>Florin 2026-10-03</t>
+        </is>
+      </c>
+      <c r="G690" t="inlineStr">
+        <is>
+          <t>PRO starts with an EMPTY library and bestek (columns only, KERN-SCHEMA-1). Hydration happens on purchase (CAT-3); ENTERPRISE may get it included.</t>
+        </is>
+      </c>
+      <c r="H690" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="I690" t="inlineStr">
+        <is>
+          <t>central catalogue — ERP → tenant only</t>
+        </is>
+      </c>
+    </row>
+    <row r="691">
+      <c r="A691" t="inlineStr">
+        <is>
+          <t>CAT-3</t>
+        </is>
+      </c>
+      <c r="B691" t="inlineStr">
+        <is>
+          <t>Library pack purchase: fill library + bestek from the catalogue (per trade), Stripe one-off; later an updates subscription.</t>
+        </is>
+      </c>
+      <c r="C691" t="inlineStr">
+        <is>
+          <t>Library</t>
+        </is>
+      </c>
+      <c r="D691" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E691" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F691" t="inlineStr">
+        <is>
+          <t>Florin 2026-10-03</t>
+        </is>
+      </c>
+      <c r="G691" t="inlineStr">
+        <is>
+          <t>Separate from the tier. Depends on ENT-FREE-1, KERN-SCHEMA-1, CAT-1/2.</t>
+        </is>
+      </c>
+      <c r="H691" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="I691" t="inlineStr">
+        <is>
+          <t>Library module</t>
+        </is>
+      </c>
+    </row>
+    <row r="692">
+      <c r="A692" t="inlineStr">
+        <is>
+          <t>CAT-NUDGE-1</t>
+        </is>
+      </c>
+      <c r="B692" t="inlineStr">
+        <is>
+          <t>Discrete, OPT-IN nudges toward the pack: empty-state card in library/bestek; a quiet "a similar item exists in the catalogue" hint in the quote line picker; an onboarding checklist item; a line on the plan/billing page.</t>
+        </is>
+      </c>
+      <c r="C692" t="inlineStr">
+        <is>
+          <t>Library</t>
+        </is>
+      </c>
+      <c r="D692" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="E692" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F692" t="inlineStr">
+        <is>
+          <t>Florin 2026-10-03</t>
+        </is>
+      </c>
+      <c r="G692" t="inlineStr">
+        <is>
+          <t>NEVER opt-out: no pop-ups, no auto-enrolment, no pre-ticked boxes, no trial that converts. Every nudge dismissible for good.</t>
+        </is>
+      </c>
+      <c r="H692" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="I692" t="inlineStr">
+        <is>
+          <t>Library module</t>
+        </is>
+      </c>
+    </row>
+    <row r="693">
+      <c r="A693" t="inlineStr">
+        <is>
+          <t>CAT-4</t>
+        </is>
+      </c>
+      <c r="B693" t="inlineStr">
+        <is>
+          <t>Price maintenance as a service: we update catalogue prices; tenants with catalogue-origin rows get a notification; applying the update is opt-in (per item or batch, with old → new shown).</t>
+        </is>
+      </c>
+      <c r="C693" t="inlineStr">
+        <is>
+          <t>Library</t>
+        </is>
+      </c>
+      <c r="D693" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="E693" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F693" t="inlineStr">
+        <is>
+          <t>Florin 2026-10-03</t>
+        </is>
+      </c>
+      <c r="G693" t="inlineStr">
+        <is>
+          <t>A tenant row edited by hand or sourced from their own supplier is never overwritten. Uses CAT-2 origin + version.</t>
+        </is>
+      </c>
+      <c r="H693" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="I693" t="inlineStr">
+        <is>
+          <t>central catalogue — ERP → tenant only</t>
+        </is>
+      </c>
+    </row>
+    <row r="694">
+      <c r="A694" t="inlineStr">
+        <is>
+          <t>SUP-1</t>
+        </is>
+      </c>
+      <c r="B694" t="inlineStr">
+        <is>
+          <t>Supplier sources for the catalogue and for tenants: Cebeo, Rexel, Facq … — inventory which offer a link / integration.</t>
+        </is>
+      </c>
+      <c r="C694" t="inlineStr">
+        <is>
+          <t>Library</t>
+        </is>
+      </c>
+      <c r="D694" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="E694" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F694" t="inlineStr">
+        <is>
+          <t>Florin 2026-10-03</t>
+        </is>
+      </c>
+      <c r="G694" t="inlineStr">
+        <is>
+          <t>Research item; feeds CAT-1 and SUP-CART-1.</t>
+        </is>
+      </c>
+      <c r="H694" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="I694" t="inlineStr">
+        <is>
+          <t>Library module</t>
+        </is>
+      </c>
+    </row>
+    <row r="695">
+      <c r="A695" t="inlineStr">
+        <is>
+          <t>SUP-CART-1</t>
+        </is>
+      </c>
+      <c r="B695" t="inlineStr">
+        <is>
+          <t>Supplier cart import: an in-app webview where the tenant is logged into a supplier shop; read the CURRENT session cart (real-time lines, their prices) and import into a quote / the library. No guessed or unofficial supplier API.</t>
+        </is>
+      </c>
+      <c r="C695" t="inlineStr">
+        <is>
+          <t>Library</t>
+        </is>
+      </c>
+      <c r="D695" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="E695" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F695" t="inlineStr">
+        <is>
+          <t>Florin 2026-10-03</t>
+        </is>
+      </c>
+      <c r="G695" t="inlineStr">
+        <is>
+          <t>Logged for later. Constraint: a web page cannot read another site's cart; needs a native shell (app webview) or a browser extension, and each shop's terms checked. Prices land in the TENANT library only (never the catalogue — CAT-1).</t>
+        </is>
+      </c>
+      <c r="H695" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="I695" t="inlineStr">
+        <is>
+          <t>Library module</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(late-tz-1): SQL to list and correct the manual entries that landed 2 h late; TD-0 with the coder; nudges approved
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/.agents/coral-roadmap.xlsx
+++ b/.agents/coral-roadmap.xlsx
@@ -26804,7 +26804,7 @@
       </c>
       <c r="E589" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="F589" t="inlineStr">
@@ -26814,7 +26814,7 @@
       </c>
       <c r="G589" t="inlineStr">
         <is>
-          <t>The only honest input to sequencing. Per file, by category: casing rename / semantic mapping / phantom field / real bug / type debt. Fix nothing. One file gave 24 errors — do not extrapolate.</t>
+          <t>The only honest input to sequencing. Per file, by category: casing rename / semantic mapping / phantom field / real bug / type debt. Fix nothing. One file gave 24 errors — do not extrapolate. Coder, from 2026-10-03.</t>
         </is>
       </c>
       <c r="H589" t="inlineStr">
@@ -30240,7 +30240,7 @@
       </c>
       <c r="G662" t="inlineStr">
         <is>
-          <t>Live 2026-10-01. Past entries since June: list offered, not fixed</t>
+          <t>Live 2026-10-01. Past entries: Florin 2026-10-03 "yes" — list + per-entry repair in .agents/workflows/sql/late-entry-tz-repair.sql (Florin runs).</t>
         </is>
       </c>
       <c r="H662" t="inlineStr">
@@ -31614,7 +31614,7 @@
       </c>
       <c r="G692" t="inlineStr">
         <is>
-          <t>NEVER opt-out: no pop-ups, no auto-enrolment, no pre-ticked boxes, no trial that converts. Every nudge dismissible for good.</t>
+          <t>NEVER opt-out: no pop-ups, no auto-enrolment, no pre-ticked boxes, no trial that converts. Every nudge dismissible for good. Florin 2026-10-03: OK on all four nudges.</t>
         </is>
       </c>
       <c r="H692" t="inlineStr">

</xml_diff>

<commit_message>
docs(roadmap): TD-0 closed after review — shift editor rebuild (WH-7) confirmed
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/.agents/coral-roadmap.xlsx
+++ b/.agents/coral-roadmap.xlsx
@@ -26804,7 +26804,7 @@
       </c>
       <c r="E589" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F589" t="inlineStr">
@@ -26814,7 +26814,7 @@
       </c>
       <c r="G589" t="inlineStr">
         <is>
-          <t>The only honest input to sequencing. Per file, by category: casing rename / semantic mapping / phantom field / real bug / type debt. Fix nothing. One file gave 24 errors — do not extrapolate. Coder, from 2026-10-03.</t>
+          <t>The only honest input to sequencing. Per file, by category: casing rename / semantic mapping / phantom field / real bug / type debt. Fix nothing. One file gave 24 errors — do not extrapolate. Coder, from 2026-10-03. Closed 2026-10-03 (report .agents/reports/TD-0.md, reviewed): 0 tsc errors, @ts-nocheck only in 2 vendor files; debt left = 5 SUPA-2-allowlisted files. Shift editor (EditShiftDialog + CreateShiftForm) carries most of it → WH-7 REBUILD confirmed. Review caveat: the report's 199 is a grep — it counts string VALUES (late_entry, clock_entry, shift_submitted, work_order_signed) that are stored data / error codes and must NOT be renamed.</t>
         </is>
       </c>
       <c r="H589" t="inlineStr">

</xml_diff>

<commit_message>
docs(roadmap): Florin's 3 Oct decisions — bestek as full work, enterprise columns, column permissions, WO-4b admin review, WO-4a-M4
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/.agents/coral-roadmap.xlsx
+++ b/.agents/coral-roadmap.xlsx
@@ -594,7 +594,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I695"/>
+  <dimension ref="A1:I699"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -30474,7 +30474,7 @@
       </c>
       <c r="G667" t="inlineStr">
         <is>
-          <t>Planner. Prints shift description + crew notes (Florin 2026-10-02)</t>
+          <t>Planner. Prints shift description + crew notes (Florin 2026-10-02) Florin 2026-10-03: sending is NOT automatic — the signed PDF passes admin review first (like hours approval), then is sent. Migration via the usual SOP.</t>
         </is>
       </c>
       <c r="H667" t="inlineStr">
@@ -30971,7 +30971,7 @@
       </c>
       <c r="G678" t="inlineStr">
         <is>
-          <t>Next (step 3)</t>
+          <t>Next (step 3) Florin 2026-10-03: GO, with VARIANT-1.</t>
         </is>
       </c>
       <c r="H678" t="inlineStr">
@@ -31018,7 +31018,7 @@
       </c>
       <c r="G679" t="inlineStr">
         <is>
-          <t>Found digging the variants logic</t>
+          <t>Found digging the variants logic Florin 2026-10-03: YES, together with WO-LIB-1 (near-zero overhead). Found: variant price is read from a fixed demo database id (db-articles) — verify on a real tenant.</t>
         </is>
       </c>
       <c r="H679" t="inlineStr">
@@ -31159,7 +31159,7 @@
       </c>
       <c r="G682" t="inlineStr">
         <is>
-          <t>Waiting Florin; Murgu had 0 fields on 10 DBs</t>
+          <t>Waiting Florin; Murgu had 0 fields on 10 DBs Florin 2026-10-03: GO — but ENT-COL-1 / COL-PERM-1 / BESTEK-COMP-1 may change the plan before release.</t>
         </is>
       </c>
       <c r="H682" t="inlineStr">
@@ -31766,6 +31766,194 @@
       <c r="I695" t="inlineStr">
         <is>
           <t>Library module</t>
+        </is>
+      </c>
+    </row>
+    <row r="696">
+      <c r="A696" t="inlineStr">
+        <is>
+          <t>BESTEK-COMP-1</t>
+        </is>
+      </c>
+      <c r="B696" t="inlineStr">
+        <is>
+          <t>Bestek post = full work: holds articles (with a QUANTITY per article) + labour, and calculates its unit price from them; picked in a quote it pulls the whole work from the library.</t>
+        </is>
+      </c>
+      <c r="C696" t="inlineStr">
+        <is>
+          <t>Library</t>
+        </is>
+      </c>
+      <c r="D696" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E696" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F696" t="inlineStr">
+        <is>
+          <t>Florin 2026-10-03</t>
+        </is>
+      </c>
+      <c r="G696" t="inlineStr">
+        <is>
+          <t>Partly exists: bestek has an "Artikelen" relation and a price formula (articles sale price + labour hours × rate), and the quote expands it into article lines. Gaps: no quantity per article (each counts once), labour rates hard-coded 35/45, and the quote expansion compares to a fixed demo id (db-bestek / db-articles) — verify it fires on a real tenant.</t>
+        </is>
+      </c>
+      <c r="H696" t="inlineStr">
+        <is>
+          <t>L3</t>
+        </is>
+      </c>
+      <c r="I696" t="inlineStr">
+        <is>
+          <t>Quotations engine</t>
+        </is>
+      </c>
+    </row>
+    <row r="697">
+      <c r="A697" t="inlineStr">
+        <is>
+          <t>ENT-COL-1</t>
+        </is>
+      </c>
+      <c r="B697" t="inlineStr">
+        <is>
+          <t>ENTERPRISE custom columns on system databases, with the same flexibility as the system columns (types, formulas, relations) — and kept apart from the kernel-owned columns so the reconcile never touches them.</t>
+        </is>
+      </c>
+      <c r="C697" t="inlineStr">
+        <is>
+          <t>Library</t>
+        </is>
+      </c>
+      <c r="D697" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="E697" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F697" t="inlineStr">
+        <is>
+          <t>Florin 2026-10-03</t>
+        </is>
+      </c>
+      <c r="G697" t="inlineStr">
+        <is>
+          <t>Interacts with KERN-SCHEMA-1 (reconcile must leave tenant columns alone).</t>
+        </is>
+      </c>
+      <c r="H697" t="inlineStr">
+        <is>
+          <t>MODULE GATE</t>
+        </is>
+      </c>
+      <c r="I697" t="inlineStr">
+        <is>
+          <t>entitlement — vocabulary &amp; grants (modules → submodules → quota)</t>
+        </is>
+      </c>
+    </row>
+    <row r="698">
+      <c r="A698" t="inlineStr">
+        <is>
+          <t>COL-PERM-1</t>
+        </is>
+      </c>
+      <c r="B698" t="inlineStr">
+        <is>
+          <t>Column-level permissions as a gating layer: per tier (which columns a plan gets) and inside the tenant (which role sees / edits which column of a database).</t>
+        </is>
+      </c>
+      <c r="C698" t="inlineStr">
+        <is>
+          <t>Platform</t>
+        </is>
+      </c>
+      <c r="D698" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E698" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F698" t="inlineStr">
+        <is>
+          <t>Florin 2026-10-03</t>
+        </is>
+      </c>
+      <c r="G698" t="inlineStr">
+        <is>
+          <t>"We were against this wall recently" (cost/margin columns, admin notes). Same canonical logic as the rest: asked, never asserted; enforced on the server read and write path, not only hidden in the UI.</t>
+        </is>
+      </c>
+      <c r="H698" t="inlineStr">
+        <is>
+          <t>MODULE GATE</t>
+        </is>
+      </c>
+      <c r="I698" t="inlineStr">
+        <is>
+          <t>entitlement — vocabulary &amp; grants (modules → submodules → quota)</t>
+        </is>
+      </c>
+    </row>
+    <row r="699">
+      <c r="A699" t="inlineStr">
+        <is>
+          <t>WO-4a-M4</t>
+        </is>
+      </c>
+      <c r="B699" t="inlineStr">
+        <is>
+          <t>Work order PDF: remove the two global patches (Math.random seeding, PDFKit deflate prototype) — determinism tested on content, not bytes.</t>
+        </is>
+      </c>
+      <c r="C699" t="inlineStr">
+        <is>
+          <t>WorkHub</t>
+        </is>
+      </c>
+      <c r="D699" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E699" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F699" t="inlineStr">
+        <is>
+          <t>Florin 2026-10-03</t>
+        </is>
+      </c>
+      <c r="G699" t="inlineStr">
+        <is>
+          <t>Required before WO-4b wires the renderer into signing; today the renderer is imported nowhere (inert).</t>
+        </is>
+      </c>
+      <c r="H699" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="I699" t="inlineStr">
+        <is>
+          <t>document engine (+ archive, attachments)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(map): task list back under every block; Florin's answers on bestek, column permissions, PDF name, KERN-TIME
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/.agents/coral-roadmap.xlsx
+++ b/.agents/coral-roadmap.xlsx
@@ -24981,7 +24981,7 @@
       </c>
       <c r="G550" t="inlineStr">
         <is>
-          <t>CreateShiftForm 1967 + EditShiftDialog 915 + ShiftViewDialog 626. BLOCKED on PROJ-0 and R1-4 — starting earlier rebuilds the [ERP] prefix and the 74 parse sites into new code. | STRONGER JUSTIFICATION (CSF-1, 2026-09-28): the ~900-line form exists TWICE in one file. Both CSF-1 defects are a fix that landed on one copy and not the other — and the copy that missed both is the matrix-+ path, which is the one actually used. | SCOPE REDUCED: ShiftViewDialog is deleted by WH-UI-1, so WH-7 is CreateShiftForm + EditShiftDialog — 2,882 lines, not 3,508.</t>
+          <t>CreateShiftForm 1967 + EditShiftDialog 915 + ShiftViewDialog 626. BLOCKED on PROJ-0 and R1-4 — starting earlier rebuilds the [ERP] prefix and the 74 parse sites into new code. | STRONGER JUSTIFICATION (CSF-1, 2026-09-28): the ~900-line form exists TWICE in one file. Both CSF-1 defects are a fix that landed on one copy and not the other — and the copy that missed both is the matrix-+ path, which is the one actually used. | SCOPE REDUCED: ShiftViewDialog is deleted by WH-UI-1, so WH-7 is CreateShiftForm + EditShiftDialog — 2,882 lines, not 3,508. Florin 2026-10-03: build on the kernel time functions now (do not wait for KERN-TIME).</t>
         </is>
       </c>
       <c r="H550" t="inlineStr">
@@ -26673,7 +26673,7 @@
       </c>
       <c r="G586" t="inlineStr">
         <is>
-          <t>ScheduledShift.shiftDate/Start/End are String; ClockEntry.clockInTime is DateTime. 25 hand-parse sites (split('-')/split(':')) exist because the text form forces every consumer to parse. The kernel owns the arithmetic (computeWorkedDuration) but no TYPE. A kernel time type makes this crash class unrepresentable. | Planner 2026-09-30: kernel/shift-time.ts created (KERN-TIME-1)</t>
+          <t>ScheduledShift.shiftDate/Start/End are String; ClockEntry.clockInTime is DateTime. 25 hand-parse sites (split('-')/split(':')) exist because the text form forces every consumer to parse. The kernel owns the arithmetic (computeWorkedDuration) but no TYPE. A kernel time type makes this crash class unrepresentable. | Planner 2026-09-30: kernel/shift-time.ts created (KERN-TIME-1) Florin 2026-10-03: WH-7 builds on the kernel time functions now; the storage change stays invisible to it.</t>
         </is>
       </c>
       <c r="H586" t="inlineStr">
@@ -30474,7 +30474,7 @@
       </c>
       <c r="G667" t="inlineStr">
         <is>
-          <t>Planner. Prints shift description + crew notes (Florin 2026-10-02) Florin 2026-10-03: sending is NOT automatic — the signed PDF passes admin review first (like hours approval), then is sent. Migration via the usual SOP.</t>
+          <t>Planner. Prints shift description + crew notes (Florin 2026-10-02) Florin 2026-10-03: sending is NOT automatic — the signed PDF passes admin review first (like hours approval), then is sent. Migration via the usual SOP. PDF file name (Florin 2026-10-03): localised "Werkbon" + work order nr + date (nl Werkbon / fr Bon de travail / en Work order).</t>
         </is>
       </c>
       <c r="H667" t="inlineStr">
@@ -30971,7 +30971,7 @@
       </c>
       <c r="G678" t="inlineStr">
         <is>
-          <t>Next (step 3) Florin 2026-10-03: GO, with VARIANT-1.</t>
+          <t>Next (step 3) Florin 2026-10-03: GO, with VARIANT-1. "CUSTOM PRIJS" (number, under the variants, not localised): a column the tenant added — not in the canonical schema, read by no engine.</t>
         </is>
       </c>
       <c r="H678" t="inlineStr">
@@ -31802,7 +31802,7 @@
       </c>
       <c r="G696" t="inlineStr">
         <is>
-          <t>Partly exists: bestek has an "Artikelen" relation and a price formula (articles sale price + labour hours × rate), and the quote expands it into article lines. Gaps: no quantity per article (each counts once), labour rates hard-coded 35/45, and the quote expansion compares to a fixed demo id (db-bestek / db-articles) — verify it fires on a real tenant.</t>
+          <t>Partly exists: bestek has an "Artikelen" relation and a price formula (articles sale price + labour hours × rate), and the quote expands it into article lines. Gaps: no quantity per article (each counts once), labour rates hard-coded 35/45, and the quote expansion compares to a fixed demo id (db-bestek / db-articles) — verify it fires on a real tenant. Florin 2026-10-03: the articles come in as SUB-ITEMS of the bestek line; the editor keeps its function; in the quote only the bestek is visible — except the DETAILED quote, which shows the entire content.</t>
         </is>
       </c>
       <c r="H696" t="inlineStr">
@@ -31896,7 +31896,7 @@
       </c>
       <c r="G698" t="inlineStr">
         <is>
-          <t>"We were against this wall recently" (cost/margin columns, admin notes). Same canonical logic as the rest: asked, never asserted; enforced on the server read and write path, not only hidden in the UI.</t>
+          <t>"We were against this wall recently" (cost/margin columns, admin notes). Same canonical logic as the rest: asked, never asserted; enforced on the server read and write path, not only hidden in the UI. Florin 2026-10-03: run it IN the canonical logic — no deviation (one gate, asked not asserted, server-side).</t>
         </is>
       </c>
       <c r="H698" t="inlineStr">

</xml_diff>

<commit_message>
docs: GEO-2 M1 approved (GO M2); TD-2 done; WEBSITES/EMAIL decision; R1-2 led by the Planner; PRO set defined as we go
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/.agents/coral-roadmap.xlsx
+++ b/.agents/coral-roadmap.xlsx
@@ -10392,7 +10392,7 @@
       </c>
       <c r="G226" s="11" t="inlineStr">
         <is>
-          <t>[P3.3] Was: denormalise tenantId column — WITHDRAWN | Planner 2026-10-01: resolveDatabaseId fail-closed in the kernel, all 11 callers converted — branch track-b/r1-2-kern-8. GATED on .agents/workflows/r1-2-binding-census.sql (Florin)</t>
+          <t>[P3.3] Was: denormalise tenantId column — WITHDRAWN | Planner 2026-10-01: resolveDatabaseId fail-closed in the kernel, all 11 callers converted — branch track-b/r1-2-kern-8. GATED on .agents/workflows/r1-2-binding-census.sql (Florin) Florin 2026-10-03: the Planner leads the binding census.</t>
         </is>
       </c>
       <c r="H226" s="28" t="inlineStr">
@@ -23148,7 +23148,7 @@
       </c>
       <c r="G511" t="inlineStr">
         <is>
-          <t>A one-way door: present in data, cannot be re-granted if ever removed. MODULES (7) omits both.</t>
+          <t>A one-way door: present in data, cannot be re-granted if ever removed. MODULES (7) omits both. Florin 2026-10-03: finish the features first, then decide what is grantable. WEBSITES/EMAIL ideally become nice-to-haves that sweeten upgrades. PRO happy path: website (lead-capture form) → lead (pipeline) ⇄ mail → quote → project → portal. Tease and squeeze, never past ethics.</t>
         </is>
       </c>
       <c r="H511" t="inlineStr">
@@ -26898,7 +26898,7 @@
       </c>
       <c r="E591" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F591" t="inlineStr">
@@ -26908,7 +26908,7 @@
       </c>
       <c r="G591" t="inlineStr">
         <is>
-          <t>source_project_id is read on ScheduleAttachment and exists in neither Prisma nor the client type — the feature it drives is already dead. Implement or delete. NEVER rename a phantom.</t>
+          <t>source_project_id is read on ScheduleAttachment and exists in neither Prisma nor the client type — the feature it drives is already dead. Implement or delete. NEVER rename a phantom. Done 2026-10-03 (Florin "gone, please"): source_project_id removed (42bd5fc) — never written; its "From Project" badge could never show.</t>
         </is>
       </c>
       <c r="H591" t="inlineStr">
@@ -29352,7 +29352,7 @@
       </c>
       <c r="G643" t="inlineStr">
         <is>
-          <t>coral-draft-pro-tier.md — awaiting Florin</t>
+          <t>coral-draft-pro-tier.md — awaiting Florin Florin 2026-10-03: PRO module set stays OPEN — defined as we go; raise it in conversations, do not force it now.</t>
         </is>
       </c>
       <c r="H643" t="inlineStr">
@@ -29760,7 +29760,7 @@
       </c>
       <c r="E652" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="F652" t="inlineStr">
@@ -29770,7 +29770,7 @@
       </c>
       <c r="G652" t="inlineStr">
         <is>
-          <t>PLANNED</t>
+          <t>PLANNED Plan approved; M1 approved 2026-10-03, GO M2.</t>
         </is>
       </c>
       <c r="H652" t="inlineStr">

</xml_diff>

<commit_message>
docs(roadmap): KERN-SCHEMA-1 released; custom columns in the permission scheme (COL-PERM-1)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/.agents/coral-roadmap.xlsx
+++ b/.agents/coral-roadmap.xlsx
@@ -29770,7 +29770,7 @@
       </c>
       <c r="G652" t="inlineStr">
         <is>
-          <t>PLANNED Plan approved; M1 approved 2026-10-03, GO M2.</t>
+          <t>PLANNED Plan approved; M1 approved 2026-10-03, GO M2. M2 reported done 2026-10-03.</t>
         </is>
       </c>
       <c r="H652" t="inlineStr">
@@ -31149,7 +31149,7 @@
       </c>
       <c r="E682" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F682" t="inlineStr">
@@ -31159,7 +31159,7 @@
       </c>
       <c r="G682" t="inlineStr">
         <is>
-          <t>Waiting Florin; Murgu had 0 fields on 10 DBs Florin 2026-10-03: GO — but ENT-COL-1 / COL-PERM-1 / BESTEK-COMP-1 may change the plan before release.</t>
+          <t>Waiting Florin; Murgu had 0 fields on 10 DBs Florin 2026-10-03: GO — but ENT-COL-1 / COL-PERM-1 / BESTEK-COMP-1 may change the plan before release. Released 2026-10-03 (832ef53) with numbered upgrade steps (system-schema-upgrades.ts, U1 = accountantExportedAt checkbox): each step applies only while the field has the old shape — no per-tenant storage, no migration; tenant-changed fields are left alone.</t>
         </is>
       </c>
       <c r="H682" t="inlineStr">
@@ -31896,7 +31896,7 @@
       </c>
       <c r="G698" t="inlineStr">
         <is>
-          <t>"We were against this wall recently" (cost/margin columns, admin notes). Same canonical logic as the rest: asked, never asserted; enforced on the server read and write path, not only hidden in the UI. Florin 2026-10-03: run it IN the canonical logic — no deviation (one gate, asked not asserted, server-side).</t>
+          <t>"We were against this wall recently" (cost/margin columns, admin notes). Same canonical logic as the rest: asked, never asserted; enforced on the server read and write path, not only hidden in the UI. Florin 2026-10-03: run it IN the canonical logic — no deviation (one gate, asked not asserted, server-side). Florin 2026-10-03: CUSTOM columns fall into the same permission scheme as the system columns — a manager can split who sees what (per team member), on custom and core columns alike. System-column permission metadata arrives via a numbered upgrade step; custom-column permissions are tenant data.</t>
         </is>
       </c>
       <c r="H698" t="inlineStr">

</xml_diff>

<commit_message>
docs(roadmap): P0 sweep — 4 holes fixed, 14 verified done, 3 trial items parked; map regenerated
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/.agents/coral-roadmap.xlsx
+++ b/.agents/coral-roadmap.xlsx
@@ -1460,7 +1460,7 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
@@ -1468,7 +1468,11 @@
           <t>coral-mem3-lazy-data.md</t>
         </is>
       </c>
-      <c r="G20" s="2" t="inlineStr"/>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>Verified 2026-10-04: getGlobalPageIndex + pageIndex loaded in the admin and mobile layouts.</t>
+        </is>
+      </c>
       <c r="H20" s="23" t="inlineStr">
         <is>
           <t>L1</t>
@@ -12148,7 +12152,7 @@
       </c>
       <c r="E264" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F264" s="11" t="inlineStr">
@@ -12158,7 +12162,7 @@
       </c>
       <c r="G264" s="11" t="inlineStr">
         <is>
-          <t>SAME TASK AS KERN-6 / pass 3a. Planner rediscovered this independently on 2026-09-25 and wrote it up as new (KERN-6a). Tonight's version is wider: five lists, 74 parse sites.</t>
+          <t>SAME TASK AS KERN-6 / pass 3a. Planner rediscovered this independently on 2026-09-25 and wrote it up as new (KERN-6a). Tonight's version is wider: five lists, 74 parse sites. Verified 2026-10-04: same as KERN-6 — one table, derived lists.</t>
         </is>
       </c>
       <c r="H264" s="28" t="inlineStr">
@@ -12610,7 +12614,7 @@
       </c>
       <c r="E274" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F274" s="11" t="inlineStr">
@@ -12620,7 +12624,7 @@
       </c>
       <c r="G274" s="11" t="inlineStr">
         <is>
-          <t>[P4.2] Landmine found 2026-09-12</t>
+          <t>[P4.2] Landmine found 2026-09-12 Fixed 2026-10-04 (3ef2e9a): updatePageServerFirst returns the row's real blocks + blocksVersion.</t>
         </is>
       </c>
       <c r="H274" s="23" t="inlineStr">
@@ -14548,7 +14552,7 @@
       </c>
       <c r="E316" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F316" s="11" t="inlineStr">
@@ -14558,7 +14562,7 @@
       </c>
       <c r="G316" s="11" t="inlineStr">
         <is>
-          <t>99 commits behind</t>
+          <t>99 commits behind Superseded 2026-10-04: develop/main separated again; every green commit promoted on its own SHA (promote.sh: CI + Vercel preview, schema ranges pushed by Florin).</t>
         </is>
       </c>
       <c r="H316" s="25" t="inlineStr">
@@ -14689,7 +14693,7 @@
       </c>
       <c r="E319" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F319" s="11" t="inlineStr">
@@ -14699,7 +14703,7 @@
       </c>
       <c r="G319" s="11" t="inlineStr">
         <is>
-          <t>Florin runs</t>
+          <t>Florin runs Superseded 2026-10-04: see PROMOTE-GATE.</t>
         </is>
       </c>
       <c r="H319" s="25" t="inlineStr">
@@ -14736,7 +14740,7 @@
       </c>
       <c r="E320" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F320" s="11" t="inlineStr">
@@ -14746,7 +14750,7 @@
       </c>
       <c r="G320" s="11" t="inlineStr">
         <is>
-          <t>pd.md Rule 8</t>
+          <t>pd.md Rule 8 Superseded 2026-10-04: see PROMOTE-GATE — the Vercel preview of the exact SHA is the staging pass.</t>
         </is>
       </c>
       <c r="H320" s="25" t="inlineStr">
@@ -15750,12 +15754,17 @@
       </c>
       <c r="E342" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F342" t="inlineStr">
         <is>
           <t>coral-r5-scheduled-work.md</t>
+        </is>
+      </c>
+      <c r="G342" t="inlineStr">
+        <is>
+          <t>Fixed 2026-10-04 (7ef1e28): isCronRequest() — one check, fail-closed, constant-time; prod CRON_SECRET confirmed set.</t>
         </is>
       </c>
       <c r="H342" s="23" t="inlineStr">
@@ -22292,7 +22301,7 @@
       </c>
       <c r="E493" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F493" t="inlineStr">
@@ -22302,7 +22311,7 @@
       </c>
       <c r="G493" t="inlineStr">
         <is>
-          <t>Five lists, five lengths: 16/16/14/8/6. Not five bugs — one missing table with columns (role, legacyBase, displayName, module).</t>
+          <t>Five lists, five lengths: 16/16/14/8/6. Not five bugs — one missing table with columns (role, legacyBase, displayName, module). Verified 2026-10-04: one SYSTEM_DATABASES table; the other lists are derived (16 each, tested).</t>
         </is>
       </c>
       <c r="H493" t="inlineStr">
@@ -22339,7 +22348,7 @@
       </c>
       <c r="E494" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F494" t="inlineStr">
@@ -22349,7 +22358,7 @@
       </c>
       <c r="G494" t="inlineStr">
         <is>
-          <t>isSystemDatabase('db-hr') === false -&gt; createPageServerFirst does not resolve them through the book; requiredModuleForDb does not gate them.</t>
+          <t>isSystemDatabase('db-hr') === false -&gt; createPageServerFirst does not resolve them through the book; requiredModuleForDb does not gate them. Verified 2026-10-04: SYSTEM_DB_PREFIXES derived from the 16 roles.</t>
         </is>
       </c>
       <c r="H494" t="inlineStr">
@@ -22433,7 +22442,7 @@
       </c>
       <c r="E496" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F496" t="inlineStr">
@@ -22443,7 +22452,7 @@
       </c>
       <c r="G496" t="inlineStr">
         <is>
-          <t>A permission decision made by string comparison. AUTHORITY DIRECTIVE — authority is never inferred from a substring. The careful batch (3b-2). | WIDER THAN LABELLED: not just how the gate reads an id — there are FOUR gates and no module vocabulary. Superseded by ENT-1..5.</t>
+          <t>A permission decision made by string comparison. AUTHORITY DIRECTIVE — authority is never inferred from a substring. The careful batch (3b-2). | WIDER THAN LABELLED: not just how the gate reads an id — there are FOUR gates and no module vocabulary. Superseded by ENT-1..5. Verified 2026-10-04: no prefix-match gate left; the create door gates by role through systemDatabaseEntitled().</t>
         </is>
       </c>
       <c r="H496" t="inlineStr">
@@ -23044,7 +23053,7 @@
       </c>
       <c r="E509" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F509" t="inlineStr">
@@ -23054,7 +23063,7 @@
       </c>
       <c r="G509" t="inlineStr">
         <is>
-          <t>Murgu (FREE, INVOICING only) has write access to projects, tasks, articles, crm, bobex, bestek, journal-general, hr. Not a decision anyone made — absence of a gate read as permission.</t>
+          <t>Murgu (FREE, INVOICING only) has write access to projects, tasks, articles, crm, bobex, bestek, journal-general, hr. Not a decision anyone made — absence of a gate read as permission. Fixed 2026-10-04 (47f7b62): one rule systemDatabaseEntitled() over SYSTEM_DATABASES.module, read by the create door and the reconcile; journal-general explicitly ungated.</t>
         </is>
       </c>
       <c r="H509" t="inlineStr">
@@ -23759,7 +23768,7 @@
       </c>
       <c r="G524" t="inlineStr">
         <is>
-          <t>Says FREE 50/mo, PRO 250, ENTERPRISE 1000. Live table PLAN_LIMITS says FREE 5 sent/10 recv, ENTERPRISE unlimited. Danger is plausibility: someone finds it first and 'fixes' the enforcing table. Delete one.</t>
+          <t>Says FREE 50/mo, PRO 250, ENTERPRISE 1000. Live table PLAN_LIMITS says FREE 5 sent/10 recv, ENTERPRISE unlimited. Danger is plausibility: someone finds it first and 'fixes' the enforcing table. Delete one. 2026-10-04: no longer zero readers — stripe.ts:200 reads it for the Peppol overage. Two Peppol tables still disagree; which survives is open in the feature matrix.</t>
         </is>
       </c>
       <c r="H524" t="inlineStr">
@@ -23979,7 +23988,7 @@
       </c>
       <c r="D529" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="E529" t="inlineStr">
@@ -23994,7 +24003,7 @@
       </c>
       <c r="G529" t="inlineStr">
         <is>
-          <t>trial.ts:40 startTrial calls syncPlanToTenant: a tenant trialling PRO BECOMES PRO, destroying their real tier. Replace with Tenant.trialGrant {tier, entitlements, expiresAt}. Expiry = overlay lapses, nothing downgraded.</t>
+          <t>trial.ts:40 startTrial calls syncPlanToTenant: a tenant trialling PRO BECOMES PRO, destroying their real tier. Replace with Tenant.trialGrant {tier, entitlements, expiresAt}. Expiry = overlay lapses, nothing downgraded. Demoted P0→P1 2026-10-04: trial mode is parked (TRIAL_MODE_ENABLED = false), so no tenant can hit it. Must be fixed BEFORE trials are switched back on.</t>
         </is>
       </c>
       <c r="H529" t="inlineStr">
@@ -24026,7 +24035,7 @@
       </c>
       <c r="D530" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="E530" t="inlineStr">
@@ -24041,7 +24050,7 @@
       </c>
       <c r="G530" t="inlineStr">
         <is>
-          <t>trial.ts:121-160. Nothing was owed and no payment failed. A lapsed trial must leave a working tenant on their own tier. Blocking a FREE tenant because they tried PRO is the bug this design prevents.</t>
+          <t>trial.ts:121-160. Nothing was owed and no payment failed. A lapsed trial must leave a working tenant on their own tier. Blocking a FREE tenant because they tried PRO is the bug this design prevents. Demoted P0→P1 2026-10-04: see TRIAL-1.</t>
         </is>
       </c>
       <c r="H530" t="inlineStr">
@@ -24120,7 +24129,7 @@
       </c>
       <c r="D532" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="E532" t="inlineStr">
@@ -24135,7 +24144,7 @@
       </c>
       <c r="G532" t="inlineStr">
         <is>
-          <t>Because planType is overwritten there is nothing to revert to. This case is the proof the overlay works. Florin 2026-09-26: a client may want to try the higher tier directly.</t>
+          <t>Because planType is overwritten there is nothing to revert to. This case is the proof the overlay works. Florin 2026-09-26: a client may want to try the higher tier directly. Demoted P0→P1 2026-10-04: see TRIAL-1.</t>
         </is>
       </c>
       <c r="H532" t="inlineStr">
@@ -24548,7 +24557,7 @@
       </c>
       <c r="E541" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F541" t="inlineStr">
@@ -24558,7 +24567,7 @@
       </c>
       <c r="G541" t="inlineStr">
         <is>
-          <t>src/lib/utils.ts does not exist. time-tracker/lib/utils.ts is 7 lines of cn(). The design system depends on the module we are deciding whether to delete. Fixing this removes 73% of the apparent coupling.</t>
+          <t>src/lib/utils.ts does not exist. time-tracker/lib/utils.ts is 7 lines of cn(). The design system depends on the module we are deciding whether to delete. Fixing this removes 73% of the apparent coupling. Verified 2026-10-04: src/lib/utils.ts exists; nothing imports time-tracker/lib/utils.</t>
         </is>
       </c>
       <c r="H541" t="inlineStr">
@@ -24924,7 +24933,7 @@
       </c>
       <c r="E549" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F549" t="inlineStr">
@@ -24934,7 +24943,7 @@
       </c>
       <c r="G549" t="inlineStr">
         <is>
-          <t>getAccessibleUserIds(tenantId, userId) NEVER USES tenantId. HrTeamMember has no tenantId (Class B via team), so neither query is tenant-constrained. Decorative tenancy in the function deciding who sees whose hours. Becomes scope.reach()/scope.reachableUserIds(), rides with R1-4.</t>
+          <t>getAccessibleUserIds(tenantId, userId) NEVER USES tenantId. HrTeamMember has no tenantId (Class B via team), so neither query is tenant-constrained. Decorative tenancy in the function deciding who sees whose hours. Becomes scope.reach()/scope.reachableUserIds(), rides with R1-4. Verified 2026-10-04: getAccessibleUserIds is tenant-constrained (team: {tenantId}); actor-reach.ts exists and gates the HR routes, write-policy, timesheet reports/export/rates.</t>
         </is>
       </c>
       <c r="H549" t="inlineStr">
@@ -26240,7 +26249,7 @@
       </c>
       <c r="E577" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F577" t="inlineStr">
@@ -26250,7 +26259,7 @@
       </c>
       <c r="G577" t="inlineStr">
         <is>
-          <t>documents+media verify the portal password server-side; messages+tasks+updates demand auth() an ERP session the client lacks; slug read checks nothing. So a client CAN upload a document and CANNOT post a message. portalScope collapses all three.</t>
+          <t>documents+media verify the portal password server-side; messages+tasks+updates demand auth() an ERP session the client lacks; slug read checks nothing. So a client CAN upload a document and CANNOT post a message. portalScope collapses all three. Verified 2026-10-04: every portal route goes through one verifyPortalAccess (lib/portal-auth).</t>
         </is>
       </c>
       <c r="H577" t="inlineStr">
@@ -26522,7 +26531,7 @@
       </c>
       <c r="E583" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F583" t="inlineStr">
@@ -26532,7 +26541,7 @@
       </c>
       <c r="G583" t="inlineStr">
         <is>
-          <t>global-databases.ts findMany returns logicalKey (no select) and the field-by-field mapper drops it. Add it to the client Database interface and EVERY mapper (at least 2 findMany sites). A missed mapper yields undefined, which reads as 'custom database' and is silently wrong. Verify all 16 roles present, none undefined, BEFORE converting anything.</t>
+          <t>global-databases.ts findMany returns logicalKey (no select) and the field-by-field mapper drops it. Add it to the client Database interface and EVERY mapper (at least 2 findMany sites). A missed mapper yields undefined, which reads as 'custom database' and is silently wrong. Verify all 16 roles present, none undefined, BEFORE converting anything. Verified 2026-10-04: logicalKey carried by the global-databases mappers.</t>
         </is>
       </c>
       <c r="H583" t="inlineStr">
@@ -26851,7 +26860,7 @@
       </c>
       <c r="E590" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F590" t="inlineStr">
@@ -26861,7 +26870,7 @@
       </c>
       <c r="G590" t="inlineStr">
         <is>
-          <t>EditShiftDialog:785 'Cannot find name fileInputRef' — an undefined variable in shipping code, a crash if that path runs. Plus a missing ProjectAttachment export. These are why the plan is urgent rather than tidy.</t>
+          <t>EditShiftDialog:785 'Cannot find name fileInputRef' — an undefined variable in shipping code, a crash if that path runs. Plus a missing ProjectAttachment export. These are why the plan is urgent rather than tidy. Verified 2026-10-04: fixed 2026-09-28 (6d55f14) — fileInputRef declared, ProjectAttachment exported.</t>
         </is>
       </c>
       <c r="H590" t="inlineStr">
@@ -26945,7 +26954,7 @@
       </c>
       <c r="E592" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F592" t="inlineStr">
@@ -26955,7 +26964,7 @@
       </c>
       <c r="G592" t="inlineStr">
         <is>
-          <t>THE CORE MOVE. Blanket silence makes readers unenumerable — that is INC-1. Line-level makes them greppable and countable WITHOUT converting one. The file becomes type-checked immediately; a new error fails the build. Order: fewest errors first. | SUPERSEDED AS A METRIC: the markers are gone (TD-4 converted those exact lines) and were never complete — local snake_case interfaces type-check and were never marked.</t>
+          <t>THE CORE MOVE. Blanket silence makes readers unenumerable — that is INC-1. Line-level makes them greppable and countable WITHOUT converting one. The file becomes type-checked immediately; a new error fails the build. Order: fewest errors first. | SUPERSEDED AS A METRIC: the markers are gone (TD-4 converted those exact lines) and were never complete — local snake_case interfaces type-check and were never marked. Verified 2026-10-04: @ts-nocheck only in 2 vendor ui files.</t>
         </is>
       </c>
       <c r="H592" t="inlineStr">

</xml_diff>

<commit_message>
docs(roadmap): no ad-hoc shifts (WH-13a/b done), SS-1 verified, superadmin reach by design + DEBUG-ROLE-1, calendar deferred
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/.agents/coral-roadmap.xlsx
+++ b/.agents/coral-roadmap.xlsx
@@ -594,7 +594,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I699"/>
+  <dimension ref="A1:I700"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -673,7 +673,7 @@
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -686,7 +686,11 @@
           <t>coral-calendar.md:64</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr"/>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Florin 2026-10-04: calendar needs a tree-shake review — it has fallen behind; not now unless it opens a security hole. Checked: events are read per user (userId), not cross-tenant; the browser cache (calendar-storage-v1) is not keyed by tenant — only matters on a shared browser / impersonation.</t>
+        </is>
+      </c>
       <c r="H2" s="22" t="inlineStr">
         <is>
           <t>L2</t>
@@ -16024,6 +16028,11 @@
           <t>pd.md AUTHORITY DIRECTIVE</t>
         </is>
       </c>
+      <c r="G348" t="inlineStr">
+        <is>
+          <t>Florin 2026-10-04: the SUPERADMIN MUST reach everything (no risk of being unable to debug a tenant) — the bypass is by design, NOT the defect. The defect is distribution: alternative = a gated DEBUG role (granted, time-boxed, audited — IMP-1/IMP-4) so superadmin is not handed out. The bypass itself must live in ONE place (ENT-4/ENT-9).</t>
+        </is>
+      </c>
       <c r="H348" s="28" t="inlineStr">
         <is>
           <t>GATE</t>
@@ -25309,7 +25318,7 @@
       </c>
       <c r="E557" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F557" t="inlineStr">
@@ -25319,7 +25328,7 @@
       </c>
       <c r="G557" t="inlineStr">
         <is>
-          <t>useScheduledShifts.ts:214. Hours attach to a shift attached to no job — 'mid air' by construction. The end time is invented regardless of reality.</t>
+          <t>useScheduledShifts.ts:214. Hours attach to a shift attached to no job — 'mid air' by construction. The end time is invented regardless of reality. Fixed 2026-10-04 (f32518b5): NO ad-hoc shifts (Florin) — the clock button no longer invents a shift; a clock-in without a planned shift is recorded as such, pending approval, note required at clock-out; the admin plans a shift in the past to match. Selecting an existing shift unchanged.</t>
         </is>
       </c>
       <c r="H557" t="inlineStr">
@@ -25356,7 +25365,7 @@
       </c>
       <c r="E558" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F558" t="inlineStr">
@@ -25366,7 +25375,7 @@
       </c>
       <c r="G558" t="inlineStr">
         <is>
-          <t>ClockButton:117-122. If the PATCH fails (dead network — the exact condition) the entry is saved unlinked. Likely source of some of the 11 orphans alongside late entry. Must be ONE atomic intent (WH-11).</t>
+          <t>ClockButton:117-122. If the PATCH fails (dead network — the exact condition) the entry is saved unlinked. Likely source of some of the 11 orphans alongside late entry. Must be ONE atomic intent (WH-11). Fixed 2026-10-04 (f32518b5): the separate link PATCH is gone with the ad-hoc shift — a clock-in carries its shiftId in the one create, or none.</t>
         </is>
       </c>
       <c r="H558" t="inlineStr">
@@ -27424,7 +27433,7 @@
       </c>
       <c r="E602" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F602" t="inlineStr">
@@ -27434,7 +27443,7 @@
       </c>
       <c r="G602" t="inlineStr">
         <is>
-          <t>Defaults usePortal=true and falls back to document.body, so ANY SearchableSelect inside ANY Radix dialog is unclickable — the focus trap eats the clicks. Fix at the component: closest('[role=dialog]') ?? body. All 56 callers correct by construction. RISK: position:fixed inside a transformed ancestor — verify placement, not just that it opens.</t>
+          <t>Defaults usePortal=true and falls back to document.body, so ANY SearchableSelect inside ANY Radix dialog is unclickable — the focus trap eats the clicks. Fix at the component: closest('[role=dialog]') ?? body. All 56 callers correct by construction. RISK: position:fixed inside a transformed ancestor — verify placement, not just that it opens. Verified 2026-10-04: SearchableSelect portals into closest([role=dialog]) — SearchableSelect.tsx:248.</t>
         </is>
       </c>
       <c r="H602" t="inlineStr">
@@ -31963,6 +31972,53 @@
       <c r="I699" t="inlineStr">
         <is>
           <t>document engine (+ archive, attachments)</t>
+        </is>
+      </c>
+    </row>
+    <row r="700">
+      <c r="A700" t="inlineStr">
+        <is>
+          <t>DEBUG-ROLE-1</t>
+        </is>
+      </c>
+      <c r="B700" t="inlineStr">
+        <is>
+          <t>A gated DEBUG role: reaches a tenant fully for debugging, granted per person (not by handing out SUPERADMIN), time-boxed, every action audited.</t>
+        </is>
+      </c>
+      <c r="C700" t="inlineStr">
+        <is>
+          <t>Platform</t>
+        </is>
+      </c>
+      <c r="D700" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E700" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F700" t="inlineStr">
+        <is>
+          <t>Florin 2026-10-04</t>
+        </is>
+      </c>
+      <c r="G700" t="inlineStr">
+        <is>
+          <t>Alternative to distributing SUPERADMIN. Builds on IMP-1 (grant lifecycle) and IMP-4 (operator log). The bypass lives once in requireModule() (ENT-4).</t>
+        </is>
+      </c>
+      <c r="H700" t="inlineStr">
+        <is>
+          <t>GATE</t>
+        </is>
+      </c>
+      <c r="I700" t="inlineStr">
+        <is>
+          <t>actor reach · platform access · operator scopes</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(roadmap): R1-2 + KERN-8 shipped (census clean), KERN-5 family closed, WO-4a-M4 done, SCHED-SYNC-1
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/.agents/coral-roadmap.xlsx
+++ b/.agents/coral-roadmap.xlsx
@@ -594,7 +594,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I700"/>
+  <dimension ref="A1:I701"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -10390,7 +10390,7 @@
       </c>
       <c r="E226" s="11" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F226" s="11" t="inlineStr">
@@ -10400,7 +10400,7 @@
       </c>
       <c r="G226" s="11" t="inlineStr">
         <is>
-          <t>[P3.3] Was: denormalise tenantId column — WITHDRAWN | Planner 2026-10-01: resolveDatabaseId fail-closed in the kernel, all 11 callers converted — branch track-b/r1-2-kern-8. GATED on .agents/workflows/r1-2-binding-census.sql (Florin) Florin 2026-10-03: the Planner leads the binding census. 2026-10-04: branch merged with develop (clean; no new getLockedDbId users). Design change after ENT-FREE: TWO reads — resolveDatabaseId THROWS (writes), lookupDatabaseId returns null = ABSENT (screens, read paths; FREE has no library/projects/CRM). tsc lists 207 sites in 28 files to handle absence. Must-fix on the branch: Peppol inbox must never throw on a missing binding (never block receive); dashboard reads CRM roles. Census SQL for Florin: .agents/workflows/sql/r1-2-binding-census.sql.</t>
+          <t>[P3.3] Was: denormalise tenantId column — WITHDRAWN | Planner 2026-10-01: resolveDatabaseId fail-closed in the kernel, all 11 callers converted — branch track-b/r1-2-kern-8. GATED on .agents/workflows/r1-2-binding-census.sql (Florin) Florin 2026-10-03: the Planner leads the binding census. 2026-10-04: branch merged with develop (clean; no new getLockedDbId users). Design change after ENT-FREE: TWO reads — resolveDatabaseId THROWS (writes), lookupDatabaseId returns null = ABSENT (screens, read paths; FREE has no library/projects/CRM). tsc lists 207 sites in 28 files to handle absence. Must-fix on the branch: Peppol inbox must never throw on a missing binding (never block receive); dashboard reads CRM roles. Census SQL for Florin: .agents/workflows/sql/r1-2-binding-census.sql. Shipped 2026-10-04 (4e04edf4): one resolver, fail-closed, no guessing. Census (Florin, 2026-10-04): 32/32 bindings OK on both tenants, so nothing throws today. The "absent" lookup for screens was dropped — needed only when ENT-FREE-1 stops provisioning. Peppol inbox can never be stopped by a missing binding.</t>
         </is>
       </c>
       <c r="H226" s="28" t="inlineStr">
@@ -21558,7 +21558,7 @@
       </c>
       <c r="E477" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F477" t="inlineStr">
@@ -21568,7 +21568,7 @@
       </c>
       <c r="G477" t="inlineStr">
         <is>
-          <t>Ids are &lt;base&gt;-&lt;tenantSuffix&gt;; tenancy recovered via split('-'). Breaches IDENTITY DIRECTIVE. Delete the function, do not fix it — 4 fallback branches = it does not know the answer.</t>
+          <t>Ids are &lt;base&gt;-&lt;tenantSuffix&gt;; tenancy recovered via split('-'). Breaches IDENTITY DIRECTIVE. Delete the function, do not fix it — 4 fallback branches = it does not know the answer. Done 2026-10-04: getLockedDbId deleted (R1-2).</t>
         </is>
       </c>
       <c r="H477" t="inlineStr">
@@ -21605,7 +21605,7 @@
       </c>
       <c r="E478" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F478" t="inlineStr">
@@ -21615,7 +21615,7 @@
       </c>
       <c r="G478" t="inlineStr">
         <is>
-          <t>Imported by TenantContext.tsx and four m/* pages. Same defect as KERN-3, fixed for creation, missed for resolution.</t>
+          <t>Imported by TenantContext.tsx and four m/* pages. Same defect as KERN-3, fixed for creation, missed for resolution. Done 2026-10-04: lockedDbUtils deleted; the browser reads the binding, computes nothing.</t>
         </is>
       </c>
       <c r="H478" t="inlineStr">
@@ -21652,7 +21652,7 @@
       </c>
       <c r="E479" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F479" t="inlineStr">
@@ -21662,7 +21662,7 @@
       </c>
       <c r="G479" t="inlineStr">
         <is>
-          <t>The resolver's last answer works for the founder and points at a foreign/nonexistent db for everyone else. Sample size of one, shipped, in a comment.</t>
+          <t>The resolver's last answer works for the founder and points at a foreign/nonexistent db for everyone else. Sample size of one, shipped, in a comment. Done 2026-10-04: the founder fallback died with getLockedDbId.</t>
         </is>
       </c>
       <c r="H479" t="inlineStr">
@@ -21793,7 +21793,7 @@
       </c>
       <c r="E482" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F482" t="inlineStr">
@@ -21803,7 +21803,7 @@
       </c>
       <c r="G482" t="inlineStr">
         <is>
-          <t>Missing: articles, bestek, bobex, crm, hr, journal-general, payments-in, payments-out, projects, tasks. getLockedDbId synthesises db-1-cmoa44mj etc., which do not exist -&gt; ten modules silently empty. Broken, NOT leaking (server paths carry database:{tenantId}). The zombie rule, observed in production.</t>
+          <t>Missing: articles, bestek, bobex, crm, hr, journal-general, payments-in, payments-out, projects, tasks. getLockedDbId synthesises db-1-cmoa44mj etc., which do not exist -&gt; ten modules silently empty. Broken, NOT leaking (server paths carry database:{tenantId}). The zombie rule, observed in production. Done 2026-10-04: census — Murgu now has all 16 bindings, each its own database.</t>
         </is>
       </c>
       <c r="H482" t="inlineStr">
@@ -22122,7 +22122,7 @@
       </c>
       <c r="E489" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F489" t="inlineStr">
@@ -22132,7 +22132,7 @@
       </c>
       <c r="G489" t="inlineStr">
         <is>
-          <t>Precondition for deleting getLockedDbId. Without it the refusal is loud instead of correct.</t>
+          <t>Precondition for deleting getLockedDbId. Without it the refusal is loud instead of correct. Done 2026-10-04: census — both tenants fully bound; no backfill needed.</t>
         </is>
       </c>
       <c r="H489" t="inlineStr">
@@ -22545,7 +22545,7 @@
       </c>
       <c r="E498" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F498" t="inlineStr">
@@ -22555,7 +22555,7 @@
       </c>
       <c r="G498" t="inlineStr">
         <is>
-          <t>Only when 3b's allowlist reaches zero. Gated on the R1-1b relation-target measurement. | Planner 2026-10-01: getLockedDbId + lockedDbUtils deleted, resolve.ts prefix searches deleted — on branch track-b/r1-2-kern-8 (b7e5853); ships with R1-2</t>
+          <t>Only when 3b's allowlist reaches zero. Gated on the R1-1b relation-target measurement. | Planner 2026-10-01: getLockedDbId + lockedDbUtils deleted, resolve.ts prefix searches deleted — on branch track-b/r1-2-kern-8 (b7e5853); ships with R1-2 Shipped 2026-10-04 with R1-2: getLockedDbId + lockedDbUtils + resolve.ts prefix searches deleted.</t>
         </is>
       </c>
       <c r="H498" t="inlineStr">
@@ -31224,7 +31224,7 @@
       </c>
       <c r="G683" t="inlineStr">
         <is>
-          <t>Provisioning creates 16 for everyone today</t>
+          <t>Provisioning creates 16 for everyone today 2026-10-04: when provisioning stops creating FREE databases, screens must handle an ABSENT database (a lookup returning null; tsc counted 207 sites in 28 files) — that work belongs here, not in R1-2.</t>
         </is>
       </c>
       <c r="H683" t="inlineStr">
@@ -31951,7 +31951,7 @@
       </c>
       <c r="E699" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F699" t="inlineStr">
@@ -31961,7 +31961,7 @@
       </c>
       <c r="G699" t="inlineStr">
         <is>
-          <t>Required before WO-4b wires the renderer into signing; today the renderer is imported nowhere (inert).</t>
+          <t>Required before WO-4b wires the renderer into signing; today the renderer is imported nowhere (inert). Done 2026-10-04 (8bb1db1e): no global patches; the test watches Math.random while renders run (throw proof re-run by the Planner).</t>
         </is>
       </c>
       <c r="H699" t="inlineStr">
@@ -32019,6 +32019,53 @@
       <c r="I700" t="inlineStr">
         <is>
           <t>actor reach · platform access · operator scopes</t>
+        </is>
+      </c>
+    </row>
+    <row r="701">
+      <c r="A701" t="inlineStr">
+        <is>
+          <t>SCHED-SYNC-1</t>
+        </is>
+      </c>
+      <c r="B701" t="inlineStr">
+        <is>
+          <t>Scheduler: an edited or deleted shift showed its old state until a page refresh (third report).</t>
+        </is>
+      </c>
+      <c r="C701" t="inlineStr">
+        <is>
+          <t>WorkHub</t>
+        </is>
+      </c>
+      <c r="D701" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E701" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F701" t="inlineStr">
+        <is>
+          <t>Florin 2026-10-04</t>
+        </is>
+      </c>
+      <c r="G701" t="inlineStr">
+        <is>
+          <t>Fixed 2026-10-04 (1adb221b): quiet reload after every change, one at a time, re-run once if a change lands meanwhile. Root cause not found by reading — symptom closed for every path.</t>
+        </is>
+      </c>
+      <c r="H701" t="inlineStr">
+        <is>
+          <t>L3</t>
+        </is>
+      </c>
+      <c r="I701" t="inlineStr">
+        <is>
+          <t>HR — scheduling</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: R2-1-CENSUS reviewed and accepted — 4 holes fixed, table corrections, dead code logged
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/.agents/coral-roadmap.xlsx
+++ b/.agents/coral-roadmap.xlsx
@@ -594,7 +594,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I701"/>
+  <dimension ref="A1:I702"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -31434,7 +31434,7 @@
       </c>
       <c r="E688" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F688" t="inlineStr">
@@ -31444,7 +31444,7 @@
       </c>
       <c r="G688" t="inlineStr">
         <is>
-          <t>Queued</t>
+          <t>Queued Done 2026-10-04: 36 writes / 19 files; 21 NONE tenant checks, 32 no OCC, 32 no audit. Reviewed: 4 real holes fixed same day (accept actions any-id, Stripe link + re-scan cross-tenant, portal tasks into BV Coral db) — 9bf19a44 · e48834a6 · a2ffa1d5. Report: .agents/reports/R2-1-CENSUS.md.</t>
         </is>
       </c>
       <c r="H688" t="inlineStr">
@@ -32066,6 +32066,53 @@
       <c r="I701" t="inlineStr">
         <is>
           <t>HR — scheduling</t>
+        </is>
+      </c>
+    </row>
+    <row r="702">
+      <c r="A702" t="inlineStr">
+        <is>
+          <t>DEAD-PAYPLAN-1</t>
+        </is>
+      </c>
+      <c r="B702" t="inlineStr">
+        <is>
+          <t>Delete updatePaymentPlanAction (lib/services/payment-plan-service.ts): no callers, unauthenticated write by page id if ever wired.</t>
+        </is>
+      </c>
+      <c r="C702" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="D702" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="E702" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F702" t="inlineStr">
+        <is>
+          <t>R2-1-CENSUS #36</t>
+        </is>
+      </c>
+      <c r="G702" t="inlineStr">
+        <is>
+          <t>Dead code found by the census — delete, do not fix.</t>
+        </is>
+      </c>
+      <c r="H702" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="I702" t="inlineStr">
+        <is>
+          <t>write path — saveRecord, intents, read model</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(roadmap): PAY-1, PAY-2, PORTAL-LINK-1 done; R1-5 first adopters; portalScope built
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/.agents/coral-roadmap.xlsx
+++ b/.agents/coral-roadmap.xlsx
@@ -594,7 +594,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I702"/>
+  <dimension ref="A1:I705"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -10541,7 +10541,7 @@
       </c>
       <c r="G229" s="11" t="inlineStr">
         <is>
-          <t>[P3.5] Revised after Florin review 2026-09-12 | Planner 2026-10-01: next: adopt scopeFromSession file by file; direct prisma outside lib/data → CI failure. Florin decides the rollout</t>
+          <t>[P3.5] Revised after Florin review 2026-09-12 | Planner 2026-10-01: next: adopt scopeFromSession file by file; direct prisma outside lib/data → CI failure. Florin decides the rollout 2026-10-04: first adopters of the scoped client — Stripe checkout + webhook, scan re-scan, portal tasks/page/create, payment matching, overdue cron, accept-by-link, quote→project; portalScope (PT-5) built.</t>
         </is>
       </c>
       <c r="H229" s="28" t="inlineStr">
@@ -26221,7 +26221,7 @@
       </c>
       <c r="G576" t="inlineStr">
         <is>
-          <t>Beside scopeFromSession and systemScope (TSC-0 D3/D5). Carries tenant AND side. No new principal type — what flows downstream is the identical TenantScopedClient. Rejected: a restricted User row (seats, db-hr projection, team pickers, 'a user who is not a user'). | CONFIRMED by Florin 2026-09-27: 'no new user then.'</t>
+          <t>Beside scopeFromSession and systemScope (TSC-0 D3/D5). Carries tenant AND side. No new principal type — what flows downstream is the identical TenantScopedClient. Rejected: a restricted User row (seats, db-hr projection, team pickers, 'a user who is not a user'). | CONFIRMED by Florin 2026-09-27: 'no new user then.' Built 2026-10-04: portalScope(verifiedAccess) in lib/data/scope.ts — opens only on a verified portal access; tested (throw proof).</t>
         </is>
       </c>
       <c r="H576" t="inlineStr">
@@ -32092,7 +32092,7 @@
       </c>
       <c r="E702" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F702" t="inlineStr">
@@ -32102,7 +32102,7 @@
       </c>
       <c r="G702" t="inlineStr">
         <is>
-          <t>Dead code found by the census — delete, do not fix.</t>
+          <t>Dead code found by the census — delete, do not fix. Deleted 2026-10-04.</t>
         </is>
       </c>
       <c r="H702" t="inlineStr">
@@ -32113,6 +32113,147 @@
       <c r="I702" t="inlineStr">
         <is>
           <t>write path — saveRecord, intents, read model</t>
+        </is>
+      </c>
+    </row>
+    <row r="703">
+      <c r="A703" t="inlineStr">
+        <is>
+          <t>PAY-1</t>
+        </is>
+      </c>
+      <c r="B703" t="inlineStr">
+        <is>
+          <t>ONE rule for invoice / expense payment status (lib/records/invoice-payment-status.ts) and ONE door (lib/data/invoice-payments.ts) on the scoped client — Stripe, bank-payment matching and the overdue cron all use it.</t>
+        </is>
+      </c>
+      <c r="C703" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="D703" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E703" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F703" t="inlineStr">
+        <is>
+          <t>Florin 2026-10-04</t>
+        </is>
+      </c>
+      <c r="G703" t="inlineStr">
+        <is>
+          <t>Done 2026-10-04 (7872a622). Semantics kept: covered by payments → paid; sent + past due (Brussels date) → overdue; paid / credited / uncollectible set by a person are never undone. A Stripe payment is now a payments-in row (idempotent on the session id). Fixed: matching could set ANY tenant's invoice paid; cron found databases by id prefix, UTC date.</t>
+        </is>
+      </c>
+      <c r="H703" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="I703" t="inlineStr">
+        <is>
+          <t>write path — saveRecord, intents, read model</t>
+        </is>
+      </c>
+    </row>
+    <row r="704">
+      <c r="A704" t="inlineStr">
+        <is>
+          <t>PAY-2</t>
+        </is>
+      </c>
+      <c r="B704" t="inlineStr">
+        <is>
+          <t>Stripe: a checkout confirmed by a TENANT's own Stripe account may only record a payment on that tenant's own invoice (lib/records/stripe-tenant-payment.ts).</t>
+        </is>
+      </c>
+      <c r="C704" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="D704" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E704" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F704" t="inlineStr">
+        <is>
+          <t>Florin 2026-10-04</t>
+        </is>
+      </c>
+      <c r="G704" t="inlineStr">
+        <is>
+          <t>Done 2026-10-04 (7872a622). Holes closed: the fallback path let a tenant mark ANOTHER tenant's invoice paid with any amount, and fell through to the platform handler — a tenant paying itself a few cents could provision ENTERPRISE. Plans/seats now react to platform-signed events only.</t>
+        </is>
+      </c>
+      <c r="H704" t="inlineStr">
+        <is>
+          <t>GATE</t>
+        </is>
+      </c>
+      <c r="I704" t="inlineStr">
+        <is>
+          <t>the seraph — resolver, logicalKey, scoped accessor</t>
+        </is>
+      </c>
+    </row>
+    <row r="705">
+      <c r="A705" t="inlineStr">
+        <is>
+          <t>PORTAL-LINK-1</t>
+        </is>
+      </c>
+      <c r="B705" t="inlineStr">
+        <is>
+          <t>Client portal: the linked project (and its quotes / invoices) read by id alone — a tenant could link and show another tenant's project.</t>
+        </is>
+      </c>
+      <c r="C705" t="inlineStr">
+        <is>
+          <t>Platform</t>
+        </is>
+      </c>
+      <c r="D705" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E705" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F705" t="inlineStr">
+        <is>
+          <t>Florin 2026-10-04</t>
+        </is>
+      </c>
+      <c r="G705" t="inlineStr">
+        <is>
+          <t>Done 2026-10-04 (2c2f3195): portal page reads through portalScope by role; create/edit accept only an own project; database = binding.</t>
+        </is>
+      </c>
+      <c r="H705" t="inlineStr">
+        <is>
+          <t>GATE</t>
+        </is>
+      </c>
+      <c r="I705" t="inlineStr">
+        <is>
+          <t>the seraph — resolver, logicalKey, scoped accessor</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(roadmap): tenant card payments dropped; LIC-1 done; STRIPE-COLS-1 queued
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/.agents/coral-roadmap.xlsx
+++ b/.agents/coral-roadmap.xlsx
@@ -594,7 +594,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I705"/>
+  <dimension ref="A1:I707"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -32149,7 +32149,7 @@
       </c>
       <c r="G703" t="inlineStr">
         <is>
-          <t>Done 2026-10-04 (7872a622). Semantics kept: covered by payments → paid; sent + past due (Brussels date) → overdue; paid / credited / uncollectible set by a person are never undone. A Stripe payment is now a payments-in row (idempotent on the session id). Fixed: matching could set ANY tenant's invoice paid; cron found databases by id prefix, UTC date.</t>
+          <t>Done 2026-10-04 (7872a622). Semantics kept: covered by payments → paid; sent + past due (Brussels date) → overdue; paid / credited / uncollectible set by a person are never undone. A Stripe payment is now a payments-in row (idempotent on the session id). Fixed: matching could set ANY tenant's invoice paid; cron found databases by id prefix, UTC date. 2026-10-04: tenants' clients pay by bank transfer only — PAY-1 serves bank-payment matching and the overdue cron.</t>
         </is>
       </c>
       <c r="H703" t="inlineStr">
@@ -32186,7 +32186,7 @@
       </c>
       <c r="E704" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Dropped</t>
         </is>
       </c>
       <c r="F704" t="inlineStr">
@@ -32196,7 +32196,7 @@
       </c>
       <c r="G704" t="inlineStr">
         <is>
-          <t>Done 2026-10-04 (7872a622). Holes closed: the fallback path let a tenant mark ANOTHER tenant's invoice paid with any amount, and fell through to the platform handler — a tenant paying itself a few cents could provision ENTERPRISE. Plans/seats now react to platform-signed events only.</t>
+          <t>Done 2026-10-04 (7872a622). Holes closed: the fallback path let a tenant mark ANOTHER tenant's invoice paid with any amount, and fell through to the platform handler — a tenant paying itself a few cents could provision ENTERPRISE. Plans/seats now react to platform-signed events only. Superseded 2026-10-04 (1400fee0): Florin — "we do not handle payments for the tenants; Stripe is ONLY our license fee." Tenant card payments removed entirely; the webhook accepts platform-signed events only.</t>
         </is>
       </c>
       <c r="H704" t="inlineStr">
@@ -32254,6 +32254,100 @@
       <c r="I705" t="inlineStr">
         <is>
           <t>the seraph — resolver, logicalKey, scoped accessor</t>
+        </is>
+      </c>
+    </row>
+    <row r="706">
+      <c r="A706" t="inlineStr">
+        <is>
+          <t>LIC-1</t>
+        </is>
+      </c>
+      <c r="B706" t="inlineStr">
+        <is>
+          <t>License fee (Stripe, platform only): the right tenant, the right plan, the current subscription, in any event order; the plan template applies only on a plan change.</t>
+        </is>
+      </c>
+      <c r="C706" t="inlineStr">
+        <is>
+          <t>Platform</t>
+        </is>
+      </c>
+      <c r="D706" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E706" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F706" t="inlineStr">
+        <is>
+          <t>Florin 2026-10-04</t>
+        </is>
+      </c>
+      <c r="G706" t="inlineStr">
+        <is>
+          <t>Done 2026-10-04 (07059eee). Fixed: unknown price → PRO default; metadata over price; old subscription's delete dropped an active tenant to FREE; out-of-order events; every renewal wiped manual module grants; tenant from metadata only. Rules: lib/records/license-subscription.ts (tested).</t>
+        </is>
+      </c>
+      <c r="H706" t="inlineStr">
+        <is>
+          <t>MODULE GATE</t>
+        </is>
+      </c>
+      <c r="I706" t="inlineStr">
+        <is>
+          <t>entitlement — vocabulary &amp; grants (modules → submodules → quota)</t>
+        </is>
+      </c>
+    </row>
+    <row r="707">
+      <c r="A707" t="inlineStr">
+        <is>
+          <t>STRIPE-COLS-1</t>
+        </is>
+      </c>
+      <c r="B707" t="inlineStr">
+        <is>
+          <t>Drop Tenant.paymentProvider / stripeSecretKey / stripePublishableKey (tenant card payments removed — code first, then this migration).</t>
+        </is>
+      </c>
+      <c r="C707" t="inlineStr">
+        <is>
+          <t>Platform</t>
+        </is>
+      </c>
+      <c r="D707" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="E707" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F707" t="inlineStr">
+        <is>
+          <t>Florin 2026-10-04</t>
+        </is>
+      </c>
+      <c r="G707" t="inlineStr">
+        <is>
+          <t>Destructive: after 1400fee0 is live. Check first that no code reads them (grep), then a migration Florin runs.</t>
+        </is>
+      </c>
+      <c r="H707" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="I707" t="inlineStr">
+        <is>
+          <t>ERP core — mixed triage</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(wo-4b): plan + Florin's decisions — WB number at signing, client language, Timesheets queue, manual send; END-CLIENT-1
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/.agents/coral-roadmap.xlsx
+++ b/.agents/coral-roadmap.xlsx
@@ -594,7 +594,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I707"/>
+  <dimension ref="A1:I708"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -30482,7 +30482,7 @@
       </c>
       <c r="E667" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="F667" t="inlineStr">
@@ -30492,7 +30492,7 @@
       </c>
       <c r="G667" t="inlineStr">
         <is>
-          <t>Planner. Prints shift description + crew notes (Florin 2026-10-02) Florin 2026-10-03: sending is NOT automatic — the signed PDF passes admin review first (like hours approval), then is sent. Migration via the usual SOP. PDF file name (Florin 2026-10-03): localised "Werkbon" + work order nr + date (nl Werkbon / fr Bon de travail / en Work order).</t>
+          <t>Planner. Prints shift description + crew notes (Florin 2026-10-02) Florin 2026-10-03: sending is NOT automatic — the signed PDF passes admin review first (like hours approval), then is sent. Migration via the usual SOP. PDF file name (Florin 2026-10-03): localised "Werkbon" + work order nr + date (nl Werkbon / fr Bon de travail / en Work order). Florin 2026-10-04: number WB-YYYY-NNNN at signing; PDF in the order giver's language; queue = Timesheets tab "Werkbonnen"; sending is a SEPARATE MANUAL act (never on approval), to the order giver (shift client → project client → typed) + copy to tenant. Plan: .agents/plans/WO-4b.md.</t>
         </is>
       </c>
       <c r="H667" t="inlineStr">
@@ -32346,6 +32346,53 @@
         </is>
       </c>
       <c r="I707" t="inlineStr">
+        <is>
+          <t>ERP core — mixed triage</t>
+        </is>
+      </c>
+    </row>
+    <row r="708">
+      <c r="A708" t="inlineStr">
+        <is>
+          <t>END-CLIENT-1</t>
+        </is>
+      </c>
+      <c r="B708" t="inlineStr">
+        <is>
+          <t>END CLIENT vs ORDER GIVER: our client may be a main contractor; documents go to the order giver, who presents them to their own client (end client) — we have no say over their rates and terms.</t>
+        </is>
+      </c>
+      <c r="C708" t="inlineStr">
+        <is>
+          <t>CRM</t>
+        </is>
+      </c>
+      <c r="D708" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E708" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F708" t="inlineStr">
+        <is>
+          <t>Florin 2026-10-04</t>
+        </is>
+      </c>
+      <c r="G708" t="inlineStr">
+        <is>
+          <t>Surfaced by WO-4b. Model both on shifts / projects (order giver = who pays us; end client = whose site it is) without merging them (pd.md 4z: each concept defined, then frozen).</t>
+        </is>
+      </c>
+      <c r="H708" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="I708" t="inlineStr">
         <is>
           <t>ERP core — mixed triage</t>
         </is>

</xml_diff>

<commit_message>
roadmap: COMMS-1 (crew + client comms platform — WhatsApp or other, undecided), COMMENTS-1, DB-DEF-1, DB-HEADER-1
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/.agents/coral-roadmap.xlsx
+++ b/.agents/coral-roadmap.xlsx
@@ -594,7 +594,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I708"/>
+  <dimension ref="A1:I712"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -32395,6 +32395,194 @@
       <c r="I708" t="inlineStr">
         <is>
           <t>ERP core — mixed triage</t>
+        </is>
+      </c>
+    </row>
+    <row r="709">
+      <c r="A709" t="inlineStr">
+        <is>
+          <t>COMMS-1</t>
+        </is>
+      </c>
+      <c r="B709" t="inlineStr">
+        <is>
+          <t>Communication with the CREW and with CLIENTS — a comms platform (WhatsApp integration or another channel). Comments (COMMENTS-1) stay internal: the crew in WorkHub and the client portals never see them, and the crew cannot be @mentioned.</t>
+        </is>
+      </c>
+      <c r="C709" t="inlineStr">
+        <is>
+          <t>Platform · Communication</t>
+        </is>
+      </c>
+      <c r="D709" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="E709" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F709" t="inlineStr">
+        <is>
+          <t>Florin 2026-10-05</t>
+        </is>
+      </c>
+      <c r="G709" t="inlineStr">
+        <is>
+          <t>Nothing decided yet — channel, provider, two-way or notify-only, cost per message, consent/GDPR (client numbers), where threads live (CoralOS vs the channel). To be looked into; do not build before Florin decides. Related: NOTIF-4…8 (transports of the same notify service), PORTAL-* (client side).</t>
+        </is>
+      </c>
+      <c r="H709" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="I709" t="inlineStr">
+        <is>
+          <t>platform services — notifications</t>
+        </is>
+      </c>
+    </row>
+    <row r="710">
+      <c r="A710" t="inlineStr">
+        <is>
+          <t>COMMENTS-1</t>
+        </is>
+      </c>
+      <c r="B710" t="inlineStr">
+        <is>
+          <t>A thread on every record (ClickUp-like) + the universal "Opmerkingen" field (latest comment, count, open count) — part of every database schema, shown per view.</t>
+        </is>
+      </c>
+      <c r="C710" t="inlineStr">
+        <is>
+          <t>Platform</t>
+        </is>
+      </c>
+      <c r="D710" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E710" t="inlineStr">
+        <is>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="F710" t="inlineStr">
+        <is>
+          <t>Florin 2026-10-05</t>
+        </is>
+      </c>
+      <c r="G710" t="inlineStr">
+        <is>
+          <t>Built 2026-10-05: migration ab608857 (additive, Comment table) + code f0b66940. Internal only (office). WAITING ON FLORIN: prisma migrate deploy, then push f0b66940 to main. Grid cell read-only until GRID-REPLACE.</t>
+        </is>
+      </c>
+      <c r="H710" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="I710" t="inlineStr">
+        <is>
+          <t>ERP core — mixed triage</t>
+        </is>
+      </c>
+    </row>
+    <row r="711">
+      <c r="A711" t="inlineStr">
+        <is>
+          <t>DB-DEF-1</t>
+        </is>
+      </c>
+      <c r="B711" t="inlineStr">
+        <is>
+          <t>A database definition (fields, views, name) changes by operations on the server, never by writing the whole definition back — schema edits stick. Decision A: the schema decides which fields exist, each view decides order and visibility.</t>
+        </is>
+      </c>
+      <c r="C711" t="inlineStr">
+        <is>
+          <t>Platform</t>
+        </is>
+      </c>
+      <c r="D711" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E711" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F711" t="inlineStr">
+        <is>
+          <t>Florin 2026-10-05</t>
+        </is>
+      </c>
+      <c r="G711" t="inlineStr">
+        <is>
+          <t>Live 2026-10-05 (c114bcf4). Step 1 of the grid replacement plan. 18 store actions sent the whole definition; a stale screen undid newer edits silently.</t>
+        </is>
+      </c>
+      <c r="H711" t="inlineStr">
+        <is>
+          <t>L0</t>
+        </is>
+      </c>
+      <c r="I711" t="inlineStr">
+        <is>
+          <t>write path — one door</t>
+        </is>
+      </c>
+    </row>
+    <row r="712">
+      <c r="A712" t="inlineStr">
+        <is>
+          <t>DB-HEADER-1</t>
+        </is>
+      </c>
+      <c r="B712" t="inlineStr">
+        <is>
+          <t>One database header across the ERP: one pure rule (role · screen · user role · plan) + one component for the 19 database screens.</t>
+        </is>
+      </c>
+      <c r="C712" t="inlineStr">
+        <is>
+          <t>Platform</t>
+        </is>
+      </c>
+      <c r="D712" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E712" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F712" t="inlineStr">
+        <is>
+          <t>Florin 2026-10-05</t>
+        </is>
+      </c>
+      <c r="G712" t="inlineStr">
+        <is>
+          <t>Coder: plan first (coder-directive-db-header-1.md), after R1-7-B1.</t>
+        </is>
+      </c>
+      <c r="H712" t="inlineStr">
+        <is>
+          <t>L4</t>
+        </is>
+      </c>
+      <c r="I712" t="inlineStr">
+        <is>
+          <t>design system</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(queue): R2-1-B plan request; roadmap R2-1 / R2-2 progress
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/.agents/coral-roadmap.xlsx
+++ b/.agents/coral-roadmap.xlsx
@@ -594,7 +594,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I712"/>
+  <dimension ref="A1:I713"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -10672,7 +10672,7 @@
       </c>
       <c r="E232" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="F232" s="11" t="inlineStr">
@@ -10682,7 +10682,7 @@
       </c>
       <c r="G232" s="11" t="inlineStr">
         <is>
-          <t>[P4.2] · R2-1-CENSUS queued for the coder (33 direct GlobalPage writes, 18 files).</t>
+          <t>[P4.2] · R2-1-CENSUS queued for the coder (33 direct GlobalPage writes, 18 files). | 2026-10-05: the ONE door is live — rule lib/records/record-intent.ts, door lib/data/records.ts saveRecord/deleteRecord (scoped, serializable, persisted state); adapters: saveGlobalPage, saveGlobalPagesBatch, deleteGlobalPage, createPageServerFirst, updatePageServerFirst (9338598a, 6b38dc93, dfdf1ddb). Remaining direct writes → coder R2-1-B.</t>
         </is>
       </c>
       <c r="H232" s="23" t="inlineStr">
@@ -10719,7 +10719,7 @@
       </c>
       <c r="E233" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="F233" s="11" t="inlineStr">
@@ -10729,7 +10729,7 @@
       </c>
       <c r="G233" s="11" t="inlineStr">
         <is>
-          <t>[P4.3]</t>
+          <t>[P4.3] | 2026-10-05: server side done — a save is an intent for the CHANGED fields (intentFromPage); different fields from one old version both land. The grid side (no whole-row diff) is GRID-REPLACE.</t>
         </is>
       </c>
       <c r="H233" s="23" t="inlineStr">
@@ -32583,6 +32583,53 @@
       <c r="I712" t="inlineStr">
         <is>
           <t>design system</t>
+        </is>
+      </c>
+    </row>
+    <row r="713">
+      <c r="A713" t="inlineStr">
+        <is>
+          <t>R2-1-B</t>
+        </is>
+      </c>
+      <c r="B713" t="inlineStr">
+        <is>
+          <t>The remaining direct GlobalPage writes (routes, crons, services) onto saveRecord / deleteRecord on the caller's scoped door — or justified in writing.</t>
+        </is>
+      </c>
+      <c r="C713" t="inlineStr">
+        <is>
+          <t>Platform</t>
+        </is>
+      </c>
+      <c r="D713" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E713" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F713" t="inlineStr">
+        <is>
+          <t>Planner 2026-10-05</t>
+        </is>
+      </c>
+      <c r="G713" t="inlineStr">
+        <is>
+          <t>Coder, plan first (coder-directive-r2-1-b.md). Input: R2-1-CENSUS.md, re-measured.</t>
+        </is>
+      </c>
+      <c r="H713" t="inlineStr">
+        <is>
+          <t>L0</t>
+        </is>
+      </c>
+      <c r="I713" t="inlineStr">
+        <is>
+          <t>write path — one door</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(map): BANK-REC-1, CONSTRUCT-1A/1B in the architecture record; today's decisions (VAT, discounts, TipTap) and Florin's open questions in the map
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/.agents/coral-roadmap.xlsx
+++ b/.agents/coral-roadmap.xlsx
@@ -594,7 +594,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I713"/>
+  <dimension ref="A1:I716"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -32630,6 +32630,147 @@
       <c r="I713" t="inlineStr">
         <is>
           <t>write path — one door</t>
+        </is>
+      </c>
+    </row>
+    <row r="714">
+      <c r="A714" t="inlineStr">
+        <is>
+          <t>BANK-REC-1</t>
+        </is>
+      </c>
+      <c r="B714" t="inlineStr">
+        <is>
+          <t>Bank reconciliation with expenses and income: import the tenant's bank movements (CODA, the Belgian bank format, or CAMT.053; later a PSD2 feed via a Belgian aggregator such as Ponto/Isabel) and match each movement to what it pays. Purchase invoices and receipts (expenses, tickets) → payments-out; sales invoices → payments-in. Match keys in order: the structured communication (OGM +++…+++), then IBAN + amount, then amount + date window + counterparty. Never books without review: proposal → confirm → payment record. Partial and over-payments, one movement for several invoices, and an unmatched queue. An invoice's paid / remaining amount follows from its payments; the accountant export stays consistent.</t>
+        </is>
+      </c>
+      <c r="C714" t="inlineStr">
+        <is>
+          <t>Finance · Bank reconciliation</t>
+        </is>
+      </c>
+      <c r="D714" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="E714" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F714" t="inlineStr">
+        <is>
+          <t>Florin 2026-10-09</t>
+        </is>
+      </c>
+      <c r="G714" t="inlineStr">
+        <is>
+          <t>Planned (ROADMAP.md § Planned modules). Placement: the matching rule pure in core (lib/records/bank-match); import and booking through lib/data doors on the scoped client; payments-in / payments-out are already kernel roles. OPEN (Florin): CODA upload first or a PSD2 feed; which banks.</t>
+        </is>
+      </c>
+      <c r="H714" t="inlineStr">
+        <is>
+          <t>L3</t>
+        </is>
+      </c>
+      <c r="I714" t="inlineStr">
+        <is>
+          <t>Finance — bank reconciliation</t>
+        </is>
+      </c>
+    </row>
+    <row r="715">
+      <c r="A715" t="inlineStr">
+        <is>
+          <t>CONSTRUCT-1A</t>
+        </is>
+      </c>
+      <c r="B715" t="inlineStr">
+        <is>
+          <t>The architect's meetstaat (bill of quantities) → a quote. In: .xlsx (most common), PDF, sometimes XML; posts carry the bestek numbering (Standaardbestek 250 / CCTB), description, unit, quantity, and VH (estimated, settled on measured quantity) or FH / forfait. Out: a quote in the ONE block model. Chapters → sections, posts → lines (newDocumentLine), the architect's post numbers kept, prices from the library / bestek. VH lines stay marked so the invoice settles them on measured quantities (vorderingsstaat).</t>
+        </is>
+      </c>
+      <c r="C715" t="inlineStr">
+        <is>
+          <t>Quotations · Construction</t>
+        </is>
+      </c>
+      <c r="D715" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="E715" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F715" t="inlineStr">
+        <is>
+          <t>Florin 2026-10-09</t>
+        </is>
+      </c>
+      <c r="G715" t="inlineStr">
+        <is>
+          <t>Planned (ROADMAP.md § CONSTRUCT-1a). ONE import door for spreadsheet, PDF/AI and meetstaat: today's SpreadsheetImportModal and PDF import fold into it, not copied. OPEN (Florin): which formats the architects send.</t>
+        </is>
+      </c>
+      <c r="H715" t="inlineStr">
+        <is>
+          <t>L3</t>
+        </is>
+      </c>
+      <c r="I715" t="inlineStr">
+        <is>
+          <t>Quotations — architect meetstaat import</t>
+        </is>
+      </c>
+    </row>
+    <row r="716">
+      <c r="A716" t="inlineStr">
+        <is>
+          <t>CONSTRUCT-1B</t>
+        </is>
+      </c>
+      <c r="B716" t="inlineStr">
+        <is>
+          <t>BIM handling: an IFC model (the open BIM standard) stored through the tenant's file door. First, viewed in the browser with an open-source IFC engine (web-ifc / That Open), no cloud service, so the tenant's model never leaves its storage. Then, a quantity takeoff from the IFC (areas, volumes, counts per element type) feeding the meetstaat / quote, with a link between a model element and its quote line.</t>
+        </is>
+      </c>
+      <c r="C716" t="inlineStr">
+        <is>
+          <t>Projects · Construction</t>
+        </is>
+      </c>
+      <c r="D716" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="E716" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F716" t="inlineStr">
+        <is>
+          <t>Florin 2026-10-09</t>
+        </is>
+      </c>
+      <c r="G716" t="inlineStr">
+        <is>
+          <t>Planned (ROADMAP.md § CONSTRUCT-1b). Feeds CONSTRUCT-1A's quote, not a second line model. OPEN (Florin): the IFC version; start with viewing only or the takeoff right away.</t>
+        </is>
+      </c>
+      <c r="H716" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="I716" t="inlineStr">
+        <is>
+          <t>Projects — BIM (IFC)</t>
         </is>
       </c>
     </row>
@@ -32650,7 +32791,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D24"/>
+  <dimension ref="A1:D26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -33182,6 +33323,50 @@
         </is>
       </c>
       <c r="D24" s="11" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>BANK-REC-Q</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>DECIDE: bank statements — start with CODA file upload, or a PSD2 bank feed (Ponto / Isabel)? Which banks do you use?</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>CONSTRUCT-Q</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>DECIDE: what do your architects send for the meetstaat (xlsx / PDF / XML)? For BIM: which IFC version, and start with viewing only or the quantity takeoff right away?</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
         <is>
           <t>P2</t>
         </is>

</xml_diff>